<commit_message>
Auto update stocks_data.xlsx [2026-09-14 09:17:27]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BR146"/>
+  <dimension ref="A1:BS146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="51"/>
@@ -604,6 +604,7 @@
     <col width="15" customWidth="1" min="68" max="68"/>
     <col width="15" customWidth="1" min="69" max="69"/>
     <col width="15" customWidth="1" min="70" max="70"/>
+    <col width="15" customWidth="1" min="71" max="71"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -957,6 +958,11 @@
           <t>2026/09/10</t>
         </is>
       </c>
+      <c r="BS1" s="15" t="inlineStr">
+        <is>
+          <t>2026/09/14</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1309,6 +1315,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="BS2" s="16" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1521,6 +1532,9 @@
       <c r="BR3" s="15" t="n">
         <v>60.57</v>
       </c>
+      <c r="BS3" s="15" t="n">
+        <v>58.64</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1732,6 +1746,9 @@
       </c>
       <c r="BR4" s="15" t="n">
         <v>3934.4</v>
+      </c>
+      <c r="BS4" s="15" t="n">
+        <v>3885.33</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1805,6 +1822,7 @@
       <c r="BP5" s="15" t="n"/>
       <c r="BQ5" s="15" t="n"/>
       <c r="BR5" s="15" t="n"/>
+      <c r="BS5" s="15" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1925,6 +1943,7 @@
       <c r="BP6" s="15" t="n"/>
       <c r="BQ6" s="15" t="n"/>
       <c r="BR6" s="15" t="n"/>
+      <c r="BS6" s="15" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -2136,6 +2155,9 @@
       </c>
       <c r="BR7" s="15" t="n">
         <v>54.29</v>
+      </c>
+      <c r="BS7" s="15" t="n">
+        <v>52.03</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -2300,6 +2322,9 @@
       </c>
       <c r="BR8" s="15" t="n">
         <v>5606.98</v>
+      </c>
+      <c r="BS8" s="15" t="n">
+        <v>5515.85</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
@@ -2421,6 +2446,7 @@
       <c r="BP9" s="15" t="n"/>
       <c r="BQ9" s="15" t="n"/>
       <c r="BR9" s="15" t="n"/>
+      <c r="BS9" s="15" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -2632,6 +2658,9 @@
       </c>
       <c r="BR10" s="15" t="n">
         <v>49.39</v>
+      </c>
+      <c r="BS10" s="15" t="n">
+        <v>47.58</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -2796,6 +2825,9 @@
       </c>
       <c r="BR11" s="15" t="n">
         <v>4548.39</v>
+      </c>
+      <c r="BS11" s="15" t="n">
+        <v>4480.08</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
@@ -2917,6 +2949,7 @@
       <c r="BP12" s="15" t="n"/>
       <c r="BQ12" s="15" t="n"/>
       <c r="BR12" s="15" t="n"/>
+      <c r="BS12" s="15" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -3128,6 +3161,9 @@
       </c>
       <c r="BR13" s="15" t="n">
         <v>60.09</v>
+      </c>
+      <c r="BS13" s="15" t="n">
+        <v>57.62</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -3292,6 +3328,9 @@
       </c>
       <c r="BR14" s="15" t="n">
         <v>7717.8</v>
+      </c>
+      <c r="BS14" s="15" t="n">
+        <v>7571.2</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
@@ -3413,6 +3452,7 @@
       <c r="BP15" s="15" t="n"/>
       <c r="BQ15" s="15" t="n"/>
       <c r="BR15" s="15" t="n"/>
+      <c r="BS15" s="15" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -3624,6 +3664,9 @@
       </c>
       <c r="BR16" s="15" t="n">
         <v>30.5</v>
+      </c>
+      <c r="BS16" s="15" t="n">
+        <v>28.7</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -3788,6 +3831,9 @@
       </c>
       <c r="BR17" s="15" t="n">
         <v>2538.76</v>
+      </c>
+      <c r="BS17" s="15" t="n">
+        <v>2515.17</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
@@ -3909,6 +3955,7 @@
       <c r="BP18" s="15" t="n"/>
       <c r="BQ18" s="15" t="n"/>
       <c r="BR18" s="15" t="n"/>
+      <c r="BS18" s="15" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -4120,6 +4167,9 @@
       </c>
       <c r="BR19" s="15" t="n">
         <v>80</v>
+      </c>
+      <c r="BS19" s="15" t="n">
+        <v>79.68000000000001</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -4284,6 +4334,9 @@
       </c>
       <c r="BR20" s="15" t="n">
         <v>7636.36</v>
+      </c>
+      <c r="BS20" s="15" t="n">
+        <v>7656.98</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
@@ -4405,6 +4458,7 @@
       <c r="BP21" s="15" t="n"/>
       <c r="BQ21" s="15" t="n"/>
       <c r="BR21" s="15" t="n"/>
+      <c r="BS21" s="15" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -4613,6 +4667,9 @@
         <v>36.34</v>
       </c>
       <c r="BR22" s="15" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="BS22" s="15" t="n">
         <v>36.34</v>
       </c>
     </row>
@@ -4778,6 +4835,9 @@
       </c>
       <c r="BR23" s="15" t="n">
         <v>74764.7</v>
+      </c>
+      <c r="BS23" s="15" t="n">
+        <v>74781.75999999999</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
@@ -4899,6 +4959,7 @@
       <c r="BP24" s="15" t="n"/>
       <c r="BQ24" s="15" t="n"/>
       <c r="BR24" s="15" t="n"/>
+      <c r="BS24" s="15" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -5109,6 +5170,9 @@
         <v>49.88</v>
       </c>
       <c r="BR25" s="15" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="BS25" s="15" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -5260,6 +5324,9 @@
       </c>
       <c r="BR26" s="15" t="n">
         <v>25550.9</v>
+      </c>
+      <c r="BS26" s="15" t="n">
+        <v>25396.13</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
@@ -5381,6 +5448,7 @@
       <c r="BP27" s="15" t="n"/>
       <c r="BQ27" s="15" t="n"/>
       <c r="BR27" s="15" t="n"/>
+      <c r="BS27" s="15" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -5591,6 +5659,9 @@
         <v>92.09</v>
       </c>
       <c r="BR28" s="15" t="n">
+        <v>92.09</v>
+      </c>
+      <c r="BS28" s="15" t="n">
         <v>92.09</v>
       </c>
     </row>
@@ -5756,6 +5827,9 @@
       </c>
       <c r="BR29" s="15" t="n">
         <v>65270.95</v>
+      </c>
+      <c r="BS29" s="15" t="n">
+        <v>63492.99</v>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
@@ -5877,6 +5951,7 @@
       <c r="BP30" s="15" t="n"/>
       <c r="BQ30" s="15" t="n"/>
       <c r="BR30" s="15" t="n"/>
+      <c r="BS30" s="15" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -6087,6 +6162,9 @@
         <v>97.44</v>
       </c>
       <c r="BR31" s="15" t="n">
+        <v>97.44</v>
+      </c>
+      <c r="BS31" s="15" t="n">
         <v>97.44</v>
       </c>
     </row>
@@ -6252,6 +6330,9 @@
       </c>
       <c r="BR32" s="15" t="n">
         <v>7033.92</v>
+      </c>
+      <c r="BS32" s="15" t="n">
+        <v>6684.37</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
@@ -6373,6 +6454,7 @@
       <c r="BP33" s="15" t="n"/>
       <c r="BQ33" s="15" t="n"/>
       <c r="BR33" s="15" t="n"/>
+      <c r="BS33" s="15" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -6584,6 +6666,9 @@
       </c>
       <c r="BR34" s="15" t="n">
         <v>45.3</v>
+      </c>
+      <c r="BS34" s="15" t="n">
+        <v>45.94</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -6748,6 +6833,9 @@
       </c>
       <c r="BR35" s="15" t="n">
         <v>5677.09</v>
+      </c>
+      <c r="BS35" s="15" t="n">
+        <v>5568.76</v>
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
@@ -6869,6 +6957,7 @@
       <c r="BP36" s="15" t="n"/>
       <c r="BQ36" s="15" t="n"/>
       <c r="BR36" s="15" t="n"/>
+      <c r="BS36" s="15" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -7080,6 +7169,9 @@
       </c>
       <c r="BR37" s="15" t="n">
         <v>51.76</v>
+      </c>
+      <c r="BS37" s="15" t="n">
+        <v>52.2</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -7244,6 +7336,9 @@
       </c>
       <c r="BR38" s="15" t="n">
         <v>11346.49</v>
+      </c>
+      <c r="BS38" s="15" t="n">
+        <v>11360.79</v>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
@@ -7365,6 +7460,7 @@
       <c r="BP39" s="15" t="n"/>
       <c r="BQ39" s="15" t="n"/>
       <c r="BR39" s="15" t="n"/>
+      <c r="BS39" s="15" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -7576,6 +7672,9 @@
       </c>
       <c r="BR40" s="15" t="n">
         <v>47.31</v>
+      </c>
+      <c r="BS40" s="15" t="n">
+        <v>48.18</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -7740,6 +7839,9 @@
       </c>
       <c r="BR41" s="15" t="n">
         <v>11161.29</v>
+      </c>
+      <c r="BS41" s="15" t="n">
+        <v>11082.15</v>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
@@ -7861,6 +7963,7 @@
       <c r="BP42" s="15" t="n"/>
       <c r="BQ42" s="15" t="n"/>
       <c r="BR42" s="15" t="n"/>
+      <c r="BS42" s="15" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -8072,6 +8175,9 @@
       </c>
       <c r="BR43" s="15" t="n">
         <v>48.92</v>
+      </c>
+      <c r="BS43" s="15" t="n">
+        <v>48.47</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -8236,6 +8342,9 @@
       </c>
       <c r="BR44" s="15" t="n">
         <v>3407.41</v>
+      </c>
+      <c r="BS44" s="15" t="n">
+        <v>3328.34</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
@@ -8357,6 +8466,7 @@
       <c r="BP45" s="15" t="n"/>
       <c r="BQ45" s="15" t="n"/>
       <c r="BR45" s="15" t="n"/>
+      <c r="BS45" s="15" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -8568,6 +8678,9 @@
       </c>
       <c r="BR46" s="15" t="n">
         <v>48.28</v>
+      </c>
+      <c r="BS46" s="15" t="n">
+        <v>51.02</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -8732,6 +8845,9 @@
       </c>
       <c r="BR47" s="15" t="n">
         <v>7038.44</v>
+      </c>
+      <c r="BS47" s="15" t="n">
+        <v>7042.77</v>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
@@ -8853,6 +8969,7 @@
       <c r="BP48" s="15" t="n"/>
       <c r="BQ48" s="15" t="n"/>
       <c r="BR48" s="15" t="n"/>
+      <c r="BS48" s="15" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -9064,6 +9181,9 @@
       </c>
       <c r="BR49" s="15" t="n">
         <v>23.4</v>
+      </c>
+      <c r="BS49" s="15" t="n">
+        <v>22.49</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -9228,6 +9348,9 @@
       </c>
       <c r="BR50" s="15" t="n">
         <v>33145.69</v>
+      </c>
+      <c r="BS50" s="15" t="n">
+        <v>32651.38</v>
       </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
@@ -9349,6 +9472,7 @@
       <c r="BP51" s="15" t="n"/>
       <c r="BQ51" s="15" t="n"/>
       <c r="BR51" s="15" t="n"/>
+      <c r="BS51" s="15" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -9560,6 +9684,9 @@
       </c>
       <c r="BR52" s="15" t="n">
         <v>38.38</v>
+      </c>
+      <c r="BS52" s="15" t="n">
+        <v>37.16</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -9724,6 +9851,9 @@
       </c>
       <c r="BR53" s="15" t="n">
         <v>3495.93</v>
+      </c>
+      <c r="BS53" s="15" t="n">
+        <v>3426.56</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
@@ -9845,6 +9975,7 @@
       <c r="BP54" s="15" t="n"/>
       <c r="BQ54" s="15" t="n"/>
       <c r="BR54" s="15" t="n"/>
+      <c r="BS54" s="15" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -10056,6 +10187,9 @@
       </c>
       <c r="BR55" s="15" t="n">
         <v>45.15</v>
+      </c>
+      <c r="BS55" s="15" t="n">
+        <v>43.56</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -10220,6 +10354,9 @@
       </c>
       <c r="BR56" s="15" t="n">
         <v>3338.42</v>
+      </c>
+      <c r="BS56" s="15" t="n">
+        <v>3285.58</v>
       </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
@@ -10341,6 +10478,7 @@
       <c r="BP57" s="15" t="n"/>
       <c r="BQ57" s="15" t="n"/>
       <c r="BR57" s="15" t="n"/>
+      <c r="BS57" s="15" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -10552,6 +10690,9 @@
       </c>
       <c r="BR58" s="15" t="n">
         <v>13.95</v>
+      </c>
+      <c r="BS58" s="15" t="n">
+        <v>10.53</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -10716,6 +10857,9 @@
       </c>
       <c r="BR59" s="15" t="n">
         <v>6582.88</v>
+      </c>
+      <c r="BS59" s="15" t="n">
+        <v>6598.37</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
@@ -10837,6 +10981,7 @@
       <c r="BP60" s="15" t="n"/>
       <c r="BQ60" s="15" t="n"/>
       <c r="BR60" s="15" t="n"/>
+      <c r="BS60" s="15" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -11048,6 +11193,9 @@
       </c>
       <c r="BR61" s="15" t="n">
         <v>31.41</v>
+      </c>
+      <c r="BS61" s="15" t="n">
+        <v>27.81</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -11212,6 +11360,9 @@
       </c>
       <c r="BR62" s="15" t="n">
         <v>7931.58</v>
+      </c>
+      <c r="BS62" s="15" t="n">
+        <v>7994.51</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
@@ -11333,6 +11484,7 @@
       <c r="BP63" s="15" t="n"/>
       <c r="BQ63" s="15" t="n"/>
       <c r="BR63" s="15" t="n"/>
+      <c r="BS63" s="15" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -11544,6 +11696,9 @@
       </c>
       <c r="BR64" s="15" t="n">
         <v>9.74</v>
+      </c>
+      <c r="BS64" s="15" t="n">
+        <v>8.380000000000001</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -11707,6 +11862,9 @@
         <v>10949.77</v>
       </c>
       <c r="BR65" s="15" t="n">
+        <v>10652.53</v>
+      </c>
+      <c r="BS65" s="15" t="n">
         <v>10652.53</v>
       </c>
     </row>
@@ -11829,6 +11987,7 @@
       <c r="BP66" s="15" t="n"/>
       <c r="BQ66" s="15" t="n"/>
       <c r="BR66" s="15" t="n"/>
+      <c r="BS66" s="15" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -12040,6 +12199,9 @@
       </c>
       <c r="BR67" s="15" t="n">
         <v>24.24</v>
+      </c>
+      <c r="BS67" s="15" t="n">
+        <v>22.02</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -12204,6 +12366,9 @@
       </c>
       <c r="BR68" s="15" t="n">
         <v>11392.59</v>
+      </c>
+      <c r="BS68" s="15" t="n">
+        <v>11215.06</v>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
@@ -12325,6 +12490,7 @@
       <c r="BP69" s="15" t="n"/>
       <c r="BQ69" s="15" t="n"/>
       <c r="BR69" s="15" t="n"/>
+      <c r="BS69" s="15" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -12536,6 +12702,9 @@
       </c>
       <c r="BR70" s="15" t="n">
         <v>18.46</v>
+      </c>
+      <c r="BS70" s="15" t="n">
+        <v>16.01</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -12700,6 +12869,9 @@
       </c>
       <c r="BR71" s="15" t="n">
         <v>6361.07</v>
+      </c>
+      <c r="BS71" s="15" t="n">
+        <v>6247.83</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
@@ -12821,6 +12993,7 @@
       <c r="BP72" s="15" t="n"/>
       <c r="BQ72" s="15" t="n"/>
       <c r="BR72" s="15" t="n"/>
+      <c r="BS72" s="15" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -13032,6 +13205,9 @@
       </c>
       <c r="BR73" s="15" t="n">
         <v>20.41</v>
+      </c>
+      <c r="BS73" s="15" t="n">
+        <v>18.12</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -13196,6 +13372,9 @@
       </c>
       <c r="BR74" s="15" t="n">
         <v>12475.28</v>
+      </c>
+      <c r="BS74" s="15" t="n">
+        <v>12324.03</v>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
@@ -13317,6 +13496,7 @@
       <c r="BP75" s="15" t="n"/>
       <c r="BQ75" s="15" t="n"/>
       <c r="BR75" s="15" t="n"/>
+      <c r="BS75" s="15" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -13528,6 +13708,9 @@
       </c>
       <c r="BR76" s="15" t="n">
         <v>52.81</v>
+      </c>
+      <c r="BS76" s="15" t="n">
+        <v>51.65</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -13692,6 +13875,9 @@
       </c>
       <c r="BR77" s="15" t="n">
         <v>15061.96</v>
+      </c>
+      <c r="BS77" s="15" t="n">
+        <v>15569.82</v>
       </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
@@ -13813,6 +13999,7 @@
       <c r="BP78" s="15" t="n"/>
       <c r="BQ78" s="15" t="n"/>
       <c r="BR78" s="15" t="n"/>
+      <c r="BS78" s="15" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -14024,6 +14211,9 @@
       </c>
       <c r="BR79" s="15" t="n">
         <v>2.48</v>
+      </c>
+      <c r="BS79" s="15" t="n">
+        <v>1.83</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -14188,6 +14378,9 @@
       </c>
       <c r="BR80" s="15" t="n">
         <v>6478.77</v>
+      </c>
+      <c r="BS80" s="15" t="n">
+        <v>6497.23</v>
       </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
@@ -14309,6 +14502,7 @@
       <c r="BP81" s="15" t="n"/>
       <c r="BQ81" s="15" t="n"/>
       <c r="BR81" s="15" t="n"/>
+      <c r="BS81" s="15" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -14520,6 +14714,9 @@
       </c>
       <c r="BR82" s="15" t="n">
         <v>4.34</v>
+      </c>
+      <c r="BS82" s="15" t="n">
+        <v>3.04</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -14684,6 +14881,9 @@
       </c>
       <c r="BR83" s="15" t="n">
         <v>8473</v>
+      </c>
+      <c r="BS83" s="15" t="n">
+        <v>8501.110000000001</v>
       </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
@@ -14805,6 +15005,7 @@
       <c r="BP84" s="15" t="n"/>
       <c r="BQ84" s="15" t="n"/>
       <c r="BR84" s="15" t="n"/>
+      <c r="BS84" s="15" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -15016,6 +15217,9 @@
       </c>
       <c r="BR85" s="15" t="n">
         <v>18.04</v>
+      </c>
+      <c r="BS85" s="15" t="n">
+        <v>17.04</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -15179,6 +15383,9 @@
         <v>2171.98</v>
       </c>
       <c r="BR86" s="15" t="n">
+        <v>2631.9</v>
+      </c>
+      <c r="BS86" s="15" t="n">
         <v>2631.9</v>
       </c>
     </row>
@@ -15301,6 +15508,7 @@
       <c r="BP87" s="15" t="n"/>
       <c r="BQ87" s="15" t="n"/>
       <c r="BR87" s="15" t="n"/>
+      <c r="BS87" s="15" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -15512,6 +15720,9 @@
       </c>
       <c r="BR88" s="15" t="n">
         <v>27.46</v>
+      </c>
+      <c r="BS88" s="15" t="n">
+        <v>25.09</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -15676,6 +15887,9 @@
       </c>
       <c r="BR89" s="15" t="n">
         <v>4333.4</v>
+      </c>
+      <c r="BS89" s="15" t="n">
+        <v>5075.31</v>
       </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
@@ -15797,6 +16011,7 @@
       <c r="BP90" s="15" t="n"/>
       <c r="BQ90" s="15" t="n"/>
       <c r="BR90" s="15" t="n"/>
+      <c r="BS90" s="15" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -16008,6 +16223,9 @@
       </c>
       <c r="BR91" s="15" t="n">
         <v>14.77</v>
+      </c>
+      <c r="BS91" s="15" t="n">
+        <v>10.73</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -16172,6 +16390,9 @@
       </c>
       <c r="BR92" s="15" t="n">
         <v>8312.059999999999</v>
+      </c>
+      <c r="BS92" s="15" t="n">
+        <v>8346.67</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
@@ -16293,6 +16514,7 @@
       <c r="BP93" s="15" t="n"/>
       <c r="BQ93" s="15" t="n"/>
       <c r="BR93" s="15" t="n"/>
+      <c r="BS93" s="15" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -16504,6 +16726,9 @@
       </c>
       <c r="BR94" s="15" t="n">
         <v>6.53</v>
+      </c>
+      <c r="BS94" s="15" t="n">
+        <v>5.07</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -16668,6 +16893,9 @@
       </c>
       <c r="BR95" s="15" t="n">
         <v>1239.83</v>
+      </c>
+      <c r="BS95" s="15" t="n">
+        <v>1212.55</v>
       </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
@@ -16789,6 +17017,7 @@
       <c r="BP96" s="15" t="n"/>
       <c r="BQ96" s="15" t="n"/>
       <c r="BR96" s="15" t="n"/>
+      <c r="BS96" s="15" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -17000,6 +17229,9 @@
       </c>
       <c r="BR97" s="15" t="n">
         <v>10.36</v>
+      </c>
+      <c r="BS97" s="15" t="n">
+        <v>8.390000000000001</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -17164,6 +17396,9 @@
       </c>
       <c r="BR98" s="15" t="n">
         <v>13914.44</v>
+      </c>
+      <c r="BS98" s="15" t="n">
+        <v>13616.29</v>
       </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
@@ -17285,6 +17520,7 @@
       <c r="BP99" s="15" t="n"/>
       <c r="BQ99" s="15" t="n"/>
       <c r="BR99" s="15" t="n"/>
+      <c r="BS99" s="15" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -17496,6 +17732,9 @@
       </c>
       <c r="BR100" s="15" t="n">
         <v>31.82</v>
+      </c>
+      <c r="BS100" s="15" t="n">
+        <v>27.7</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -17660,6 +17899,9 @@
       </c>
       <c r="BR101" s="15" t="n">
         <v>3203.69</v>
+      </c>
+      <c r="BS101" s="15" t="n">
+        <v>3093.74</v>
       </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
@@ -17781,6 +18023,7 @@
       <c r="BP102" s="15" t="n"/>
       <c r="BQ102" s="15" t="n"/>
       <c r="BR102" s="15" t="n"/>
+      <c r="BS102" s="15" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -17992,6 +18235,9 @@
       </c>
       <c r="BR103" s="15" t="n">
         <v>29.75</v>
+      </c>
+      <c r="BS103" s="15" t="n">
+        <v>28.31</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -18156,6 +18402,9 @@
       </c>
       <c r="BR104" s="15" t="n">
         <v>2281.11</v>
+      </c>
+      <c r="BS104" s="15" t="n">
+        <v>2257.6</v>
       </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
@@ -18277,6 +18526,7 @@
       <c r="BP105" s="15" t="n"/>
       <c r="BQ105" s="15" t="n"/>
       <c r="BR105" s="15" t="n"/>
+      <c r="BS105" s="15" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -18488,6 +18738,9 @@
       </c>
       <c r="BR106" s="15" t="n">
         <v>14.18</v>
+      </c>
+      <c r="BS106" s="15" t="n">
+        <v>11.74</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -18651,6 +18904,9 @@
         <v>2412.23</v>
       </c>
       <c r="BR107" s="15" t="n">
+        <v>2413.21</v>
+      </c>
+      <c r="BS107" s="15" t="n">
         <v>2413.21</v>
       </c>
     </row>
@@ -18773,6 +19029,7 @@
       <c r="BP108" s="15" t="n"/>
       <c r="BQ108" s="15" t="n"/>
       <c r="BR108" s="15" t="n"/>
+      <c r="BS108" s="15" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -18984,6 +19241,9 @@
       </c>
       <c r="BR109" s="15" t="n">
         <v>30.04</v>
+      </c>
+      <c r="BS109" s="15" t="n">
+        <v>28.33</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -19148,6 +19408,9 @@
       </c>
       <c r="BR110" s="15" t="n">
         <v>2419.39</v>
+      </c>
+      <c r="BS110" s="15" t="n">
+        <v>2397.17</v>
       </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
@@ -19269,6 +19532,7 @@
       <c r="BP111" s="15" t="n"/>
       <c r="BQ111" s="15" t="n"/>
       <c r="BR111" s="15" t="n"/>
+      <c r="BS111" s="15" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -19480,6 +19744,9 @@
       </c>
       <c r="BR112" s="15" t="n">
         <v>45.48</v>
+      </c>
+      <c r="BS112" s="15" t="n">
+        <v>38.92</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -19642,6 +19909,9 @@
       </c>
       <c r="BR113" s="15" t="n">
         <v>1883.01</v>
+      </c>
+      <c r="BS113" s="15" t="n">
+        <v>1869.95</v>
       </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
@@ -19763,6 +20033,7 @@
       <c r="BP114" s="15" t="n"/>
       <c r="BQ114" s="15" t="n"/>
       <c r="BR114" s="15" t="n"/>
+      <c r="BS114" s="15" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -19974,6 +20245,9 @@
       </c>
       <c r="BR115" s="15" t="n">
         <v>16.45</v>
+      </c>
+      <c r="BS115" s="15" t="n">
+        <v>14.47</v>
       </c>
     </row>
     <row r="116" ht="14.25" customHeight="1">
@@ -20123,6 +20397,9 @@
       </c>
       <c r="BR116" s="15" t="n">
         <v>8587.74</v>
+      </c>
+      <c r="BS116" s="15" t="n">
+        <v>8794.76</v>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1">
@@ -20199,6 +20476,7 @@
       <c r="BP117" s="15" t="n"/>
       <c r="BQ117" s="15" t="n"/>
       <c r="BR117" s="15" t="n"/>
+      <c r="BS117" s="15" t="n"/>
     </row>
     <row r="118" ht="14.25" customHeight="1">
       <c r="P118" s="13" t="n">
@@ -20366,6 +20644,9 @@
       <c r="BR118" s="15" t="n">
         <v>72.06999999999999</v>
       </c>
+      <c r="BS118" s="15" t="n">
+        <v>70.45999999999999</v>
+      </c>
     </row>
     <row r="119" ht="14.25" customHeight="1">
       <c r="Y119" s="13" t="n">
@@ -20505,6 +20786,9 @@
       </c>
       <c r="BR119" s="15" t="n">
         <v>12348.16</v>
+      </c>
+      <c r="BS119" s="15" t="n">
+        <v>11938.17</v>
       </c>
     </row>
     <row r="120" ht="14.25" customHeight="1">
@@ -20530,6 +20814,7 @@
       <c r="BP120" s="15" t="n"/>
       <c r="BQ120" s="15" t="n"/>
       <c r="BR120" s="15" t="n"/>
+      <c r="BS120" s="15" t="n"/>
     </row>
     <row r="121" ht="14.25" customHeight="1">
       <c r="AW121" s="13" t="n">
@@ -20598,6 +20883,9 @@
       <c r="BR121" s="15" t="n">
         <v>27.45</v>
       </c>
+      <c r="BS121" s="15" t="n">
+        <v>24.98</v>
+      </c>
     </row>
     <row r="122" ht="14.25" customHeight="1">
       <c r="AW122" s="13" t="n">
@@ -20665,6 +20953,9 @@
       </c>
       <c r="BR122" s="15" t="n">
         <v>1242.48</v>
+      </c>
+      <c r="BS122" s="15" t="n">
+        <v>1212.12</v>
       </c>
     </row>
     <row r="123" ht="14.25" customHeight="1">
@@ -20690,6 +20981,7 @@
       <c r="BP123" s="15" t="n"/>
       <c r="BQ123" s="15" t="n"/>
       <c r="BR123" s="15" t="n"/>
+      <c r="BS123" s="15" t="n"/>
     </row>
     <row r="124" ht="14.25" customHeight="1">
       <c r="AW124" s="13" t="n">
@@ -20758,6 +21050,9 @@
       <c r="BR124" s="15" t="n">
         <v>52.69</v>
       </c>
+      <c r="BS124" s="15" t="n">
+        <v>50.63</v>
+      </c>
     </row>
     <row r="125" ht="14.25" customHeight="1">
       <c r="AW125" s="13" t="n">
@@ -20825,6 +21120,9 @@
       </c>
       <c r="BR125" s="15" t="n">
         <v>11914.41</v>
+      </c>
+      <c r="BS125" s="15" t="n">
+        <v>11643.01</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1">
@@ -20850,6 +21148,7 @@
       <c r="BP126" s="15" t="n"/>
       <c r="BQ126" s="15" t="n"/>
       <c r="BR126" s="15" t="n"/>
+      <c r="BS126" s="15" t="n"/>
     </row>
     <row r="127" ht="14.25" customHeight="1">
       <c r="AW127" s="13" t="n">
@@ -20918,6 +21217,9 @@
       <c r="BR127" s="15" t="n">
         <v>8.48</v>
       </c>
+      <c r="BS127" s="15" t="n">
+        <v>5.63</v>
+      </c>
     </row>
     <row r="128" ht="14.25" customHeight="1">
       <c r="AW128" s="13" t="n">
@@ -20985,6 +21287,9 @@
       </c>
       <c r="BR128" s="15" t="n">
         <v>1943.68</v>
+      </c>
+      <c r="BS128" s="15" t="n">
+        <v>1894.86</v>
       </c>
     </row>
     <row r="129" ht="14.25" customHeight="1">
@@ -21010,6 +21315,7 @@
       <c r="BP129" s="15" t="n"/>
       <c r="BQ129" s="15" t="n"/>
       <c r="BR129" s="15" t="n"/>
+      <c r="BS129" s="15" t="n"/>
     </row>
     <row r="130" ht="14.25" customHeight="1">
       <c r="AW130" s="13" t="n">
@@ -21078,6 +21384,9 @@
       <c r="BR130" s="15" t="n">
         <v>10.29</v>
       </c>
+      <c r="BS130" s="15" t="n">
+        <v>7.77</v>
+      </c>
     </row>
     <row r="131" ht="14.25" customHeight="1">
       <c r="AW131" s="13" t="n">
@@ -21145,6 +21454,9 @@
       </c>
       <c r="BR131" s="15" t="n">
         <v>759.02</v>
+      </c>
+      <c r="BS131" s="15" t="n">
+        <v>732.6</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1">
@@ -21170,6 +21482,7 @@
       <c r="BP132" s="15" t="n"/>
       <c r="BQ132" s="15" t="n"/>
       <c r="BR132" s="15" t="n"/>
+      <c r="BS132" s="15" t="n"/>
     </row>
     <row r="133" ht="14.25" customHeight="1">
       <c r="AW133" s="13" t="n">
@@ -21238,6 +21551,9 @@
       <c r="BR133" s="15" t="n">
         <v>65.87</v>
       </c>
+      <c r="BS133" s="15" t="n">
+        <v>58.68</v>
+      </c>
     </row>
     <row r="134" ht="14.25" customHeight="1">
       <c r="AW134" s="13" t="n">
@@ -21305,6 +21621,9 @@
       </c>
       <c r="BR134" s="15" t="n">
         <v>3015.83</v>
+      </c>
+      <c r="BS134" s="15" t="n">
+        <v>3050.14</v>
       </c>
     </row>
     <row r="135" ht="14.25" customHeight="1">
@@ -21330,6 +21649,7 @@
       <c r="BP135" s="15" t="n"/>
       <c r="BQ135" s="15" t="n"/>
       <c r="BR135" s="15" t="n"/>
+      <c r="BS135" s="15" t="n"/>
     </row>
     <row r="136" ht="14.25" customHeight="1">
       <c r="AW136" s="13" t="n">
@@ -21398,6 +21718,9 @@
       <c r="BR136" s="15" t="n">
         <v>22.65</v>
       </c>
+      <c r="BS136" s="15" t="n">
+        <v>21.83</v>
+      </c>
     </row>
     <row r="137" ht="14.25" customHeight="1">
       <c r="AW137" s="13" t="n">
@@ -21465,6 +21788,9 @@
       </c>
       <c r="BR137" s="15" t="n">
         <v>3616.98</v>
+      </c>
+      <c r="BS137" s="15" t="n">
+        <v>3522.7</v>
       </c>
     </row>
     <row r="138">
@@ -21482,6 +21808,7 @@
       <c r="BP138" s="15" t="n"/>
       <c r="BQ138" s="15" t="n"/>
       <c r="BR138" s="15" t="n"/>
+      <c r="BS138" s="15" t="n"/>
     </row>
     <row r="139">
       <c r="BE139" s="15" t="n">
@@ -21526,6 +21853,9 @@
       <c r="BR139" s="15" t="n">
         <v>4.25</v>
       </c>
+      <c r="BS139" s="15" t="n">
+        <v>3.27</v>
+      </c>
     </row>
     <row r="140">
       <c r="BE140" s="15" t="n">
@@ -21568,6 +21898,9 @@
         <v>2412.96</v>
       </c>
       <c r="BR140" s="15" t="n">
+        <v>2431.48</v>
+      </c>
+      <c r="BS140" s="15" t="n">
         <v>2431.48</v>
       </c>
     </row>
@@ -21586,6 +21919,7 @@
       <c r="BP141" s="15" t="n"/>
       <c r="BQ141" s="15" t="n"/>
       <c r="BR141" s="15" t="n"/>
+      <c r="BS141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="BE142" s="15" t="n">
@@ -21630,6 +21964,9 @@
       <c r="BR142" s="15" t="n">
         <v>23.64</v>
       </c>
+      <c r="BS142" s="15" t="n">
+        <v>22.98</v>
+      </c>
     </row>
     <row r="143">
       <c r="BE143" s="15" t="n">
@@ -21673,6 +22010,9 @@
       </c>
       <c r="BR143" s="15" t="n">
         <v>5803.28</v>
+      </c>
+      <c r="BS143" s="15" t="n">
+        <v>5852.64</v>
       </c>
     </row>
     <row r="144">
@@ -21685,6 +22025,7 @@
       <c r="BP144" s="15" t="n"/>
       <c r="BQ144" s="15" t="n"/>
       <c r="BR144" s="15" t="n"/>
+      <c r="BS144" s="15" t="n"/>
     </row>
     <row r="145">
       <c r="BJ145" s="15" t="n">
@@ -21714,6 +22055,9 @@
       <c r="BR145" s="15" t="n">
         <v>3.22</v>
       </c>
+      <c r="BS145" s="15" t="n">
+        <v>2.09</v>
+      </c>
     </row>
     <row r="146">
       <c r="BJ146" s="15" t="n">
@@ -21742,6 +22086,9 @@
       </c>
       <c r="BR146" s="15" t="n">
         <v>2354.67</v>
+      </c>
+      <c r="BS146" s="15" t="n">
+        <v>2277.18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-09-17 08:57:44]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BS146"/>
+  <dimension ref="A1:BT146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="51"/>
@@ -605,6 +605,7 @@
     <col width="15" customWidth="1" min="69" max="69"/>
     <col width="15" customWidth="1" min="70" max="70"/>
     <col width="15" customWidth="1" min="71" max="71"/>
+    <col width="15" customWidth="1" min="72" max="72"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -963,6 +964,11 @@
           <t>2026/09/14</t>
         </is>
       </c>
+      <c r="BT1" s="15" t="inlineStr">
+        <is>
+          <t>2026/09/17</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1320,6 +1326,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="BT2" s="16" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1535,6 +1546,9 @@
       <c r="BS3" s="15" t="n">
         <v>58.64</v>
       </c>
+      <c r="BT3" s="15" t="n">
+        <v>58.56</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1749,6 +1763,9 @@
       </c>
       <c r="BS4" s="15" t="n">
         <v>3885.33</v>
+      </c>
+      <c r="BT4" s="15" t="n">
+        <v>3875.6</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1823,6 +1840,7 @@
       <c r="BQ5" s="15" t="n"/>
       <c r="BR5" s="15" t="n"/>
       <c r="BS5" s="15" t="n"/>
+      <c r="BT5" s="15" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1944,6 +1962,7 @@
       <c r="BQ6" s="15" t="n"/>
       <c r="BR6" s="15" t="n"/>
       <c r="BS6" s="15" t="n"/>
+      <c r="BT6" s="15" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -2158,6 +2177,9 @@
       </c>
       <c r="BS7" s="15" t="n">
         <v>52.03</v>
+      </c>
+      <c r="BT7" s="15" t="n">
+        <v>51.56</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -2325,6 +2347,9 @@
       </c>
       <c r="BS8" s="15" t="n">
         <v>5515.85</v>
+      </c>
+      <c r="BT8" s="15" t="n">
+        <v>5515.99</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
@@ -2447,6 +2472,7 @@
       <c r="BQ9" s="15" t="n"/>
       <c r="BR9" s="15" t="n"/>
       <c r="BS9" s="15" t="n"/>
+      <c r="BT9" s="15" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -2661,6 +2687,9 @@
       </c>
       <c r="BS10" s="15" t="n">
         <v>47.58</v>
+      </c>
+      <c r="BT10" s="15" t="n">
+        <v>45.56</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -2828,6 +2857,9 @@
       </c>
       <c r="BS11" s="15" t="n">
         <v>4480.08</v>
+      </c>
+      <c r="BT11" s="15" t="n">
+        <v>4460.16</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
@@ -2950,6 +2982,7 @@
       <c r="BQ12" s="15" t="n"/>
       <c r="BR12" s="15" t="n"/>
       <c r="BS12" s="15" t="n"/>
+      <c r="BT12" s="15" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -3164,6 +3197,9 @@
       </c>
       <c r="BS13" s="15" t="n">
         <v>57.62</v>
+      </c>
+      <c r="BT13" s="15" t="n">
+        <v>59.23</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -3331,6 +3367,9 @@
       </c>
       <c r="BS14" s="15" t="n">
         <v>7571.2</v>
+      </c>
+      <c r="BT14" s="15" t="n">
+        <v>7654.98</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
@@ -3453,6 +3492,7 @@
       <c r="BQ15" s="15" t="n"/>
       <c r="BR15" s="15" t="n"/>
       <c r="BS15" s="15" t="n"/>
+      <c r="BT15" s="15" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -3667,6 +3707,9 @@
       </c>
       <c r="BS16" s="15" t="n">
         <v>28.7</v>
+      </c>
+      <c r="BT16" s="15" t="n">
+        <v>28.08</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -3834,6 +3877,9 @@
       </c>
       <c r="BS17" s="15" t="n">
         <v>2515.17</v>
+      </c>
+      <c r="BT17" s="15" t="n">
+        <v>2491.04</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
@@ -3956,6 +4002,7 @@
       <c r="BQ18" s="15" t="n"/>
       <c r="BR18" s="15" t="n"/>
       <c r="BS18" s="15" t="n"/>
+      <c r="BT18" s="15" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -4170,6 +4217,9 @@
       </c>
       <c r="BS19" s="15" t="n">
         <v>79.68000000000001</v>
+      </c>
+      <c r="BT19" s="15" t="n">
+        <v>79.83</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -4337,6 +4387,9 @@
       </c>
       <c r="BS20" s="15" t="n">
         <v>7656.98</v>
+      </c>
+      <c r="BT20" s="15" t="n">
+        <v>7551.81</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
@@ -4459,6 +4512,7 @@
       <c r="BQ21" s="15" t="n"/>
       <c r="BR21" s="15" t="n"/>
       <c r="BS21" s="15" t="n"/>
+      <c r="BT21" s="15" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -4670,6 +4724,9 @@
         <v>36.34</v>
       </c>
       <c r="BS22" s="15" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="BT22" s="15" t="n">
         <v>36.34</v>
       </c>
     </row>
@@ -4838,6 +4895,9 @@
       </c>
       <c r="BS23" s="15" t="n">
         <v>74781.75999999999</v>
+      </c>
+      <c r="BT23" s="15" t="n">
+        <v>74383.59</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
@@ -4960,6 +5020,7 @@
       <c r="BQ24" s="15" t="n"/>
       <c r="BR24" s="15" t="n"/>
       <c r="BS24" s="15" t="n"/>
+      <c r="BT24" s="15" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -5173,6 +5234,9 @@
         <v>49.88</v>
       </c>
       <c r="BS25" s="15" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="BT25" s="15" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -5327,6 +5391,9 @@
       </c>
       <c r="BS26" s="15" t="n">
         <v>25396.13</v>
+      </c>
+      <c r="BT26" s="15" t="n">
+        <v>25673.14</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
@@ -5449,6 +5516,7 @@
       <c r="BQ27" s="15" t="n"/>
       <c r="BR27" s="15" t="n"/>
       <c r="BS27" s="15" t="n"/>
+      <c r="BT27" s="15" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -5662,6 +5730,9 @@
         <v>92.09</v>
       </c>
       <c r="BS28" s="15" t="n">
+        <v>92.09</v>
+      </c>
+      <c r="BT28" s="15" t="n">
         <v>92.09</v>
       </c>
     </row>
@@ -5830,6 +5901,9 @@
       </c>
       <c r="BS29" s="15" t="n">
         <v>63492.99</v>
+      </c>
+      <c r="BT29" s="15" t="n">
+        <v>64136.25</v>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
@@ -5952,6 +6026,7 @@
       <c r="BQ30" s="15" t="n"/>
       <c r="BR30" s="15" t="n"/>
       <c r="BS30" s="15" t="n"/>
+      <c r="BT30" s="15" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -6165,6 +6240,9 @@
         <v>97.44</v>
       </c>
       <c r="BS31" s="15" t="n">
+        <v>97.44</v>
+      </c>
+      <c r="BT31" s="15" t="n">
         <v>97.44</v>
       </c>
     </row>
@@ -6333,6 +6411,9 @@
       </c>
       <c r="BS32" s="15" t="n">
         <v>6684.37</v>
+      </c>
+      <c r="BT32" s="15" t="n">
+        <v>6715.41</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
@@ -6455,6 +6536,7 @@
       <c r="BQ33" s="15" t="n"/>
       <c r="BR33" s="15" t="n"/>
       <c r="BS33" s="15" t="n"/>
+      <c r="BT33" s="15" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -6669,6 +6751,9 @@
       </c>
       <c r="BS34" s="15" t="n">
         <v>45.94</v>
+      </c>
+      <c r="BT34" s="15" t="n">
+        <v>48.41</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -6836,6 +6921,9 @@
       </c>
       <c r="BS35" s="15" t="n">
         <v>5568.76</v>
+      </c>
+      <c r="BT35" s="15" t="n">
+        <v>5473.85</v>
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
@@ -6958,6 +7046,7 @@
       <c r="BQ36" s="15" t="n"/>
       <c r="BR36" s="15" t="n"/>
       <c r="BS36" s="15" t="n"/>
+      <c r="BT36" s="15" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -7172,6 +7261,9 @@
       </c>
       <c r="BS37" s="15" t="n">
         <v>52.2</v>
+      </c>
+      <c r="BT37" s="15" t="n">
+        <v>49.73</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -7339,6 +7431,9 @@
       </c>
       <c r="BS38" s="15" t="n">
         <v>11360.79</v>
+      </c>
+      <c r="BT38" s="15" t="n">
+        <v>11175.12</v>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
@@ -7461,6 +7556,7 @@
       <c r="BQ39" s="15" t="n"/>
       <c r="BR39" s="15" t="n"/>
       <c r="BS39" s="15" t="n"/>
+      <c r="BT39" s="15" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -7675,6 +7771,9 @@
       </c>
       <c r="BS40" s="15" t="n">
         <v>48.18</v>
+      </c>
+      <c r="BT40" s="15" t="n">
+        <v>51.11</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -7842,6 +7941,9 @@
       </c>
       <c r="BS41" s="15" t="n">
         <v>11082.15</v>
+      </c>
+      <c r="BT41" s="15" t="n">
+        <v>10931.94</v>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
@@ -7964,6 +8066,7 @@
       <c r="BQ42" s="15" t="n"/>
       <c r="BR42" s="15" t="n"/>
       <c r="BS42" s="15" t="n"/>
+      <c r="BT42" s="15" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -8178,6 +8281,9 @@
       </c>
       <c r="BS43" s="15" t="n">
         <v>48.47</v>
+      </c>
+      <c r="BT43" s="15" t="n">
+        <v>52.01</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -8345,6 +8451,9 @@
       </c>
       <c r="BS44" s="15" t="n">
         <v>3328.34</v>
+      </c>
+      <c r="BT44" s="15" t="n">
+        <v>3277.88</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
@@ -8467,6 +8576,7 @@
       <c r="BQ45" s="15" t="n"/>
       <c r="BR45" s="15" t="n"/>
       <c r="BS45" s="15" t="n"/>
+      <c r="BT45" s="15" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -8681,6 +8791,9 @@
       </c>
       <c r="BS46" s="15" t="n">
         <v>51.02</v>
+      </c>
+      <c r="BT46" s="15" t="n">
+        <v>52.11</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -8848,6 +8961,9 @@
       </c>
       <c r="BS47" s="15" t="n">
         <v>7042.77</v>
+      </c>
+      <c r="BT47" s="15" t="n">
+        <v>6983.47</v>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
@@ -8970,6 +9086,7 @@
       <c r="BQ48" s="15" t="n"/>
       <c r="BR48" s="15" t="n"/>
       <c r="BS48" s="15" t="n"/>
+      <c r="BT48" s="15" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -9184,6 +9301,9 @@
       </c>
       <c r="BS49" s="15" t="n">
         <v>22.49</v>
+      </c>
+      <c r="BT49" s="15" t="n">
+        <v>20.4</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -9351,6 +9471,9 @@
       </c>
       <c r="BS50" s="15" t="n">
         <v>32651.38</v>
+      </c>
+      <c r="BT50" s="15" t="n">
+        <v>32316.77</v>
       </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
@@ -9473,6 +9596,7 @@
       <c r="BQ51" s="15" t="n"/>
       <c r="BR51" s="15" t="n"/>
       <c r="BS51" s="15" t="n"/>
+      <c r="BT51" s="15" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -9687,6 +9811,9 @@
       </c>
       <c r="BS52" s="15" t="n">
         <v>37.16</v>
+      </c>
+      <c r="BT52" s="15" t="n">
+        <v>35.83</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -9854,6 +9981,9 @@
       </c>
       <c r="BS53" s="15" t="n">
         <v>3426.56</v>
+      </c>
+      <c r="BT53" s="15" t="n">
+        <v>3429.26</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
@@ -9976,6 +10106,7 @@
       <c r="BQ54" s="15" t="n"/>
       <c r="BR54" s="15" t="n"/>
       <c r="BS54" s="15" t="n"/>
+      <c r="BT54" s="15" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -10190,6 +10321,9 @@
       </c>
       <c r="BS55" s="15" t="n">
         <v>43.56</v>
+      </c>
+      <c r="BT55" s="15" t="n">
+        <v>43.21</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -10357,6 +10491,9 @@
       </c>
       <c r="BS56" s="15" t="n">
         <v>3285.58</v>
+      </c>
+      <c r="BT56" s="15" t="n">
+        <v>3298.31</v>
       </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
@@ -10479,6 +10616,7 @@
       <c r="BQ57" s="15" t="n"/>
       <c r="BR57" s="15" t="n"/>
       <c r="BS57" s="15" t="n"/>
+      <c r="BT57" s="15" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -10693,6 +10831,9 @@
       </c>
       <c r="BS58" s="15" t="n">
         <v>10.53</v>
+      </c>
+      <c r="BT58" s="15" t="n">
+        <v>13.68</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -10860,6 +11001,9 @@
       </c>
       <c r="BS59" s="15" t="n">
         <v>6598.37</v>
+      </c>
+      <c r="BT59" s="15" t="n">
+        <v>6638.7</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
@@ -10982,6 +11126,7 @@
       <c r="BQ60" s="15" t="n"/>
       <c r="BR60" s="15" t="n"/>
       <c r="BS60" s="15" t="n"/>
+      <c r="BT60" s="15" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -11196,6 +11341,9 @@
       </c>
       <c r="BS61" s="15" t="n">
         <v>27.81</v>
+      </c>
+      <c r="BT61" s="15" t="n">
+        <v>29.3</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -11363,6 +11511,9 @@
       </c>
       <c r="BS62" s="15" t="n">
         <v>7994.51</v>
+      </c>
+      <c r="BT62" s="15" t="n">
+        <v>7970.45</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
@@ -11485,6 +11636,7 @@
       <c r="BQ63" s="15" t="n"/>
       <c r="BR63" s="15" t="n"/>
       <c r="BS63" s="15" t="n"/>
+      <c r="BT63" s="15" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -11699,6 +11851,9 @@
       </c>
       <c r="BS64" s="15" t="n">
         <v>8.380000000000001</v>
+      </c>
+      <c r="BT64" s="15" t="n">
+        <v>6.58</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -11866,6 +12021,9 @@
       </c>
       <c r="BS65" s="15" t="n">
         <v>10652.53</v>
+      </c>
+      <c r="BT65" s="15" t="n">
+        <v>10472.93</v>
       </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
@@ -11988,6 +12146,7 @@
       <c r="BQ66" s="15" t="n"/>
       <c r="BR66" s="15" t="n"/>
       <c r="BS66" s="15" t="n"/>
+      <c r="BT66" s="15" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -12202,6 +12361,9 @@
       </c>
       <c r="BS67" s="15" t="n">
         <v>22.02</v>
+      </c>
+      <c r="BT67" s="15" t="n">
+        <v>18.18</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -12368,6 +12530,9 @@
         <v>11392.59</v>
       </c>
       <c r="BS68" s="15" t="n">
+        <v>11215.06</v>
+      </c>
+      <c r="BT68" s="15" t="n">
         <v>11215.06</v>
       </c>
     </row>
@@ -12491,6 +12656,7 @@
       <c r="BQ69" s="15" t="n"/>
       <c r="BR69" s="15" t="n"/>
       <c r="BS69" s="15" t="n"/>
+      <c r="BT69" s="15" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -12705,6 +12871,9 @@
       </c>
       <c r="BS70" s="15" t="n">
         <v>16.01</v>
+      </c>
+      <c r="BT70" s="15" t="n">
+        <v>14.47</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -12872,6 +13041,9 @@
       </c>
       <c r="BS71" s="15" t="n">
         <v>6247.83</v>
+      </c>
+      <c r="BT71" s="15" t="n">
+        <v>6164.84</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
@@ -12994,6 +13166,7 @@
       <c r="BQ72" s="15" t="n"/>
       <c r="BR72" s="15" t="n"/>
       <c r="BS72" s="15" t="n"/>
+      <c r="BT72" s="15" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -13208,6 +13381,9 @@
       </c>
       <c r="BS73" s="15" t="n">
         <v>18.12</v>
+      </c>
+      <c r="BT73" s="15" t="n">
+        <v>16.83</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -13375,6 +13551,9 @@
       </c>
       <c r="BS74" s="15" t="n">
         <v>12324.03</v>
+      </c>
+      <c r="BT74" s="15" t="n">
+        <v>12162.26</v>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
@@ -13497,6 +13676,7 @@
       <c r="BQ75" s="15" t="n"/>
       <c r="BR75" s="15" t="n"/>
       <c r="BS75" s="15" t="n"/>
+      <c r="BT75" s="15" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -13711,6 +13891,9 @@
       </c>
       <c r="BS76" s="15" t="n">
         <v>51.65</v>
+      </c>
+      <c r="BT76" s="15" t="n">
+        <v>51.91</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -13877,6 +14060,9 @@
         <v>15061.96</v>
       </c>
       <c r="BS77" s="15" t="n">
+        <v>15569.82</v>
+      </c>
+      <c r="BT77" s="15" t="n">
         <v>15569.82</v>
       </c>
     </row>
@@ -14000,6 +14186,7 @@
       <c r="BQ78" s="15" t="n"/>
       <c r="BR78" s="15" t="n"/>
       <c r="BS78" s="15" t="n"/>
+      <c r="BT78" s="15" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -14214,6 +14401,9 @@
       </c>
       <c r="BS79" s="15" t="n">
         <v>1.83</v>
+      </c>
+      <c r="BT79" s="15" t="n">
+        <v>2.32</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -14381,6 +14571,9 @@
       </c>
       <c r="BS80" s="15" t="n">
         <v>6497.23</v>
+      </c>
+      <c r="BT80" s="15" t="n">
+        <v>6501.74</v>
       </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
@@ -14503,6 +14696,7 @@
       <c r="BQ81" s="15" t="n"/>
       <c r="BR81" s="15" t="n"/>
       <c r="BS81" s="15" t="n"/>
+      <c r="BT81" s="15" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -14717,6 +14911,9 @@
       </c>
       <c r="BS82" s="15" t="n">
         <v>3.04</v>
+      </c>
+      <c r="BT82" s="15" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -14884,6 +15081,9 @@
       </c>
       <c r="BS83" s="15" t="n">
         <v>8501.110000000001</v>
+      </c>
+      <c r="BT83" s="15" t="n">
+        <v>8203.559999999999</v>
       </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
@@ -15006,6 +15206,7 @@
       <c r="BQ84" s="15" t="n"/>
       <c r="BR84" s="15" t="n"/>
       <c r="BS84" s="15" t="n"/>
+      <c r="BT84" s="15" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -15220,6 +15421,9 @@
       </c>
       <c r="BS85" s="15" t="n">
         <v>17.04</v>
+      </c>
+      <c r="BT85" s="15" t="n">
+        <v>16.63</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -15386,6 +15590,9 @@
         <v>2631.9</v>
       </c>
       <c r="BS86" s="15" t="n">
+        <v>2631.9</v>
+      </c>
+      <c r="BT86" s="15" t="n">
         <v>2631.9</v>
       </c>
     </row>
@@ -15509,6 +15716,7 @@
       <c r="BQ87" s="15" t="n"/>
       <c r="BR87" s="15" t="n"/>
       <c r="BS87" s="15" t="n"/>
+      <c r="BT87" s="15" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -15723,6 +15931,9 @@
       </c>
       <c r="BS88" s="15" t="n">
         <v>25.09</v>
+      </c>
+      <c r="BT88" s="15" t="n">
+        <v>26.75</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -15890,6 +16101,9 @@
       </c>
       <c r="BS89" s="15" t="n">
         <v>5075.31</v>
+      </c>
+      <c r="BT89" s="15" t="n">
+        <v>4310.74</v>
       </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
@@ -16012,6 +16226,7 @@
       <c r="BQ90" s="15" t="n"/>
       <c r="BR90" s="15" t="n"/>
       <c r="BS90" s="15" t="n"/>
+      <c r="BT90" s="15" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -16226,6 +16441,9 @@
       </c>
       <c r="BS91" s="15" t="n">
         <v>10.73</v>
+      </c>
+      <c r="BT91" s="15" t="n">
+        <v>12.68</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -16393,6 +16611,9 @@
       </c>
       <c r="BS92" s="15" t="n">
         <v>8346.67</v>
+      </c>
+      <c r="BT92" s="15" t="n">
+        <v>8336.48</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
@@ -16515,6 +16736,7 @@
       <c r="BQ93" s="15" t="n"/>
       <c r="BR93" s="15" t="n"/>
       <c r="BS93" s="15" t="n"/>
+      <c r="BT93" s="15" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -16729,6 +16951,9 @@
       </c>
       <c r="BS94" s="15" t="n">
         <v>5.07</v>
+      </c>
+      <c r="BT94" s="15" t="n">
+        <v>4.25</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -16896,6 +17121,9 @@
       </c>
       <c r="BS95" s="15" t="n">
         <v>1212.55</v>
+      </c>
+      <c r="BT95" s="15" t="n">
+        <v>1184.06</v>
       </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
@@ -17018,6 +17246,7 @@
       <c r="BQ96" s="15" t="n"/>
       <c r="BR96" s="15" t="n"/>
       <c r="BS96" s="15" t="n"/>
+      <c r="BT96" s="15" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -17232,6 +17461,9 @@
       </c>
       <c r="BS97" s="15" t="n">
         <v>8.390000000000001</v>
+      </c>
+      <c r="BT97" s="15" t="n">
+        <v>7.8</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -17399,6 +17631,9 @@
       </c>
       <c r="BS98" s="15" t="n">
         <v>13616.29</v>
+      </c>
+      <c r="BT98" s="15" t="n">
+        <v>13486.33</v>
       </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
@@ -17521,6 +17756,7 @@
       <c r="BQ99" s="15" t="n"/>
       <c r="BR99" s="15" t="n"/>
       <c r="BS99" s="15" t="n"/>
+      <c r="BT99" s="15" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -17735,6 +17971,9 @@
       </c>
       <c r="BS100" s="15" t="n">
         <v>27.7</v>
+      </c>
+      <c r="BT100" s="15" t="n">
+        <v>30.57</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -17902,6 +18141,9 @@
       </c>
       <c r="BS101" s="15" t="n">
         <v>3093.74</v>
+      </c>
+      <c r="BT101" s="15" t="n">
+        <v>3159.21</v>
       </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
@@ -18024,6 +18266,7 @@
       <c r="BQ102" s="15" t="n"/>
       <c r="BR102" s="15" t="n"/>
       <c r="BS102" s="15" t="n"/>
+      <c r="BT102" s="15" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -18238,6 +18481,9 @@
       </c>
       <c r="BS103" s="15" t="n">
         <v>28.31</v>
+      </c>
+      <c r="BT103" s="15" t="n">
+        <v>26.81</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -18405,6 +18651,9 @@
       </c>
       <c r="BS104" s="15" t="n">
         <v>2257.6</v>
+      </c>
+      <c r="BT104" s="15" t="n">
+        <v>2229.3</v>
       </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
@@ -18527,6 +18776,7 @@
       <c r="BQ105" s="15" t="n"/>
       <c r="BR105" s="15" t="n"/>
       <c r="BS105" s="15" t="n"/>
+      <c r="BT105" s="15" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -18741,6 +18991,9 @@
       </c>
       <c r="BS106" s="15" t="n">
         <v>11.74</v>
+      </c>
+      <c r="BT106" s="15" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -18908,6 +19161,9 @@
       </c>
       <c r="BS107" s="15" t="n">
         <v>2413.21</v>
+      </c>
+      <c r="BT107" s="15" t="n">
+        <v>2330.22</v>
       </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
@@ -19030,6 +19286,7 @@
       <c r="BQ108" s="15" t="n"/>
       <c r="BR108" s="15" t="n"/>
       <c r="BS108" s="15" t="n"/>
+      <c r="BT108" s="15" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -19244,6 +19501,9 @@
       </c>
       <c r="BS109" s="15" t="n">
         <v>28.33</v>
+      </c>
+      <c r="BT109" s="15" t="n">
+        <v>25.87</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -19411,6 +19671,9 @@
       </c>
       <c r="BS110" s="15" t="n">
         <v>2397.17</v>
+      </c>
+      <c r="BT110" s="15" t="n">
+        <v>2419.39</v>
       </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
@@ -19533,6 +19796,7 @@
       <c r="BQ111" s="15" t="n"/>
       <c r="BR111" s="15" t="n"/>
       <c r="BS111" s="15" t="n"/>
+      <c r="BT111" s="15" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -19747,6 +20011,9 @@
       </c>
       <c r="BS112" s="15" t="n">
         <v>38.92</v>
+      </c>
+      <c r="BT112" s="15" t="n">
+        <v>44.11</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -19912,6 +20179,9 @@
       </c>
       <c r="BS113" s="15" t="n">
         <v>1869.95</v>
+      </c>
+      <c r="BT113" s="15" t="n">
+        <v>1869.55</v>
       </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
@@ -20034,6 +20304,7 @@
       <c r="BQ114" s="15" t="n"/>
       <c r="BR114" s="15" t="n"/>
       <c r="BS114" s="15" t="n"/>
+      <c r="BT114" s="15" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -20248,6 +20519,9 @@
       </c>
       <c r="BS115" s="15" t="n">
         <v>14.47</v>
+      </c>
+      <c r="BT115" s="15" t="n">
+        <v>14.51</v>
       </c>
     </row>
     <row r="116" ht="14.25" customHeight="1">
@@ -20400,6 +20674,9 @@
       </c>
       <c r="BS116" s="15" t="n">
         <v>8794.76</v>
+      </c>
+      <c r="BT116" s="15" t="n">
+        <v>8467.52</v>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1">
@@ -20477,6 +20754,7 @@
       <c r="BQ117" s="15" t="n"/>
       <c r="BR117" s="15" t="n"/>
       <c r="BS117" s="15" t="n"/>
+      <c r="BT117" s="15" t="n"/>
     </row>
     <row r="118" ht="14.25" customHeight="1">
       <c r="P118" s="13" t="n">
@@ -20647,6 +20925,9 @@
       <c r="BS118" s="15" t="n">
         <v>70.45999999999999</v>
       </c>
+      <c r="BT118" s="15" t="n">
+        <v>73.77</v>
+      </c>
     </row>
     <row r="119" ht="14.25" customHeight="1">
       <c r="Y119" s="13" t="n">
@@ -20789,6 +21070,9 @@
       </c>
       <c r="BS119" s="15" t="n">
         <v>11938.17</v>
+      </c>
+      <c r="BT119" s="15" t="n">
+        <v>12632.71</v>
       </c>
     </row>
     <row r="120" ht="14.25" customHeight="1">
@@ -20815,6 +21099,7 @@
       <c r="BQ120" s="15" t="n"/>
       <c r="BR120" s="15" t="n"/>
       <c r="BS120" s="15" t="n"/>
+      <c r="BT120" s="15" t="n"/>
     </row>
     <row r="121" ht="14.25" customHeight="1">
       <c r="AW121" s="13" t="n">
@@ -20886,6 +21171,9 @@
       <c r="BS121" s="15" t="n">
         <v>24.98</v>
       </c>
+      <c r="BT121" s="15" t="n">
+        <v>22.38</v>
+      </c>
     </row>
     <row r="122" ht="14.25" customHeight="1">
       <c r="AW122" s="13" t="n">
@@ -20956,6 +21244,9 @@
       </c>
       <c r="BS122" s="15" t="n">
         <v>1212.12</v>
+      </c>
+      <c r="BT122" s="15" t="n">
+        <v>1188.27</v>
       </c>
     </row>
     <row r="123" ht="14.25" customHeight="1">
@@ -20982,6 +21273,7 @@
       <c r="BQ123" s="15" t="n"/>
       <c r="BR123" s="15" t="n"/>
       <c r="BS123" s="15" t="n"/>
+      <c r="BT123" s="15" t="n"/>
     </row>
     <row r="124" ht="14.25" customHeight="1">
       <c r="AW124" s="13" t="n">
@@ -21053,6 +21345,9 @@
       <c r="BS124" s="15" t="n">
         <v>50.63</v>
       </c>
+      <c r="BT124" s="15" t="n">
+        <v>47.17</v>
+      </c>
     </row>
     <row r="125" ht="14.25" customHeight="1">
       <c r="AW125" s="13" t="n">
@@ -21123,6 +21418,9 @@
       </c>
       <c r="BS125" s="15" t="n">
         <v>11643.01</v>
+      </c>
+      <c r="BT125" s="15" t="n">
+        <v>11570.27</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1">
@@ -21149,6 +21447,7 @@
       <c r="BQ126" s="15" t="n"/>
       <c r="BR126" s="15" t="n"/>
       <c r="BS126" s="15" t="n"/>
+      <c r="BT126" s="15" t="n"/>
     </row>
     <row r="127" ht="14.25" customHeight="1">
       <c r="AW127" s="13" t="n">
@@ -21220,6 +21519,9 @@
       <c r="BS127" s="15" t="n">
         <v>5.63</v>
       </c>
+      <c r="BT127" s="15" t="n">
+        <v>4.26</v>
+      </c>
     </row>
     <row r="128" ht="14.25" customHeight="1">
       <c r="AW128" s="13" t="n">
@@ -21290,6 +21592,9 @@
       </c>
       <c r="BS128" s="15" t="n">
         <v>1894.86</v>
+      </c>
+      <c r="BT128" s="15" t="n">
+        <v>1854.4</v>
       </c>
     </row>
     <row r="129" ht="14.25" customHeight="1">
@@ -21316,6 +21621,7 @@
       <c r="BQ129" s="15" t="n"/>
       <c r="BR129" s="15" t="n"/>
       <c r="BS129" s="15" t="n"/>
+      <c r="BT129" s="15" t="n"/>
     </row>
     <row r="130" ht="14.25" customHeight="1">
       <c r="AW130" s="13" t="n">
@@ -21387,6 +21693,9 @@
       <c r="BS130" s="15" t="n">
         <v>7.77</v>
       </c>
+      <c r="BT130" s="15" t="n">
+        <v>7.74</v>
+      </c>
     </row>
     <row r="131" ht="14.25" customHeight="1">
       <c r="AW131" s="13" t="n">
@@ -21457,6 +21766,9 @@
       </c>
       <c r="BS131" s="15" t="n">
         <v>732.6</v>
+      </c>
+      <c r="BT131" s="15" t="n">
+        <v>724.78</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1">
@@ -21483,6 +21795,7 @@
       <c r="BQ132" s="15" t="n"/>
       <c r="BR132" s="15" t="n"/>
       <c r="BS132" s="15" t="n"/>
+      <c r="BT132" s="15" t="n"/>
     </row>
     <row r="133" ht="14.25" customHeight="1">
       <c r="AW133" s="13" t="n">
@@ -21554,6 +21867,9 @@
       <c r="BS133" s="15" t="n">
         <v>58.68</v>
       </c>
+      <c r="BT133" s="15" t="n">
+        <v>58.73</v>
+      </c>
     </row>
     <row r="134" ht="14.25" customHeight="1">
       <c r="AW134" s="13" t="n">
@@ -21624,6 +21940,9 @@
       </c>
       <c r="BS134" s="15" t="n">
         <v>3050.14</v>
+      </c>
+      <c r="BT134" s="15" t="n">
+        <v>3015.83</v>
       </c>
     </row>
     <row r="135" ht="14.25" customHeight="1">
@@ -21650,6 +21969,7 @@
       <c r="BQ135" s="15" t="n"/>
       <c r="BR135" s="15" t="n"/>
       <c r="BS135" s="15" t="n"/>
+      <c r="BT135" s="15" t="n"/>
     </row>
     <row r="136" ht="14.25" customHeight="1">
       <c r="AW136" s="13" t="n">
@@ -21721,6 +22041,9 @@
       <c r="BS136" s="15" t="n">
         <v>21.83</v>
       </c>
+      <c r="BT136" s="15" t="n">
+        <v>21.34</v>
+      </c>
     </row>
     <row r="137" ht="14.25" customHeight="1">
       <c r="AW137" s="13" t="n">
@@ -21791,6 +22114,9 @@
       </c>
       <c r="BS137" s="15" t="n">
         <v>3522.7</v>
+      </c>
+      <c r="BT137" s="15" t="n">
+        <v>3513.37</v>
       </c>
     </row>
     <row r="138">
@@ -21809,6 +22135,7 @@
       <c r="BQ138" s="15" t="n"/>
       <c r="BR138" s="15" t="n"/>
       <c r="BS138" s="15" t="n"/>
+      <c r="BT138" s="15" t="n"/>
     </row>
     <row r="139">
       <c r="BE139" s="15" t="n">
@@ -21856,6 +22183,9 @@
       <c r="BS139" s="15" t="n">
         <v>3.27</v>
       </c>
+      <c r="BT139" s="15" t="n">
+        <v>3.52</v>
+      </c>
     </row>
     <row r="140">
       <c r="BE140" s="15" t="n">
@@ -21902,6 +22232,9 @@
       </c>
       <c r="BS140" s="15" t="n">
         <v>2431.48</v>
+      </c>
+      <c r="BT140" s="15" t="n">
+        <v>2351.96</v>
       </c>
     </row>
     <row r="141">
@@ -21920,6 +22253,7 @@
       <c r="BQ141" s="15" t="n"/>
       <c r="BR141" s="15" t="n"/>
       <c r="BS141" s="15" t="n"/>
+      <c r="BT141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="BE142" s="15" t="n">
@@ -21967,6 +22301,9 @@
       <c r="BS142" s="15" t="n">
         <v>22.98</v>
       </c>
+      <c r="BT142" s="15" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="143">
       <c r="BE143" s="15" t="n">
@@ -22013,6 +22350,9 @@
       </c>
       <c r="BS143" s="15" t="n">
         <v>5852.64</v>
+      </c>
+      <c r="BT143" s="15" t="n">
+        <v>5685.82</v>
       </c>
     </row>
     <row r="144">
@@ -22026,6 +22366,7 @@
       <c r="BQ144" s="15" t="n"/>
       <c r="BR144" s="15" t="n"/>
       <c r="BS144" s="15" t="n"/>
+      <c r="BT144" s="15" t="n"/>
     </row>
     <row r="145">
       <c r="BJ145" s="15" t="n">
@@ -22058,6 +22399,9 @@
       <c r="BS145" s="15" t="n">
         <v>2.09</v>
       </c>
+      <c r="BT145" s="15" t="n">
+        <v>1.4</v>
+      </c>
     </row>
     <row r="146">
       <c r="BJ146" s="15" t="n">
@@ -22089,6 +22433,9 @@
       </c>
       <c r="BS146" s="15" t="n">
         <v>2277.18</v>
+      </c>
+      <c r="BT146" s="15" t="n">
+        <v>2197.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-09-21 09:20:08]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BT146"/>
+  <dimension ref="A1:BU146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="51"/>
@@ -606,6 +606,7 @@
     <col width="15" customWidth="1" min="70" max="70"/>
     <col width="15" customWidth="1" min="71" max="71"/>
     <col width="15" customWidth="1" min="72" max="72"/>
+    <col width="15" customWidth="1" min="73" max="73"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -969,6 +970,11 @@
           <t>2026/09/17</t>
         </is>
       </c>
+      <c r="BU1" s="15" t="inlineStr">
+        <is>
+          <t>2026/09/21</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1331,6 +1337,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="BU2" s="16" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1549,6 +1560,9 @@
       <c r="BT3" s="15" t="n">
         <v>58.56</v>
       </c>
+      <c r="BU3" s="15" t="n">
+        <v>59.93</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1766,6 +1780,9 @@
       </c>
       <c r="BT4" s="15" t="n">
         <v>3875.6</v>
+      </c>
+      <c r="BU4" s="15" t="n">
+        <v>3949.91</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1841,6 +1858,7 @@
       <c r="BR5" s="15" t="n"/>
       <c r="BS5" s="15" t="n"/>
       <c r="BT5" s="15" t="n"/>
+      <c r="BU5" s="15" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1963,6 +1981,7 @@
       <c r="BR6" s="15" t="n"/>
       <c r="BS6" s="15" t="n"/>
       <c r="BT6" s="15" t="n"/>
+      <c r="BU6" s="15" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -2180,6 +2199,9 @@
       </c>
       <c r="BT7" s="15" t="n">
         <v>51.56</v>
+      </c>
+      <c r="BU7" s="15" t="n">
+        <v>51.86</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -2350,6 +2372,9 @@
       </c>
       <c r="BT8" s="15" t="n">
         <v>5515.99</v>
+      </c>
+      <c r="BU8" s="15" t="n">
+        <v>5626.57</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
@@ -2473,6 +2498,7 @@
       <c r="BR9" s="15" t="n"/>
       <c r="BS9" s="15" t="n"/>
       <c r="BT9" s="15" t="n"/>
+      <c r="BU9" s="15" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -2690,6 +2716,9 @@
       </c>
       <c r="BT10" s="15" t="n">
         <v>45.56</v>
+      </c>
+      <c r="BU10" s="15" t="n">
+        <v>46.1</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -2860,6 +2889,9 @@
       </c>
       <c r="BT11" s="15" t="n">
         <v>4460.16</v>
+      </c>
+      <c r="BU11" s="15" t="n">
+        <v>4539.57</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
@@ -2983,6 +3015,7 @@
       <c r="BR12" s="15" t="n"/>
       <c r="BS12" s="15" t="n"/>
       <c r="BT12" s="15" t="n"/>
+      <c r="BU12" s="15" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -3200,6 +3233,9 @@
       </c>
       <c r="BT13" s="15" t="n">
         <v>59.23</v>
+      </c>
+      <c r="BU13" s="15" t="n">
+        <v>60.72</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -3370,6 +3406,9 @@
       </c>
       <c r="BT14" s="15" t="n">
         <v>7654.98</v>
+      </c>
+      <c r="BU14" s="15" t="n">
+        <v>7850.48</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
@@ -3493,6 +3532,7 @@
       <c r="BR15" s="15" t="n"/>
       <c r="BS15" s="15" t="n"/>
       <c r="BT15" s="15" t="n"/>
+      <c r="BU15" s="15" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -3710,6 +3750,9 @@
       </c>
       <c r="BT16" s="15" t="n">
         <v>28.08</v>
+      </c>
+      <c r="BU16" s="15" t="n">
+        <v>27.95</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -3880,6 +3923,9 @@
       </c>
       <c r="BT17" s="15" t="n">
         <v>2491.04</v>
+      </c>
+      <c r="BU17" s="15" t="n">
+        <v>2538.47</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
@@ -4003,6 +4049,7 @@
       <c r="BR18" s="15" t="n"/>
       <c r="BS18" s="15" t="n"/>
       <c r="BT18" s="15" t="n"/>
+      <c r="BU18" s="15" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -4220,6 +4267,9 @@
       </c>
       <c r="BT19" s="15" t="n">
         <v>79.83</v>
+      </c>
+      <c r="BU19" s="15" t="n">
+        <v>80.12</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -4390,6 +4440,9 @@
       </c>
       <c r="BT20" s="15" t="n">
         <v>7551.81</v>
+      </c>
+      <c r="BU20" s="15" t="n">
+        <v>7650.5</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
@@ -4513,6 +4566,7 @@
       <c r="BR21" s="15" t="n"/>
       <c r="BS21" s="15" t="n"/>
       <c r="BT21" s="15" t="n"/>
+      <c r="BU21" s="15" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -4727,6 +4781,9 @@
         <v>36.34</v>
       </c>
       <c r="BT22" s="15" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="BU22" s="15" t="n">
         <v>36.34</v>
       </c>
     </row>
@@ -4898,6 +4955,9 @@
       </c>
       <c r="BT23" s="15" t="n">
         <v>74383.59</v>
+      </c>
+      <c r="BU23" s="15" t="n">
+        <v>74928.75</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
@@ -5021,6 +5081,7 @@
       <c r="BR24" s="15" t="n"/>
       <c r="BS24" s="15" t="n"/>
       <c r="BT24" s="15" t="n"/>
+      <c r="BU24" s="15" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -5237,6 +5298,9 @@
         <v>49.88</v>
       </c>
       <c r="BT25" s="15" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="BU25" s="15" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -5394,6 +5458,9 @@
       </c>
       <c r="BT26" s="15" t="n">
         <v>25673.14</v>
+      </c>
+      <c r="BU26" s="15" t="n">
+        <v>25544.8</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
@@ -5517,6 +5584,7 @@
       <c r="BR27" s="15" t="n"/>
       <c r="BS27" s="15" t="n"/>
       <c r="BT27" s="15" t="n"/>
+      <c r="BU27" s="15" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -5733,6 +5801,9 @@
         <v>92.09</v>
       </c>
       <c r="BT28" s="15" t="n">
+        <v>92.09</v>
+      </c>
+      <c r="BU28" s="15" t="n">
         <v>92.09</v>
       </c>
     </row>
@@ -5904,6 +5975,9 @@
       </c>
       <c r="BT29" s="15" t="n">
         <v>64136.25</v>
+      </c>
+      <c r="BU29" s="15" t="n">
+        <v>65018.95</v>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
@@ -6027,6 +6101,7 @@
       <c r="BR30" s="15" t="n"/>
       <c r="BS30" s="15" t="n"/>
       <c r="BT30" s="15" t="n"/>
+      <c r="BU30" s="15" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -6243,6 +6318,9 @@
         <v>97.44</v>
       </c>
       <c r="BT31" s="15" t="n">
+        <v>97.44</v>
+      </c>
+      <c r="BU31" s="15" t="n">
         <v>97.44</v>
       </c>
     </row>
@@ -6414,6 +6492,9 @@
       </c>
       <c r="BT32" s="15" t="n">
         <v>6715.41</v>
+      </c>
+      <c r="BU32" s="15" t="n">
+        <v>7007.72</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
@@ -6537,6 +6618,7 @@
       <c r="BR33" s="15" t="n"/>
       <c r="BS33" s="15" t="n"/>
       <c r="BT33" s="15" t="n"/>
+      <c r="BU33" s="15" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -6754,6 +6836,9 @@
       </c>
       <c r="BT34" s="15" t="n">
         <v>48.41</v>
+      </c>
+      <c r="BU34" s="15" t="n">
+        <v>45.3</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -6924,6 +7009,9 @@
       </c>
       <c r="BT35" s="15" t="n">
         <v>5473.85</v>
+      </c>
+      <c r="BU35" s="15" t="n">
+        <v>5527.38</v>
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
@@ -7047,6 +7135,7 @@
       <c r="BR36" s="15" t="n"/>
       <c r="BS36" s="15" t="n"/>
       <c r="BT36" s="15" t="n"/>
+      <c r="BU36" s="15" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -7264,6 +7353,9 @@
       </c>
       <c r="BT37" s="15" t="n">
         <v>49.73</v>
+      </c>
+      <c r="BU37" s="15" t="n">
+        <v>49.69</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -7433,6 +7525,9 @@
         <v>11360.79</v>
       </c>
       <c r="BT38" s="15" t="n">
+        <v>11175.12</v>
+      </c>
+      <c r="BU38" s="15" t="n">
         <v>11175.12</v>
       </c>
     </row>
@@ -7557,6 +7652,7 @@
       <c r="BR39" s="15" t="n"/>
       <c r="BS39" s="15" t="n"/>
       <c r="BT39" s="15" t="n"/>
+      <c r="BU39" s="15" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -7774,6 +7870,9 @@
       </c>
       <c r="BT40" s="15" t="n">
         <v>51.11</v>
+      </c>
+      <c r="BU40" s="15" t="n">
+        <v>47.86</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -7944,6 +8043,9 @@
       </c>
       <c r="BT41" s="15" t="n">
         <v>10931.94</v>
+      </c>
+      <c r="BU41" s="15" t="n">
+        <v>10871.21</v>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
@@ -8067,6 +8169,7 @@
       <c r="BR42" s="15" t="n"/>
       <c r="BS42" s="15" t="n"/>
       <c r="BT42" s="15" t="n"/>
+      <c r="BU42" s="15" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -8284,6 +8387,9 @@
       </c>
       <c r="BT43" s="15" t="n">
         <v>52.01</v>
+      </c>
+      <c r="BU43" s="15" t="n">
+        <v>49</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -8454,6 +8560,9 @@
       </c>
       <c r="BT44" s="15" t="n">
         <v>3277.88</v>
+      </c>
+      <c r="BU44" s="15" t="n">
+        <v>3246.18</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
@@ -8577,6 +8686,7 @@
       <c r="BR45" s="15" t="n"/>
       <c r="BS45" s="15" t="n"/>
       <c r="BT45" s="15" t="n"/>
+      <c r="BU45" s="15" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -8794,6 +8904,9 @@
       </c>
       <c r="BT46" s="15" t="n">
         <v>52.11</v>
+      </c>
+      <c r="BU46" s="15" t="n">
+        <v>51.61</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -8964,6 +9077,9 @@
       </c>
       <c r="BT47" s="15" t="n">
         <v>6983.47</v>
+      </c>
+      <c r="BU47" s="15" t="n">
+        <v>6948.44</v>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
@@ -9087,6 +9203,7 @@
       <c r="BR48" s="15" t="n"/>
       <c r="BS48" s="15" t="n"/>
       <c r="BT48" s="15" t="n"/>
+      <c r="BU48" s="15" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -9304,6 +9421,9 @@
       </c>
       <c r="BT49" s="15" t="n">
         <v>20.4</v>
+      </c>
+      <c r="BU49" s="15" t="n">
+        <v>19.69</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -9474,6 +9594,9 @@
       </c>
       <c r="BT50" s="15" t="n">
         <v>32316.77</v>
+      </c>
+      <c r="BU50" s="15" t="n">
+        <v>32761.47</v>
       </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
@@ -9597,6 +9720,7 @@
       <c r="BR51" s="15" t="n"/>
       <c r="BS51" s="15" t="n"/>
       <c r="BT51" s="15" t="n"/>
+      <c r="BU51" s="15" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -9814,6 +9938,9 @@
       </c>
       <c r="BT52" s="15" t="n">
         <v>35.83</v>
+      </c>
+      <c r="BU52" s="15" t="n">
+        <v>37.41</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -9984,6 +10111,9 @@
       </c>
       <c r="BT53" s="15" t="n">
         <v>3429.26</v>
+      </c>
+      <c r="BU53" s="15" t="n">
+        <v>3538.47</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
@@ -10107,6 +10237,7 @@
       <c r="BR54" s="15" t="n"/>
       <c r="BS54" s="15" t="n"/>
       <c r="BT54" s="15" t="n"/>
+      <c r="BU54" s="15" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -10324,6 +10455,9 @@
       </c>
       <c r="BT55" s="15" t="n">
         <v>43.21</v>
+      </c>
+      <c r="BU55" s="15" t="n">
+        <v>45.41</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -10494,6 +10628,9 @@
       </c>
       <c r="BT56" s="15" t="n">
         <v>3298.31</v>
+      </c>
+      <c r="BU56" s="15" t="n">
+        <v>3399.59</v>
       </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
@@ -10617,6 +10754,7 @@
       <c r="BR57" s="15" t="n"/>
       <c r="BS57" s="15" t="n"/>
       <c r="BT57" s="15" t="n"/>
+      <c r="BU57" s="15" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -10834,6 +10972,9 @@
       </c>
       <c r="BT58" s="15" t="n">
         <v>13.68</v>
+      </c>
+      <c r="BU58" s="15" t="n">
+        <v>15.41</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -11004,6 +11145,9 @@
       </c>
       <c r="BT59" s="15" t="n">
         <v>6638.7</v>
+      </c>
+      <c r="BU59" s="15" t="n">
+        <v>6869.19</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
@@ -11127,6 +11271,7 @@
       <c r="BR60" s="15" t="n"/>
       <c r="BS60" s="15" t="n"/>
       <c r="BT60" s="15" t="n"/>
+      <c r="BU60" s="15" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -11344,6 +11489,9 @@
       </c>
       <c r="BT61" s="15" t="n">
         <v>29.3</v>
+      </c>
+      <c r="BU61" s="15" t="n">
+        <v>30.48</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -11514,6 +11662,9 @@
       </c>
       <c r="BT62" s="15" t="n">
         <v>7970.45</v>
+      </c>
+      <c r="BU62" s="15" t="n">
+        <v>8282.4</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
@@ -11637,6 +11788,7 @@
       <c r="BR63" s="15" t="n"/>
       <c r="BS63" s="15" t="n"/>
       <c r="BT63" s="15" t="n"/>
+      <c r="BU63" s="15" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -11854,6 +12006,9 @@
       </c>
       <c r="BT64" s="15" t="n">
         <v>6.58</v>
+      </c>
+      <c r="BU64" s="15" t="n">
+        <v>6.92</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -12024,6 +12179,9 @@
       </c>
       <c r="BT65" s="15" t="n">
         <v>10472.93</v>
+      </c>
+      <c r="BU65" s="15" t="n">
+        <v>10420.45</v>
       </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
@@ -12147,6 +12305,7 @@
       <c r="BR66" s="15" t="n"/>
       <c r="BS66" s="15" t="n"/>
       <c r="BT66" s="15" t="n"/>
+      <c r="BU66" s="15" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -12364,6 +12523,9 @@
       </c>
       <c r="BT67" s="15" t="n">
         <v>18.18</v>
+      </c>
+      <c r="BU67" s="15" t="n">
+        <v>20.05</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -12534,6 +12696,9 @@
       </c>
       <c r="BT68" s="15" t="n">
         <v>11215.06</v>
+      </c>
+      <c r="BU68" s="15" t="n">
+        <v>11220.97</v>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
@@ -12657,6 +12822,7 @@
       <c r="BR69" s="15" t="n"/>
       <c r="BS69" s="15" t="n"/>
       <c r="BT69" s="15" t="n"/>
+      <c r="BU69" s="15" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -12874,6 +13040,9 @@
       </c>
       <c r="BT70" s="15" t="n">
         <v>14.47</v>
+      </c>
+      <c r="BU70" s="15" t="n">
+        <v>14.61</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -13044,6 +13213,9 @@
       </c>
       <c r="BT71" s="15" t="n">
         <v>6164.84</v>
+      </c>
+      <c r="BU71" s="15" t="n">
+        <v>6254.47</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
@@ -13167,6 +13339,7 @@
       <c r="BR72" s="15" t="n"/>
       <c r="BS72" s="15" t="n"/>
       <c r="BT72" s="15" t="n"/>
+      <c r="BU72" s="15" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -13384,6 +13557,9 @@
       </c>
       <c r="BT73" s="15" t="n">
         <v>16.83</v>
+      </c>
+      <c r="BU73" s="15" t="n">
+        <v>17.07</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -13554,6 +13730,9 @@
       </c>
       <c r="BT74" s="15" t="n">
         <v>12162.26</v>
+      </c>
+      <c r="BU74" s="15" t="n">
+        <v>12321.63</v>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
@@ -13677,6 +13856,7 @@
       <c r="BR75" s="15" t="n"/>
       <c r="BS75" s="15" t="n"/>
       <c r="BT75" s="15" t="n"/>
+      <c r="BU75" s="15" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -13894,6 +14074,9 @@
       </c>
       <c r="BT76" s="15" t="n">
         <v>51.91</v>
+      </c>
+      <c r="BU76" s="15" t="n">
+        <v>52.73</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -14064,6 +14247,9 @@
       </c>
       <c r="BT77" s="15" t="n">
         <v>15569.82</v>
+      </c>
+      <c r="BU77" s="15" t="n">
+        <v>16449.57</v>
       </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
@@ -14187,6 +14373,7 @@
       <c r="BR78" s="15" t="n"/>
       <c r="BS78" s="15" t="n"/>
       <c r="BT78" s="15" t="n"/>
+      <c r="BU78" s="15" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -14404,6 +14591,9 @@
       </c>
       <c r="BT79" s="15" t="n">
         <v>2.32</v>
+      </c>
+      <c r="BU79" s="15" t="n">
+        <v>1.89</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -14574,6 +14764,9 @@
       </c>
       <c r="BT80" s="15" t="n">
         <v>6501.74</v>
+      </c>
+      <c r="BU80" s="15" t="n">
+        <v>6593.43</v>
       </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
@@ -14697,6 +14890,7 @@
       <c r="BR81" s="15" t="n"/>
       <c r="BS81" s="15" t="n"/>
       <c r="BT81" s="15" t="n"/>
+      <c r="BU81" s="15" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -14914,6 +15108,9 @@
       </c>
       <c r="BT82" s="15" t="n">
         <v>3</v>
+      </c>
+      <c r="BU82" s="15" t="n">
+        <v>3.19</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -15084,6 +15281,9 @@
       </c>
       <c r="BT83" s="15" t="n">
         <v>8203.559999999999</v>
+      </c>
+      <c r="BU83" s="15" t="n">
+        <v>8391.32</v>
       </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
@@ -15207,6 +15407,7 @@
       <c r="BR84" s="15" t="n"/>
       <c r="BS84" s="15" t="n"/>
       <c r="BT84" s="15" t="n"/>
+      <c r="BU84" s="15" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -15424,6 +15625,9 @@
       </c>
       <c r="BT85" s="15" t="n">
         <v>16.63</v>
+      </c>
+      <c r="BU85" s="15" t="n">
+        <v>16.53</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -15593,6 +15797,9 @@
         <v>2631.9</v>
       </c>
       <c r="BT86" s="15" t="n">
+        <v>2631.9</v>
+      </c>
+      <c r="BU86" s="15" t="n">
         <v>2631.9</v>
       </c>
     </row>
@@ -15717,6 +15924,7 @@
       <c r="BR87" s="15" t="n"/>
       <c r="BS87" s="15" t="n"/>
       <c r="BT87" s="15" t="n"/>
+      <c r="BU87" s="15" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -15934,6 +16142,9 @@
       </c>
       <c r="BT88" s="15" t="n">
         <v>26.75</v>
+      </c>
+      <c r="BU88" s="15" t="n">
+        <v>27.45</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -16104,6 +16315,9 @@
       </c>
       <c r="BT89" s="15" t="n">
         <v>4310.74</v>
+      </c>
+      <c r="BU89" s="15" t="n">
+        <v>4423.29</v>
       </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
@@ -16227,6 +16441,7 @@
       <c r="BR90" s="15" t="n"/>
       <c r="BS90" s="15" t="n"/>
       <c r="BT90" s="15" t="n"/>
+      <c r="BU90" s="15" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -16444,6 +16659,9 @@
       </c>
       <c r="BT91" s="15" t="n">
         <v>12.68</v>
+      </c>
+      <c r="BU91" s="15" t="n">
+        <v>14.11</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -16614,6 +16832,9 @@
       </c>
       <c r="BT92" s="15" t="n">
         <v>8336.48</v>
+      </c>
+      <c r="BU92" s="15" t="n">
+        <v>8645.5</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
@@ -16737,6 +16958,7 @@
       <c r="BR93" s="15" t="n"/>
       <c r="BS93" s="15" t="n"/>
       <c r="BT93" s="15" t="n"/>
+      <c r="BU93" s="15" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -16954,6 +17176,9 @@
       </c>
       <c r="BT94" s="15" t="n">
         <v>4.25</v>
+      </c>
+      <c r="BU94" s="15" t="n">
+        <v>4.46</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -17124,6 +17349,9 @@
       </c>
       <c r="BT95" s="15" t="n">
         <v>1184.06</v>
+      </c>
+      <c r="BU95" s="15" t="n">
+        <v>1184.75</v>
       </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
@@ -17247,6 +17475,7 @@
       <c r="BR96" s="15" t="n"/>
       <c r="BS96" s="15" t="n"/>
       <c r="BT96" s="15" t="n"/>
+      <c r="BU96" s="15" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -17464,6 +17693,9 @@
       </c>
       <c r="BT97" s="15" t="n">
         <v>7.8</v>
+      </c>
+      <c r="BU97" s="15" t="n">
+        <v>8.050000000000001</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -17634,6 +17866,9 @@
       </c>
       <c r="BT98" s="15" t="n">
         <v>13486.33</v>
+      </c>
+      <c r="BU98" s="15" t="n">
+        <v>13547.29</v>
       </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
@@ -17757,6 +17992,7 @@
       <c r="BR99" s="15" t="n"/>
       <c r="BS99" s="15" t="n"/>
       <c r="BT99" s="15" t="n"/>
+      <c r="BU99" s="15" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -17974,6 +18210,9 @@
       </c>
       <c r="BT100" s="15" t="n">
         <v>30.57</v>
+      </c>
+      <c r="BU100" s="15" t="n">
+        <v>32.58</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -18144,6 +18383,9 @@
       </c>
       <c r="BT101" s="15" t="n">
         <v>3159.21</v>
+      </c>
+      <c r="BU101" s="15" t="n">
+        <v>3212.94</v>
       </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
@@ -18267,6 +18509,7 @@
       <c r="BR102" s="15" t="n"/>
       <c r="BS102" s="15" t="n"/>
       <c r="BT102" s="15" t="n"/>
+      <c r="BU102" s="15" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -18484,6 +18727,9 @@
       </c>
       <c r="BT103" s="15" t="n">
         <v>26.81</v>
+      </c>
+      <c r="BU103" s="15" t="n">
+        <v>27.59</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -18654,6 +18900,9 @@
       </c>
       <c r="BT104" s="15" t="n">
         <v>2229.3</v>
+      </c>
+      <c r="BU104" s="15" t="n">
+        <v>2267.47</v>
       </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
@@ -18777,6 +19026,7 @@
       <c r="BR105" s="15" t="n"/>
       <c r="BS105" s="15" t="n"/>
       <c r="BT105" s="15" t="n"/>
+      <c r="BU105" s="15" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -18994,6 +19244,9 @@
       </c>
       <c r="BT106" s="15" t="n">
         <v>13</v>
+      </c>
+      <c r="BU106" s="15" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -19163,6 +19416,9 @@
         <v>2413.21</v>
       </c>
       <c r="BT107" s="15" t="n">
+        <v>2330.22</v>
+      </c>
+      <c r="BU107" s="15" t="n">
         <v>2330.22</v>
       </c>
     </row>
@@ -19287,6 +19543,7 @@
       <c r="BR108" s="15" t="n"/>
       <c r="BS108" s="15" t="n"/>
       <c r="BT108" s="15" t="n"/>
+      <c r="BU108" s="15" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -19504,6 +19761,9 @@
       </c>
       <c r="BT109" s="15" t="n">
         <v>25.87</v>
+      </c>
+      <c r="BU109" s="15" t="n">
+        <v>26.46</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -19674,6 +19934,9 @@
       </c>
       <c r="BT110" s="15" t="n">
         <v>2419.39</v>
+      </c>
+      <c r="BU110" s="15" t="n">
+        <v>2391.89</v>
       </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
@@ -19797,6 +20060,7 @@
       <c r="BR111" s="15" t="n"/>
       <c r="BS111" s="15" t="n"/>
       <c r="BT111" s="15" t="n"/>
+      <c r="BU111" s="15" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -20014,6 +20278,9 @@
       </c>
       <c r="BT112" s="15" t="n">
         <v>44.11</v>
+      </c>
+      <c r="BU112" s="15" t="n">
+        <v>46.42</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -20182,6 +20449,9 @@
       </c>
       <c r="BT113" s="15" t="n">
         <v>1869.55</v>
+      </c>
+      <c r="BU113" s="15" t="n">
+        <v>1880.2</v>
       </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
@@ -20305,6 +20575,7 @@
       <c r="BR114" s="15" t="n"/>
       <c r="BS114" s="15" t="n"/>
       <c r="BT114" s="15" t="n"/>
+      <c r="BU114" s="15" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -20522,6 +20793,9 @@
       </c>
       <c r="BT115" s="15" t="n">
         <v>14.51</v>
+      </c>
+      <c r="BU115" s="15" t="n">
+        <v>15.53</v>
       </c>
     </row>
     <row r="116" ht="14.25" customHeight="1">
@@ -20677,6 +20951,9 @@
       </c>
       <c r="BT116" s="15" t="n">
         <v>8467.52</v>
+      </c>
+      <c r="BU116" s="15" t="n">
+        <v>8691.26</v>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1">
@@ -20755,6 +21032,7 @@
       <c r="BR117" s="15" t="n"/>
       <c r="BS117" s="15" t="n"/>
       <c r="BT117" s="15" t="n"/>
+      <c r="BU117" s="15" t="n"/>
     </row>
     <row r="118" ht="14.25" customHeight="1">
       <c r="P118" s="13" t="n">
@@ -20928,6 +21206,9 @@
       <c r="BT118" s="15" t="n">
         <v>73.77</v>
       </c>
+      <c r="BU118" s="15" t="n">
+        <v>75.48999999999999</v>
+      </c>
     </row>
     <row r="119" ht="14.25" customHeight="1">
       <c r="Y119" s="13" t="n">
@@ -21073,6 +21354,9 @@
       </c>
       <c r="BT119" s="15" t="n">
         <v>12632.71</v>
+      </c>
+      <c r="BU119" s="15" t="n">
+        <v>13163.37</v>
       </c>
     </row>
     <row r="120" ht="14.25" customHeight="1">
@@ -21100,6 +21384,7 @@
       <c r="BR120" s="15" t="n"/>
       <c r="BS120" s="15" t="n"/>
       <c r="BT120" s="15" t="n"/>
+      <c r="BU120" s="15" t="n"/>
     </row>
     <row r="121" ht="14.25" customHeight="1">
       <c r="AW121" s="13" t="n">
@@ -21174,6 +21459,9 @@
       <c r="BT121" s="15" t="n">
         <v>22.38</v>
       </c>
+      <c r="BU121" s="15" t="n">
+        <v>23.75</v>
+      </c>
     </row>
     <row r="122" ht="14.25" customHeight="1">
       <c r="AW122" s="13" t="n">
@@ -21247,6 +21535,9 @@
       </c>
       <c r="BT122" s="15" t="n">
         <v>1188.27</v>
+      </c>
+      <c r="BU122" s="15" t="n">
+        <v>1198.64</v>
       </c>
     </row>
     <row r="123" ht="14.25" customHeight="1">
@@ -21274,6 +21565,7 @@
       <c r="BR123" s="15" t="n"/>
       <c r="BS123" s="15" t="n"/>
       <c r="BT123" s="15" t="n"/>
+      <c r="BU123" s="15" t="n"/>
     </row>
     <row r="124" ht="14.25" customHeight="1">
       <c r="AW124" s="13" t="n">
@@ -21348,6 +21640,9 @@
       <c r="BT124" s="15" t="n">
         <v>47.17</v>
       </c>
+      <c r="BU124" s="15" t="n">
+        <v>48.61</v>
+      </c>
     </row>
     <row r="125" ht="14.25" customHeight="1">
       <c r="AW125" s="13" t="n">
@@ -21421,6 +21716,9 @@
       </c>
       <c r="BT125" s="15" t="n">
         <v>11570.27</v>
+      </c>
+      <c r="BU125" s="15" t="n">
+        <v>11895.94</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1">
@@ -21448,6 +21746,7 @@
       <c r="BR126" s="15" t="n"/>
       <c r="BS126" s="15" t="n"/>
       <c r="BT126" s="15" t="n"/>
+      <c r="BU126" s="15" t="n"/>
     </row>
     <row r="127" ht="14.25" customHeight="1">
       <c r="AW127" s="13" t="n">
@@ -21522,6 +21821,9 @@
       <c r="BT127" s="15" t="n">
         <v>4.26</v>
       </c>
+      <c r="BU127" s="15" t="n">
+        <v>4.25</v>
+      </c>
     </row>
     <row r="128" ht="14.25" customHeight="1">
       <c r="AW128" s="13" t="n">
@@ -21595,6 +21897,9 @@
       </c>
       <c r="BT128" s="15" t="n">
         <v>1854.4</v>
+      </c>
+      <c r="BU128" s="15" t="n">
+        <v>1855.25</v>
       </c>
     </row>
     <row r="129" ht="14.25" customHeight="1">
@@ -21622,6 +21927,7 @@
       <c r="BR129" s="15" t="n"/>
       <c r="BS129" s="15" t="n"/>
       <c r="BT129" s="15" t="n"/>
+      <c r="BU129" s="15" t="n"/>
     </row>
     <row r="130" ht="14.25" customHeight="1">
       <c r="AW130" s="13" t="n">
@@ -21696,6 +22002,9 @@
       <c r="BT130" s="15" t="n">
         <v>7.74</v>
       </c>
+      <c r="BU130" s="15" t="n">
+        <v>7.3</v>
+      </c>
     </row>
     <row r="131" ht="14.25" customHeight="1">
       <c r="AW131" s="13" t="n">
@@ -21769,6 +22078,9 @@
       </c>
       <c r="BT131" s="15" t="n">
         <v>724.78</v>
+      </c>
+      <c r="BU131" s="15" t="n">
+        <v>742.3099999999999</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1">
@@ -21796,6 +22108,7 @@
       <c r="BR132" s="15" t="n"/>
       <c r="BS132" s="15" t="n"/>
       <c r="BT132" s="15" t="n"/>
+      <c r="BU132" s="15" t="n"/>
     </row>
     <row r="133" ht="14.25" customHeight="1">
       <c r="AW133" s="13" t="n">
@@ -21870,6 +22183,9 @@
       <c r="BT133" s="15" t="n">
         <v>58.73</v>
       </c>
+      <c r="BU133" s="15" t="n">
+        <v>56.92</v>
+      </c>
     </row>
     <row r="134" ht="14.25" customHeight="1">
       <c r="AW134" s="13" t="n">
@@ -21943,6 +22259,9 @@
       </c>
       <c r="BT134" s="15" t="n">
         <v>3015.83</v>
+      </c>
+      <c r="BU134" s="15" t="n">
+        <v>2851.18</v>
       </c>
     </row>
     <row r="135" ht="14.25" customHeight="1">
@@ -21970,6 +22289,7 @@
       <c r="BR135" s="15" t="n"/>
       <c r="BS135" s="15" t="n"/>
       <c r="BT135" s="15" t="n"/>
+      <c r="BU135" s="15" t="n"/>
     </row>
     <row r="136" ht="14.25" customHeight="1">
       <c r="AW136" s="13" t="n">
@@ -22044,6 +22364,9 @@
       <c r="BT136" s="15" t="n">
         <v>21.34</v>
       </c>
+      <c r="BU136" s="15" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="137" ht="14.25" customHeight="1">
       <c r="AW137" s="13" t="n">
@@ -22117,6 +22440,9 @@
       </c>
       <c r="BT137" s="15" t="n">
         <v>3513.37</v>
+      </c>
+      <c r="BU137" s="15" t="n">
+        <v>3561.44</v>
       </c>
     </row>
     <row r="138">
@@ -22136,6 +22462,7 @@
       <c r="BR138" s="15" t="n"/>
       <c r="BS138" s="15" t="n"/>
       <c r="BT138" s="15" t="n"/>
+      <c r="BU138" s="15" t="n"/>
     </row>
     <row r="139">
       <c r="BE139" s="15" t="n">
@@ -22186,6 +22513,9 @@
       <c r="BT139" s="15" t="n">
         <v>3.52</v>
       </c>
+      <c r="BU139" s="15" t="n">
+        <v>4.44</v>
+      </c>
     </row>
     <row r="140">
       <c r="BE140" s="15" t="n">
@@ -22234,6 +22564,9 @@
         <v>2431.48</v>
       </c>
       <c r="BT140" s="15" t="n">
+        <v>2351.96</v>
+      </c>
+      <c r="BU140" s="15" t="n">
         <v>2351.96</v>
       </c>
     </row>
@@ -22254,6 +22587,7 @@
       <c r="BR141" s="15" t="n"/>
       <c r="BS141" s="15" t="n"/>
       <c r="BT141" s="15" t="n"/>
+      <c r="BU141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="BE142" s="15" t="n">
@@ -22304,6 +22638,9 @@
       <c r="BT142" s="15" t="n">
         <v>17.95</v>
       </c>
+      <c r="BU142" s="15" t="n">
+        <v>17.94</v>
+      </c>
     </row>
     <row r="143">
       <c r="BE143" s="15" t="n">
@@ -22353,6 +22690,9 @@
       </c>
       <c r="BT143" s="15" t="n">
         <v>5685.82</v>
+      </c>
+      <c r="BU143" s="15" t="n">
+        <v>5687.43</v>
       </c>
     </row>
     <row r="144">
@@ -22367,6 +22707,7 @@
       <c r="BR144" s="15" t="n"/>
       <c r="BS144" s="15" t="n"/>
       <c r="BT144" s="15" t="n"/>
+      <c r="BU144" s="15" t="n"/>
     </row>
     <row r="145">
       <c r="BJ145" s="15" t="n">
@@ -22402,6 +22743,9 @@
       <c r="BT145" s="15" t="n">
         <v>1.4</v>
       </c>
+      <c r="BU145" s="15" t="n">
+        <v>1.86</v>
+      </c>
     </row>
     <row r="146">
       <c r="BJ146" s="15" t="n">
@@ -22436,6 +22780,9 @@
       </c>
       <c r="BT146" s="15" t="n">
         <v>2197.8</v>
+      </c>
+      <c r="BU146" s="15" t="n">
+        <v>2232.84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-09-24 08:48:05]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BU146"/>
+  <dimension ref="A1:BV146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="51"/>
@@ -607,6 +607,7 @@
     <col width="15" customWidth="1" min="71" max="71"/>
     <col width="15" customWidth="1" min="72" max="72"/>
     <col width="15" customWidth="1" min="73" max="73"/>
+    <col width="15" customWidth="1" min="74" max="74"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -975,6 +976,11 @@
           <t>2026/09/21</t>
         </is>
       </c>
+      <c r="BV1" s="15" t="inlineStr">
+        <is>
+          <t>2026/09/24</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1342,6 +1348,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="BV2" s="16" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1563,6 +1574,9 @@
       <c r="BU3" s="15" t="n">
         <v>59.93</v>
       </c>
+      <c r="BV3" s="15" t="n">
+        <v>60.52</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1783,6 +1797,9 @@
       </c>
       <c r="BU4" s="15" t="n">
         <v>3949.91</v>
+      </c>
+      <c r="BV4" s="15" t="n">
+        <v>3888.37</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1859,6 +1876,7 @@
       <c r="BS5" s="15" t="n"/>
       <c r="BT5" s="15" t="n"/>
       <c r="BU5" s="15" t="n"/>
+      <c r="BV5" s="15" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1982,6 +2000,7 @@
       <c r="BS6" s="15" t="n"/>
       <c r="BT6" s="15" t="n"/>
       <c r="BU6" s="15" t="n"/>
+      <c r="BV6" s="15" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -2202,6 +2221,9 @@
       </c>
       <c r="BU7" s="15" t="n">
         <v>51.86</v>
+      </c>
+      <c r="BV7" s="15" t="n">
+        <v>52.98</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -2375,6 +2397,9 @@
       </c>
       <c r="BU8" s="15" t="n">
         <v>5626.57</v>
+      </c>
+      <c r="BV8" s="15" t="n">
+        <v>5486.01</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
@@ -2499,6 +2524,7 @@
       <c r="BS9" s="15" t="n"/>
       <c r="BT9" s="15" t="n"/>
       <c r="BU9" s="15" t="n"/>
+      <c r="BV9" s="15" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -2719,6 +2745,9 @@
       </c>
       <c r="BU10" s="15" t="n">
         <v>46.1</v>
+      </c>
+      <c r="BV10" s="15" t="n">
+        <v>47.36</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -2892,6 +2921,9 @@
       </c>
       <c r="BU11" s="15" t="n">
         <v>4539.57</v>
+      </c>
+      <c r="BV11" s="15" t="n">
+        <v>4439.14</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
@@ -3016,6 +3048,7 @@
       <c r="BS12" s="15" t="n"/>
       <c r="BT12" s="15" t="n"/>
       <c r="BU12" s="15" t="n"/>
+      <c r="BV12" s="15" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -3236,6 +3269,9 @@
       </c>
       <c r="BU13" s="15" t="n">
         <v>60.72</v>
+      </c>
+      <c r="BV13" s="15" t="n">
+        <v>60.7</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -3409,6 +3445,9 @@
       </c>
       <c r="BU14" s="15" t="n">
         <v>7850.48</v>
+      </c>
+      <c r="BV14" s="15" t="n">
+        <v>7624.07</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
@@ -3533,6 +3572,7 @@
       <c r="BS15" s="15" t="n"/>
       <c r="BT15" s="15" t="n"/>
       <c r="BU15" s="15" t="n"/>
+      <c r="BV15" s="15" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -3753,6 +3793,9 @@
       </c>
       <c r="BU16" s="15" t="n">
         <v>27.95</v>
+      </c>
+      <c r="BV16" s="15" t="n">
+        <v>27.98</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -3926,6 +3969,9 @@
       </c>
       <c r="BU17" s="15" t="n">
         <v>2538.47</v>
+      </c>
+      <c r="BV17" s="15" t="n">
+        <v>2495.36</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
@@ -4050,6 +4096,7 @@
       <c r="BS18" s="15" t="n"/>
       <c r="BT18" s="15" t="n"/>
       <c r="BU18" s="15" t="n"/>
+      <c r="BV18" s="15" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -4270,6 +4317,9 @@
       </c>
       <c r="BU19" s="15" t="n">
         <v>80.12</v>
+      </c>
+      <c r="BV19" s="15" t="n">
+        <v>80.64</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -4443,6 +4493,9 @@
       </c>
       <c r="BU20" s="15" t="n">
         <v>7650.5</v>
+      </c>
+      <c r="BV20" s="15" t="n">
+        <v>7706.03</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
@@ -4567,6 +4620,7 @@
       <c r="BS21" s="15" t="n"/>
       <c r="BT21" s="15" t="n"/>
       <c r="BU21" s="15" t="n"/>
+      <c r="BV21" s="15" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -4784,6 +4838,9 @@
         <v>36.34</v>
       </c>
       <c r="BU22" s="15" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="BV22" s="15" t="n">
         <v>36.34</v>
       </c>
     </row>
@@ -4958,6 +5015,9 @@
       </c>
       <c r="BU23" s="15" t="n">
         <v>74928.75</v>
+      </c>
+      <c r="BV23" s="15" t="n">
+        <v>73647.46000000001</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
@@ -5082,6 +5142,7 @@
       <c r="BS24" s="15" t="n"/>
       <c r="BT24" s="15" t="n"/>
       <c r="BU24" s="15" t="n"/>
+      <c r="BV24" s="15" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -5301,6 +5362,9 @@
         <v>49.88</v>
       </c>
       <c r="BU25" s="15" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="BV25" s="15" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -5461,6 +5525,9 @@
       </c>
       <c r="BU26" s="15" t="n">
         <v>25544.8</v>
+      </c>
+      <c r="BV26" s="15" t="n">
+        <v>25178.08</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
@@ -5585,6 +5652,7 @@
       <c r="BS27" s="15" t="n"/>
       <c r="BT27" s="15" t="n"/>
       <c r="BU27" s="15" t="n"/>
+      <c r="BV27" s="15" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -5804,6 +5872,9 @@
         <v>92.09</v>
       </c>
       <c r="BU28" s="15" t="n">
+        <v>92.09</v>
+      </c>
+      <c r="BV28" s="15" t="n">
         <v>92.09</v>
       </c>
     </row>
@@ -5978,6 +6049,9 @@
       </c>
       <c r="BU29" s="15" t="n">
         <v>65018.95</v>
+      </c>
+      <c r="BV29" s="15" t="n">
+        <v>65513.99</v>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
@@ -6102,6 +6176,7 @@
       <c r="BS30" s="15" t="n"/>
       <c r="BT30" s="15" t="n"/>
       <c r="BU30" s="15" t="n"/>
+      <c r="BV30" s="15" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -6321,6 +6396,9 @@
         <v>97.44</v>
       </c>
       <c r="BU31" s="15" t="n">
+        <v>97.44</v>
+      </c>
+      <c r="BV31" s="15" t="n">
         <v>97.44</v>
       </c>
     </row>
@@ -6495,6 +6573,9 @@
       </c>
       <c r="BU32" s="15" t="n">
         <v>7007.72</v>
+      </c>
+      <c r="BV32" s="15" t="n">
+        <v>7080.92</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
@@ -6619,6 +6700,7 @@
       <c r="BS33" s="15" t="n"/>
       <c r="BT33" s="15" t="n"/>
       <c r="BU33" s="15" t="n"/>
+      <c r="BV33" s="15" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -6839,6 +6921,9 @@
       </c>
       <c r="BU34" s="15" t="n">
         <v>45.3</v>
+      </c>
+      <c r="BV34" s="15" t="n">
+        <v>45.66</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -7012,6 +7097,9 @@
       </c>
       <c r="BU35" s="15" t="n">
         <v>5527.38</v>
+      </c>
+      <c r="BV35" s="15" t="n">
+        <v>5469.4</v>
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
@@ -7136,6 +7224,7 @@
       <c r="BS36" s="15" t="n"/>
       <c r="BT36" s="15" t="n"/>
       <c r="BU36" s="15" t="n"/>
+      <c r="BV36" s="15" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -7356,6 +7445,9 @@
       </c>
       <c r="BU37" s="15" t="n">
         <v>49.69</v>
+      </c>
+      <c r="BV37" s="15" t="n">
+        <v>49.82</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -7529,6 +7621,9 @@
       </c>
       <c r="BU38" s="15" t="n">
         <v>11175.12</v>
+      </c>
+      <c r="BV38" s="15" t="n">
+        <v>11114.77</v>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
@@ -7653,6 +7748,7 @@
       <c r="BS39" s="15" t="n"/>
       <c r="BT39" s="15" t="n"/>
       <c r="BU39" s="15" t="n"/>
+      <c r="BV39" s="15" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -7873,6 +7969,9 @@
       </c>
       <c r="BU40" s="15" t="n">
         <v>47.86</v>
+      </c>
+      <c r="BV40" s="15" t="n">
+        <v>47.88</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -8046,6 +8145,9 @@
       </c>
       <c r="BU41" s="15" t="n">
         <v>10871.21</v>
+      </c>
+      <c r="BV41" s="15" t="n">
+        <v>10847.74</v>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
@@ -8170,6 +8272,7 @@
       <c r="BS42" s="15" t="n"/>
       <c r="BT42" s="15" t="n"/>
       <c r="BU42" s="15" t="n"/>
+      <c r="BV42" s="15" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -8390,6 +8493,9 @@
       </c>
       <c r="BU43" s="15" t="n">
         <v>49</v>
+      </c>
+      <c r="BV43" s="15" t="n">
+        <v>48.53</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -8563,6 +8669,9 @@
       </c>
       <c r="BU44" s="15" t="n">
         <v>3246.18</v>
+      </c>
+      <c r="BV44" s="15" t="n">
+        <v>3261.84</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
@@ -8687,6 +8796,7 @@
       <c r="BS45" s="15" t="n"/>
       <c r="BT45" s="15" t="n"/>
       <c r="BU45" s="15" t="n"/>
+      <c r="BV45" s="15" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -8907,6 +9017,9 @@
       </c>
       <c r="BU46" s="15" t="n">
         <v>51.61</v>
+      </c>
+      <c r="BV46" s="15" t="n">
+        <v>50.8</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -9080,6 +9193,9 @@
       </c>
       <c r="BU47" s="15" t="n">
         <v>6948.44</v>
+      </c>
+      <c r="BV47" s="15" t="n">
+        <v>6925.02</v>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
@@ -9204,6 +9320,7 @@
       <c r="BS48" s="15" t="n"/>
       <c r="BT48" s="15" t="n"/>
       <c r="BU48" s="15" t="n"/>
+      <c r="BV48" s="15" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -9424,6 +9541,9 @@
       </c>
       <c r="BU49" s="15" t="n">
         <v>19.69</v>
+      </c>
+      <c r="BV49" s="15" t="n">
+        <v>20.39</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -9597,6 +9717,9 @@
       </c>
       <c r="BU50" s="15" t="n">
         <v>32761.47</v>
+      </c>
+      <c r="BV50" s="15" t="n">
+        <v>32800.06</v>
       </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
@@ -9721,6 +9844,7 @@
       <c r="BS51" s="15" t="n"/>
       <c r="BT51" s="15" t="n"/>
       <c r="BU51" s="15" t="n"/>
+      <c r="BV51" s="15" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -9941,6 +10065,9 @@
       </c>
       <c r="BU52" s="15" t="n">
         <v>37.41</v>
+      </c>
+      <c r="BV52" s="15" t="n">
+        <v>37.73</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -10114,6 +10241,9 @@
       </c>
       <c r="BU53" s="15" t="n">
         <v>3538.47</v>
+      </c>
+      <c r="BV53" s="15" t="n">
+        <v>3415.1</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
@@ -10238,6 +10368,7 @@
       <c r="BS54" s="15" t="n"/>
       <c r="BT54" s="15" t="n"/>
       <c r="BU54" s="15" t="n"/>
+      <c r="BV54" s="15" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -10458,6 +10589,9 @@
       </c>
       <c r="BU55" s="15" t="n">
         <v>45.41</v>
+      </c>
+      <c r="BV55" s="15" t="n">
+        <v>45.69</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -10631,6 +10765,9 @@
       </c>
       <c r="BU56" s="15" t="n">
         <v>3399.59</v>
+      </c>
+      <c r="BV56" s="15" t="n">
+        <v>3288.95</v>
       </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
@@ -10755,6 +10892,7 @@
       <c r="BS57" s="15" t="n"/>
       <c r="BT57" s="15" t="n"/>
       <c r="BU57" s="15" t="n"/>
+      <c r="BV57" s="15" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -10975,6 +11113,9 @@
       </c>
       <c r="BU58" s="15" t="n">
         <v>15.41</v>
+      </c>
+      <c r="BV58" s="15" t="n">
+        <v>19.43</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -11148,6 +11289,9 @@
       </c>
       <c r="BU59" s="15" t="n">
         <v>6869.19</v>
+      </c>
+      <c r="BV59" s="15" t="n">
+        <v>6731.18</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
@@ -11272,6 +11416,7 @@
       <c r="BS60" s="15" t="n"/>
       <c r="BT60" s="15" t="n"/>
       <c r="BU60" s="15" t="n"/>
+      <c r="BV60" s="15" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -11492,6 +11637,9 @@
       </c>
       <c r="BU61" s="15" t="n">
         <v>30.48</v>
+      </c>
+      <c r="BV61" s="15" t="n">
+        <v>34.86</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -11665,6 +11813,9 @@
       </c>
       <c r="BU62" s="15" t="n">
         <v>8282.4</v>
+      </c>
+      <c r="BV62" s="15" t="n">
+        <v>8034.61</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
@@ -11789,6 +11940,7 @@
       <c r="BS63" s="15" t="n"/>
       <c r="BT63" s="15" t="n"/>
       <c r="BU63" s="15" t="n"/>
+      <c r="BV63" s="15" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -12009,6 +12161,9 @@
       </c>
       <c r="BU64" s="15" t="n">
         <v>6.92</v>
+      </c>
+      <c r="BV64" s="15" t="n">
+        <v>6.6</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -12182,6 +12337,9 @@
       </c>
       <c r="BU65" s="15" t="n">
         <v>10420.45</v>
+      </c>
+      <c r="BV65" s="15" t="n">
+        <v>10367.63</v>
       </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
@@ -12306,6 +12464,7 @@
       <c r="BS66" s="15" t="n"/>
       <c r="BT66" s="15" t="n"/>
       <c r="BU66" s="15" t="n"/>
+      <c r="BV66" s="15" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -12526,6 +12685,9 @@
       </c>
       <c r="BU67" s="15" t="n">
         <v>20.05</v>
+      </c>
+      <c r="BV67" s="15" t="n">
+        <v>19.38</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -12699,6 +12861,9 @@
       </c>
       <c r="BU68" s="15" t="n">
         <v>11220.97</v>
+      </c>
+      <c r="BV68" s="15" t="n">
+        <v>11219.09</v>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
@@ -12823,6 +12988,7 @@
       <c r="BS69" s="15" t="n"/>
       <c r="BT69" s="15" t="n"/>
       <c r="BU69" s="15" t="n"/>
+      <c r="BV69" s="15" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -13043,6 +13209,9 @@
       </c>
       <c r="BU70" s="15" t="n">
         <v>14.61</v>
+      </c>
+      <c r="BV70" s="15" t="n">
+        <v>14.62</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -13216,6 +13385,9 @@
       </c>
       <c r="BU71" s="15" t="n">
         <v>6254.47</v>
+      </c>
+      <c r="BV71" s="15" t="n">
+        <v>6105.76</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
@@ -13340,6 +13512,7 @@
       <c r="BS72" s="15" t="n"/>
       <c r="BT72" s="15" t="n"/>
       <c r="BU72" s="15" t="n"/>
+      <c r="BV72" s="15" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -13560,6 +13733,9 @@
       </c>
       <c r="BU73" s="15" t="n">
         <v>17.07</v>
+      </c>
+      <c r="BV73" s="15" t="n">
+        <v>17.53</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -13733,6 +13909,9 @@
       </c>
       <c r="BU74" s="15" t="n">
         <v>12321.63</v>
+      </c>
+      <c r="BV74" s="15" t="n">
+        <v>12109.54</v>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
@@ -13857,6 +14036,7 @@
       <c r="BS75" s="15" t="n"/>
       <c r="BT75" s="15" t="n"/>
       <c r="BU75" s="15" t="n"/>
+      <c r="BV75" s="15" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -14077,6 +14257,9 @@
       </c>
       <c r="BU76" s="15" t="n">
         <v>52.73</v>
+      </c>
+      <c r="BV76" s="15" t="n">
+        <v>53.91</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -14250,6 +14433,9 @@
       </c>
       <c r="BU77" s="15" t="n">
         <v>16449.57</v>
+      </c>
+      <c r="BV77" s="15" t="n">
+        <v>15569.82</v>
       </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
@@ -14374,6 +14560,7 @@
       <c r="BS78" s="15" t="n"/>
       <c r="BT78" s="15" t="n"/>
       <c r="BU78" s="15" t="n"/>
+      <c r="BV78" s="15" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -14594,6 +14781,9 @@
       </c>
       <c r="BU79" s="15" t="n">
         <v>1.89</v>
+      </c>
+      <c r="BV79" s="15" t="n">
+        <v>3.05</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -14767,6 +14957,9 @@
       </c>
       <c r="BU80" s="15" t="n">
         <v>6593.43</v>
+      </c>
+      <c r="BV80" s="15" t="n">
+        <v>6557.96</v>
       </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
@@ -14891,6 +15084,7 @@
       <c r="BS81" s="15" t="n"/>
       <c r="BT81" s="15" t="n"/>
       <c r="BU81" s="15" t="n"/>
+      <c r="BV81" s="15" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -15111,6 +15305,9 @@
       </c>
       <c r="BU82" s="15" t="n">
         <v>3.19</v>
+      </c>
+      <c r="BV82" s="15" t="n">
+        <v>3.64</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -15284,6 +15481,9 @@
       </c>
       <c r="BU83" s="15" t="n">
         <v>8391.32</v>
+      </c>
+      <c r="BV83" s="15" t="n">
+        <v>8201.43</v>
       </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
@@ -15408,6 +15608,7 @@
       <c r="BS84" s="15" t="n"/>
       <c r="BT84" s="15" t="n"/>
       <c r="BU84" s="15" t="n"/>
+      <c r="BV84" s="15" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -15628,6 +15829,9 @@
       </c>
       <c r="BU85" s="15" t="n">
         <v>16.53</v>
+      </c>
+      <c r="BV85" s="15" t="n">
+        <v>17.32</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -15801,6 +16005,9 @@
       </c>
       <c r="BU86" s="15" t="n">
         <v>2631.9</v>
+      </c>
+      <c r="BV86" s="15" t="n">
+        <v>2071.42</v>
       </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
@@ -15925,6 +16132,7 @@
       <c r="BS87" s="15" t="n"/>
       <c r="BT87" s="15" t="n"/>
       <c r="BU87" s="15" t="n"/>
+      <c r="BV87" s="15" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -16145,6 +16353,9 @@
       </c>
       <c r="BU88" s="15" t="n">
         <v>27.45</v>
+      </c>
+      <c r="BV88" s="15" t="n">
+        <v>27.98</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -16318,6 +16529,9 @@
       </c>
       <c r="BU89" s="15" t="n">
         <v>4423.29</v>
+      </c>
+      <c r="BV89" s="15" t="n">
+        <v>4361.13</v>
       </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
@@ -16442,6 +16656,7 @@
       <c r="BS90" s="15" t="n"/>
       <c r="BT90" s="15" t="n"/>
       <c r="BU90" s="15" t="n"/>
+      <c r="BV90" s="15" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -16662,6 +16877,9 @@
       </c>
       <c r="BU91" s="15" t="n">
         <v>14.11</v>
+      </c>
+      <c r="BV91" s="15" t="n">
+        <v>18.46</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -16835,6 +17053,9 @@
       </c>
       <c r="BU92" s="15" t="n">
         <v>8645.5</v>
+      </c>
+      <c r="BV92" s="15" t="n">
+        <v>8420.93</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
@@ -16959,6 +17180,7 @@
       <c r="BS93" s="15" t="n"/>
       <c r="BT93" s="15" t="n"/>
       <c r="BU93" s="15" t="n"/>
+      <c r="BV93" s="15" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -17179,6 +17401,9 @@
       </c>
       <c r="BU94" s="15" t="n">
         <v>4.46</v>
+      </c>
+      <c r="BV94" s="15" t="n">
+        <v>4.83</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -17352,6 +17577,9 @@
       </c>
       <c r="BU95" s="15" t="n">
         <v>1184.75</v>
+      </c>
+      <c r="BV95" s="15" t="n">
+        <v>1193.12</v>
       </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
@@ -17476,6 +17704,7 @@
       <c r="BS96" s="15" t="n"/>
       <c r="BT96" s="15" t="n"/>
       <c r="BU96" s="15" t="n"/>
+      <c r="BV96" s="15" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -17696,6 +17925,9 @@
       </c>
       <c r="BU97" s="15" t="n">
         <v>8.050000000000001</v>
+      </c>
+      <c r="BV97" s="15" t="n">
+        <v>8.59</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -17869,6 +18101,9 @@
       </c>
       <c r="BU98" s="15" t="n">
         <v>13547.29</v>
+      </c>
+      <c r="BV98" s="15" t="n">
+        <v>13636.38</v>
       </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
@@ -17993,6 +18228,7 @@
       <c r="BS99" s="15" t="n"/>
       <c r="BT99" s="15" t="n"/>
       <c r="BU99" s="15" t="n"/>
+      <c r="BV99" s="15" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -18213,6 +18449,9 @@
       </c>
       <c r="BU100" s="15" t="n">
         <v>32.58</v>
+      </c>
+      <c r="BV100" s="15" t="n">
+        <v>39.06</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -18386,6 +18625,9 @@
       </c>
       <c r="BU101" s="15" t="n">
         <v>3212.94</v>
+      </c>
+      <c r="BV101" s="15" t="n">
+        <v>3342.43</v>
       </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
@@ -18510,6 +18752,7 @@
       <c r="BS102" s="15" t="n"/>
       <c r="BT102" s="15" t="n"/>
       <c r="BU102" s="15" t="n"/>
+      <c r="BV102" s="15" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -18730,6 +18973,9 @@
       </c>
       <c r="BU103" s="15" t="n">
         <v>27.59</v>
+      </c>
+      <c r="BV103" s="15" t="n">
+        <v>26.8</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -18903,6 +19149,9 @@
       </c>
       <c r="BU104" s="15" t="n">
         <v>2267.47</v>
+      </c>
+      <c r="BV104" s="15" t="n">
+        <v>2196.75</v>
       </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
@@ -19027,6 +19276,7 @@
       <c r="BS105" s="15" t="n"/>
       <c r="BT105" s="15" t="n"/>
       <c r="BU105" s="15" t="n"/>
+      <c r="BV105" s="15" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -19247,6 +19497,9 @@
       </c>
       <c r="BU106" s="15" t="n">
         <v>15</v>
+      </c>
+      <c r="BV106" s="15" t="n">
+        <v>14.61</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -19420,6 +19673,9 @@
       </c>
       <c r="BU107" s="15" t="n">
         <v>2330.22</v>
+      </c>
+      <c r="BV107" s="15" t="n">
+        <v>2354.65</v>
       </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
@@ -19544,6 +19800,7 @@
       <c r="BS108" s="15" t="n"/>
       <c r="BT108" s="15" t="n"/>
       <c r="BU108" s="15" t="n"/>
+      <c r="BV108" s="15" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -19764,6 +20021,9 @@
       </c>
       <c r="BU109" s="15" t="n">
         <v>26.46</v>
+      </c>
+      <c r="BV109" s="15" t="n">
+        <v>26.55</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -19937,6 +20197,9 @@
       </c>
       <c r="BU110" s="15" t="n">
         <v>2391.89</v>
+      </c>
+      <c r="BV110" s="15" t="n">
+        <v>2335.61</v>
       </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
@@ -20061,6 +20324,7 @@
       <c r="BS111" s="15" t="n"/>
       <c r="BT111" s="15" t="n"/>
       <c r="BU111" s="15" t="n"/>
+      <c r="BV111" s="15" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -20281,6 +20545,9 @@
       </c>
       <c r="BU112" s="15" t="n">
         <v>46.42</v>
+      </c>
+      <c r="BV112" s="15" t="n">
+        <v>53.44</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -20452,6 +20719,9 @@
       </c>
       <c r="BU113" s="15" t="n">
         <v>1880.2</v>
+      </c>
+      <c r="BV113" s="15" t="n">
+        <v>1959.69</v>
       </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
@@ -20576,6 +20846,7 @@
       <c r="BS114" s="15" t="n"/>
       <c r="BT114" s="15" t="n"/>
       <c r="BU114" s="15" t="n"/>
+      <c r="BV114" s="15" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -20796,6 +21067,9 @@
       </c>
       <c r="BU115" s="15" t="n">
         <v>15.53</v>
+      </c>
+      <c r="BV115" s="15" t="n">
+        <v>18.2</v>
       </c>
     </row>
     <row r="116" ht="14.25" customHeight="1">
@@ -20954,6 +21228,9 @@
       </c>
       <c r="BU116" s="15" t="n">
         <v>8691.26</v>
+      </c>
+      <c r="BV116" s="15" t="n">
+        <v>8784.530000000001</v>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1">
@@ -21033,6 +21310,7 @@
       <c r="BS117" s="15" t="n"/>
       <c r="BT117" s="15" t="n"/>
       <c r="BU117" s="15" t="n"/>
+      <c r="BV117" s="15" t="n"/>
     </row>
     <row r="118" ht="14.25" customHeight="1">
       <c r="P118" s="13" t="n">
@@ -21209,6 +21487,9 @@
       <c r="BU118" s="15" t="n">
         <v>75.48999999999999</v>
       </c>
+      <c r="BV118" s="15" t="n">
+        <v>75.87</v>
+      </c>
     </row>
     <row r="119" ht="14.25" customHeight="1">
       <c r="Y119" s="13" t="n">
@@ -21357,6 +21638,9 @@
       </c>
       <c r="BU119" s="15" t="n">
         <v>13163.37</v>
+      </c>
+      <c r="BV119" s="15" t="n">
+        <v>12900.98</v>
       </c>
     </row>
     <row r="120" ht="14.25" customHeight="1">
@@ -21385,6 +21669,7 @@
       <c r="BS120" s="15" t="n"/>
       <c r="BT120" s="15" t="n"/>
       <c r="BU120" s="15" t="n"/>
+      <c r="BV120" s="15" t="n"/>
     </row>
     <row r="121" ht="14.25" customHeight="1">
       <c r="AW121" s="13" t="n">
@@ -21462,6 +21747,9 @@
       <c r="BU121" s="15" t="n">
         <v>23.75</v>
       </c>
+      <c r="BV121" s="15" t="n">
+        <v>24.19</v>
+      </c>
     </row>
     <row r="122" ht="14.25" customHeight="1">
       <c r="AW122" s="13" t="n">
@@ -21538,6 +21826,9 @@
       </c>
       <c r="BU122" s="15" t="n">
         <v>1198.64</v>
+      </c>
+      <c r="BV122" s="15" t="n">
+        <v>1196.23</v>
       </c>
     </row>
     <row r="123" ht="14.25" customHeight="1">
@@ -21566,6 +21857,7 @@
       <c r="BS123" s="15" t="n"/>
       <c r="BT123" s="15" t="n"/>
       <c r="BU123" s="15" t="n"/>
+      <c r="BV123" s="15" t="n"/>
     </row>
     <row r="124" ht="14.25" customHeight="1">
       <c r="AW124" s="13" t="n">
@@ -21643,6 +21935,9 @@
       <c r="BU124" s="15" t="n">
         <v>48.61</v>
       </c>
+      <c r="BV124" s="15" t="n">
+        <v>47.15</v>
+      </c>
     </row>
     <row r="125" ht="14.25" customHeight="1">
       <c r="AW125" s="13" t="n">
@@ -21719,6 +22014,9 @@
       </c>
       <c r="BU125" s="15" t="n">
         <v>11895.94</v>
+      </c>
+      <c r="BV125" s="15" t="n">
+        <v>11436.37</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1">
@@ -21747,6 +22045,7 @@
       <c r="BS126" s="15" t="n"/>
       <c r="BT126" s="15" t="n"/>
       <c r="BU126" s="15" t="n"/>
+      <c r="BV126" s="15" t="n"/>
     </row>
     <row r="127" ht="14.25" customHeight="1">
       <c r="AW127" s="13" t="n">
@@ -21824,6 +22123,9 @@
       <c r="BU127" s="15" t="n">
         <v>4.25</v>
       </c>
+      <c r="BV127" s="15" t="n">
+        <v>4.31</v>
+      </c>
     </row>
     <row r="128" ht="14.25" customHeight="1">
       <c r="AW128" s="13" t="n">
@@ -21900,6 +22202,9 @@
       </c>
       <c r="BU128" s="15" t="n">
         <v>1855.25</v>
+      </c>
+      <c r="BV128" s="15" t="n">
+        <v>1813.99</v>
       </c>
     </row>
     <row r="129" ht="14.25" customHeight="1">
@@ -21928,6 +22233,7 @@
       <c r="BS129" s="15" t="n"/>
       <c r="BT129" s="15" t="n"/>
       <c r="BU129" s="15" t="n"/>
+      <c r="BV129" s="15" t="n"/>
     </row>
     <row r="130" ht="14.25" customHeight="1">
       <c r="AW130" s="13" t="n">
@@ -22005,6 +22311,9 @@
       <c r="BU130" s="15" t="n">
         <v>7.3</v>
       </c>
+      <c r="BV130" s="15" t="n">
+        <v>8.26</v>
+      </c>
     </row>
     <row r="131" ht="14.25" customHeight="1">
       <c r="AW131" s="13" t="n">
@@ -22081,6 +22390,9 @@
       </c>
       <c r="BU131" s="15" t="n">
         <v>742.3099999999999</v>
+      </c>
+      <c r="BV131" s="15" t="n">
+        <v>726.62</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1">
@@ -22109,6 +22421,7 @@
       <c r="BS132" s="15" t="n"/>
       <c r="BT132" s="15" t="n"/>
       <c r="BU132" s="15" t="n"/>
+      <c r="BV132" s="15" t="n"/>
     </row>
     <row r="133" ht="14.25" customHeight="1">
       <c r="AW133" s="13" t="n">
@@ -22186,6 +22499,9 @@
       <c r="BU133" s="15" t="n">
         <v>56.92</v>
       </c>
+      <c r="BV133" s="15" t="n">
+        <v>54.57</v>
+      </c>
     </row>
     <row r="134" ht="14.25" customHeight="1">
       <c r="AW134" s="13" t="n">
@@ -22262,6 +22578,9 @@
       </c>
       <c r="BU134" s="15" t="n">
         <v>2851.18</v>
+      </c>
+      <c r="BV134" s="15" t="n">
+        <v>2738.48</v>
       </c>
     </row>
     <row r="135" ht="14.25" customHeight="1">
@@ -22290,6 +22609,7 @@
       <c r="BS135" s="15" t="n"/>
       <c r="BT135" s="15" t="n"/>
       <c r="BU135" s="15" t="n"/>
+      <c r="BV135" s="15" t="n"/>
     </row>
     <row r="136" ht="14.25" customHeight="1">
       <c r="AW136" s="13" t="n">
@@ -22367,6 +22687,9 @@
       <c r="BU136" s="15" t="n">
         <v>21.89</v>
       </c>
+      <c r="BV136" s="15" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="137" ht="14.25" customHeight="1">
       <c r="AW137" s="13" t="n">
@@ -22443,6 +22766,9 @@
       </c>
       <c r="BU137" s="15" t="n">
         <v>3561.44</v>
+      </c>
+      <c r="BV137" s="15" t="n">
+        <v>3486.51</v>
       </c>
     </row>
     <row r="138">
@@ -22463,6 +22789,7 @@
       <c r="BS138" s="15" t="n"/>
       <c r="BT138" s="15" t="n"/>
       <c r="BU138" s="15" t="n"/>
+      <c r="BV138" s="15" t="n"/>
     </row>
     <row r="139">
       <c r="BE139" s="15" t="n">
@@ -22516,6 +22843,9 @@
       <c r="BU139" s="15" t="n">
         <v>4.44</v>
       </c>
+      <c r="BV139" s="15" t="n">
+        <v>5.02</v>
+      </c>
     </row>
     <row r="140">
       <c r="BE140" s="15" t="n">
@@ -22569,6 +22899,7 @@
       <c r="BU140" s="15" t="n">
         <v>2351.96</v>
       </c>
+      <c r="BV140" s="15" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="BE141" s="15" t="n"/>
@@ -22588,6 +22919,7 @@
       <c r="BS141" s="15" t="n"/>
       <c r="BT141" s="15" t="n"/>
       <c r="BU141" s="15" t="n"/>
+      <c r="BV141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="BE142" s="15" t="n">
@@ -22641,6 +22973,9 @@
       <c r="BU142" s="15" t="n">
         <v>17.94</v>
       </c>
+      <c r="BV142" s="15" t="n">
+        <v>17.48</v>
+      </c>
     </row>
     <row r="143">
       <c r="BE143" s="15" t="n">
@@ -22693,6 +23028,9 @@
       </c>
       <c r="BU143" s="15" t="n">
         <v>5687.43</v>
+      </c>
+      <c r="BV143" s="15" t="n">
+        <v>5654.84</v>
       </c>
     </row>
     <row r="144">
@@ -22708,6 +23046,7 @@
       <c r="BS144" s="15" t="n"/>
       <c r="BT144" s="15" t="n"/>
       <c r="BU144" s="15" t="n"/>
+      <c r="BV144" s="15" t="n"/>
     </row>
     <row r="145">
       <c r="BJ145" s="15" t="n">
@@ -22746,6 +23085,9 @@
       <c r="BU145" s="15" t="n">
         <v>1.86</v>
       </c>
+      <c r="BV145" s="15" t="n">
+        <v>2.26</v>
+      </c>
     </row>
     <row r="146">
       <c r="BJ146" s="15" t="n">
@@ -22783,6 +23125,9 @@
       </c>
       <c r="BU146" s="15" t="n">
         <v>2232.84</v>
+      </c>
+      <c r="BV146" s="15" t="n">
+        <v>2248.48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-09-26 11:53:45]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BV146"/>
+  <dimension ref="A1:BW146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="51"/>
@@ -608,6 +608,7 @@
     <col width="15" customWidth="1" min="72" max="72"/>
     <col width="15" customWidth="1" min="73" max="73"/>
     <col width="15" customWidth="1" min="74" max="74"/>
+    <col width="15" customWidth="1" min="75" max="75"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -981,6 +982,11 @@
           <t>2026/09/24</t>
         </is>
       </c>
+      <c r="BW1" s="15" t="inlineStr">
+        <is>
+          <t>2026/09/26</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1353,6 +1359,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="BW2" s="16" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1577,6 +1588,9 @@
       <c r="BV3" s="15" t="n">
         <v>60.52</v>
       </c>
+      <c r="BW3" s="15" t="n">
+        <v>59.66</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1799,6 +1813,9 @@
         <v>3949.91</v>
       </c>
       <c r="BV4" s="15" t="n">
+        <v>3888.37</v>
+      </c>
+      <c r="BW4" s="15" t="n">
         <v>3888.37</v>
       </c>
     </row>
@@ -1877,6 +1894,7 @@
       <c r="BT5" s="15" t="n"/>
       <c r="BU5" s="15" t="n"/>
       <c r="BV5" s="15" t="n"/>
+      <c r="BW5" s="15" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -2001,6 +2019,7 @@
       <c r="BT6" s="15" t="n"/>
       <c r="BU6" s="15" t="n"/>
       <c r="BV6" s="15" t="n"/>
+      <c r="BW6" s="15" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -2224,6 +2243,9 @@
       </c>
       <c r="BV7" s="15" t="n">
         <v>52.98</v>
+      </c>
+      <c r="BW7" s="15" t="n">
+        <v>49.88</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -2399,6 +2421,9 @@
         <v>5626.57</v>
       </c>
       <c r="BV8" s="15" t="n">
+        <v>5486.01</v>
+      </c>
+      <c r="BW8" s="15" t="n">
         <v>5486.01</v>
       </c>
     </row>
@@ -2525,6 +2550,7 @@
       <c r="BT9" s="15" t="n"/>
       <c r="BU9" s="15" t="n"/>
       <c r="BV9" s="15" t="n"/>
+      <c r="BW9" s="15" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -2748,6 +2774,9 @@
       </c>
       <c r="BV10" s="15" t="n">
         <v>47.36</v>
+      </c>
+      <c r="BW10" s="15" t="n">
+        <v>44.58</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -2923,6 +2952,9 @@
         <v>4539.57</v>
       </c>
       <c r="BV11" s="15" t="n">
+        <v>4439.14</v>
+      </c>
+      <c r="BW11" s="15" t="n">
         <v>4439.14</v>
       </c>
     </row>
@@ -3049,6 +3081,7 @@
       <c r="BT12" s="15" t="n"/>
       <c r="BU12" s="15" t="n"/>
       <c r="BV12" s="15" t="n"/>
+      <c r="BW12" s="15" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -3272,6 +3305,9 @@
       </c>
       <c r="BV13" s="15" t="n">
         <v>60.7</v>
+      </c>
+      <c r="BW13" s="15" t="n">
+        <v>58.12</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -3447,6 +3483,9 @@
         <v>7850.48</v>
       </c>
       <c r="BV14" s="15" t="n">
+        <v>7624.07</v>
+      </c>
+      <c r="BW14" s="15" t="n">
         <v>7624.07</v>
       </c>
     </row>
@@ -3573,6 +3612,7 @@
       <c r="BT15" s="15" t="n"/>
       <c r="BU15" s="15" t="n"/>
       <c r="BV15" s="15" t="n"/>
+      <c r="BW15" s="15" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -3796,6 +3836,9 @@
       </c>
       <c r="BV16" s="15" t="n">
         <v>27.98</v>
+      </c>
+      <c r="BW16" s="15" t="n">
+        <v>27.42</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -3971,6 +4014,9 @@
         <v>2538.47</v>
       </c>
       <c r="BV17" s="15" t="n">
+        <v>2495.36</v>
+      </c>
+      <c r="BW17" s="15" t="n">
         <v>2495.36</v>
       </c>
     </row>
@@ -4097,6 +4143,7 @@
       <c r="BT18" s="15" t="n"/>
       <c r="BU18" s="15" t="n"/>
       <c r="BV18" s="15" t="n"/>
+      <c r="BW18" s="15" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -4319,6 +4366,9 @@
         <v>80.12</v>
       </c>
       <c r="BV19" s="15" t="n">
+        <v>80.64</v>
+      </c>
+      <c r="BW19" s="15" t="n">
         <v>80.64</v>
       </c>
     </row>
@@ -4496,6 +4546,9 @@
       </c>
       <c r="BV20" s="15" t="n">
         <v>7706.03</v>
+      </c>
+      <c r="BW20" s="15" t="n">
+        <v>7743.41</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
@@ -4621,6 +4674,7 @@
       <c r="BT21" s="15" t="n"/>
       <c r="BU21" s="15" t="n"/>
       <c r="BV21" s="15" t="n"/>
+      <c r="BW21" s="15" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -4841,6 +4895,9 @@
         <v>36.34</v>
       </c>
       <c r="BV22" s="15" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="BW22" s="15" t="n">
         <v>36.34</v>
       </c>
     </row>
@@ -5018,6 +5075,9 @@
       </c>
       <c r="BV23" s="15" t="n">
         <v>73647.46000000001</v>
+      </c>
+      <c r="BW23" s="15" t="n">
+        <v>73895.74000000001</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
@@ -5143,6 +5203,7 @@
       <c r="BT24" s="15" t="n"/>
       <c r="BU24" s="15" t="n"/>
       <c r="BV24" s="15" t="n"/>
+      <c r="BW24" s="15" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -5365,6 +5426,9 @@
         <v>49.88</v>
       </c>
       <c r="BV25" s="15" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="BW25" s="15" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -5528,6 +5592,9 @@
       </c>
       <c r="BV26" s="15" t="n">
         <v>25178.08</v>
+      </c>
+      <c r="BW26" s="15" t="n">
+        <v>25408.64</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
@@ -5653,6 +5720,7 @@
       <c r="BT27" s="15" t="n"/>
       <c r="BU27" s="15" t="n"/>
       <c r="BV27" s="15" t="n"/>
+      <c r="BW27" s="15" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -5875,6 +5943,9 @@
         <v>92.09</v>
       </c>
       <c r="BV28" s="15" t="n">
+        <v>92.09</v>
+      </c>
+      <c r="BW28" s="15" t="n">
         <v>92.09</v>
       </c>
     </row>
@@ -6052,6 +6123,9 @@
       </c>
       <c r="BV29" s="15" t="n">
         <v>65513.99</v>
+      </c>
+      <c r="BW29" s="15" t="n">
+        <v>66364.2</v>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
@@ -6177,6 +6251,7 @@
       <c r="BT30" s="15" t="n"/>
       <c r="BU30" s="15" t="n"/>
       <c r="BV30" s="15" t="n"/>
+      <c r="BW30" s="15" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -6399,6 +6474,9 @@
         <v>97.44</v>
       </c>
       <c r="BV31" s="15" t="n">
+        <v>97.44</v>
+      </c>
+      <c r="BW31" s="15" t="n">
         <v>97.44</v>
       </c>
     </row>
@@ -6575,6 +6653,9 @@
         <v>7007.72</v>
       </c>
       <c r="BV32" s="15" t="n">
+        <v>7080.92</v>
+      </c>
+      <c r="BW32" s="15" t="n">
         <v>7080.92</v>
       </c>
     </row>
@@ -6701,6 +6782,7 @@
       <c r="BT33" s="15" t="n"/>
       <c r="BU33" s="15" t="n"/>
       <c r="BV33" s="15" t="n"/>
+      <c r="BW33" s="15" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -6924,6 +7006,9 @@
       </c>
       <c r="BV34" s="15" t="n">
         <v>45.66</v>
+      </c>
+      <c r="BW34" s="15" t="n">
+        <v>45.51</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -7099,6 +7184,9 @@
         <v>5527.38</v>
       </c>
       <c r="BV35" s="15" t="n">
+        <v>5469.4</v>
+      </c>
+      <c r="BW35" s="15" t="n">
         <v>5469.4</v>
       </c>
     </row>
@@ -7225,6 +7313,7 @@
       <c r="BT36" s="15" t="n"/>
       <c r="BU36" s="15" t="n"/>
       <c r="BV36" s="15" t="n"/>
+      <c r="BW36" s="15" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -7448,6 +7537,9 @@
       </c>
       <c r="BV37" s="15" t="n">
         <v>49.82</v>
+      </c>
+      <c r="BW37" s="15" t="n">
+        <v>50.37</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -7623,6 +7715,9 @@
         <v>11175.12</v>
       </c>
       <c r="BV38" s="15" t="n">
+        <v>11114.77</v>
+      </c>
+      <c r="BW38" s="15" t="n">
         <v>11114.77</v>
       </c>
     </row>
@@ -7749,6 +7844,7 @@
       <c r="BT39" s="15" t="n"/>
       <c r="BU39" s="15" t="n"/>
       <c r="BV39" s="15" t="n"/>
+      <c r="BW39" s="15" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -7972,6 +8068,9 @@
       </c>
       <c r="BV40" s="15" t="n">
         <v>47.88</v>
+      </c>
+      <c r="BW40" s="15" t="n">
+        <v>48.39</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -8148,6 +8247,9 @@
       </c>
       <c r="BV41" s="15" t="n">
         <v>10847.74</v>
+      </c>
+      <c r="BW41" s="15" t="n">
+        <v>10848.95</v>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
@@ -8273,6 +8375,7 @@
       <c r="BT42" s="15" t="n"/>
       <c r="BU42" s="15" t="n"/>
       <c r="BV42" s="15" t="n"/>
+      <c r="BW42" s="15" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -8496,6 +8599,9 @@
       </c>
       <c r="BV43" s="15" t="n">
         <v>48.53</v>
+      </c>
+      <c r="BW43" s="15" t="n">
+        <v>48.99</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -8672,6 +8778,9 @@
       </c>
       <c r="BV44" s="15" t="n">
         <v>3261.84</v>
+      </c>
+      <c r="BW44" s="15" t="n">
+        <v>3263.3</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
@@ -8797,6 +8906,7 @@
       <c r="BT45" s="15" t="n"/>
       <c r="BU45" s="15" t="n"/>
       <c r="BV45" s="15" t="n"/>
+      <c r="BW45" s="15" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -9020,6 +9130,9 @@
       </c>
       <c r="BV46" s="15" t="n">
         <v>50.8</v>
+      </c>
+      <c r="BW46" s="15" t="n">
+        <v>52.54</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -9196,6 +9309,9 @@
       </c>
       <c r="BV47" s="15" t="n">
         <v>6925.02</v>
+      </c>
+      <c r="BW47" s="15" t="n">
+        <v>6935.79</v>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
@@ -9321,6 +9437,7 @@
       <c r="BT48" s="15" t="n"/>
       <c r="BU48" s="15" t="n"/>
       <c r="BV48" s="15" t="n"/>
+      <c r="BW48" s="15" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -9544,6 +9661,9 @@
       </c>
       <c r="BV49" s="15" t="n">
         <v>20.39</v>
+      </c>
+      <c r="BW49" s="15" t="n">
+        <v>19.41</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -9720,6 +9840,9 @@
       </c>
       <c r="BV50" s="15" t="n">
         <v>32800.06</v>
+      </c>
+      <c r="BW50" s="15" t="n">
+        <v>32175.64</v>
       </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
@@ -9845,6 +9968,7 @@
       <c r="BT51" s="15" t="n"/>
       <c r="BU51" s="15" t="n"/>
       <c r="BV51" s="15" t="n"/>
+      <c r="BW51" s="15" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -10068,6 +10192,9 @@
       </c>
       <c r="BV52" s="15" t="n">
         <v>37.73</v>
+      </c>
+      <c r="BW52" s="15" t="n">
+        <v>34.84</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -10243,6 +10370,9 @@
         <v>3538.47</v>
       </c>
       <c r="BV53" s="15" t="n">
+        <v>3415.1</v>
+      </c>
+      <c r="BW53" s="15" t="n">
         <v>3415.1</v>
       </c>
     </row>
@@ -10369,6 +10499,7 @@
       <c r="BT54" s="15" t="n"/>
       <c r="BU54" s="15" t="n"/>
       <c r="BV54" s="15" t="n"/>
+      <c r="BW54" s="15" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -10592,6 +10723,9 @@
       </c>
       <c r="BV55" s="15" t="n">
         <v>45.69</v>
+      </c>
+      <c r="BW55" s="15" t="n">
+        <v>42.37</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -10767,6 +10901,9 @@
         <v>3399.59</v>
       </c>
       <c r="BV56" s="15" t="n">
+        <v>3288.95</v>
+      </c>
+      <c r="BW56" s="15" t="n">
         <v>3288.95</v>
       </c>
     </row>
@@ -10893,6 +11030,7 @@
       <c r="BT57" s="15" t="n"/>
       <c r="BU57" s="15" t="n"/>
       <c r="BV57" s="15" t="n"/>
+      <c r="BW57" s="15" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -11116,6 +11254,9 @@
       </c>
       <c r="BV58" s="15" t="n">
         <v>19.43</v>
+      </c>
+      <c r="BW58" s="15" t="n">
+        <v>16.66</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -11291,6 +11432,9 @@
         <v>6869.19</v>
       </c>
       <c r="BV59" s="15" t="n">
+        <v>6731.18</v>
+      </c>
+      <c r="BW59" s="15" t="n">
         <v>6731.18</v>
       </c>
     </row>
@@ -11417,6 +11561,7 @@
       <c r="BT60" s="15" t="n"/>
       <c r="BU60" s="15" t="n"/>
       <c r="BV60" s="15" t="n"/>
+      <c r="BW60" s="15" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -11640,6 +11785,9 @@
       </c>
       <c r="BV61" s="15" t="n">
         <v>34.86</v>
+      </c>
+      <c r="BW61" s="15" t="n">
+        <v>30.91</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -11815,6 +11963,9 @@
         <v>8282.4</v>
       </c>
       <c r="BV62" s="15" t="n">
+        <v>8034.61</v>
+      </c>
+      <c r="BW62" s="15" t="n">
         <v>8034.61</v>
       </c>
     </row>
@@ -11941,6 +12092,7 @@
       <c r="BT63" s="15" t="n"/>
       <c r="BU63" s="15" t="n"/>
       <c r="BV63" s="15" t="n"/>
+      <c r="BW63" s="15" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -12164,6 +12316,9 @@
       </c>
       <c r="BV64" s="15" t="n">
         <v>6.6</v>
+      </c>
+      <c r="BW64" s="15" t="n">
+        <v>5.41</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -12339,6 +12494,9 @@
         <v>10420.45</v>
       </c>
       <c r="BV65" s="15" t="n">
+        <v>10367.63</v>
+      </c>
+      <c r="BW65" s="15" t="n">
         <v>10367.63</v>
       </c>
     </row>
@@ -12465,6 +12623,7 @@
       <c r="BT66" s="15" t="n"/>
       <c r="BU66" s="15" t="n"/>
       <c r="BV66" s="15" t="n"/>
+      <c r="BW66" s="15" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -12688,6 +12847,9 @@
       </c>
       <c r="BV67" s="15" t="n">
         <v>19.38</v>
+      </c>
+      <c r="BW67" s="15" t="n">
+        <v>19.02</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -12863,6 +13025,9 @@
         <v>11220.97</v>
       </c>
       <c r="BV68" s="15" t="n">
+        <v>11219.09</v>
+      </c>
+      <c r="BW68" s="15" t="n">
         <v>11219.09</v>
       </c>
     </row>
@@ -12989,6 +13154,7 @@
       <c r="BT69" s="15" t="n"/>
       <c r="BU69" s="15" t="n"/>
       <c r="BV69" s="15" t="n"/>
+      <c r="BW69" s="15" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -13212,6 +13378,9 @@
       </c>
       <c r="BV70" s="15" t="n">
         <v>14.62</v>
+      </c>
+      <c r="BW70" s="15" t="n">
+        <v>12.82</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -13387,6 +13556,9 @@
         <v>6254.47</v>
       </c>
       <c r="BV71" s="15" t="n">
+        <v>6105.76</v>
+      </c>
+      <c r="BW71" s="15" t="n">
         <v>6105.76</v>
       </c>
     </row>
@@ -13513,6 +13685,7 @@
       <c r="BT72" s="15" t="n"/>
       <c r="BU72" s="15" t="n"/>
       <c r="BV72" s="15" t="n"/>
+      <c r="BW72" s="15" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -13736,6 +13909,9 @@
       </c>
       <c r="BV73" s="15" t="n">
         <v>17.53</v>
+      </c>
+      <c r="BW73" s="15" t="n">
+        <v>16.36</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -13911,6 +14087,9 @@
         <v>12321.63</v>
       </c>
       <c r="BV74" s="15" t="n">
+        <v>12109.54</v>
+      </c>
+      <c r="BW74" s="15" t="n">
         <v>12109.54</v>
       </c>
     </row>
@@ -14037,6 +14216,7 @@
       <c r="BT75" s="15" t="n"/>
       <c r="BU75" s="15" t="n"/>
       <c r="BV75" s="15" t="n"/>
+      <c r="BW75" s="15" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -14260,6 +14440,9 @@
       </c>
       <c r="BV76" s="15" t="n">
         <v>53.91</v>
+      </c>
+      <c r="BW76" s="15" t="n">
+        <v>53.09</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -14435,6 +14618,9 @@
         <v>16449.57</v>
       </c>
       <c r="BV77" s="15" t="n">
+        <v>15569.82</v>
+      </c>
+      <c r="BW77" s="15" t="n">
         <v>15569.82</v>
       </c>
     </row>
@@ -14561,6 +14747,7 @@
       <c r="BT78" s="15" t="n"/>
       <c r="BU78" s="15" t="n"/>
       <c r="BV78" s="15" t="n"/>
+      <c r="BW78" s="15" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -14784,6 +14971,9 @@
       </c>
       <c r="BV79" s="15" t="n">
         <v>3.05</v>
+      </c>
+      <c r="BW79" s="15" t="n">
+        <v>2.88</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -14959,6 +15149,9 @@
         <v>6593.43</v>
       </c>
       <c r="BV80" s="15" t="n">
+        <v>6557.96</v>
+      </c>
+      <c r="BW80" s="15" t="n">
         <v>6557.96</v>
       </c>
     </row>
@@ -15085,6 +15278,7 @@
       <c r="BT81" s="15" t="n"/>
       <c r="BU81" s="15" t="n"/>
       <c r="BV81" s="15" t="n"/>
+      <c r="BW81" s="15" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -15308,6 +15502,9 @@
       </c>
       <c r="BV82" s="15" t="n">
         <v>3.64</v>
+      </c>
+      <c r="BW82" s="15" t="n">
+        <v>2.92</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -15484,6 +15681,9 @@
       </c>
       <c r="BV83" s="15" t="n">
         <v>8201.43</v>
+      </c>
+      <c r="BW83" s="15" t="n">
+        <v>8161.87</v>
       </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
@@ -15609,6 +15809,7 @@
       <c r="BT84" s="15" t="n"/>
       <c r="BU84" s="15" t="n"/>
       <c r="BV84" s="15" t="n"/>
+      <c r="BW84" s="15" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -15832,6 +16033,9 @@
       </c>
       <c r="BV85" s="15" t="n">
         <v>17.32</v>
+      </c>
+      <c r="BW85" s="15" t="n">
+        <v>16.57</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -16008,6 +16212,9 @@
       </c>
       <c r="BV86" s="15" t="n">
         <v>2071.42</v>
+      </c>
+      <c r="BW86" s="15" t="n">
+        <v>2040.14</v>
       </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
@@ -16133,6 +16340,7 @@
       <c r="BT87" s="15" t="n"/>
       <c r="BU87" s="15" t="n"/>
       <c r="BV87" s="15" t="n"/>
+      <c r="BW87" s="15" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -16356,6 +16564,9 @@
       </c>
       <c r="BV88" s="15" t="n">
         <v>27.98</v>
+      </c>
+      <c r="BW88" s="15" t="n">
+        <v>26.28</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -16532,6 +16743,9 @@
       </c>
       <c r="BV89" s="15" t="n">
         <v>4361.13</v>
+      </c>
+      <c r="BW89" s="15" t="n">
+        <v>5075.31</v>
       </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
@@ -16657,6 +16871,7 @@
       <c r="BT90" s="15" t="n"/>
       <c r="BU90" s="15" t="n"/>
       <c r="BV90" s="15" t="n"/>
+      <c r="BW90" s="15" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -16880,6 +17095,9 @@
       </c>
       <c r="BV91" s="15" t="n">
         <v>18.46</v>
+      </c>
+      <c r="BW91" s="15" t="n">
+        <v>14.86</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -17055,6 +17273,9 @@
         <v>8645.5</v>
       </c>
       <c r="BV92" s="15" t="n">
+        <v>8420.93</v>
+      </c>
+      <c r="BW92" s="15" t="n">
         <v>8420.93</v>
       </c>
     </row>
@@ -17181,6 +17402,7 @@
       <c r="BT93" s="15" t="n"/>
       <c r="BU93" s="15" t="n"/>
       <c r="BV93" s="15" t="n"/>
+      <c r="BW93" s="15" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -17404,6 +17626,9 @@
       </c>
       <c r="BV94" s="15" t="n">
         <v>4.83</v>
+      </c>
+      <c r="BW94" s="15" t="n">
+        <v>3.9</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -17580,6 +17805,9 @@
       </c>
       <c r="BV95" s="15" t="n">
         <v>1193.12</v>
+      </c>
+      <c r="BW95" s="15" t="n">
+        <v>1176.71</v>
       </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
@@ -17705,6 +17933,7 @@
       <c r="BT96" s="15" t="n"/>
       <c r="BU96" s="15" t="n"/>
       <c r="BV96" s="15" t="n"/>
+      <c r="BW96" s="15" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -17928,6 +18157,9 @@
       </c>
       <c r="BV97" s="15" t="n">
         <v>8.59</v>
+      </c>
+      <c r="BW97" s="15" t="n">
+        <v>7.75</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -18104,6 +18336,9 @@
       </c>
       <c r="BV98" s="15" t="n">
         <v>13636.38</v>
+      </c>
+      <c r="BW98" s="15" t="n">
+        <v>13458.58</v>
       </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
@@ -18229,6 +18464,7 @@
       <c r="BT99" s="15" t="n"/>
       <c r="BU99" s="15" t="n"/>
       <c r="BV99" s="15" t="n"/>
+      <c r="BW99" s="15" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -18452,6 +18688,9 @@
       </c>
       <c r="BV100" s="15" t="n">
         <v>39.06</v>
+      </c>
+      <c r="BW100" s="15" t="n">
+        <v>34.57</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -18628,6 +18867,9 @@
       </c>
       <c r="BV101" s="15" t="n">
         <v>3342.43</v>
+      </c>
+      <c r="BW101" s="15" t="n">
+        <v>3257.76</v>
       </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
@@ -18753,6 +18995,7 @@
       <c r="BT102" s="15" t="n"/>
       <c r="BU102" s="15" t="n"/>
       <c r="BV102" s="15" t="n"/>
+      <c r="BW102" s="15" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -18976,6 +19219,9 @@
       </c>
       <c r="BV103" s="15" t="n">
         <v>26.8</v>
+      </c>
+      <c r="BW103" s="15" t="n">
+        <v>24.74</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -19151,6 +19397,9 @@
         <v>2267.47</v>
       </c>
       <c r="BV104" s="15" t="n">
+        <v>2196.75</v>
+      </c>
+      <c r="BW104" s="15" t="n">
         <v>2196.75</v>
       </c>
     </row>
@@ -19277,6 +19526,7 @@
       <c r="BT105" s="15" t="n"/>
       <c r="BU105" s="15" t="n"/>
       <c r="BV105" s="15" t="n"/>
+      <c r="BW105" s="15" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -19500,6 +19750,9 @@
       </c>
       <c r="BV106" s="15" t="n">
         <v>14.61</v>
+      </c>
+      <c r="BW106" s="15" t="n">
+        <v>15.91</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -19676,6 +19929,9 @@
       </c>
       <c r="BV107" s="15" t="n">
         <v>2354.65</v>
+      </c>
+      <c r="BW107" s="15" t="n">
+        <v>2333.92</v>
       </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
@@ -19801,6 +20057,7 @@
       <c r="BT108" s="15" t="n"/>
       <c r="BU108" s="15" t="n"/>
       <c r="BV108" s="15" t="n"/>
+      <c r="BW108" s="15" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -20024,6 +20281,9 @@
       </c>
       <c r="BV109" s="15" t="n">
         <v>26.55</v>
+      </c>
+      <c r="BW109" s="15" t="n">
+        <v>25.78</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -20200,6 +20460,9 @@
       </c>
       <c r="BV110" s="15" t="n">
         <v>2335.61</v>
+      </c>
+      <c r="BW110" s="15" t="n">
+        <v>2391.95</v>
       </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
@@ -20325,6 +20588,7 @@
       <c r="BT111" s="15" t="n"/>
       <c r="BU111" s="15" t="n"/>
       <c r="BV111" s="15" t="n"/>
+      <c r="BW111" s="15" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -20548,6 +20812,9 @@
       </c>
       <c r="BV112" s="15" t="n">
         <v>53.44</v>
+      </c>
+      <c r="BW112" s="15" t="n">
+        <v>47.56</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -20722,6 +20989,9 @@
       </c>
       <c r="BV113" s="15" t="n">
         <v>1959.69</v>
+      </c>
+      <c r="BW113" s="15" t="n">
+        <v>1892.25</v>
       </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
@@ -20847,6 +21117,7 @@
       <c r="BT114" s="15" t="n"/>
       <c r="BU114" s="15" t="n"/>
       <c r="BV114" s="15" t="n"/>
+      <c r="BW114" s="15" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -21070,6 +21341,9 @@
       </c>
       <c r="BV115" s="15" t="n">
         <v>18.2</v>
+      </c>
+      <c r="BW115" s="15" t="n">
+        <v>16.88</v>
       </c>
     </row>
     <row r="116" ht="14.25" customHeight="1">
@@ -21231,6 +21505,9 @@
       </c>
       <c r="BV116" s="15" t="n">
         <v>8784.530000000001</v>
+      </c>
+      <c r="BW116" s="15" t="n">
+        <v>8720.299999999999</v>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1">
@@ -21311,6 +21588,7 @@
       <c r="BT117" s="15" t="n"/>
       <c r="BU117" s="15" t="n"/>
       <c r="BV117" s="15" t="n"/>
+      <c r="BW117" s="15" t="n"/>
     </row>
     <row r="118" ht="14.25" customHeight="1">
       <c r="P118" s="13" t="n">
@@ -21490,6 +21768,9 @@
       <c r="BV118" s="15" t="n">
         <v>75.87</v>
       </c>
+      <c r="BW118" s="15" t="n">
+        <v>74.56</v>
+      </c>
     </row>
     <row r="119" ht="14.25" customHeight="1">
       <c r="Y119" s="13" t="n">
@@ -21640,6 +21921,9 @@
         <v>13163.37</v>
       </c>
       <c r="BV119" s="15" t="n">
+        <v>12900.98</v>
+      </c>
+      <c r="BW119" s="15" t="n">
         <v>12900.98</v>
       </c>
     </row>
@@ -21670,6 +21954,7 @@
       <c r="BT120" s="15" t="n"/>
       <c r="BU120" s="15" t="n"/>
       <c r="BV120" s="15" t="n"/>
+      <c r="BW120" s="15" t="n"/>
     </row>
     <row r="121" ht="14.25" customHeight="1">
       <c r="AW121" s="13" t="n">
@@ -21750,6 +22035,9 @@
       <c r="BV121" s="15" t="n">
         <v>24.19</v>
       </c>
+      <c r="BW121" s="15" t="n">
+        <v>22.04</v>
+      </c>
     </row>
     <row r="122" ht="14.25" customHeight="1">
       <c r="AW122" s="13" t="n">
@@ -21829,6 +22117,9 @@
       </c>
       <c r="BV122" s="15" t="n">
         <v>1196.23</v>
+      </c>
+      <c r="BW122" s="15" t="n">
+        <v>1179.2</v>
       </c>
     </row>
     <row r="123" ht="14.25" customHeight="1">
@@ -21858,6 +22149,7 @@
       <c r="BT123" s="15" t="n"/>
       <c r="BU123" s="15" t="n"/>
       <c r="BV123" s="15" t="n"/>
+      <c r="BW123" s="15" t="n"/>
     </row>
     <row r="124" ht="14.25" customHeight="1">
       <c r="AW124" s="13" t="n">
@@ -21938,6 +22230,9 @@
       <c r="BV124" s="15" t="n">
         <v>47.15</v>
       </c>
+      <c r="BW124" s="15" t="n">
+        <v>43.4</v>
+      </c>
     </row>
     <row r="125" ht="14.25" customHeight="1">
       <c r="AW125" s="13" t="n">
@@ -22016,6 +22311,9 @@
         <v>11895.94</v>
       </c>
       <c r="BV125" s="15" t="n">
+        <v>11436.37</v>
+      </c>
+      <c r="BW125" s="15" t="n">
         <v>11436.37</v>
       </c>
     </row>
@@ -22046,6 +22344,7 @@
       <c r="BT126" s="15" t="n"/>
       <c r="BU126" s="15" t="n"/>
       <c r="BV126" s="15" t="n"/>
+      <c r="BW126" s="15" t="n"/>
     </row>
     <row r="127" ht="14.25" customHeight="1">
       <c r="AW127" s="13" t="n">
@@ -22126,6 +22425,9 @@
       <c r="BV127" s="15" t="n">
         <v>4.31</v>
       </c>
+      <c r="BW127" s="15" t="n">
+        <v>2.32</v>
+      </c>
     </row>
     <row r="128" ht="14.25" customHeight="1">
       <c r="AW128" s="13" t="n">
@@ -22204,6 +22506,9 @@
         <v>1855.25</v>
       </c>
       <c r="BV128" s="15" t="n">
+        <v>1813.99</v>
+      </c>
+      <c r="BW128" s="15" t="n">
         <v>1813.99</v>
       </c>
     </row>
@@ -22234,6 +22539,7 @@
       <c r="BT129" s="15" t="n"/>
       <c r="BU129" s="15" t="n"/>
       <c r="BV129" s="15" t="n"/>
+      <c r="BW129" s="15" t="n"/>
     </row>
     <row r="130" ht="14.25" customHeight="1">
       <c r="AW130" s="13" t="n">
@@ -22314,6 +22620,9 @@
       <c r="BV130" s="15" t="n">
         <v>8.26</v>
       </c>
+      <c r="BW130" s="15" t="n">
+        <v>6.5</v>
+      </c>
     </row>
     <row r="131" ht="14.25" customHeight="1">
       <c r="AW131" s="13" t="n">
@@ -22392,6 +22701,9 @@
         <v>742.3099999999999</v>
       </c>
       <c r="BV131" s="15" t="n">
+        <v>726.62</v>
+      </c>
+      <c r="BW131" s="15" t="n">
         <v>726.62</v>
       </c>
     </row>
@@ -22422,6 +22734,7 @@
       <c r="BT132" s="15" t="n"/>
       <c r="BU132" s="15" t="n"/>
       <c r="BV132" s="15" t="n"/>
+      <c r="BW132" s="15" t="n"/>
     </row>
     <row r="133" ht="14.25" customHeight="1">
       <c r="AW133" s="13" t="n">
@@ -22502,6 +22815,9 @@
       <c r="BV133" s="15" t="n">
         <v>54.57</v>
       </c>
+      <c r="BW133" s="15" t="n">
+        <v>47.6</v>
+      </c>
     </row>
     <row r="134" ht="14.25" customHeight="1">
       <c r="AW134" s="13" t="n">
@@ -22580,6 +22896,9 @@
         <v>2851.18</v>
       </c>
       <c r="BV134" s="15" t="n">
+        <v>2738.48</v>
+      </c>
+      <c r="BW134" s="15" t="n">
         <v>2738.48</v>
       </c>
     </row>
@@ -22610,6 +22929,7 @@
       <c r="BT135" s="15" t="n"/>
       <c r="BU135" s="15" t="n"/>
       <c r="BV135" s="15" t="n"/>
+      <c r="BW135" s="15" t="n"/>
     </row>
     <row r="136" ht="14.25" customHeight="1">
       <c r="AW136" s="13" t="n">
@@ -22690,6 +23010,9 @@
       <c r="BV136" s="15" t="n">
         <v>21.66</v>
       </c>
+      <c r="BW136" s="15" t="n">
+        <v>21.14</v>
+      </c>
     </row>
     <row r="137" ht="14.25" customHeight="1">
       <c r="AW137" s="13" t="n">
@@ -22768,6 +23091,9 @@
         <v>3561.44</v>
       </c>
       <c r="BV137" s="15" t="n">
+        <v>3486.51</v>
+      </c>
+      <c r="BW137" s="15" t="n">
         <v>3486.51</v>
       </c>
     </row>
@@ -22790,6 +23116,7 @@
       <c r="BT138" s="15" t="n"/>
       <c r="BU138" s="15" t="n"/>
       <c r="BV138" s="15" t="n"/>
+      <c r="BW138" s="15" t="n"/>
     </row>
     <row r="139">
       <c r="BE139" s="15" t="n">
@@ -22846,6 +23173,9 @@
       <c r="BV139" s="15" t="n">
         <v>5.02</v>
       </c>
+      <c r="BW139" s="15" t="n">
+        <v>4.56</v>
+      </c>
     </row>
     <row r="140">
       <c r="BE140" s="15" t="n">
@@ -22900,6 +23230,9 @@
         <v>2351.96</v>
       </c>
       <c r="BV140" s="15" t="inlineStr"/>
+      <c r="BW140" s="15" t="n">
+        <v>2497.34</v>
+      </c>
     </row>
     <row r="141">
       <c r="BE141" s="15" t="n"/>
@@ -22920,6 +23253,7 @@
       <c r="BT141" s="15" t="n"/>
       <c r="BU141" s="15" t="n"/>
       <c r="BV141" s="15" t="n"/>
+      <c r="BW141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="BE142" s="15" t="n">
@@ -22976,6 +23310,9 @@
       <c r="BV142" s="15" t="n">
         <v>17.48</v>
       </c>
+      <c r="BW142" s="15" t="n">
+        <v>17.48</v>
+      </c>
     </row>
     <row r="143">
       <c r="BE143" s="15" t="n">
@@ -23031,6 +23368,9 @@
       </c>
       <c r="BV143" s="15" t="n">
         <v>5654.84</v>
+      </c>
+      <c r="BW143" s="15" t="n">
+        <v>5561.12</v>
       </c>
     </row>
     <row r="144">
@@ -23047,6 +23387,7 @@
       <c r="BT144" s="15" t="n"/>
       <c r="BU144" s="15" t="n"/>
       <c r="BV144" s="15" t="n"/>
+      <c r="BW144" s="15" t="n"/>
     </row>
     <row r="145">
       <c r="BJ145" s="15" t="n">
@@ -23088,6 +23429,9 @@
       <c r="BV145" s="15" t="n">
         <v>2.26</v>
       </c>
+      <c r="BW145" s="15" t="n">
+        <v>1.59</v>
+      </c>
     </row>
     <row r="146">
       <c r="BJ146" s="15" t="n">
@@ -23128,6 +23472,9 @@
       </c>
       <c r="BV146" s="15" t="n">
         <v>2248.48</v>
+      </c>
+      <c r="BW146" s="15" t="n">
+        <v>2207.48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-09-28 06:01:53]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BW146"/>
+  <dimension ref="A1:BX146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="51"/>
@@ -609,6 +609,7 @@
     <col width="15" customWidth="1" min="73" max="73"/>
     <col width="15" customWidth="1" min="74" max="74"/>
     <col width="15" customWidth="1" min="75" max="75"/>
+    <col width="15" customWidth="1" min="76" max="76"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -987,6 +988,11 @@
           <t>2026/09/26</t>
         </is>
       </c>
+      <c r="BX1" s="15" t="inlineStr">
+        <is>
+          <t>2026/09/28</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1364,6 +1370,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="BX2" s="16" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1591,6 +1602,9 @@
       <c r="BW3" s="15" t="n">
         <v>59.66</v>
       </c>
+      <c r="BX3" s="15" t="n">
+        <v>58.63</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1817,6 +1831,9 @@
       </c>
       <c r="BW4" s="15" t="n">
         <v>3888.37</v>
+      </c>
+      <c r="BX4" s="15" t="n">
+        <v>3812.65</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1895,6 +1912,7 @@
       <c r="BU5" s="15" t="n"/>
       <c r="BV5" s="15" t="n"/>
       <c r="BW5" s="15" t="n"/>
+      <c r="BX5" s="15" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -2020,6 +2038,7 @@
       <c r="BU6" s="15" t="n"/>
       <c r="BV6" s="15" t="n"/>
       <c r="BW6" s="15" t="n"/>
+      <c r="BX6" s="15" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -2245,6 +2264,9 @@
         <v>52.98</v>
       </c>
       <c r="BW7" s="15" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="BX7" s="15" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -2425,6 +2447,9 @@
       </c>
       <c r="BW8" s="15" t="n">
         <v>5486.01</v>
+      </c>
+      <c r="BX8" s="15" t="n">
+        <v>5332.89</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
@@ -2551,6 +2576,7 @@
       <c r="BU9" s="15" t="n"/>
       <c r="BV9" s="15" t="n"/>
       <c r="BW9" s="15" t="n"/>
+      <c r="BX9" s="15" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -2776,6 +2802,9 @@
         <v>47.36</v>
       </c>
       <c r="BW10" s="15" t="n">
+        <v>44.58</v>
+      </c>
+      <c r="BX10" s="15" t="n">
         <v>44.58</v>
       </c>
     </row>
@@ -2956,6 +2985,9 @@
       </c>
       <c r="BW11" s="15" t="n">
         <v>4439.14</v>
+      </c>
+      <c r="BX11" s="15" t="n">
+        <v>4330.78</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
@@ -3082,6 +3114,7 @@
       <c r="BU12" s="15" t="n"/>
       <c r="BV12" s="15" t="n"/>
       <c r="BW12" s="15" t="n"/>
+      <c r="BX12" s="15" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -3307,6 +3340,9 @@
         <v>60.7</v>
       </c>
       <c r="BW13" s="15" t="n">
+        <v>58.12</v>
+      </c>
+      <c r="BX13" s="15" t="n">
         <v>58.12</v>
       </c>
     </row>
@@ -3487,6 +3523,9 @@
       </c>
       <c r="BW14" s="15" t="n">
         <v>7624.07</v>
+      </c>
+      <c r="BX14" s="15" t="n">
+        <v>7379.28</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
@@ -3613,6 +3652,7 @@
       <c r="BU15" s="15" t="n"/>
       <c r="BV15" s="15" t="n"/>
       <c r="BW15" s="15" t="n"/>
+      <c r="BX15" s="15" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -3838,6 +3878,9 @@
         <v>27.98</v>
       </c>
       <c r="BW16" s="15" t="n">
+        <v>27.42</v>
+      </c>
+      <c r="BX16" s="15" t="n">
         <v>27.42</v>
       </c>
     </row>
@@ -4017,6 +4060,9 @@
         <v>2495.36</v>
       </c>
       <c r="BW17" s="15" t="n">
+        <v>2495.36</v>
+      </c>
+      <c r="BX17" s="15" t="n">
         <v>2495.36</v>
       </c>
     </row>
@@ -4144,6 +4190,7 @@
       <c r="BU18" s="15" t="n"/>
       <c r="BV18" s="15" t="n"/>
       <c r="BW18" s="15" t="n"/>
+      <c r="BX18" s="15" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -4369,6 +4416,9 @@
         <v>80.64</v>
       </c>
       <c r="BW19" s="15" t="n">
+        <v>80.64</v>
+      </c>
+      <c r="BX19" s="15" t="n">
         <v>80.64</v>
       </c>
     </row>
@@ -4548,6 +4598,9 @@
         <v>7706.03</v>
       </c>
       <c r="BW20" s="15" t="n">
+        <v>7743.41</v>
+      </c>
+      <c r="BX20" s="15" t="n">
         <v>7743.41</v>
       </c>
     </row>
@@ -4675,6 +4728,7 @@
       <c r="BU21" s="15" t="n"/>
       <c r="BV21" s="15" t="n"/>
       <c r="BW21" s="15" t="n"/>
+      <c r="BX21" s="15" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -4898,6 +4952,9 @@
         <v>36.34</v>
       </c>
       <c r="BW22" s="15" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="BX22" s="15" t="n">
         <v>36.34</v>
       </c>
     </row>
@@ -5078,6 +5135,9 @@
       </c>
       <c r="BW23" s="15" t="n">
         <v>73895.74000000001</v>
+      </c>
+      <c r="BX23" s="15" t="n">
+        <v>72881.84</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
@@ -5204,6 +5264,7 @@
       <c r="BU24" s="15" t="n"/>
       <c r="BV24" s="15" t="n"/>
       <c r="BW24" s="15" t="n"/>
+      <c r="BX24" s="15" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -5429,6 +5490,9 @@
         <v>49.88</v>
       </c>
       <c r="BW25" s="15" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="BX25" s="15" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -5594,6 +5658,9 @@
         <v>25178.08</v>
       </c>
       <c r="BW26" s="15" t="n">
+        <v>25408.64</v>
+      </c>
+      <c r="BX26" s="15" t="n">
         <v>25408.64</v>
       </c>
     </row>
@@ -5721,6 +5788,7 @@
       <c r="BU27" s="15" t="n"/>
       <c r="BV27" s="15" t="n"/>
       <c r="BW27" s="15" t="n"/>
+      <c r="BX27" s="15" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -5946,6 +6014,9 @@
         <v>92.09</v>
       </c>
       <c r="BW28" s="15" t="n">
+        <v>92.09</v>
+      </c>
+      <c r="BX28" s="15" t="n">
         <v>92.09</v>
       </c>
     </row>
@@ -6126,6 +6197,9 @@
       </c>
       <c r="BW29" s="15" t="n">
         <v>66364.2</v>
+      </c>
+      <c r="BX29" s="15" t="n">
+        <v>66215.06</v>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
@@ -6252,6 +6326,7 @@
       <c r="BU30" s="15" t="n"/>
       <c r="BV30" s="15" t="n"/>
       <c r="BW30" s="15" t="n"/>
+      <c r="BX30" s="15" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -6477,6 +6552,9 @@
         <v>97.44</v>
       </c>
       <c r="BW31" s="15" t="n">
+        <v>97.44</v>
+      </c>
+      <c r="BX31" s="15" t="n">
         <v>97.44</v>
       </c>
     </row>
@@ -6657,6 +6735,9 @@
       </c>
       <c r="BW32" s="15" t="n">
         <v>7080.92</v>
+      </c>
+      <c r="BX32" s="15" t="n">
+        <v>6912.38</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
@@ -6783,6 +6864,7 @@
       <c r="BU33" s="15" t="n"/>
       <c r="BV33" s="15" t="n"/>
       <c r="BW33" s="15" t="n"/>
+      <c r="BX33" s="15" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -7008,6 +7090,9 @@
         <v>45.66</v>
       </c>
       <c r="BW34" s="15" t="n">
+        <v>45.51</v>
+      </c>
+      <c r="BX34" s="15" t="n">
         <v>45.51</v>
       </c>
     </row>
@@ -7188,6 +7273,9 @@
       </c>
       <c r="BW35" s="15" t="n">
         <v>5469.4</v>
+      </c>
+      <c r="BX35" s="15" t="n">
+        <v>5424.43</v>
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
@@ -7314,6 +7402,7 @@
       <c r="BU36" s="15" t="n"/>
       <c r="BV36" s="15" t="n"/>
       <c r="BW36" s="15" t="n"/>
+      <c r="BX36" s="15" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -7539,6 +7628,9 @@
         <v>49.82</v>
       </c>
       <c r="BW37" s="15" t="n">
+        <v>50.37</v>
+      </c>
+      <c r="BX37" s="15" t="n">
         <v>50.37</v>
       </c>
     </row>
@@ -7719,6 +7811,9 @@
       </c>
       <c r="BW38" s="15" t="n">
         <v>11114.77</v>
+      </c>
+      <c r="BX38" s="15" t="n">
+        <v>11089.32</v>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
@@ -7845,6 +7940,7 @@
       <c r="BU39" s="15" t="n"/>
       <c r="BV39" s="15" t="n"/>
       <c r="BW39" s="15" t="n"/>
+      <c r="BX39" s="15" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -8070,6 +8166,9 @@
         <v>47.88</v>
       </c>
       <c r="BW40" s="15" t="n">
+        <v>48.39</v>
+      </c>
+      <c r="BX40" s="15" t="n">
         <v>48.39</v>
       </c>
     </row>
@@ -8249,6 +8348,9 @@
         <v>10847.74</v>
       </c>
       <c r="BW41" s="15" t="n">
+        <v>10848.95</v>
+      </c>
+      <c r="BX41" s="15" t="n">
         <v>10848.95</v>
       </c>
     </row>
@@ -8376,6 +8478,7 @@
       <c r="BU42" s="15" t="n"/>
       <c r="BV42" s="15" t="n"/>
       <c r="BW42" s="15" t="n"/>
+      <c r="BX42" s="15" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -8601,6 +8704,9 @@
         <v>48.53</v>
       </c>
       <c r="BW43" s="15" t="n">
+        <v>48.99</v>
+      </c>
+      <c r="BX43" s="15" t="n">
         <v>48.99</v>
       </c>
     </row>
@@ -8780,6 +8886,9 @@
         <v>3261.84</v>
       </c>
       <c r="BW44" s="15" t="n">
+        <v>3263.3</v>
+      </c>
+      <c r="BX44" s="15" t="n">
         <v>3263.3</v>
       </c>
     </row>
@@ -8907,6 +9016,7 @@
       <c r="BU45" s="15" t="n"/>
       <c r="BV45" s="15" t="n"/>
       <c r="BW45" s="15" t="n"/>
+      <c r="BX45" s="15" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -9132,6 +9242,9 @@
         <v>50.8</v>
       </c>
       <c r="BW46" s="15" t="n">
+        <v>52.54</v>
+      </c>
+      <c r="BX46" s="15" t="n">
         <v>52.54</v>
       </c>
     </row>
@@ -9311,6 +9424,9 @@
         <v>6925.02</v>
       </c>
       <c r="BW47" s="15" t="n">
+        <v>6935.79</v>
+      </c>
+      <c r="BX47" s="15" t="n">
         <v>6935.79</v>
       </c>
     </row>
@@ -9438,6 +9554,7 @@
       <c r="BU48" s="15" t="n"/>
       <c r="BV48" s="15" t="n"/>
       <c r="BW48" s="15" t="n"/>
+      <c r="BX48" s="15" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -9663,6 +9780,9 @@
         <v>20.39</v>
       </c>
       <c r="BW49" s="15" t="n">
+        <v>19.41</v>
+      </c>
+      <c r="BX49" s="15" t="n">
         <v>19.41</v>
       </c>
     </row>
@@ -9843,6 +9963,9 @@
       </c>
       <c r="BW50" s="15" t="n">
         <v>32175.64</v>
+      </c>
+      <c r="BX50" s="15" t="n">
+        <v>31648.99</v>
       </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
@@ -9969,6 +10092,7 @@
       <c r="BU51" s="15" t="n"/>
       <c r="BV51" s="15" t="n"/>
       <c r="BW51" s="15" t="n"/>
+      <c r="BX51" s="15" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -10194,6 +10318,9 @@
         <v>37.73</v>
       </c>
       <c r="BW52" s="15" t="n">
+        <v>34.84</v>
+      </c>
+      <c r="BX52" s="15" t="n">
         <v>34.84</v>
       </c>
     </row>
@@ -10374,6 +10501,9 @@
       </c>
       <c r="BW53" s="15" t="n">
         <v>3415.1</v>
+      </c>
+      <c r="BX53" s="15" t="n">
+        <v>3239.07</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
@@ -10500,6 +10630,7 @@
       <c r="BU54" s="15" t="n"/>
       <c r="BV54" s="15" t="n"/>
       <c r="BW54" s="15" t="n"/>
+      <c r="BX54" s="15" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -10726,6 +10857,9 @@
       </c>
       <c r="BW55" s="15" t="n">
         <v>42.37</v>
+      </c>
+      <c r="BX55" s="15" t="n">
+        <v>42.28</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -10905,6 +11039,9 @@
       </c>
       <c r="BW56" s="15" t="n">
         <v>3288.95</v>
+      </c>
+      <c r="BX56" s="15" t="n">
+        <v>3132.47</v>
       </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
@@ -11031,6 +11168,7 @@
       <c r="BU57" s="15" t="n"/>
       <c r="BV57" s="15" t="n"/>
       <c r="BW57" s="15" t="n"/>
+      <c r="BX57" s="15" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -11257,6 +11395,9 @@
       </c>
       <c r="BW58" s="15" t="n">
         <v>16.66</v>
+      </c>
+      <c r="BX58" s="15" t="n">
+        <v>15.91</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -11436,6 +11577,9 @@
       </c>
       <c r="BW59" s="15" t="n">
         <v>6731.18</v>
+      </c>
+      <c r="BX59" s="15" t="n">
+        <v>6698.71</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
@@ -11562,6 +11706,7 @@
       <c r="BU60" s="15" t="n"/>
       <c r="BV60" s="15" t="n"/>
       <c r="BW60" s="15" t="n"/>
+      <c r="BX60" s="15" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -11787,6 +11932,9 @@
         <v>34.86</v>
       </c>
       <c r="BW61" s="15" t="n">
+        <v>30.91</v>
+      </c>
+      <c r="BX61" s="15" t="n">
         <v>30.91</v>
       </c>
     </row>
@@ -11967,6 +12115,9 @@
       </c>
       <c r="BW62" s="15" t="n">
         <v>8034.61</v>
+      </c>
+      <c r="BX62" s="15" t="n">
+        <v>8025.71</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
@@ -12093,6 +12244,7 @@
       <c r="BU63" s="15" t="n"/>
       <c r="BV63" s="15" t="n"/>
       <c r="BW63" s="15" t="n"/>
+      <c r="BX63" s="15" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -12318,6 +12470,9 @@
         <v>6.6</v>
       </c>
       <c r="BW64" s="15" t="n">
+        <v>5.41</v>
+      </c>
+      <c r="BX64" s="15" t="n">
         <v>5.41</v>
       </c>
     </row>
@@ -12498,6 +12653,9 @@
       </c>
       <c r="BW65" s="15" t="n">
         <v>10367.63</v>
+      </c>
+      <c r="BX65" s="15" t="n">
+        <v>10320.59</v>
       </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
@@ -12624,6 +12782,7 @@
       <c r="BU66" s="15" t="n"/>
       <c r="BV66" s="15" t="n"/>
       <c r="BW66" s="15" t="n"/>
+      <c r="BX66" s="15" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -12849,6 +13008,9 @@
         <v>19.38</v>
       </c>
       <c r="BW67" s="15" t="n">
+        <v>19.02</v>
+      </c>
+      <c r="BX67" s="15" t="n">
         <v>19.02</v>
       </c>
     </row>
@@ -13028,6 +13190,9 @@
         <v>11219.09</v>
       </c>
       <c r="BW68" s="15" t="n">
+        <v>11219.09</v>
+      </c>
+      <c r="BX68" s="15" t="n">
         <v>11219.09</v>
       </c>
     </row>
@@ -13155,6 +13320,7 @@
       <c r="BU69" s="15" t="n"/>
       <c r="BV69" s="15" t="n"/>
       <c r="BW69" s="15" t="n"/>
+      <c r="BX69" s="15" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -13380,6 +13546,9 @@
         <v>14.62</v>
       </c>
       <c r="BW70" s="15" t="n">
+        <v>12.82</v>
+      </c>
+      <c r="BX70" s="15" t="n">
         <v>12.82</v>
       </c>
     </row>
@@ -13560,6 +13729,9 @@
       </c>
       <c r="BW71" s="15" t="n">
         <v>6105.76</v>
+      </c>
+      <c r="BX71" s="15" t="n">
+        <v>6044</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
@@ -13686,6 +13858,7 @@
       <c r="BU72" s="15" t="n"/>
       <c r="BV72" s="15" t="n"/>
       <c r="BW72" s="15" t="n"/>
+      <c r="BX72" s="15" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -13911,6 +14084,9 @@
         <v>17.53</v>
       </c>
       <c r="BW73" s="15" t="n">
+        <v>16.36</v>
+      </c>
+      <c r="BX73" s="15" t="n">
         <v>16.36</v>
       </c>
     </row>
@@ -14091,6 +14267,9 @@
       </c>
       <c r="BW74" s="15" t="n">
         <v>12109.54</v>
+      </c>
+      <c r="BX74" s="15" t="n">
+        <v>12078.68</v>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
@@ -14217,6 +14396,7 @@
       <c r="BU75" s="15" t="n"/>
       <c r="BV75" s="15" t="n"/>
       <c r="BW75" s="15" t="n"/>
+      <c r="BX75" s="15" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -14442,6 +14622,9 @@
         <v>53.91</v>
       </c>
       <c r="BW76" s="15" t="n">
+        <v>53.09</v>
+      </c>
+      <c r="BX76" s="15" t="n">
         <v>53.09</v>
       </c>
     </row>
@@ -14621,6 +14804,9 @@
         <v>15569.82</v>
       </c>
       <c r="BW77" s="15" t="n">
+        <v>15569.82</v>
+      </c>
+      <c r="BX77" s="15" t="n">
         <v>15569.82</v>
       </c>
     </row>
@@ -14748,6 +14934,7 @@
       <c r="BU78" s="15" t="n"/>
       <c r="BV78" s="15" t="n"/>
       <c r="BW78" s="15" t="n"/>
+      <c r="BX78" s="15" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -14973,6 +15160,9 @@
         <v>3.05</v>
       </c>
       <c r="BW79" s="15" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="BX79" s="15" t="n">
         <v>2.88</v>
       </c>
     </row>
@@ -15153,6 +15343,9 @@
       </c>
       <c r="BW80" s="15" t="n">
         <v>6557.96</v>
+      </c>
+      <c r="BX80" s="15" t="n">
+        <v>6485.64</v>
       </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
@@ -15279,6 +15472,7 @@
       <c r="BU81" s="15" t="n"/>
       <c r="BV81" s="15" t="n"/>
       <c r="BW81" s="15" t="n"/>
+      <c r="BX81" s="15" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -15504,6 +15698,9 @@
         <v>3.64</v>
       </c>
       <c r="BW82" s="15" t="n">
+        <v>2.92</v>
+      </c>
+      <c r="BX82" s="15" t="n">
         <v>2.92</v>
       </c>
     </row>
@@ -15683,6 +15880,9 @@
         <v>8201.43</v>
       </c>
       <c r="BW83" s="15" t="n">
+        <v>8161.87</v>
+      </c>
+      <c r="BX83" s="15" t="n">
         <v>8161.87</v>
       </c>
     </row>
@@ -15810,6 +16010,7 @@
       <c r="BU84" s="15" t="n"/>
       <c r="BV84" s="15" t="n"/>
       <c r="BW84" s="15" t="n"/>
+      <c r="BX84" s="15" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -16035,6 +16236,9 @@
         <v>17.32</v>
       </c>
       <c r="BW85" s="15" t="n">
+        <v>16.57</v>
+      </c>
+      <c r="BX85" s="15" t="n">
         <v>16.57</v>
       </c>
     </row>
@@ -16215,6 +16419,9 @@
       </c>
       <c r="BW86" s="15" t="n">
         <v>2040.14</v>
+      </c>
+      <c r="BX86" s="15" t="n">
+        <v>2041.04</v>
       </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
@@ -16341,6 +16548,7 @@
       <c r="BU87" s="15" t="n"/>
       <c r="BV87" s="15" t="n"/>
       <c r="BW87" s="15" t="n"/>
+      <c r="BX87" s="15" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -16566,6 +16774,9 @@
         <v>27.98</v>
       </c>
       <c r="BW88" s="15" t="n">
+        <v>26.28</v>
+      </c>
+      <c r="BX88" s="15" t="n">
         <v>26.28</v>
       </c>
     </row>
@@ -16745,6 +16956,9 @@
         <v>4361.13</v>
       </c>
       <c r="BW89" s="15" t="n">
+        <v>5075.31</v>
+      </c>
+      <c r="BX89" s="15" t="n">
         <v>5075.31</v>
       </c>
     </row>
@@ -16872,6 +17086,7 @@
       <c r="BU90" s="15" t="n"/>
       <c r="BV90" s="15" t="n"/>
       <c r="BW90" s="15" t="n"/>
+      <c r="BX90" s="15" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -17098,6 +17313,9 @@
       </c>
       <c r="BW91" s="15" t="n">
         <v>14.86</v>
+      </c>
+      <c r="BX91" s="15" t="n">
+        <v>14.68</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -17277,6 +17495,9 @@
       </c>
       <c r="BW92" s="15" t="n">
         <v>8420.93</v>
+      </c>
+      <c r="BX92" s="15" t="n">
+        <v>8392.030000000001</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
@@ -17403,6 +17624,7 @@
       <c r="BU93" s="15" t="n"/>
       <c r="BV93" s="15" t="n"/>
       <c r="BW93" s="15" t="n"/>
+      <c r="BX93" s="15" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -17628,6 +17850,9 @@
         <v>4.83</v>
       </c>
       <c r="BW94" s="15" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="BX94" s="15" t="n">
         <v>3.9</v>
       </c>
     </row>
@@ -17807,6 +18032,9 @@
         <v>1193.12</v>
       </c>
       <c r="BW95" s="15" t="n">
+        <v>1176.71</v>
+      </c>
+      <c r="BX95" s="15" t="n">
         <v>1176.71</v>
       </c>
     </row>
@@ -17934,6 +18162,7 @@
       <c r="BU96" s="15" t="n"/>
       <c r="BV96" s="15" t="n"/>
       <c r="BW96" s="15" t="n"/>
+      <c r="BX96" s="15" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -18159,6 +18388,9 @@
         <v>8.59</v>
       </c>
       <c r="BW97" s="15" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="BX97" s="15" t="n">
         <v>7.75</v>
       </c>
     </row>
@@ -18338,6 +18570,9 @@
         <v>13636.38</v>
       </c>
       <c r="BW98" s="15" t="n">
+        <v>13458.58</v>
+      </c>
+      <c r="BX98" s="15" t="n">
         <v>13458.58</v>
       </c>
     </row>
@@ -18465,6 +18700,7 @@
       <c r="BU99" s="15" t="n"/>
       <c r="BV99" s="15" t="n"/>
       <c r="BW99" s="15" t="n"/>
+      <c r="BX99" s="15" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -18690,6 +18926,9 @@
         <v>39.06</v>
       </c>
       <c r="BW100" s="15" t="n">
+        <v>34.57</v>
+      </c>
+      <c r="BX100" s="15" t="n">
         <v>34.57</v>
       </c>
     </row>
@@ -18869,6 +19108,9 @@
         <v>3342.43</v>
       </c>
       <c r="BW101" s="15" t="n">
+        <v>3257.76</v>
+      </c>
+      <c r="BX101" s="15" t="n">
         <v>3257.76</v>
       </c>
     </row>
@@ -18996,6 +19238,7 @@
       <c r="BU102" s="15" t="n"/>
       <c r="BV102" s="15" t="n"/>
       <c r="BW102" s="15" t="n"/>
+      <c r="BX102" s="15" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -19221,6 +19464,9 @@
         <v>26.8</v>
       </c>
       <c r="BW103" s="15" t="n">
+        <v>24.74</v>
+      </c>
+      <c r="BX103" s="15" t="n">
         <v>24.74</v>
       </c>
     </row>
@@ -19401,6 +19647,9 @@
       </c>
       <c r="BW104" s="15" t="n">
         <v>2196.75</v>
+      </c>
+      <c r="BX104" s="15" t="n">
+        <v>2136</v>
       </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
@@ -19527,6 +19776,7 @@
       <c r="BU105" s="15" t="n"/>
       <c r="BV105" s="15" t="n"/>
       <c r="BW105" s="15" t="n"/>
+      <c r="BX105" s="15" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -19752,6 +20002,9 @@
         <v>14.61</v>
       </c>
       <c r="BW106" s="15" t="n">
+        <v>15.91</v>
+      </c>
+      <c r="BX106" s="15" t="n">
         <v>15.91</v>
       </c>
     </row>
@@ -19932,6 +20185,9 @@
       </c>
       <c r="BW107" s="15" t="n">
         <v>2333.92</v>
+      </c>
+      <c r="BX107" s="15" t="n">
+        <v>2265.14</v>
       </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
@@ -20058,6 +20314,7 @@
       <c r="BU108" s="15" t="n"/>
       <c r="BV108" s="15" t="n"/>
       <c r="BW108" s="15" t="n"/>
+      <c r="BX108" s="15" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -20283,6 +20540,9 @@
         <v>26.55</v>
       </c>
       <c r="BW109" s="15" t="n">
+        <v>25.78</v>
+      </c>
+      <c r="BX109" s="15" t="n">
         <v>25.78</v>
       </c>
     </row>
@@ -20463,6 +20723,9 @@
       </c>
       <c r="BW110" s="15" t="n">
         <v>2391.95</v>
+      </c>
+      <c r="BX110" s="15" t="n">
+        <v>2276.69</v>
       </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
@@ -20589,6 +20852,7 @@
       <c r="BU111" s="15" t="n"/>
       <c r="BV111" s="15" t="n"/>
       <c r="BW111" s="15" t="n"/>
+      <c r="BX111" s="15" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -20814,6 +21078,9 @@
         <v>53.44</v>
       </c>
       <c r="BW112" s="15" t="n">
+        <v>47.56</v>
+      </c>
+      <c r="BX112" s="15" t="n">
         <v>47.56</v>
       </c>
     </row>
@@ -20992,6 +21259,9 @@
       </c>
       <c r="BW113" s="15" t="n">
         <v>1892.25</v>
+      </c>
+      <c r="BX113" s="15" t="n">
+        <v>1885.92</v>
       </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
@@ -21118,6 +21388,7 @@
       <c r="BU114" s="15" t="n"/>
       <c r="BV114" s="15" t="n"/>
       <c r="BW114" s="15" t="n"/>
+      <c r="BX114" s="15" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -21344,6 +21615,9 @@
       </c>
       <c r="BW115" s="15" t="n">
         <v>16.88</v>
+      </c>
+      <c r="BX115" s="15" t="n">
+        <v>16.55</v>
       </c>
     </row>
     <row r="116" ht="14.25" customHeight="1">
@@ -21507,6 +21781,9 @@
         <v>8784.530000000001</v>
       </c>
       <c r="BW116" s="15" t="n">
+        <v>8720.299999999999</v>
+      </c>
+      <c r="BX116" s="15" t="n">
         <v>8720.299999999999</v>
       </c>
     </row>
@@ -21589,6 +21866,7 @@
       <c r="BU117" s="15" t="n"/>
       <c r="BV117" s="15" t="n"/>
       <c r="BW117" s="15" t="n"/>
+      <c r="BX117" s="15" t="n"/>
     </row>
     <row r="118" ht="14.25" customHeight="1">
       <c r="P118" s="13" t="n">
@@ -21771,6 +22049,9 @@
       <c r="BW118" s="15" t="n">
         <v>74.56</v>
       </c>
+      <c r="BX118" s="15" t="n">
+        <v>74.56</v>
+      </c>
     </row>
     <row r="119" ht="14.25" customHeight="1">
       <c r="Y119" s="13" t="n">
@@ -21925,6 +22206,9 @@
       </c>
       <c r="BW119" s="15" t="n">
         <v>12900.98</v>
+      </c>
+      <c r="BX119" s="15" t="n">
+        <v>12333.91</v>
       </c>
     </row>
     <row r="120" ht="14.25" customHeight="1">
@@ -21955,6 +22239,7 @@
       <c r="BU120" s="15" t="n"/>
       <c r="BV120" s="15" t="n"/>
       <c r="BW120" s="15" t="n"/>
+      <c r="BX120" s="15" t="n"/>
     </row>
     <row r="121" ht="14.25" customHeight="1">
       <c r="AW121" s="13" t="n">
@@ -22038,6 +22323,9 @@
       <c r="BW121" s="15" t="n">
         <v>22.04</v>
       </c>
+      <c r="BX121" s="15" t="n">
+        <v>22.04</v>
+      </c>
     </row>
     <row r="122" ht="14.25" customHeight="1">
       <c r="AW122" s="13" t="n">
@@ -22119,6 +22407,9 @@
         <v>1196.23</v>
       </c>
       <c r="BW122" s="15" t="n">
+        <v>1179.2</v>
+      </c>
+      <c r="BX122" s="15" t="n">
         <v>1179.2</v>
       </c>
     </row>
@@ -22150,6 +22441,7 @@
       <c r="BU123" s="15" t="n"/>
       <c r="BV123" s="15" t="n"/>
       <c r="BW123" s="15" t="n"/>
+      <c r="BX123" s="15" t="n"/>
     </row>
     <row r="124" ht="14.25" customHeight="1">
       <c r="AW124" s="13" t="n">
@@ -22233,6 +22525,9 @@
       <c r="BW124" s="15" t="n">
         <v>43.4</v>
       </c>
+      <c r="BX124" s="15" t="n">
+        <v>43.4</v>
+      </c>
     </row>
     <row r="125" ht="14.25" customHeight="1">
       <c r="AW125" s="13" t="n">
@@ -22315,6 +22610,9 @@
       </c>
       <c r="BW125" s="15" t="n">
         <v>11436.37</v>
+      </c>
+      <c r="BX125" s="15" t="n">
+        <v>11125.13</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1">
@@ -22345,6 +22643,7 @@
       <c r="BU126" s="15" t="n"/>
       <c r="BV126" s="15" t="n"/>
       <c r="BW126" s="15" t="n"/>
+      <c r="BX126" s="15" t="n"/>
     </row>
     <row r="127" ht="14.25" customHeight="1">
       <c r="AW127" s="13" t="n">
@@ -22428,6 +22727,9 @@
       <c r="BW127" s="15" t="n">
         <v>2.32</v>
       </c>
+      <c r="BX127" s="15" t="n">
+        <v>2.32</v>
+      </c>
     </row>
     <row r="128" ht="14.25" customHeight="1">
       <c r="AW128" s="13" t="n">
@@ -22509,6 +22811,9 @@
         <v>1813.99</v>
       </c>
       <c r="BW128" s="15" t="n">
+        <v>1813.99</v>
+      </c>
+      <c r="BX128" s="15" t="n">
         <v>1813.99</v>
       </c>
     </row>
@@ -22540,6 +22845,7 @@
       <c r="BU129" s="15" t="n"/>
       <c r="BV129" s="15" t="n"/>
       <c r="BW129" s="15" t="n"/>
+      <c r="BX129" s="15" t="n"/>
     </row>
     <row r="130" ht="14.25" customHeight="1">
       <c r="AW130" s="13" t="n">
@@ -22623,6 +22929,9 @@
       <c r="BW130" s="15" t="n">
         <v>6.5</v>
       </c>
+      <c r="BX130" s="15" t="n">
+        <v>6.5</v>
+      </c>
     </row>
     <row r="131" ht="14.25" customHeight="1">
       <c r="AW131" s="13" t="n">
@@ -22705,6 +23014,9 @@
       </c>
       <c r="BW131" s="15" t="n">
         <v>726.62</v>
+      </c>
+      <c r="BX131" s="15" t="n">
+        <v>712.1</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1">
@@ -22735,6 +23047,7 @@
       <c r="BU132" s="15" t="n"/>
       <c r="BV132" s="15" t="n"/>
       <c r="BW132" s="15" t="n"/>
+      <c r="BX132" s="15" t="n"/>
     </row>
     <row r="133" ht="14.25" customHeight="1">
       <c r="AW133" s="13" t="n">
@@ -22818,6 +23131,9 @@
       <c r="BW133" s="15" t="n">
         <v>47.6</v>
       </c>
+      <c r="BX133" s="15" t="n">
+        <v>47.6</v>
+      </c>
     </row>
     <row r="134" ht="14.25" customHeight="1">
       <c r="AW134" s="13" t="n">
@@ -22899,6 +23215,9 @@
         <v>2738.48</v>
       </c>
       <c r="BW134" s="15" t="n">
+        <v>2738.48</v>
+      </c>
+      <c r="BX134" s="15" t="n">
         <v>2738.48</v>
       </c>
     </row>
@@ -22930,6 +23249,7 @@
       <c r="BU135" s="15" t="n"/>
       <c r="BV135" s="15" t="n"/>
       <c r="BW135" s="15" t="n"/>
+      <c r="BX135" s="15" t="n"/>
     </row>
     <row r="136" ht="14.25" customHeight="1">
       <c r="AW136" s="13" t="n">
@@ -23013,6 +23333,9 @@
       <c r="BW136" s="15" t="n">
         <v>21.14</v>
       </c>
+      <c r="BX136" s="15" t="n">
+        <v>21.14</v>
+      </c>
     </row>
     <row r="137" ht="14.25" customHeight="1">
       <c r="AW137" s="13" t="n">
@@ -23095,6 +23418,9 @@
       </c>
       <c r="BW137" s="15" t="n">
         <v>3486.51</v>
+      </c>
+      <c r="BX137" s="15" t="n">
+        <v>3404.06</v>
       </c>
     </row>
     <row r="138">
@@ -23117,6 +23443,7 @@
       <c r="BU138" s="15" t="n"/>
       <c r="BV138" s="15" t="n"/>
       <c r="BW138" s="15" t="n"/>
+      <c r="BX138" s="15" t="n"/>
     </row>
     <row r="139">
       <c r="BE139" s="15" t="n">
@@ -23176,6 +23503,9 @@
       <c r="BW139" s="15" t="n">
         <v>4.56</v>
       </c>
+      <c r="BX139" s="15" t="n">
+        <v>4.56</v>
+      </c>
     </row>
     <row r="140">
       <c r="BE140" s="15" t="n">
@@ -23231,6 +23561,9 @@
       </c>
       <c r="BV140" s="15" t="inlineStr"/>
       <c r="BW140" s="15" t="n">
+        <v>2497.34</v>
+      </c>
+      <c r="BX140" s="15" t="n">
         <v>2497.34</v>
       </c>
     </row>
@@ -23254,6 +23587,7 @@
       <c r="BU141" s="15" t="n"/>
       <c r="BV141" s="15" t="n"/>
       <c r="BW141" s="15" t="n"/>
+      <c r="BX141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="BE142" s="15" t="n">
@@ -23313,6 +23647,9 @@
       <c r="BW142" s="15" t="n">
         <v>17.48</v>
       </c>
+      <c r="BX142" s="15" t="n">
+        <v>15.3</v>
+      </c>
     </row>
     <row r="143">
       <c r="BE143" s="15" t="n">
@@ -23370,6 +23707,9 @@
         <v>5654.84</v>
       </c>
       <c r="BW143" s="15" t="n">
+        <v>5561.12</v>
+      </c>
+      <c r="BX143" s="15" t="n">
         <v>5561.12</v>
       </c>
     </row>
@@ -23388,6 +23728,7 @@
       <c r="BU144" s="15" t="n"/>
       <c r="BV144" s="15" t="n"/>
       <c r="BW144" s="15" t="n"/>
+      <c r="BX144" s="15" t="n"/>
     </row>
     <row r="145">
       <c r="BJ145" s="15" t="n">
@@ -23432,6 +23773,9 @@
       <c r="BW145" s="15" t="n">
         <v>1.59</v>
       </c>
+      <c r="BX145" s="15" t="n">
+        <v>1.59</v>
+      </c>
     </row>
     <row r="146">
       <c r="BJ146" s="15" t="n">
@@ -23474,6 +23818,9 @@
         <v>2248.48</v>
       </c>
       <c r="BW146" s="15" t="n">
+        <v>2207.48</v>
+      </c>
+      <c r="BX146" s="15" t="n">
         <v>2207.48</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-09-28 10:11:43]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BX146"/>
+  <dimension ref="A1:BY146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="51"/>
@@ -610,6 +610,7 @@
     <col width="15" customWidth="1" min="74" max="74"/>
     <col width="15" customWidth="1" min="75" max="75"/>
     <col width="15" customWidth="1" min="76" max="76"/>
+    <col width="15" customWidth="1" min="77" max="77"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -993,6 +994,11 @@
           <t>2026/09/28</t>
         </is>
       </c>
+      <c r="BY1" s="15" t="inlineStr">
+        <is>
+          <t>2026/09/28</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1375,6 +1381,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="BY2" s="16" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1605,6 +1616,9 @@
       <c r="BX3" s="15" t="n">
         <v>58.63</v>
       </c>
+      <c r="BY3" s="15" t="n">
+        <v>58.63</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1834,6 +1848,9 @@
       </c>
       <c r="BX4" s="15" t="n">
         <v>3812.65</v>
+      </c>
+      <c r="BY4" s="15" t="n">
+        <v>3823.62</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1913,6 +1930,7 @@
       <c r="BV5" s="15" t="n"/>
       <c r="BW5" s="15" t="n"/>
       <c r="BX5" s="15" t="n"/>
+      <c r="BY5" s="15" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -2039,6 +2057,7 @@
       <c r="BV6" s="15" t="n"/>
       <c r="BW6" s="15" t="n"/>
       <c r="BX6" s="15" t="n"/>
+      <c r="BY6" s="15" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -2267,6 +2286,9 @@
         <v>49.88</v>
       </c>
       <c r="BX7" s="15" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="BY7" s="15" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -2450,6 +2472,9 @@
       </c>
       <c r="BX8" s="15" t="n">
         <v>5332.89</v>
+      </c>
+      <c r="BY8" s="15" t="n">
+        <v>5348.5</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
@@ -2577,6 +2602,7 @@
       <c r="BV9" s="15" t="n"/>
       <c r="BW9" s="15" t="n"/>
       <c r="BX9" s="15" t="n"/>
+      <c r="BY9" s="15" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -2805,6 +2831,9 @@
         <v>44.58</v>
       </c>
       <c r="BX10" s="15" t="n">
+        <v>44.58</v>
+      </c>
+      <c r="BY10" s="15" t="n">
         <v>44.58</v>
       </c>
     </row>
@@ -2988,6 +3017,9 @@
       </c>
       <c r="BX11" s="15" t="n">
         <v>4330.78</v>
+      </c>
+      <c r="BY11" s="15" t="n">
+        <v>4340.76</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
@@ -3115,6 +3147,7 @@
       <c r="BV12" s="15" t="n"/>
       <c r="BW12" s="15" t="n"/>
       <c r="BX12" s="15" t="n"/>
+      <c r="BY12" s="15" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -3343,6 +3376,9 @@
         <v>58.12</v>
       </c>
       <c r="BX13" s="15" t="n">
+        <v>58.12</v>
+      </c>
+      <c r="BY13" s="15" t="n">
         <v>58.12</v>
       </c>
     </row>
@@ -3526,6 +3562,9 @@
       </c>
       <c r="BX14" s="15" t="n">
         <v>7379.28</v>
+      </c>
+      <c r="BY14" s="15" t="n">
+        <v>7402.3</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
@@ -3653,6 +3692,7 @@
       <c r="BV15" s="15" t="n"/>
       <c r="BW15" s="15" t="n"/>
       <c r="BX15" s="15" t="n"/>
+      <c r="BY15" s="15" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -3881,6 +3921,9 @@
         <v>27.42</v>
       </c>
       <c r="BX16" s="15" t="n">
+        <v>27.42</v>
+      </c>
+      <c r="BY16" s="15" t="n">
         <v>27.42</v>
       </c>
     </row>
@@ -4063,6 +4106,9 @@
         <v>2495.36</v>
       </c>
       <c r="BX17" s="15" t="n">
+        <v>2495.36</v>
+      </c>
+      <c r="BY17" s="15" t="n">
         <v>2495.36</v>
       </c>
     </row>
@@ -4191,6 +4237,7 @@
       <c r="BV18" s="15" t="n"/>
       <c r="BW18" s="15" t="n"/>
       <c r="BX18" s="15" t="n"/>
+      <c r="BY18" s="15" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -4419,6 +4466,9 @@
         <v>80.64</v>
       </c>
       <c r="BX19" s="15" t="n">
+        <v>80.64</v>
+      </c>
+      <c r="BY19" s="15" t="n">
         <v>80.64</v>
       </c>
     </row>
@@ -4601,6 +4651,9 @@
         <v>7743.41</v>
       </c>
       <c r="BX20" s="15" t="n">
+        <v>7743.41</v>
+      </c>
+      <c r="BY20" s="15" t="n">
         <v>7743.41</v>
       </c>
     </row>
@@ -4729,6 +4782,7 @@
       <c r="BV21" s="15" t="n"/>
       <c r="BW21" s="15" t="n"/>
       <c r="BX21" s="15" t="n"/>
+      <c r="BY21" s="15" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -4955,6 +5009,9 @@
         <v>36.34</v>
       </c>
       <c r="BX22" s="15" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="BY22" s="15" t="n">
         <v>36.34</v>
       </c>
     </row>
@@ -5138,6 +5195,9 @@
       </c>
       <c r="BX23" s="15" t="n">
         <v>72881.84</v>
+      </c>
+      <c r="BY23" s="15" t="n">
+        <v>72805.78</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
@@ -5265,6 +5325,7 @@
       <c r="BV24" s="15" t="n"/>
       <c r="BW24" s="15" t="n"/>
       <c r="BX24" s="15" t="n"/>
+      <c r="BY24" s="15" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -5493,6 +5554,9 @@
         <v>49.88</v>
       </c>
       <c r="BX25" s="15" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="BY25" s="15" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -5662,6 +5726,9 @@
       </c>
       <c r="BX26" s="15" t="n">
         <v>25408.64</v>
+      </c>
+      <c r="BY26" s="15" t="n">
+        <v>25419.65</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
@@ -5789,6 +5856,7 @@
       <c r="BV27" s="15" t="n"/>
       <c r="BW27" s="15" t="n"/>
       <c r="BX27" s="15" t="n"/>
+      <c r="BY27" s="15" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -6017,6 +6085,9 @@
         <v>92.09</v>
       </c>
       <c r="BX28" s="15" t="n">
+        <v>92.09</v>
+      </c>
+      <c r="BY28" s="15" t="n">
         <v>92.09</v>
       </c>
     </row>
@@ -6200,6 +6271,9 @@
       </c>
       <c r="BX29" s="15" t="n">
         <v>66215.06</v>
+      </c>
+      <c r="BY29" s="15" t="n">
+        <v>65877.62</v>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
@@ -6327,6 +6401,7 @@
       <c r="BV30" s="15" t="n"/>
       <c r="BW30" s="15" t="n"/>
       <c r="BX30" s="15" t="n"/>
+      <c r="BY30" s="15" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -6555,6 +6630,9 @@
         <v>97.44</v>
       </c>
       <c r="BX31" s="15" t="n">
+        <v>97.44</v>
+      </c>
+      <c r="BY31" s="15" t="n">
         <v>97.44</v>
       </c>
     </row>
@@ -6738,6 +6816,9 @@
       </c>
       <c r="BX32" s="15" t="n">
         <v>6912.38</v>
+      </c>
+      <c r="BY32" s="15" t="n">
+        <v>6889.74</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
@@ -6865,6 +6946,7 @@
       <c r="BV33" s="15" t="n"/>
       <c r="BW33" s="15" t="n"/>
       <c r="BX33" s="15" t="n"/>
+      <c r="BY33" s="15" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -7093,6 +7175,9 @@
         <v>45.51</v>
       </c>
       <c r="BX34" s="15" t="n">
+        <v>45.51</v>
+      </c>
+      <c r="BY34" s="15" t="n">
         <v>45.51</v>
       </c>
     </row>
@@ -7276,6 +7361,9 @@
       </c>
       <c r="BX35" s="15" t="n">
         <v>5424.43</v>
+      </c>
+      <c r="BY35" s="15" t="n">
+        <v>5439.6</v>
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
@@ -7403,6 +7491,7 @@
       <c r="BV36" s="15" t="n"/>
       <c r="BW36" s="15" t="n"/>
       <c r="BX36" s="15" t="n"/>
+      <c r="BY36" s="15" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -7631,6 +7720,9 @@
         <v>50.37</v>
       </c>
       <c r="BX37" s="15" t="n">
+        <v>50.37</v>
+      </c>
+      <c r="BY37" s="15" t="n">
         <v>50.37</v>
       </c>
     </row>
@@ -7814,6 +7906,9 @@
       </c>
       <c r="BX38" s="15" t="n">
         <v>11089.32</v>
+      </c>
+      <c r="BY38" s="15" t="n">
+        <v>11122.04</v>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
@@ -7941,6 +8036,7 @@
       <c r="BV39" s="15" t="n"/>
       <c r="BW39" s="15" t="n"/>
       <c r="BX39" s="15" t="n"/>
+      <c r="BY39" s="15" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -8169,6 +8265,9 @@
         <v>48.39</v>
       </c>
       <c r="BX40" s="15" t="n">
+        <v>48.39</v>
+      </c>
+      <c r="BY40" s="15" t="n">
         <v>48.39</v>
       </c>
     </row>
@@ -8351,6 +8450,9 @@
         <v>10848.95</v>
       </c>
       <c r="BX41" s="15" t="n">
+        <v>10848.95</v>
+      </c>
+      <c r="BY41" s="15" t="n">
         <v>10848.95</v>
       </c>
     </row>
@@ -8479,6 +8581,7 @@
       <c r="BV42" s="15" t="n"/>
       <c r="BW42" s="15" t="n"/>
       <c r="BX42" s="15" t="n"/>
+      <c r="BY42" s="15" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -8707,6 +8810,9 @@
         <v>48.99</v>
       </c>
       <c r="BX43" s="15" t="n">
+        <v>48.99</v>
+      </c>
+      <c r="BY43" s="15" t="n">
         <v>48.99</v>
       </c>
     </row>
@@ -8889,6 +8995,9 @@
         <v>3263.3</v>
       </c>
       <c r="BX44" s="15" t="n">
+        <v>3263.3</v>
+      </c>
+      <c r="BY44" s="15" t="n">
         <v>3263.3</v>
       </c>
     </row>
@@ -9017,6 +9126,7 @@
       <c r="BV45" s="15" t="n"/>
       <c r="BW45" s="15" t="n"/>
       <c r="BX45" s="15" t="n"/>
+      <c r="BY45" s="15" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -9245,6 +9355,9 @@
         <v>52.54</v>
       </c>
       <c r="BX46" s="15" t="n">
+        <v>52.54</v>
+      </c>
+      <c r="BY46" s="15" t="n">
         <v>52.54</v>
       </c>
     </row>
@@ -9427,6 +9540,9 @@
         <v>6935.79</v>
       </c>
       <c r="BX47" s="15" t="n">
+        <v>6935.79</v>
+      </c>
+      <c r="BY47" s="15" t="n">
         <v>6935.79</v>
       </c>
     </row>
@@ -9555,6 +9671,7 @@
       <c r="BV48" s="15" t="n"/>
       <c r="BW48" s="15" t="n"/>
       <c r="BX48" s="15" t="n"/>
+      <c r="BY48" s="15" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -9783,6 +9900,9 @@
         <v>19.41</v>
       </c>
       <c r="BX49" s="15" t="n">
+        <v>19.41</v>
+      </c>
+      <c r="BY49" s="15" t="n">
         <v>19.41</v>
       </c>
     </row>
@@ -9966,6 +10086,9 @@
       </c>
       <c r="BX50" s="15" t="n">
         <v>31648.99</v>
+      </c>
+      <c r="BY50" s="15" t="n">
+        <v>31738.74</v>
       </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
@@ -10093,6 +10216,7 @@
       <c r="BV51" s="15" t="n"/>
       <c r="BW51" s="15" t="n"/>
       <c r="BX51" s="15" t="n"/>
+      <c r="BY51" s="15" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -10321,6 +10445,9 @@
         <v>34.84</v>
       </c>
       <c r="BX52" s="15" t="n">
+        <v>34.84</v>
+      </c>
+      <c r="BY52" s="15" t="n">
         <v>34.84</v>
       </c>
     </row>
@@ -10504,6 +10631,9 @@
       </c>
       <c r="BX53" s="15" t="n">
         <v>3239.07</v>
+      </c>
+      <c r="BY53" s="15" t="n">
+        <v>3246.03</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
@@ -10631,6 +10761,7 @@
       <c r="BV54" s="15" t="n"/>
       <c r="BW54" s="15" t="n"/>
       <c r="BX54" s="15" t="n"/>
+      <c r="BY54" s="15" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -10859,6 +10990,9 @@
         <v>42.37</v>
       </c>
       <c r="BX55" s="15" t="n">
+        <v>42.28</v>
+      </c>
+      <c r="BY55" s="15" t="n">
         <v>42.28</v>
       </c>
     </row>
@@ -11042,6 +11176,9 @@
       </c>
       <c r="BX56" s="15" t="n">
         <v>3132.47</v>
+      </c>
+      <c r="BY56" s="15" t="n">
+        <v>3139.82</v>
       </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
@@ -11169,6 +11306,7 @@
       <c r="BV57" s="15" t="n"/>
       <c r="BW57" s="15" t="n"/>
       <c r="BX57" s="15" t="n"/>
+      <c r="BY57" s="15" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -11397,6 +11535,9 @@
         <v>16.66</v>
       </c>
       <c r="BX58" s="15" t="n">
+        <v>15.91</v>
+      </c>
+      <c r="BY58" s="15" t="n">
         <v>15.91</v>
       </c>
     </row>
@@ -11580,6 +11721,9 @@
       </c>
       <c r="BX59" s="15" t="n">
         <v>6698.71</v>
+      </c>
+      <c r="BY59" s="15" t="n">
+        <v>6721.58</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
@@ -11707,6 +11851,7 @@
       <c r="BV60" s="15" t="n"/>
       <c r="BW60" s="15" t="n"/>
       <c r="BX60" s="15" t="n"/>
+      <c r="BY60" s="15" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -11935,6 +12080,9 @@
         <v>30.91</v>
       </c>
       <c r="BX61" s="15" t="n">
+        <v>30.91</v>
+      </c>
+      <c r="BY61" s="15" t="n">
         <v>30.91</v>
       </c>
     </row>
@@ -12118,6 +12266,9 @@
       </c>
       <c r="BX62" s="15" t="n">
         <v>8025.71</v>
+      </c>
+      <c r="BY62" s="15" t="n">
+        <v>8052.78</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
@@ -12245,6 +12396,7 @@
       <c r="BV63" s="15" t="n"/>
       <c r="BW63" s="15" t="n"/>
       <c r="BX63" s="15" t="n"/>
+      <c r="BY63" s="15" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -12473,6 +12625,9 @@
         <v>5.41</v>
       </c>
       <c r="BX64" s="15" t="n">
+        <v>5.41</v>
+      </c>
+      <c r="BY64" s="15" t="n">
         <v>5.41</v>
       </c>
     </row>
@@ -12656,6 +12811,9 @@
       </c>
       <c r="BX65" s="15" t="n">
         <v>10320.59</v>
+      </c>
+      <c r="BY65" s="15" t="n">
+        <v>10367.63</v>
       </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
@@ -12783,6 +12941,7 @@
       <c r="BV66" s="15" t="n"/>
       <c r="BW66" s="15" t="n"/>
       <c r="BX66" s="15" t="n"/>
+      <c r="BY66" s="15" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -13011,6 +13170,9 @@
         <v>19.02</v>
       </c>
       <c r="BX67" s="15" t="n">
+        <v>19.02</v>
+      </c>
+      <c r="BY67" s="15" t="n">
         <v>19.02</v>
       </c>
     </row>
@@ -13193,6 +13355,9 @@
         <v>11219.09</v>
       </c>
       <c r="BX68" s="15" t="n">
+        <v>11219.09</v>
+      </c>
+      <c r="BY68" s="15" t="n">
         <v>11219.09</v>
       </c>
     </row>
@@ -13321,6 +13486,7 @@
       <c r="BV69" s="15" t="n"/>
       <c r="BW69" s="15" t="n"/>
       <c r="BX69" s="15" t="n"/>
+      <c r="BY69" s="15" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -13549,6 +13715,9 @@
         <v>12.82</v>
       </c>
       <c r="BX70" s="15" t="n">
+        <v>12.82</v>
+      </c>
+      <c r="BY70" s="15" t="n">
         <v>12.82</v>
       </c>
     </row>
@@ -13732,6 +13901,9 @@
       </c>
       <c r="BX71" s="15" t="n">
         <v>6044</v>
+      </c>
+      <c r="BY71" s="15" t="n">
+        <v>6049.99</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
@@ -13859,6 +14031,7 @@
       <c r="BV72" s="15" t="n"/>
       <c r="BW72" s="15" t="n"/>
       <c r="BX72" s="15" t="n"/>
+      <c r="BY72" s="15" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -14087,6 +14260,9 @@
         <v>16.36</v>
       </c>
       <c r="BX73" s="15" t="n">
+        <v>16.36</v>
+      </c>
+      <c r="BY73" s="15" t="n">
         <v>16.36</v>
       </c>
     </row>
@@ -14270,6 +14446,9 @@
       </c>
       <c r="BX74" s="15" t="n">
         <v>12078.68</v>
+      </c>
+      <c r="BY74" s="15" t="n">
+        <v>12096.02</v>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
@@ -14397,6 +14576,7 @@
       <c r="BV75" s="15" t="n"/>
       <c r="BW75" s="15" t="n"/>
       <c r="BX75" s="15" t="n"/>
+      <c r="BY75" s="15" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -14625,6 +14805,9 @@
         <v>53.09</v>
       </c>
       <c r="BX76" s="15" t="n">
+        <v>53.09</v>
+      </c>
+      <c r="BY76" s="15" t="n">
         <v>53.09</v>
       </c>
     </row>
@@ -14808,6 +14991,9 @@
       </c>
       <c r="BX77" s="15" t="n">
         <v>15569.82</v>
+      </c>
+      <c r="BY77" s="15" t="n">
+        <v>15805.57</v>
       </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
@@ -14935,6 +15121,7 @@
       <c r="BV78" s="15" t="n"/>
       <c r="BW78" s="15" t="n"/>
       <c r="BX78" s="15" t="n"/>
+      <c r="BY78" s="15" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -15163,6 +15350,9 @@
         <v>2.88</v>
       </c>
       <c r="BX79" s="15" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="BY79" s="15" t="n">
         <v>2.88</v>
       </c>
     </row>
@@ -15346,6 +15536,9 @@
       </c>
       <c r="BX80" s="15" t="n">
         <v>6485.64</v>
+      </c>
+      <c r="BY80" s="15" t="n">
+        <v>6495.47</v>
       </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
@@ -15473,6 +15666,7 @@
       <c r="BV81" s="15" t="n"/>
       <c r="BW81" s="15" t="n"/>
       <c r="BX81" s="15" t="n"/>
+      <c r="BY81" s="15" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -15701,6 +15895,9 @@
         <v>2.92</v>
       </c>
       <c r="BX82" s="15" t="n">
+        <v>2.92</v>
+      </c>
+      <c r="BY82" s="15" t="n">
         <v>2.92</v>
       </c>
     </row>
@@ -15883,6 +16080,9 @@
         <v>8161.87</v>
       </c>
       <c r="BX83" s="15" t="n">
+        <v>8161.87</v>
+      </c>
+      <c r="BY83" s="15" t="n">
         <v>8161.87</v>
       </c>
     </row>
@@ -16011,6 +16211,7 @@
       <c r="BV84" s="15" t="n"/>
       <c r="BW84" s="15" t="n"/>
       <c r="BX84" s="15" t="n"/>
+      <c r="BY84" s="15" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -16239,6 +16440,9 @@
         <v>16.57</v>
       </c>
       <c r="BX85" s="15" t="n">
+        <v>16.57</v>
+      </c>
+      <c r="BY85" s="15" t="n">
         <v>16.57</v>
       </c>
     </row>
@@ -16422,6 +16626,9 @@
       </c>
       <c r="BX86" s="15" t="n">
         <v>2041.04</v>
+      </c>
+      <c r="BY86" s="15" t="n">
+        <v>2631.9</v>
       </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
@@ -16549,6 +16756,7 @@
       <c r="BV87" s="15" t="n"/>
       <c r="BW87" s="15" t="n"/>
       <c r="BX87" s="15" t="n"/>
+      <c r="BY87" s="15" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -16777,6 +16985,9 @@
         <v>26.28</v>
       </c>
       <c r="BX88" s="15" t="n">
+        <v>26.28</v>
+      </c>
+      <c r="BY88" s="15" t="n">
         <v>26.28</v>
       </c>
     </row>
@@ -16960,6 +17171,9 @@
       </c>
       <c r="BX89" s="15" t="n">
         <v>5075.31</v>
+      </c>
+      <c r="BY89" s="15" t="n">
+        <v>4296</v>
       </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
@@ -17087,6 +17301,7 @@
       <c r="BV90" s="15" t="n"/>
       <c r="BW90" s="15" t="n"/>
       <c r="BX90" s="15" t="n"/>
+      <c r="BY90" s="15" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -17315,6 +17530,9 @@
         <v>14.86</v>
       </c>
       <c r="BX91" s="15" t="n">
+        <v>14.68</v>
+      </c>
+      <c r="BY91" s="15" t="n">
         <v>14.68</v>
       </c>
     </row>
@@ -17498,6 +17716,9 @@
       </c>
       <c r="BX92" s="15" t="n">
         <v>8392.030000000001</v>
+      </c>
+      <c r="BY92" s="15" t="n">
+        <v>8420.24</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
@@ -17625,6 +17846,7 @@
       <c r="BV93" s="15" t="n"/>
       <c r="BW93" s="15" t="n"/>
       <c r="BX93" s="15" t="n"/>
+      <c r="BY93" s="15" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -17853,6 +18075,9 @@
         <v>3.9</v>
       </c>
       <c r="BX94" s="15" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="BY94" s="15" t="n">
         <v>3.9</v>
       </c>
     </row>
@@ -18035,6 +18260,9 @@
         <v>1176.71</v>
       </c>
       <c r="BX95" s="15" t="n">
+        <v>1176.71</v>
+      </c>
+      <c r="BY95" s="15" t="n">
         <v>1176.71</v>
       </c>
     </row>
@@ -18163,6 +18391,7 @@
       <c r="BV96" s="15" t="n"/>
       <c r="BW96" s="15" t="n"/>
       <c r="BX96" s="15" t="n"/>
+      <c r="BY96" s="15" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -18391,6 +18620,9 @@
         <v>7.75</v>
       </c>
       <c r="BX97" s="15" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="BY97" s="15" t="n">
         <v>7.75</v>
       </c>
     </row>
@@ -18573,6 +18805,9 @@
         <v>13458.58</v>
       </c>
       <c r="BX98" s="15" t="n">
+        <v>13458.58</v>
+      </c>
+      <c r="BY98" s="15" t="n">
         <v>13458.58</v>
       </c>
     </row>
@@ -18701,6 +18936,7 @@
       <c r="BV99" s="15" t="n"/>
       <c r="BW99" s="15" t="n"/>
       <c r="BX99" s="15" t="n"/>
+      <c r="BY99" s="15" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -18929,6 +19165,9 @@
         <v>34.57</v>
       </c>
       <c r="BX100" s="15" t="n">
+        <v>34.57</v>
+      </c>
+      <c r="BY100" s="15" t="n">
         <v>34.57</v>
       </c>
     </row>
@@ -19111,6 +19350,9 @@
         <v>3257.76</v>
       </c>
       <c r="BX101" s="15" t="n">
+        <v>3257.76</v>
+      </c>
+      <c r="BY101" s="15" t="n">
         <v>3257.76</v>
       </c>
     </row>
@@ -19239,6 +19481,7 @@
       <c r="BV102" s="15" t="n"/>
       <c r="BW102" s="15" t="n"/>
       <c r="BX102" s="15" t="n"/>
+      <c r="BY102" s="15" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -19467,6 +19710,9 @@
         <v>24.74</v>
       </c>
       <c r="BX103" s="15" t="n">
+        <v>24.74</v>
+      </c>
+      <c r="BY103" s="15" t="n">
         <v>24.74</v>
       </c>
     </row>
@@ -19650,6 +19896,9 @@
       </c>
       <c r="BX104" s="15" t="n">
         <v>2136</v>
+      </c>
+      <c r="BY104" s="15" t="n">
+        <v>2138.4</v>
       </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
@@ -19777,6 +20026,7 @@
       <c r="BV105" s="15" t="n"/>
       <c r="BW105" s="15" t="n"/>
       <c r="BX105" s="15" t="n"/>
+      <c r="BY105" s="15" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -20005,6 +20255,9 @@
         <v>15.91</v>
       </c>
       <c r="BX106" s="15" t="n">
+        <v>15.91</v>
+      </c>
+      <c r="BY106" s="15" t="n">
         <v>15.91</v>
       </c>
     </row>
@@ -20188,6 +20441,9 @@
       </c>
       <c r="BX107" s="15" t="n">
         <v>2265.14</v>
+      </c>
+      <c r="BY107" s="15" t="n">
+        <v>2267.7</v>
       </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
@@ -20315,6 +20571,7 @@
       <c r="BV108" s="15" t="n"/>
       <c r="BW108" s="15" t="n"/>
       <c r="BX108" s="15" t="n"/>
+      <c r="BY108" s="15" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -20543,6 +20800,9 @@
         <v>25.78</v>
       </c>
       <c r="BX109" s="15" t="n">
+        <v>25.78</v>
+      </c>
+      <c r="BY109" s="15" t="n">
         <v>25.78</v>
       </c>
     </row>
@@ -20725,6 +20985,9 @@
         <v>2391.95</v>
       </c>
       <c r="BX110" s="15" t="n">
+        <v>2276.69</v>
+      </c>
+      <c r="BY110" s="15" t="n">
         <v>2276.69</v>
       </c>
     </row>
@@ -20853,6 +21116,7 @@
       <c r="BV111" s="15" t="n"/>
       <c r="BW111" s="15" t="n"/>
       <c r="BX111" s="15" t="n"/>
+      <c r="BY111" s="15" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -21081,6 +21345,9 @@
         <v>47.56</v>
       </c>
       <c r="BX112" s="15" t="n">
+        <v>47.56</v>
+      </c>
+      <c r="BY112" s="15" t="n">
         <v>47.56</v>
       </c>
     </row>
@@ -21262,6 +21529,9 @@
       </c>
       <c r="BX113" s="15" t="n">
         <v>1885.92</v>
+      </c>
+      <c r="BY113" s="15" t="n">
+        <v>1892.25</v>
       </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
@@ -21389,6 +21659,7 @@
       <c r="BV114" s="15" t="n"/>
       <c r="BW114" s="15" t="n"/>
       <c r="BX114" s="15" t="n"/>
+      <c r="BY114" s="15" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -21617,6 +21888,9 @@
         <v>16.88</v>
       </c>
       <c r="BX115" s="15" t="n">
+        <v>16.55</v>
+      </c>
+      <c r="BY115" s="15" t="n">
         <v>16.55</v>
       </c>
     </row>
@@ -21785,6 +22059,9 @@
       </c>
       <c r="BX116" s="15" t="n">
         <v>8720.299999999999</v>
+      </c>
+      <c r="BY116" s="15" t="n">
+        <v>8701.969999999999</v>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1">
@@ -21867,6 +22144,7 @@
       <c r="BV117" s="15" t="n"/>
       <c r="BW117" s="15" t="n"/>
       <c r="BX117" s="15" t="n"/>
+      <c r="BY117" s="15" t="n"/>
     </row>
     <row r="118" ht="14.25" customHeight="1">
       <c r="P118" s="13" t="n">
@@ -22052,6 +22330,9 @@
       <c r="BX118" s="15" t="n">
         <v>74.56</v>
       </c>
+      <c r="BY118" s="15" t="n">
+        <v>74.56</v>
+      </c>
     </row>
     <row r="119" ht="14.25" customHeight="1">
       <c r="Y119" s="13" t="n">
@@ -22209,6 +22490,9 @@
       </c>
       <c r="BX119" s="15" t="n">
         <v>12333.91</v>
+      </c>
+      <c r="BY119" s="15" t="n">
+        <v>12354.37</v>
       </c>
     </row>
     <row r="120" ht="14.25" customHeight="1">
@@ -22240,6 +22524,7 @@
       <c r="BV120" s="15" t="n"/>
       <c r="BW120" s="15" t="n"/>
       <c r="BX120" s="15" t="n"/>
+      <c r="BY120" s="15" t="n"/>
     </row>
     <row r="121" ht="14.25" customHeight="1">
       <c r="AW121" s="13" t="n">
@@ -22326,6 +22611,9 @@
       <c r="BX121" s="15" t="n">
         <v>22.04</v>
       </c>
+      <c r="BY121" s="15" t="n">
+        <v>22.04</v>
+      </c>
     </row>
     <row r="122" ht="14.25" customHeight="1">
       <c r="AW122" s="13" t="n">
@@ -22410,6 +22698,9 @@
         <v>1179.2</v>
       </c>
       <c r="BX122" s="15" t="n">
+        <v>1179.2</v>
+      </c>
+      <c r="BY122" s="15" t="n">
         <v>1179.2</v>
       </c>
     </row>
@@ -22442,6 +22733,7 @@
       <c r="BV123" s="15" t="n"/>
       <c r="BW123" s="15" t="n"/>
       <c r="BX123" s="15" t="n"/>
+      <c r="BY123" s="15" t="n"/>
     </row>
     <row r="124" ht="14.25" customHeight="1">
       <c r="AW124" s="13" t="n">
@@ -22528,6 +22820,9 @@
       <c r="BX124" s="15" t="n">
         <v>43.4</v>
       </c>
+      <c r="BY124" s="15" t="n">
+        <v>43.4</v>
+      </c>
     </row>
     <row r="125" ht="14.25" customHeight="1">
       <c r="AW125" s="13" t="n">
@@ -22613,6 +22908,9 @@
       </c>
       <c r="BX125" s="15" t="n">
         <v>11125.13</v>
+      </c>
+      <c r="BY125" s="15" t="n">
+        <v>11132.25</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1">
@@ -22644,6 +22942,7 @@
       <c r="BV126" s="15" t="n"/>
       <c r="BW126" s="15" t="n"/>
       <c r="BX126" s="15" t="n"/>
+      <c r="BY126" s="15" t="n"/>
     </row>
     <row r="127" ht="14.25" customHeight="1">
       <c r="AW127" s="13" t="n">
@@ -22730,6 +23029,9 @@
       <c r="BX127" s="15" t="n">
         <v>2.32</v>
       </c>
+      <c r="BY127" s="15" t="n">
+        <v>2.32</v>
+      </c>
     </row>
     <row r="128" ht="14.25" customHeight="1">
       <c r="AW128" s="13" t="n">
@@ -22815,6 +23117,9 @@
       </c>
       <c r="BX128" s="15" t="n">
         <v>1813.99</v>
+      </c>
+      <c r="BY128" s="15" t="n">
+        <v>1823.05</v>
       </c>
     </row>
     <row r="129" ht="14.25" customHeight="1">
@@ -22846,6 +23151,7 @@
       <c r="BV129" s="15" t="n"/>
       <c r="BW129" s="15" t="n"/>
       <c r="BX129" s="15" t="n"/>
+      <c r="BY129" s="15" t="n"/>
     </row>
     <row r="130" ht="14.25" customHeight="1">
       <c r="AW130" s="13" t="n">
@@ -22932,6 +23238,9 @@
       <c r="BX130" s="15" t="n">
         <v>6.5</v>
       </c>
+      <c r="BY130" s="15" t="n">
+        <v>6.5</v>
+      </c>
     </row>
     <row r="131" ht="14.25" customHeight="1">
       <c r="AW131" s="13" t="n">
@@ -23017,6 +23326,9 @@
       </c>
       <c r="BX131" s="15" t="n">
         <v>712.1</v>
+      </c>
+      <c r="BY131" s="15" t="n">
+        <v>712.95</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1">
@@ -23048,6 +23360,7 @@
       <c r="BV132" s="15" t="n"/>
       <c r="BW132" s="15" t="n"/>
       <c r="BX132" s="15" t="n"/>
+      <c r="BY132" s="15" t="n"/>
     </row>
     <row r="133" ht="14.25" customHeight="1">
       <c r="AW133" s="13" t="n">
@@ -23134,6 +23447,9 @@
       <c r="BX133" s="15" t="n">
         <v>47.6</v>
       </c>
+      <c r="BY133" s="15" t="n">
+        <v>47.6</v>
+      </c>
     </row>
     <row r="134" ht="14.25" customHeight="1">
       <c r="AW134" s="13" t="n">
@@ -23219,6 +23535,9 @@
       </c>
       <c r="BX134" s="15" t="n">
         <v>2738.48</v>
+      </c>
+      <c r="BY134" s="15" t="n">
+        <v>2638.92</v>
       </c>
     </row>
     <row r="135" ht="14.25" customHeight="1">
@@ -23250,6 +23569,7 @@
       <c r="BV135" s="15" t="n"/>
       <c r="BW135" s="15" t="n"/>
       <c r="BX135" s="15" t="n"/>
+      <c r="BY135" s="15" t="n"/>
     </row>
     <row r="136" ht="14.25" customHeight="1">
       <c r="AW136" s="13" t="n">
@@ -23336,6 +23656,9 @@
       <c r="BX136" s="15" t="n">
         <v>21.14</v>
       </c>
+      <c r="BY136" s="15" t="n">
+        <v>21.14</v>
+      </c>
     </row>
     <row r="137" ht="14.25" customHeight="1">
       <c r="AW137" s="13" t="n">
@@ -23421,6 +23744,9 @@
       </c>
       <c r="BX137" s="15" t="n">
         <v>3404.06</v>
+      </c>
+      <c r="BY137" s="15" t="n">
+        <v>3409.69</v>
       </c>
     </row>
     <row r="138">
@@ -23444,6 +23770,7 @@
       <c r="BV138" s="15" t="n"/>
       <c r="BW138" s="15" t="n"/>
       <c r="BX138" s="15" t="n"/>
+      <c r="BY138" s="15" t="n"/>
     </row>
     <row r="139">
       <c r="BE139" s="15" t="n">
@@ -23506,6 +23833,9 @@
       <c r="BX139" s="15" t="n">
         <v>4.56</v>
       </c>
+      <c r="BY139" s="15" t="n">
+        <v>4.56</v>
+      </c>
     </row>
     <row r="140">
       <c r="BE140" s="15" t="n">
@@ -23564,6 +23894,9 @@
         <v>2497.34</v>
       </c>
       <c r="BX140" s="15" t="n">
+        <v>2497.34</v>
+      </c>
+      <c r="BY140" s="15" t="n">
         <v>2497.34</v>
       </c>
     </row>
@@ -23588,6 +23921,7 @@
       <c r="BV141" s="15" t="n"/>
       <c r="BW141" s="15" t="n"/>
       <c r="BX141" s="15" t="n"/>
+      <c r="BY141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="BE142" s="15" t="n">
@@ -23650,6 +23984,9 @@
       <c r="BX142" s="15" t="n">
         <v>15.3</v>
       </c>
+      <c r="BY142" s="15" t="n">
+        <v>15.3</v>
+      </c>
     </row>
     <row r="143">
       <c r="BE143" s="15" t="n">
@@ -23710,6 +24047,9 @@
         <v>5561.12</v>
       </c>
       <c r="BX143" s="15" t="n">
+        <v>5561.12</v>
+      </c>
+      <c r="BY143" s="15" t="n">
         <v>5561.12</v>
       </c>
     </row>
@@ -23729,6 +24069,7 @@
       <c r="BV144" s="15" t="n"/>
       <c r="BW144" s="15" t="n"/>
       <c r="BX144" s="15" t="n"/>
+      <c r="BY144" s="15" t="n"/>
     </row>
     <row r="145">
       <c r="BJ145" s="15" t="n">
@@ -23776,6 +24117,9 @@
       <c r="BX145" s="15" t="n">
         <v>1.59</v>
       </c>
+      <c r="BY145" s="15" t="n">
+        <v>1.59</v>
+      </c>
     </row>
     <row r="146">
       <c r="BJ146" s="15" t="n">
@@ -23821,6 +24165,9 @@
         <v>2207.48</v>
       </c>
       <c r="BX146" s="15" t="n">
+        <v>2207.48</v>
+      </c>
+      <c r="BY146" s="15" t="n">
         <v>2207.48</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-10-01 10:29:57]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BY146"/>
+  <dimension ref="A1:BZ146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="51"/>
@@ -611,6 +611,7 @@
     <col width="15" customWidth="1" min="75" max="75"/>
     <col width="15" customWidth="1" min="76" max="76"/>
     <col width="15" customWidth="1" min="77" max="77"/>
+    <col width="15" customWidth="1" min="78" max="78"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -999,6 +1000,11 @@
           <t>2026/09/28</t>
         </is>
       </c>
+      <c r="BZ1" s="15" t="inlineStr">
+        <is>
+          <t>2026/10/01</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1386,6 +1392,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="BZ2" s="16" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1619,6 +1630,9 @@
       <c r="BY3" s="15" t="n">
         <v>58.63</v>
       </c>
+      <c r="BZ3" s="15" t="n">
+        <v>57.07</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1851,6 +1865,9 @@
       </c>
       <c r="BY4" s="15" t="n">
         <v>3823.62</v>
+      </c>
+      <c r="BZ4" s="15" t="n">
+        <v>3842.19</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1931,6 +1948,7 @@
       <c r="BW5" s="15" t="n"/>
       <c r="BX5" s="15" t="n"/>
       <c r="BY5" s="15" t="n"/>
+      <c r="BZ5" s="15" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -2058,6 +2076,7 @@
       <c r="BW6" s="15" t="n"/>
       <c r="BX6" s="15" t="n"/>
       <c r="BY6" s="15" t="n"/>
+      <c r="BZ6" s="15" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -2290,6 +2309,9 @@
       </c>
       <c r="BY7" s="15" t="n">
         <v>49.88</v>
+      </c>
+      <c r="BZ7" s="15" t="n">
+        <v>47.39</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -2475,6 +2497,9 @@
       </c>
       <c r="BY8" s="15" t="n">
         <v>5348.5</v>
+      </c>
+      <c r="BZ8" s="15" t="n">
+        <v>5370.26</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
@@ -2603,6 +2628,7 @@
       <c r="BW9" s="15" t="n"/>
       <c r="BX9" s="15" t="n"/>
       <c r="BY9" s="15" t="n"/>
+      <c r="BZ9" s="15" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -2835,6 +2861,9 @@
       </c>
       <c r="BY10" s="15" t="n">
         <v>44.58</v>
+      </c>
+      <c r="BZ10" s="15" t="n">
+        <v>43.3</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -3020,6 +3049,9 @@
       </c>
       <c r="BY11" s="15" t="n">
         <v>4340.76</v>
+      </c>
+      <c r="BZ11" s="15" t="n">
+        <v>4357.62</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
@@ -3148,6 +3180,7 @@
       <c r="BW12" s="15" t="n"/>
       <c r="BX12" s="15" t="n"/>
       <c r="BY12" s="15" t="n"/>
+      <c r="BZ12" s="15" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -3380,6 +3413,9 @@
       </c>
       <c r="BY13" s="15" t="n">
         <v>58.12</v>
+      </c>
+      <c r="BZ13" s="15" t="n">
+        <v>55.81</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -3565,6 +3601,9 @@
       </c>
       <c r="BY14" s="15" t="n">
         <v>7402.3</v>
+      </c>
+      <c r="BZ14" s="15" t="n">
+        <v>7435.16</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
@@ -3693,6 +3732,7 @@
       <c r="BW15" s="15" t="n"/>
       <c r="BX15" s="15" t="n"/>
       <c r="BY15" s="15" t="n"/>
+      <c r="BZ15" s="15" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -3925,6 +3965,9 @@
       </c>
       <c r="BY16" s="15" t="n">
         <v>27.42</v>
+      </c>
+      <c r="BZ16" s="15" t="n">
+        <v>25.62</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -4110,6 +4153,9 @@
       </c>
       <c r="BY17" s="15" t="n">
         <v>2495.36</v>
+      </c>
+      <c r="BZ17" s="15" t="n">
+        <v>2461.21</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
@@ -4238,6 +4284,7 @@
       <c r="BW18" s="15" t="n"/>
       <c r="BX18" s="15" t="n"/>
       <c r="BY18" s="15" t="n"/>
+      <c r="BZ18" s="15" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -4470,6 +4517,9 @@
       </c>
       <c r="BY19" s="15" t="n">
         <v>80.64</v>
+      </c>
+      <c r="BZ19" s="15" t="n">
+        <v>79.77</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -4655,6 +4705,9 @@
       </c>
       <c r="BY20" s="15" t="n">
         <v>7743.41</v>
+      </c>
+      <c r="BZ20" s="15" t="n">
+        <v>7651.54</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
@@ -4783,6 +4836,7 @@
       <c r="BW21" s="15" t="n"/>
       <c r="BX21" s="15" t="n"/>
       <c r="BY21" s="15" t="n"/>
+      <c r="BZ21" s="15" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -5012,6 +5066,9 @@
         <v>36.34</v>
       </c>
       <c r="BY22" s="15" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="BZ22" s="15" t="n">
         <v>36.34</v>
       </c>
     </row>
@@ -5198,6 +5255,9 @@
       </c>
       <c r="BY23" s="15" t="n">
         <v>72805.78</v>
+      </c>
+      <c r="BZ23" s="15" t="n">
+        <v>71909.7</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
@@ -5326,6 +5386,7 @@
       <c r="BW24" s="15" t="n"/>
       <c r="BX24" s="15" t="n"/>
       <c r="BY24" s="15" t="n"/>
+      <c r="BZ24" s="15" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -5557,6 +5618,9 @@
         <v>49.88</v>
       </c>
       <c r="BY25" s="15" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="BZ25" s="15" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -5729,6 +5793,9 @@
       </c>
       <c r="BY26" s="15" t="n">
         <v>25419.65</v>
+      </c>
+      <c r="BZ26" s="15" t="n">
+        <v>25025.14</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
@@ -5857,6 +5924,7 @@
       <c r="BW27" s="15" t="n"/>
       <c r="BX27" s="15" t="n"/>
       <c r="BY27" s="15" t="n"/>
+      <c r="BZ27" s="15" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -6088,6 +6156,9 @@
         <v>92.09</v>
       </c>
       <c r="BY28" s="15" t="n">
+        <v>92.09</v>
+      </c>
+      <c r="BZ28" s="15" t="n">
         <v>92.09</v>
       </c>
     </row>
@@ -6274,6 +6345,9 @@
       </c>
       <c r="BY29" s="15" t="n">
         <v>65877.62</v>
+      </c>
+      <c r="BZ29" s="15" t="n">
+        <v>68956.72</v>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
@@ -6402,6 +6476,7 @@
       <c r="BW30" s="15" t="n"/>
       <c r="BX30" s="15" t="n"/>
       <c r="BY30" s="15" t="n"/>
+      <c r="BZ30" s="15" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -6633,6 +6708,9 @@
         <v>97.44</v>
       </c>
       <c r="BY31" s="15" t="n">
+        <v>97.44</v>
+      </c>
+      <c r="BZ31" s="15" t="n">
         <v>97.44</v>
       </c>
     </row>
@@ -6819,6 +6897,9 @@
       </c>
       <c r="BY32" s="15" t="n">
         <v>6889.74</v>
+      </c>
+      <c r="BZ32" s="15" t="n">
+        <v>6971.35</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
@@ -6947,6 +7028,7 @@
       <c r="BW33" s="15" t="n"/>
       <c r="BX33" s="15" t="n"/>
       <c r="BY33" s="15" t="n"/>
+      <c r="BZ33" s="15" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -7179,6 +7261,9 @@
       </c>
       <c r="BY34" s="15" t="n">
         <v>45.51</v>
+      </c>
+      <c r="BZ34" s="15" t="n">
+        <v>47.21</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -7364,6 +7449,9 @@
       </c>
       <c r="BY35" s="15" t="n">
         <v>5439.6</v>
+      </c>
+      <c r="BZ35" s="15" t="n">
+        <v>5493.34</v>
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
@@ -7492,6 +7580,7 @@
       <c r="BW36" s="15" t="n"/>
       <c r="BX36" s="15" t="n"/>
       <c r="BY36" s="15" t="n"/>
+      <c r="BZ36" s="15" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -7724,6 +7813,9 @@
       </c>
       <c r="BY37" s="15" t="n">
         <v>50.37</v>
+      </c>
+      <c r="BZ37" s="15" t="n">
+        <v>55.99</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -7909,6 +8001,9 @@
       </c>
       <c r="BY38" s="15" t="n">
         <v>11122.04</v>
+      </c>
+      <c r="BZ38" s="15" t="n">
+        <v>11285.61</v>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
@@ -8037,6 +8132,7 @@
       <c r="BW39" s="15" t="n"/>
       <c r="BX39" s="15" t="n"/>
       <c r="BY39" s="15" t="n"/>
+      <c r="BZ39" s="15" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -8269,6 +8365,9 @@
       </c>
       <c r="BY40" s="15" t="n">
         <v>48.39</v>
+      </c>
+      <c r="BZ40" s="15" t="n">
+        <v>52.27</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -8454,6 +8553,9 @@
       </c>
       <c r="BY41" s="15" t="n">
         <v>10848.95</v>
+      </c>
+      <c r="BZ41" s="15" t="n">
+        <v>10971.43</v>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
@@ -8582,6 +8684,7 @@
       <c r="BW42" s="15" t="n"/>
       <c r="BX42" s="15" t="n"/>
       <c r="BY42" s="15" t="n"/>
+      <c r="BZ42" s="15" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -8814,6 +8917,9 @@
       </c>
       <c r="BY43" s="15" t="n">
         <v>48.99</v>
+      </c>
+      <c r="BZ43" s="15" t="n">
+        <v>49.8</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -8999,6 +9105,9 @@
       </c>
       <c r="BY44" s="15" t="n">
         <v>3263.3</v>
+      </c>
+      <c r="BZ44" s="15" t="n">
+        <v>3271.9</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
@@ -9127,6 +9236,7 @@
       <c r="BW45" s="15" t="n"/>
       <c r="BX45" s="15" t="n"/>
       <c r="BY45" s="15" t="n"/>
+      <c r="BZ45" s="15" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -9359,6 +9469,9 @@
       </c>
       <c r="BY46" s="15" t="n">
         <v>52.54</v>
+      </c>
+      <c r="BZ46" s="15" t="n">
+        <v>61.04</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -9544,6 +9657,9 @@
       </c>
       <c r="BY47" s="15" t="n">
         <v>6935.79</v>
+      </c>
+      <c r="BZ47" s="15" t="n">
+        <v>7025.76</v>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
@@ -9672,6 +9788,7 @@
       <c r="BW48" s="15" t="n"/>
       <c r="BX48" s="15" t="n"/>
       <c r="BY48" s="15" t="n"/>
+      <c r="BZ48" s="15" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -9904,6 +10021,9 @@
       </c>
       <c r="BY49" s="15" t="n">
         <v>19.41</v>
+      </c>
+      <c r="BZ49" s="15" t="n">
+        <v>19.57</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -10089,6 +10209,9 @@
       </c>
       <c r="BY50" s="15" t="n">
         <v>31738.74</v>
+      </c>
+      <c r="BZ50" s="15" t="n">
+        <v>32172.27</v>
       </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
@@ -10217,6 +10340,7 @@
       <c r="BW51" s="15" t="n"/>
       <c r="BX51" s="15" t="n"/>
       <c r="BY51" s="15" t="n"/>
+      <c r="BZ51" s="15" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -10449,6 +10573,9 @@
       </c>
       <c r="BY52" s="15" t="n">
         <v>34.84</v>
+      </c>
+      <c r="BZ52" s="15" t="n">
+        <v>29.77</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -10634,6 +10761,9 @@
       </c>
       <c r="BY53" s="15" t="n">
         <v>3246.03</v>
+      </c>
+      <c r="BZ53" s="15" t="n">
+        <v>3240.53</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
@@ -10762,6 +10892,7 @@
       <c r="BW54" s="15" t="n"/>
       <c r="BX54" s="15" t="n"/>
       <c r="BY54" s="15" t="n"/>
+      <c r="BZ54" s="15" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -10994,6 +11125,9 @@
       </c>
       <c r="BY55" s="15" t="n">
         <v>42.28</v>
+      </c>
+      <c r="BZ55" s="15" t="n">
+        <v>38.37</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -11179,6 +11313,9 @@
       </c>
       <c r="BY56" s="15" t="n">
         <v>3139.82</v>
+      </c>
+      <c r="BZ56" s="15" t="n">
+        <v>3135.28</v>
       </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
@@ -11307,6 +11444,7 @@
       <c r="BW57" s="15" t="n"/>
       <c r="BX57" s="15" t="n"/>
       <c r="BY57" s="15" t="n"/>
+      <c r="BZ57" s="15" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -11539,6 +11677,9 @@
       </c>
       <c r="BY58" s="15" t="n">
         <v>15.91</v>
+      </c>
+      <c r="BZ58" s="15" t="n">
+        <v>19.41</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -11724,6 +11865,9 @@
       </c>
       <c r="BY59" s="15" t="n">
         <v>6721.58</v>
+      </c>
+      <c r="BZ59" s="15" t="n">
+        <v>6883.56</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
@@ -11852,6 +11996,7 @@
       <c r="BW60" s="15" t="n"/>
       <c r="BX60" s="15" t="n"/>
       <c r="BY60" s="15" t="n"/>
+      <c r="BZ60" s="15" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -12084,6 +12229,9 @@
       </c>
       <c r="BY61" s="15" t="n">
         <v>30.91</v>
+      </c>
+      <c r="BZ61" s="15" t="n">
+        <v>37.19</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -12269,6 +12417,9 @@
       </c>
       <c r="BY62" s="15" t="n">
         <v>8052.78</v>
+      </c>
+      <c r="BZ62" s="15" t="n">
+        <v>8323.309999999999</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
@@ -12397,6 +12548,7 @@
       <c r="BW63" s="15" t="n"/>
       <c r="BX63" s="15" t="n"/>
       <c r="BY63" s="15" t="n"/>
+      <c r="BZ63" s="15" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -12629,6 +12781,9 @@
       </c>
       <c r="BY64" s="15" t="n">
         <v>5.41</v>
+      </c>
+      <c r="BZ64" s="15" t="n">
+        <v>6.29</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -12814,6 +12969,9 @@
       </c>
       <c r="BY65" s="15" t="n">
         <v>10367.63</v>
+      </c>
+      <c r="BZ65" s="15" t="n">
+        <v>10401.01</v>
       </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
@@ -12942,6 +13100,7 @@
       <c r="BW66" s="15" t="n"/>
       <c r="BX66" s="15" t="n"/>
       <c r="BY66" s="15" t="n"/>
+      <c r="BZ66" s="15" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -13174,6 +13333,9 @@
       </c>
       <c r="BY67" s="15" t="n">
         <v>19.02</v>
+      </c>
+      <c r="BZ67" s="15" t="n">
+        <v>15.25</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -13359,6 +13521,9 @@
       </c>
       <c r="BY68" s="15" t="n">
         <v>11219.09</v>
+      </c>
+      <c r="BZ68" s="15" t="n">
+        <v>11058.05</v>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
@@ -13487,6 +13652,7 @@
       <c r="BW69" s="15" t="n"/>
       <c r="BX69" s="15" t="n"/>
       <c r="BY69" s="15" t="n"/>
+      <c r="BZ69" s="15" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -13719,6 +13885,9 @@
       </c>
       <c r="BY70" s="15" t="n">
         <v>12.82</v>
+      </c>
+      <c r="BZ70" s="15" t="n">
+        <v>15.18</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -13904,6 +14073,9 @@
       </c>
       <c r="BY71" s="15" t="n">
         <v>6049.99</v>
+      </c>
+      <c r="BZ71" s="15" t="n">
+        <v>6228.9</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
@@ -14032,6 +14204,7 @@
       <c r="BW72" s="15" t="n"/>
       <c r="BX72" s="15" t="n"/>
       <c r="BY72" s="15" t="n"/>
+      <c r="BZ72" s="15" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -14264,6 +14437,9 @@
       </c>
       <c r="BY73" s="15" t="n">
         <v>16.36</v>
+      </c>
+      <c r="BZ73" s="15" t="n">
+        <v>17.67</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -14449,6 +14625,9 @@
       </c>
       <c r="BY74" s="15" t="n">
         <v>12096.02</v>
+      </c>
+      <c r="BZ74" s="15" t="n">
+        <v>12295.96</v>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
@@ -14577,6 +14756,7 @@
       <c r="BW75" s="15" t="n"/>
       <c r="BX75" s="15" t="n"/>
       <c r="BY75" s="15" t="n"/>
+      <c r="BZ75" s="15" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -14808,6 +14988,9 @@
         <v>53.09</v>
       </c>
       <c r="BY76" s="15" t="n">
+        <v>53.09</v>
+      </c>
+      <c r="BZ76" s="15" t="n">
         <v>53.09</v>
       </c>
     </row>
@@ -14994,6 +15177,9 @@
       </c>
       <c r="BY77" s="15" t="n">
         <v>15805.57</v>
+      </c>
+      <c r="BZ77" s="15" t="n">
+        <v>16651.14</v>
       </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
@@ -15122,6 +15308,7 @@
       <c r="BW78" s="15" t="n"/>
       <c r="BX78" s="15" t="n"/>
       <c r="BY78" s="15" t="n"/>
+      <c r="BZ78" s="15" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -15354,6 +15541,9 @@
       </c>
       <c r="BY79" s="15" t="n">
         <v>2.88</v>
+      </c>
+      <c r="BZ79" s="15" t="n">
+        <v>1.79</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -15539,6 +15729,9 @@
       </c>
       <c r="BY80" s="15" t="n">
         <v>6495.47</v>
+      </c>
+      <c r="BZ80" s="15" t="n">
+        <v>6406.02</v>
       </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
@@ -15667,6 +15860,7 @@
       <c r="BW81" s="15" t="n"/>
       <c r="BX81" s="15" t="n"/>
       <c r="BY81" s="15" t="n"/>
+      <c r="BZ81" s="15" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -15899,6 +16093,9 @@
       </c>
       <c r="BY82" s="15" t="n">
         <v>2.92</v>
+      </c>
+      <c r="BZ82" s="15" t="n">
+        <v>3.58</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -16084,6 +16281,9 @@
       </c>
       <c r="BY83" s="15" t="n">
         <v>8161.87</v>
+      </c>
+      <c r="BZ83" s="15" t="n">
+        <v>8284.629999999999</v>
       </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
@@ -16212,6 +16412,7 @@
       <c r="BW84" s="15" t="n"/>
       <c r="BX84" s="15" t="n"/>
       <c r="BY84" s="15" t="n"/>
+      <c r="BZ84" s="15" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -16444,6 +16645,9 @@
       </c>
       <c r="BY85" s="15" t="n">
         <v>16.57</v>
+      </c>
+      <c r="BZ85" s="15" t="n">
+        <v>16.02</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -16629,6 +16833,9 @@
       </c>
       <c r="BY86" s="15" t="n">
         <v>2631.9</v>
+      </c>
+      <c r="BZ86" s="15" t="n">
+        <v>2038.77</v>
       </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
@@ -16757,6 +16964,7 @@
       <c r="BW87" s="15" t="n"/>
       <c r="BX87" s="15" t="n"/>
       <c r="BY87" s="15" t="n"/>
+      <c r="BZ87" s="15" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -16989,6 +17197,9 @@
       </c>
       <c r="BY88" s="15" t="n">
         <v>26.28</v>
+      </c>
+      <c r="BZ88" s="15" t="n">
+        <v>23.92</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -17174,6 +17385,9 @@
       </c>
       <c r="BY89" s="15" t="n">
         <v>4296</v>
+      </c>
+      <c r="BZ89" s="15" t="n">
+        <v>4253.89</v>
       </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
@@ -17302,6 +17516,7 @@
       <c r="BW90" s="15" t="n"/>
       <c r="BX90" s="15" t="n"/>
       <c r="BY90" s="15" t="n"/>
+      <c r="BZ90" s="15" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -17534,6 +17749,9 @@
       </c>
       <c r="BY91" s="15" t="n">
         <v>14.68</v>
+      </c>
+      <c r="BZ91" s="15" t="n">
+        <v>19.19</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -17719,6 +17937,9 @@
       </c>
       <c r="BY92" s="15" t="n">
         <v>8420.24</v>
+      </c>
+      <c r="BZ92" s="15" t="n">
+        <v>8679.559999999999</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
@@ -17847,6 +18068,7 @@
       <c r="BW93" s="15" t="n"/>
       <c r="BX93" s="15" t="n"/>
       <c r="BY93" s="15" t="n"/>
+      <c r="BZ93" s="15" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -18079,6 +18301,9 @@
       </c>
       <c r="BY94" s="15" t="n">
         <v>3.9</v>
+      </c>
+      <c r="BZ94" s="15" t="n">
+        <v>4.22</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -18264,6 +18489,9 @@
       </c>
       <c r="BY95" s="15" t="n">
         <v>1176.71</v>
+      </c>
+      <c r="BZ95" s="15" t="n">
+        <v>1174.56</v>
       </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
@@ -18392,6 +18620,7 @@
       <c r="BW96" s="15" t="n"/>
       <c r="BX96" s="15" t="n"/>
       <c r="BY96" s="15" t="n"/>
+      <c r="BZ96" s="15" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -18624,6 +18853,9 @@
       </c>
       <c r="BY97" s="15" t="n">
         <v>7.75</v>
+      </c>
+      <c r="BZ97" s="15" t="n">
+        <v>8.539999999999999</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -18809,6 +19041,9 @@
       </c>
       <c r="BY98" s="15" t="n">
         <v>13458.58</v>
+      </c>
+      <c r="BZ98" s="15" t="n">
+        <v>13618.21</v>
       </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
@@ -18937,6 +19172,7 @@
       <c r="BW99" s="15" t="n"/>
       <c r="BX99" s="15" t="n"/>
       <c r="BY99" s="15" t="n"/>
+      <c r="BZ99" s="15" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -19169,6 +19405,9 @@
       </c>
       <c r="BY100" s="15" t="n">
         <v>34.57</v>
+      </c>
+      <c r="BZ100" s="15" t="n">
+        <v>39.69</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -19354,6 +19593,9 @@
       </c>
       <c r="BY101" s="15" t="n">
         <v>3257.76</v>
+      </c>
+      <c r="BZ101" s="15" t="n">
+        <v>3360.25</v>
       </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
@@ -19482,6 +19724,7 @@
       <c r="BW102" s="15" t="n"/>
       <c r="BX102" s="15" t="n"/>
       <c r="BY102" s="15" t="n"/>
+      <c r="BZ102" s="15" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -19714,6 +19957,9 @@
       </c>
       <c r="BY103" s="15" t="n">
         <v>24.74</v>
+      </c>
+      <c r="BZ103" s="15" t="n">
+        <v>23.92</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -19899,6 +20145,9 @@
       </c>
       <c r="BY104" s="15" t="n">
         <v>2138.4</v>
+      </c>
+      <c r="BZ104" s="15" t="n">
+        <v>2173.93</v>
       </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
@@ -20027,6 +20276,7 @@
       <c r="BW105" s="15" t="n"/>
       <c r="BX105" s="15" t="n"/>
       <c r="BY105" s="15" t="n"/>
+      <c r="BZ105" s="15" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -20259,6 +20509,9 @@
       </c>
       <c r="BY106" s="15" t="n">
         <v>15.91</v>
+      </c>
+      <c r="BZ106" s="15" t="n">
+        <v>11.98</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -20444,6 +20697,9 @@
       </c>
       <c r="BY107" s="15" t="n">
         <v>2267.7</v>
+      </c>
+      <c r="BZ107" s="15" t="n">
+        <v>2289.53</v>
       </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
@@ -20572,6 +20828,7 @@
       <c r="BW108" s="15" t="n"/>
       <c r="BX108" s="15" t="n"/>
       <c r="BY108" s="15" t="n"/>
+      <c r="BZ108" s="15" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -20804,6 +21061,9 @@
       </c>
       <c r="BY109" s="15" t="n">
         <v>25.78</v>
+      </c>
+      <c r="BZ109" s="15" t="n">
+        <v>24.89</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -20989,6 +21249,9 @@
       </c>
       <c r="BY110" s="15" t="n">
         <v>2276.69</v>
+      </c>
+      <c r="BZ110" s="15" t="n">
+        <v>2312.43</v>
       </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
@@ -21117,6 +21380,7 @@
       <c r="BW111" s="15" t="n"/>
       <c r="BX111" s="15" t="n"/>
       <c r="BY111" s="15" t="n"/>
+      <c r="BZ111" s="15" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -21349,6 +21613,9 @@
       </c>
       <c r="BY112" s="15" t="n">
         <v>47.56</v>
+      </c>
+      <c r="BZ112" s="15" t="n">
+        <v>53.65</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -21532,6 +21799,9 @@
       </c>
       <c r="BY113" s="15" t="n">
         <v>1892.25</v>
+      </c>
+      <c r="BZ113" s="15" t="n">
+        <v>1963.8</v>
       </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
@@ -21660,6 +21930,7 @@
       <c r="BW114" s="15" t="n"/>
       <c r="BX114" s="15" t="n"/>
       <c r="BY114" s="15" t="n"/>
+      <c r="BZ114" s="15" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -21892,6 +22163,9 @@
       </c>
       <c r="BY115" s="15" t="n">
         <v>16.55</v>
+      </c>
+      <c r="BZ115" s="15" t="n">
+        <v>18.24</v>
       </c>
     </row>
     <row r="116" ht="14.25" customHeight="1">
@@ -22061,6 +22335,9 @@
         <v>8720.299999999999</v>
       </c>
       <c r="BY116" s="15" t="n">
+        <v>8701.969999999999</v>
+      </c>
+      <c r="BZ116" s="15" t="n">
         <v>8701.969999999999</v>
       </c>
     </row>
@@ -22145,6 +22422,7 @@
       <c r="BW117" s="15" t="n"/>
       <c r="BX117" s="15" t="n"/>
       <c r="BY117" s="15" t="n"/>
+      <c r="BZ117" s="15" t="n"/>
     </row>
     <row r="118" ht="14.25" customHeight="1">
       <c r="P118" s="13" t="n">
@@ -22333,6 +22611,9 @@
       <c r="BY118" s="15" t="n">
         <v>74.56</v>
       </c>
+      <c r="BZ118" s="15" t="n">
+        <v>69.3</v>
+      </c>
     </row>
     <row r="119" ht="14.25" customHeight="1">
       <c r="Y119" s="13" t="n">
@@ -22493,6 +22774,9 @@
       </c>
       <c r="BY119" s="15" t="n">
         <v>12354.37</v>
+      </c>
+      <c r="BZ119" s="15" t="n">
+        <v>12036.57</v>
       </c>
     </row>
     <row r="120" ht="14.25" customHeight="1">
@@ -22525,6 +22809,7 @@
       <c r="BW120" s="15" t="n"/>
       <c r="BX120" s="15" t="n"/>
       <c r="BY120" s="15" t="n"/>
+      <c r="BZ120" s="15" t="n"/>
     </row>
     <row r="121" ht="14.25" customHeight="1">
       <c r="AW121" s="13" t="n">
@@ -22614,6 +22899,9 @@
       <c r="BY121" s="15" t="n">
         <v>22.04</v>
       </c>
+      <c r="BZ121" s="15" t="n">
+        <v>21.06</v>
+      </c>
     </row>
     <row r="122" ht="14.25" customHeight="1">
       <c r="AW122" s="13" t="n">
@@ -22702,6 +22990,9 @@
       </c>
       <c r="BY122" s="15" t="n">
         <v>1179.2</v>
+      </c>
+      <c r="BZ122" s="15" t="n">
+        <v>1161.09</v>
       </c>
     </row>
     <row r="123" ht="14.25" customHeight="1">
@@ -22734,6 +23025,7 @@
       <c r="BW123" s="15" t="n"/>
       <c r="BX123" s="15" t="n"/>
       <c r="BY123" s="15" t="n"/>
+      <c r="BZ123" s="15" t="n"/>
     </row>
     <row r="124" ht="14.25" customHeight="1">
       <c r="AW124" s="13" t="n">
@@ -22823,6 +23115,9 @@
       <c r="BY124" s="15" t="n">
         <v>43.4</v>
       </c>
+      <c r="BZ124" s="15" t="n">
+        <v>39.15</v>
+      </c>
     </row>
     <row r="125" ht="14.25" customHeight="1">
       <c r="AW125" s="13" t="n">
@@ -22911,6 +23206,9 @@
       </c>
       <c r="BY125" s="15" t="n">
         <v>11132.25</v>
+      </c>
+      <c r="BZ125" s="15" t="n">
+        <v>11144.03</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1">
@@ -22943,6 +23241,7 @@
       <c r="BW126" s="15" t="n"/>
       <c r="BX126" s="15" t="n"/>
       <c r="BY126" s="15" t="n"/>
+      <c r="BZ126" s="15" t="n"/>
     </row>
     <row r="127" ht="14.25" customHeight="1">
       <c r="AW127" s="13" t="n">
@@ -23032,6 +23331,9 @@
       <c r="BY127" s="15" t="n">
         <v>2.32</v>
       </c>
+      <c r="BZ127" s="15" t="n">
+        <v>4.78</v>
+      </c>
     </row>
     <row r="128" ht="14.25" customHeight="1">
       <c r="AW128" s="13" t="n">
@@ -23120,6 +23422,9 @@
       </c>
       <c r="BY128" s="15" t="n">
         <v>1823.05</v>
+      </c>
+      <c r="BZ128" s="15" t="n">
+        <v>1843.6</v>
       </c>
     </row>
     <row r="129" ht="14.25" customHeight="1">
@@ -23152,6 +23457,7 @@
       <c r="BW129" s="15" t="n"/>
       <c r="BX129" s="15" t="n"/>
       <c r="BY129" s="15" t="n"/>
+      <c r="BZ129" s="15" t="n"/>
     </row>
     <row r="130" ht="14.25" customHeight="1">
       <c r="AW130" s="13" t="n">
@@ -23241,6 +23547,9 @@
       <c r="BY130" s="15" t="n">
         <v>6.5</v>
       </c>
+      <c r="BZ130" s="15" t="n">
+        <v>5.3</v>
+      </c>
     </row>
     <row r="131" ht="14.25" customHeight="1">
       <c r="AW131" s="13" t="n">
@@ -23329,6 +23638,9 @@
       </c>
       <c r="BY131" s="15" t="n">
         <v>712.95</v>
+      </c>
+      <c r="BZ131" s="15" t="n">
+        <v>715.39</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1">
@@ -23361,6 +23673,7 @@
       <c r="BW132" s="15" t="n"/>
       <c r="BX132" s="15" t="n"/>
       <c r="BY132" s="15" t="n"/>
+      <c r="BZ132" s="15" t="n"/>
     </row>
     <row r="133" ht="14.25" customHeight="1">
       <c r="AW133" s="13" t="n">
@@ -23450,6 +23763,9 @@
       <c r="BY133" s="15" t="n">
         <v>47.6</v>
       </c>
+      <c r="BZ133" s="15" t="n">
+        <v>45.48</v>
+      </c>
     </row>
     <row r="134" ht="14.25" customHeight="1">
       <c r="AW134" s="13" t="n">
@@ -23537,6 +23853,9 @@
         <v>2738.48</v>
       </c>
       <c r="BY134" s="15" t="n">
+        <v>2638.92</v>
+      </c>
+      <c r="BZ134" s="15" t="n">
         <v>2638.92</v>
       </c>
     </row>
@@ -23570,6 +23889,7 @@
       <c r="BW135" s="15" t="n"/>
       <c r="BX135" s="15" t="n"/>
       <c r="BY135" s="15" t="n"/>
+      <c r="BZ135" s="15" t="n"/>
     </row>
     <row r="136" ht="14.25" customHeight="1">
       <c r="AW136" s="13" t="n">
@@ -23659,6 +23979,9 @@
       <c r="BY136" s="15" t="n">
         <v>21.14</v>
       </c>
+      <c r="BZ136" s="15" t="n">
+        <v>21.18</v>
+      </c>
     </row>
     <row r="137" ht="14.25" customHeight="1">
       <c r="AW137" s="13" t="n">
@@ -23747,6 +24070,9 @@
       </c>
       <c r="BY137" s="15" t="n">
         <v>3409.69</v>
+      </c>
+      <c r="BZ137" s="15" t="n">
+        <v>3452.7</v>
       </c>
     </row>
     <row r="138">
@@ -23771,6 +24097,7 @@
       <c r="BW138" s="15" t="n"/>
       <c r="BX138" s="15" t="n"/>
       <c r="BY138" s="15" t="n"/>
+      <c r="BZ138" s="15" t="n"/>
     </row>
     <row r="139">
       <c r="BE139" s="15" t="n">
@@ -23836,6 +24163,9 @@
       <c r="BY139" s="15" t="n">
         <v>4.56</v>
       </c>
+      <c r="BZ139" s="15" t="n">
+        <v>5.7</v>
+      </c>
     </row>
     <row r="140">
       <c r="BE140" s="15" t="n">
@@ -23898,6 +24228,9 @@
       </c>
       <c r="BY140" s="15" t="n">
         <v>2497.34</v>
+      </c>
+      <c r="BZ140" s="15" t="n">
+        <v>2589.89</v>
       </c>
     </row>
     <row r="141">
@@ -23922,6 +24255,7 @@
       <c r="BW141" s="15" t="n"/>
       <c r="BX141" s="15" t="n"/>
       <c r="BY141" s="15" t="n"/>
+      <c r="BZ141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="BE142" s="15" t="n">
@@ -23987,6 +24321,9 @@
       <c r="BY142" s="15" t="n">
         <v>15.3</v>
       </c>
+      <c r="BZ142" s="15" t="n">
+        <v>11.17</v>
+      </c>
     </row>
     <row r="143">
       <c r="BE143" s="15" t="n">
@@ -24051,6 +24388,9 @@
       </c>
       <c r="BY143" s="15" t="n">
         <v>5561.12</v>
+      </c>
+      <c r="BZ143" s="15" t="n">
+        <v>5405.58</v>
       </c>
     </row>
     <row r="144">
@@ -24070,6 +24410,7 @@
       <c r="BW144" s="15" t="n"/>
       <c r="BX144" s="15" t="n"/>
       <c r="BY144" s="15" t="n"/>
+      <c r="BZ144" s="15" t="n"/>
     </row>
     <row r="145">
       <c r="BJ145" s="15" t="n">
@@ -24120,6 +24461,9 @@
       <c r="BY145" s="15" t="n">
         <v>1.59</v>
       </c>
+      <c r="BZ145" s="15" t="n">
+        <v>1.89</v>
+      </c>
     </row>
     <row r="146">
       <c r="BJ146" s="15" t="n">
@@ -24169,6 +24513,9 @@
       </c>
       <c r="BY146" s="15" t="n">
         <v>2207.48</v>
+      </c>
+      <c r="BZ146" s="15" t="n">
+        <v>2207.65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-10-05 10:52:56]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BZ146"/>
+  <dimension ref="A1:CA146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="51"/>
@@ -612,6 +612,7 @@
     <col width="15" customWidth="1" min="76" max="76"/>
     <col width="15" customWidth="1" min="77" max="77"/>
     <col width="15" customWidth="1" min="78" max="78"/>
+    <col width="15" customWidth="1" min="79" max="79"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -1005,6 +1006,11 @@
           <t>2026/10/01</t>
         </is>
       </c>
+      <c r="CA1" s="15" t="inlineStr">
+        <is>
+          <t>2026/10/05</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1397,6 +1403,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="CA2" s="16" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1633,6 +1644,9 @@
       <c r="BZ3" s="15" t="n">
         <v>57.07</v>
       </c>
+      <c r="CA3" s="15" t="n">
+        <v>57.07</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1867,6 +1881,9 @@
         <v>3823.62</v>
       </c>
       <c r="BZ4" s="15" t="n">
+        <v>3842.19</v>
+      </c>
+      <c r="CA4" s="15" t="n">
         <v>3842.19</v>
       </c>
     </row>
@@ -1949,6 +1966,7 @@
       <c r="BX5" s="15" t="n"/>
       <c r="BY5" s="15" t="n"/>
       <c r="BZ5" s="15" t="n"/>
+      <c r="CA5" s="15" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -2077,6 +2095,7 @@
       <c r="BX6" s="15" t="n"/>
       <c r="BY6" s="15" t="n"/>
       <c r="BZ6" s="15" t="n"/>
+      <c r="CA6" s="15" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -2311,6 +2330,9 @@
         <v>49.88</v>
       </c>
       <c r="BZ7" s="15" t="n">
+        <v>47.39</v>
+      </c>
+      <c r="CA7" s="15" t="n">
         <v>47.39</v>
       </c>
     </row>
@@ -2499,6 +2521,9 @@
         <v>5348.5</v>
       </c>
       <c r="BZ8" s="15" t="n">
+        <v>5370.26</v>
+      </c>
+      <c r="CA8" s="15" t="n">
         <v>5370.26</v>
       </c>
     </row>
@@ -2629,6 +2654,7 @@
       <c r="BX9" s="15" t="n"/>
       <c r="BY9" s="15" t="n"/>
       <c r="BZ9" s="15" t="n"/>
+      <c r="CA9" s="15" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -2863,6 +2889,9 @@
         <v>44.58</v>
       </c>
       <c r="BZ10" s="15" t="n">
+        <v>43.3</v>
+      </c>
+      <c r="CA10" s="15" t="n">
         <v>43.3</v>
       </c>
     </row>
@@ -3051,6 +3080,9 @@
         <v>4340.76</v>
       </c>
       <c r="BZ11" s="15" t="n">
+        <v>4357.62</v>
+      </c>
+      <c r="CA11" s="15" t="n">
         <v>4357.62</v>
       </c>
     </row>
@@ -3181,6 +3213,7 @@
       <c r="BX12" s="15" t="n"/>
       <c r="BY12" s="15" t="n"/>
       <c r="BZ12" s="15" t="n"/>
+      <c r="CA12" s="15" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -3415,6 +3448,9 @@
         <v>58.12</v>
       </c>
       <c r="BZ13" s="15" t="n">
+        <v>55.81</v>
+      </c>
+      <c r="CA13" s="15" t="n">
         <v>55.81</v>
       </c>
     </row>
@@ -3603,6 +3639,9 @@
         <v>7402.3</v>
       </c>
       <c r="BZ14" s="15" t="n">
+        <v>7435.16</v>
+      </c>
+      <c r="CA14" s="15" t="n">
         <v>7435.16</v>
       </c>
     </row>
@@ -3733,6 +3772,7 @@
       <c r="BX15" s="15" t="n"/>
       <c r="BY15" s="15" t="n"/>
       <c r="BZ15" s="15" t="n"/>
+      <c r="CA15" s="15" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -3968,6 +4008,9 @@
       </c>
       <c r="BZ16" s="15" t="n">
         <v>25.62</v>
+      </c>
+      <c r="CA16" s="15" t="n">
+        <v>25.39</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -4155,6 +4198,9 @@
         <v>2495.36</v>
       </c>
       <c r="BZ17" s="15" t="n">
+        <v>2461.21</v>
+      </c>
+      <c r="CA17" s="15" t="n">
         <v>2461.21</v>
       </c>
     </row>
@@ -4285,6 +4331,7 @@
       <c r="BX18" s="15" t="n"/>
       <c r="BY18" s="15" t="n"/>
       <c r="BZ18" s="15" t="n"/>
+      <c r="CA18" s="15" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -4519,6 +4566,9 @@
         <v>80.64</v>
       </c>
       <c r="BZ19" s="15" t="n">
+        <v>79.77</v>
+      </c>
+      <c r="CA19" s="15" t="n">
         <v>79.77</v>
       </c>
     </row>
@@ -4708,6 +4758,9 @@
       </c>
       <c r="BZ20" s="15" t="n">
         <v>7651.54</v>
+      </c>
+      <c r="CA20" s="15" t="n">
+        <v>7722.72</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
@@ -4837,6 +4890,7 @@
       <c r="BX21" s="15" t="n"/>
       <c r="BY21" s="15" t="n"/>
       <c r="BZ21" s="15" t="n"/>
+      <c r="CA21" s="15" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -5069,6 +5123,9 @@
         <v>36.34</v>
       </c>
       <c r="BZ22" s="15" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="CA22" s="15" t="n">
         <v>36.34</v>
       </c>
     </row>
@@ -5258,6 +5315,9 @@
       </c>
       <c r="BZ23" s="15" t="n">
         <v>71909.7</v>
+      </c>
+      <c r="CA23" s="15" t="n">
+        <v>72382.47</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
@@ -5387,6 +5447,7 @@
       <c r="BX24" s="15" t="n"/>
       <c r="BY24" s="15" t="n"/>
       <c r="BZ24" s="15" t="n"/>
+      <c r="CA24" s="15" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -5621,6 +5682,9 @@
         <v>49.88</v>
       </c>
       <c r="BZ25" s="15" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="CA25" s="15" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -5796,6 +5860,9 @@
       </c>
       <c r="BZ26" s="15" t="n">
         <v>25025.14</v>
+      </c>
+      <c r="CA26" s="15" t="n">
+        <v>25194.01</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
@@ -5925,6 +5992,7 @@
       <c r="BX27" s="15" t="n"/>
       <c r="BY27" s="15" t="n"/>
       <c r="BZ27" s="15" t="n"/>
+      <c r="CA27" s="15" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -6159,6 +6227,9 @@
         <v>92.09</v>
       </c>
       <c r="BZ28" s="15" t="n">
+        <v>92.09</v>
+      </c>
+      <c r="CA28" s="15" t="n">
         <v>92.09</v>
       </c>
     </row>
@@ -6348,6 +6419,9 @@
       </c>
       <c r="BZ29" s="15" t="n">
         <v>68956.72</v>
+      </c>
+      <c r="CA29" s="15" t="n">
+        <v>69946.86</v>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
@@ -6477,6 +6551,7 @@
       <c r="BX30" s="15" t="n"/>
       <c r="BY30" s="15" t="n"/>
       <c r="BZ30" s="15" t="n"/>
+      <c r="CA30" s="15" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -6711,6 +6786,9 @@
         <v>97.44</v>
       </c>
       <c r="BZ31" s="15" t="n">
+        <v>97.44</v>
+      </c>
+      <c r="CA31" s="15" t="n">
         <v>97.44</v>
       </c>
     </row>
@@ -6900,6 +6978,9 @@
       </c>
       <c r="BZ32" s="15" t="n">
         <v>6971.35</v>
+      </c>
+      <c r="CA32" s="15" t="n">
+        <v>7003.74</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
@@ -7029,6 +7110,7 @@
       <c r="BX33" s="15" t="n"/>
       <c r="BY33" s="15" t="n"/>
       <c r="BZ33" s="15" t="n"/>
+      <c r="CA33" s="15" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -7263,6 +7345,9 @@
         <v>45.51</v>
       </c>
       <c r="BZ34" s="15" t="n">
+        <v>47.21</v>
+      </c>
+      <c r="CA34" s="15" t="n">
         <v>47.21</v>
       </c>
     </row>
@@ -7451,6 +7536,9 @@
         <v>5439.6</v>
       </c>
       <c r="BZ35" s="15" t="n">
+        <v>5493.34</v>
+      </c>
+      <c r="CA35" s="15" t="n">
         <v>5493.34</v>
       </c>
     </row>
@@ -7581,6 +7669,7 @@
       <c r="BX36" s="15" t="n"/>
       <c r="BY36" s="15" t="n"/>
       <c r="BZ36" s="15" t="n"/>
+      <c r="CA36" s="15" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -7815,6 +7904,9 @@
         <v>50.37</v>
       </c>
       <c r="BZ37" s="15" t="n">
+        <v>55.99</v>
+      </c>
+      <c r="CA37" s="15" t="n">
         <v>55.99</v>
       </c>
     </row>
@@ -8003,6 +8095,9 @@
         <v>11122.04</v>
       </c>
       <c r="BZ38" s="15" t="n">
+        <v>11285.61</v>
+      </c>
+      <c r="CA38" s="15" t="n">
         <v>11285.61</v>
       </c>
     </row>
@@ -8133,6 +8228,7 @@
       <c r="BX39" s="15" t="n"/>
       <c r="BY39" s="15" t="n"/>
       <c r="BZ39" s="15" t="n"/>
+      <c r="CA39" s="15" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -8367,6 +8463,9 @@
         <v>48.39</v>
       </c>
       <c r="BZ40" s="15" t="n">
+        <v>52.27</v>
+      </c>
+      <c r="CA40" s="15" t="n">
         <v>52.27</v>
       </c>
     </row>
@@ -8555,6 +8654,9 @@
         <v>10848.95</v>
       </c>
       <c r="BZ41" s="15" t="n">
+        <v>10971.43</v>
+      </c>
+      <c r="CA41" s="15" t="n">
         <v>10971.43</v>
       </c>
     </row>
@@ -8685,6 +8787,7 @@
       <c r="BX42" s="15" t="n"/>
       <c r="BY42" s="15" t="n"/>
       <c r="BZ42" s="15" t="n"/>
+      <c r="CA42" s="15" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -8919,6 +9022,9 @@
         <v>48.99</v>
       </c>
       <c r="BZ43" s="15" t="n">
+        <v>49.8</v>
+      </c>
+      <c r="CA43" s="15" t="n">
         <v>49.8</v>
       </c>
     </row>
@@ -9107,6 +9213,9 @@
         <v>3263.3</v>
       </c>
       <c r="BZ44" s="15" t="n">
+        <v>3271.9</v>
+      </c>
+      <c r="CA44" s="15" t="n">
         <v>3271.9</v>
       </c>
     </row>
@@ -9237,6 +9346,7 @@
       <c r="BX45" s="15" t="n"/>
       <c r="BY45" s="15" t="n"/>
       <c r="BZ45" s="15" t="n"/>
+      <c r="CA45" s="15" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -9471,6 +9581,9 @@
         <v>52.54</v>
       </c>
       <c r="BZ46" s="15" t="n">
+        <v>61.04</v>
+      </c>
+      <c r="CA46" s="15" t="n">
         <v>61.04</v>
       </c>
     </row>
@@ -9659,6 +9772,9 @@
         <v>6935.79</v>
       </c>
       <c r="BZ47" s="15" t="n">
+        <v>7025.76</v>
+      </c>
+      <c r="CA47" s="15" t="n">
         <v>7025.76</v>
       </c>
     </row>
@@ -9789,6 +9905,7 @@
       <c r="BX48" s="15" t="n"/>
       <c r="BY48" s="15" t="n"/>
       <c r="BZ48" s="15" t="n"/>
+      <c r="CA48" s="15" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -10023,6 +10140,9 @@
         <v>19.41</v>
       </c>
       <c r="BZ49" s="15" t="n">
+        <v>19.57</v>
+      </c>
+      <c r="CA49" s="15" t="n">
         <v>19.57</v>
       </c>
     </row>
@@ -10211,6 +10331,9 @@
         <v>31738.74</v>
       </c>
       <c r="BZ50" s="15" t="n">
+        <v>32172.27</v>
+      </c>
+      <c r="CA50" s="15" t="n">
         <v>32172.27</v>
       </c>
     </row>
@@ -10341,6 +10464,7 @@
       <c r="BX51" s="15" t="n"/>
       <c r="BY51" s="15" t="n"/>
       <c r="BZ51" s="15" t="n"/>
+      <c r="CA51" s="15" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -10575,6 +10699,9 @@
         <v>34.84</v>
       </c>
       <c r="BZ52" s="15" t="n">
+        <v>29.77</v>
+      </c>
+      <c r="CA52" s="15" t="n">
         <v>29.77</v>
       </c>
     </row>
@@ -10763,6 +10890,9 @@
         <v>3246.03</v>
       </c>
       <c r="BZ53" s="15" t="n">
+        <v>3240.53</v>
+      </c>
+      <c r="CA53" s="15" t="n">
         <v>3240.53</v>
       </c>
     </row>
@@ -10893,6 +11023,7 @@
       <c r="BX54" s="15" t="n"/>
       <c r="BY54" s="15" t="n"/>
       <c r="BZ54" s="15" t="n"/>
+      <c r="CA54" s="15" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -11127,6 +11258,9 @@
         <v>42.28</v>
       </c>
       <c r="BZ55" s="15" t="n">
+        <v>38.37</v>
+      </c>
+      <c r="CA55" s="15" t="n">
         <v>38.37</v>
       </c>
     </row>
@@ -11315,6 +11449,9 @@
         <v>3139.82</v>
       </c>
       <c r="BZ56" s="15" t="n">
+        <v>3135.28</v>
+      </c>
+      <c r="CA56" s="15" t="n">
         <v>3135.28</v>
       </c>
     </row>
@@ -11445,6 +11582,7 @@
       <c r="BX57" s="15" t="n"/>
       <c r="BY57" s="15" t="n"/>
       <c r="BZ57" s="15" t="n"/>
+      <c r="CA57" s="15" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -11679,6 +11817,9 @@
         <v>15.91</v>
       </c>
       <c r="BZ58" s="15" t="n">
+        <v>19.41</v>
+      </c>
+      <c r="CA58" s="15" t="n">
         <v>19.41</v>
       </c>
     </row>
@@ -11867,6 +12008,9 @@
         <v>6721.58</v>
       </c>
       <c r="BZ59" s="15" t="n">
+        <v>6883.56</v>
+      </c>
+      <c r="CA59" s="15" t="n">
         <v>6883.56</v>
       </c>
     </row>
@@ -11997,6 +12141,7 @@
       <c r="BX60" s="15" t="n"/>
       <c r="BY60" s="15" t="n"/>
       <c r="BZ60" s="15" t="n"/>
+      <c r="CA60" s="15" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -12231,6 +12376,9 @@
         <v>30.91</v>
       </c>
       <c r="BZ61" s="15" t="n">
+        <v>37.19</v>
+      </c>
+      <c r="CA61" s="15" t="n">
         <v>37.19</v>
       </c>
     </row>
@@ -12419,6 +12567,9 @@
         <v>8052.78</v>
       </c>
       <c r="BZ62" s="15" t="n">
+        <v>8323.309999999999</v>
+      </c>
+      <c r="CA62" s="15" t="n">
         <v>8323.309999999999</v>
       </c>
     </row>
@@ -12549,6 +12700,7 @@
       <c r="BX63" s="15" t="n"/>
       <c r="BY63" s="15" t="n"/>
       <c r="BZ63" s="15" t="n"/>
+      <c r="CA63" s="15" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -12783,6 +12935,9 @@
         <v>5.41</v>
       </c>
       <c r="BZ64" s="15" t="n">
+        <v>6.29</v>
+      </c>
+      <c r="CA64" s="15" t="n">
         <v>6.29</v>
       </c>
     </row>
@@ -12971,6 +13126,9 @@
         <v>10367.63</v>
       </c>
       <c r="BZ65" s="15" t="n">
+        <v>10401.01</v>
+      </c>
+      <c r="CA65" s="15" t="n">
         <v>10401.01</v>
       </c>
     </row>
@@ -13101,6 +13259,7 @@
       <c r="BX66" s="15" t="n"/>
       <c r="BY66" s="15" t="n"/>
       <c r="BZ66" s="15" t="n"/>
+      <c r="CA66" s="15" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -13335,6 +13494,9 @@
         <v>19.02</v>
       </c>
       <c r="BZ67" s="15" t="n">
+        <v>15.25</v>
+      </c>
+      <c r="CA67" s="15" t="n">
         <v>15.25</v>
       </c>
     </row>
@@ -13523,6 +13685,9 @@
         <v>11219.09</v>
       </c>
       <c r="BZ68" s="15" t="n">
+        <v>11058.05</v>
+      </c>
+      <c r="CA68" s="15" t="n">
         <v>11058.05</v>
       </c>
     </row>
@@ -13653,6 +13818,7 @@
       <c r="BX69" s="15" t="n"/>
       <c r="BY69" s="15" t="n"/>
       <c r="BZ69" s="15" t="n"/>
+      <c r="CA69" s="15" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -13887,6 +14053,9 @@
         <v>12.82</v>
       </c>
       <c r="BZ70" s="15" t="n">
+        <v>15.18</v>
+      </c>
+      <c r="CA70" s="15" t="n">
         <v>15.18</v>
       </c>
     </row>
@@ -14075,6 +14244,9 @@
         <v>6049.99</v>
       </c>
       <c r="BZ71" s="15" t="n">
+        <v>6228.9</v>
+      </c>
+      <c r="CA71" s="15" t="n">
         <v>6228.9</v>
       </c>
     </row>
@@ -14205,6 +14377,7 @@
       <c r="BX72" s="15" t="n"/>
       <c r="BY72" s="15" t="n"/>
       <c r="BZ72" s="15" t="n"/>
+      <c r="CA72" s="15" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -14439,6 +14612,9 @@
         <v>16.36</v>
       </c>
       <c r="BZ73" s="15" t="n">
+        <v>17.67</v>
+      </c>
+      <c r="CA73" s="15" t="n">
         <v>17.67</v>
       </c>
     </row>
@@ -14627,6 +14803,9 @@
         <v>12096.02</v>
       </c>
       <c r="BZ74" s="15" t="n">
+        <v>12295.96</v>
+      </c>
+      <c r="CA74" s="15" t="n">
         <v>12295.96</v>
       </c>
     </row>
@@ -14757,6 +14936,7 @@
       <c r="BX75" s="15" t="n"/>
       <c r="BY75" s="15" t="n"/>
       <c r="BZ75" s="15" t="n"/>
+      <c r="CA75" s="15" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -14992,6 +15172,9 @@
       </c>
       <c r="BZ76" s="15" t="n">
         <v>53.09</v>
+      </c>
+      <c r="CA76" s="15" t="n">
+        <v>53.36</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -15180,6 +15363,9 @@
       </c>
       <c r="BZ77" s="15" t="n">
         <v>16651.14</v>
+      </c>
+      <c r="CA77" s="15" t="n">
+        <v>15569.82</v>
       </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
@@ -15309,6 +15495,7 @@
       <c r="BX78" s="15" t="n"/>
       <c r="BY78" s="15" t="n"/>
       <c r="BZ78" s="15" t="n"/>
+      <c r="CA78" s="15" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -15544,6 +15731,9 @@
       </c>
       <c r="BZ79" s="15" t="n">
         <v>1.79</v>
+      </c>
+      <c r="CA79" s="15" t="n">
+        <v>1.74</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -15731,6 +15921,9 @@
         <v>6495.47</v>
       </c>
       <c r="BZ80" s="15" t="n">
+        <v>6406.02</v>
+      </c>
+      <c r="CA80" s="15" t="n">
         <v>6406.02</v>
       </c>
     </row>
@@ -15861,6 +16054,7 @@
       <c r="BX81" s="15" t="n"/>
       <c r="BY81" s="15" t="n"/>
       <c r="BZ81" s="15" t="n"/>
+      <c r="CA81" s="15" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -16095,6 +16289,9 @@
         <v>2.92</v>
       </c>
       <c r="BZ82" s="15" t="n">
+        <v>3.58</v>
+      </c>
+      <c r="CA82" s="15" t="n">
         <v>3.58</v>
       </c>
     </row>
@@ -16283,6 +16480,9 @@
         <v>8161.87</v>
       </c>
       <c r="BZ83" s="15" t="n">
+        <v>8284.629999999999</v>
+      </c>
+      <c r="CA83" s="15" t="n">
         <v>8284.629999999999</v>
       </c>
     </row>
@@ -16413,6 +16613,7 @@
       <c r="BX84" s="15" t="n"/>
       <c r="BY84" s="15" t="n"/>
       <c r="BZ84" s="15" t="n"/>
+      <c r="CA84" s="15" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -16648,6 +16849,9 @@
       </c>
       <c r="BZ85" s="15" t="n">
         <v>16.02</v>
+      </c>
+      <c r="CA85" s="15" t="n">
+        <v>14.91</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -16836,6 +17040,9 @@
       </c>
       <c r="BZ86" s="15" t="n">
         <v>2038.77</v>
+      </c>
+      <c r="CA86" s="15" t="n">
+        <v>2631.9</v>
       </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
@@ -16965,6 +17172,7 @@
       <c r="BX87" s="15" t="n"/>
       <c r="BY87" s="15" t="n"/>
       <c r="BZ87" s="15" t="n"/>
+      <c r="CA87" s="15" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -17200,6 +17408,9 @@
       </c>
       <c r="BZ88" s="15" t="n">
         <v>23.92</v>
+      </c>
+      <c r="CA88" s="15" t="n">
+        <v>22.01</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -17388,6 +17599,9 @@
       </c>
       <c r="BZ89" s="15" t="n">
         <v>4253.89</v>
+      </c>
+      <c r="CA89" s="15" t="n">
+        <v>5075.31</v>
       </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
@@ -17517,6 +17731,7 @@
       <c r="BX90" s="15" t="n"/>
       <c r="BY90" s="15" t="n"/>
       <c r="BZ90" s="15" t="n"/>
+      <c r="CA90" s="15" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -17751,6 +17966,9 @@
         <v>14.68</v>
       </c>
       <c r="BZ91" s="15" t="n">
+        <v>19.19</v>
+      </c>
+      <c r="CA91" s="15" t="n">
         <v>19.19</v>
       </c>
     </row>
@@ -17939,6 +18157,9 @@
         <v>8420.24</v>
       </c>
       <c r="BZ92" s="15" t="n">
+        <v>8679.559999999999</v>
+      </c>
+      <c r="CA92" s="15" t="n">
         <v>8679.559999999999</v>
       </c>
     </row>
@@ -18069,6 +18290,7 @@
       <c r="BX93" s="15" t="n"/>
       <c r="BY93" s="15" t="n"/>
       <c r="BZ93" s="15" t="n"/>
+      <c r="CA93" s="15" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -18303,6 +18525,9 @@
         <v>3.9</v>
       </c>
       <c r="BZ94" s="15" t="n">
+        <v>4.22</v>
+      </c>
+      <c r="CA94" s="15" t="n">
         <v>4.22</v>
       </c>
     </row>
@@ -18491,6 +18716,9 @@
         <v>1176.71</v>
       </c>
       <c r="BZ95" s="15" t="n">
+        <v>1174.56</v>
+      </c>
+      <c r="CA95" s="15" t="n">
         <v>1174.56</v>
       </c>
     </row>
@@ -18621,6 +18849,7 @@
       <c r="BX96" s="15" t="n"/>
       <c r="BY96" s="15" t="n"/>
       <c r="BZ96" s="15" t="n"/>
+      <c r="CA96" s="15" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -18855,6 +19084,9 @@
         <v>7.75</v>
       </c>
       <c r="BZ97" s="15" t="n">
+        <v>8.539999999999999</v>
+      </c>
+      <c r="CA97" s="15" t="n">
         <v>8.539999999999999</v>
       </c>
     </row>
@@ -19043,6 +19275,9 @@
         <v>13458.58</v>
       </c>
       <c r="BZ98" s="15" t="n">
+        <v>13618.21</v>
+      </c>
+      <c r="CA98" s="15" t="n">
         <v>13618.21</v>
       </c>
     </row>
@@ -19173,6 +19408,7 @@
       <c r="BX99" s="15" t="n"/>
       <c r="BY99" s="15" t="n"/>
       <c r="BZ99" s="15" t="n"/>
+      <c r="CA99" s="15" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -19407,6 +19643,9 @@
         <v>34.57</v>
       </c>
       <c r="BZ100" s="15" t="n">
+        <v>39.69</v>
+      </c>
+      <c r="CA100" s="15" t="n">
         <v>39.69</v>
       </c>
     </row>
@@ -19595,6 +19834,9 @@
         <v>3257.76</v>
       </c>
       <c r="BZ101" s="15" t="n">
+        <v>3360.25</v>
+      </c>
+      <c r="CA101" s="15" t="n">
         <v>3360.25</v>
       </c>
     </row>
@@ -19725,6 +19967,7 @@
       <c r="BX102" s="15" t="n"/>
       <c r="BY102" s="15" t="n"/>
       <c r="BZ102" s="15" t="n"/>
+      <c r="CA102" s="15" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -19959,6 +20202,9 @@
         <v>24.74</v>
       </c>
       <c r="BZ103" s="15" t="n">
+        <v>23.92</v>
+      </c>
+      <c r="CA103" s="15" t="n">
         <v>23.92</v>
       </c>
     </row>
@@ -20147,6 +20393,9 @@
         <v>2138.4</v>
       </c>
       <c r="BZ104" s="15" t="n">
+        <v>2173.93</v>
+      </c>
+      <c r="CA104" s="15" t="n">
         <v>2173.93</v>
       </c>
     </row>
@@ -20277,6 +20526,7 @@
       <c r="BX105" s="15" t="n"/>
       <c r="BY105" s="15" t="n"/>
       <c r="BZ105" s="15" t="n"/>
+      <c r="CA105" s="15" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -20511,6 +20761,9 @@
         <v>15.91</v>
       </c>
       <c r="BZ106" s="15" t="n">
+        <v>11.98</v>
+      </c>
+      <c r="CA106" s="15" t="n">
         <v>11.98</v>
       </c>
     </row>
@@ -20700,6 +20953,9 @@
       </c>
       <c r="BZ107" s="15" t="n">
         <v>2289.53</v>
+      </c>
+      <c r="CA107" s="15" t="n">
+        <v>2285.3</v>
       </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
@@ -20829,6 +21085,7 @@
       <c r="BX108" s="15" t="n"/>
       <c r="BY108" s="15" t="n"/>
       <c r="BZ108" s="15" t="n"/>
+      <c r="CA108" s="15" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -21063,6 +21320,9 @@
         <v>25.78</v>
       </c>
       <c r="BZ109" s="15" t="n">
+        <v>24.89</v>
+      </c>
+      <c r="CA109" s="15" t="n">
         <v>24.89</v>
       </c>
     </row>
@@ -21251,6 +21511,9 @@
         <v>2276.69</v>
       </c>
       <c r="BZ110" s="15" t="n">
+        <v>2312.43</v>
+      </c>
+      <c r="CA110" s="15" t="n">
         <v>2312.43</v>
       </c>
     </row>
@@ -21381,6 +21644,7 @@
       <c r="BX111" s="15" t="n"/>
       <c r="BY111" s="15" t="n"/>
       <c r="BZ111" s="15" t="n"/>
+      <c r="CA111" s="15" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -21615,6 +21879,9 @@
         <v>47.56</v>
       </c>
       <c r="BZ112" s="15" t="n">
+        <v>53.65</v>
+      </c>
+      <c r="CA112" s="15" t="n">
         <v>53.65</v>
       </c>
     </row>
@@ -21801,6 +22068,9 @@
         <v>1892.25</v>
       </c>
       <c r="BZ113" s="15" t="n">
+        <v>1963.8</v>
+      </c>
+      <c r="CA113" s="15" t="n">
         <v>1963.8</v>
       </c>
     </row>
@@ -21931,6 +22201,7 @@
       <c r="BX114" s="15" t="n"/>
       <c r="BY114" s="15" t="n"/>
       <c r="BZ114" s="15" t="n"/>
+      <c r="CA114" s="15" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -22165,6 +22436,9 @@
         <v>16.55</v>
       </c>
       <c r="BZ115" s="15" t="n">
+        <v>18.24</v>
+      </c>
+      <c r="CA115" s="15" t="n">
         <v>18.24</v>
       </c>
     </row>
@@ -22338,6 +22612,9 @@
         <v>8701.969999999999</v>
       </c>
       <c r="BZ116" s="15" t="n">
+        <v>8701.969999999999</v>
+      </c>
+      <c r="CA116" s="15" t="n">
         <v>8701.969999999999</v>
       </c>
     </row>
@@ -22423,6 +22700,7 @@
       <c r="BX117" s="15" t="n"/>
       <c r="BY117" s="15" t="n"/>
       <c r="BZ117" s="15" t="n"/>
+      <c r="CA117" s="15" t="n"/>
     </row>
     <row r="118" ht="14.25" customHeight="1">
       <c r="P118" s="13" t="n">
@@ -22614,6 +22892,9 @@
       <c r="BZ118" s="15" t="n">
         <v>69.3</v>
       </c>
+      <c r="CA118" s="15" t="n">
+        <v>69.3</v>
+      </c>
     </row>
     <row r="119" ht="14.25" customHeight="1">
       <c r="Y119" s="13" t="n">
@@ -22776,6 +23057,9 @@
         <v>12354.37</v>
       </c>
       <c r="BZ119" s="15" t="n">
+        <v>12036.57</v>
+      </c>
+      <c r="CA119" s="15" t="n">
         <v>12036.57</v>
       </c>
     </row>
@@ -22810,6 +23094,7 @@
       <c r="BX120" s="15" t="n"/>
       <c r="BY120" s="15" t="n"/>
       <c r="BZ120" s="15" t="n"/>
+      <c r="CA120" s="15" t="n"/>
     </row>
     <row r="121" ht="14.25" customHeight="1">
       <c r="AW121" s="13" t="n">
@@ -22902,6 +23187,9 @@
       <c r="BZ121" s="15" t="n">
         <v>21.06</v>
       </c>
+      <c r="CA121" s="15" t="n">
+        <v>21.06</v>
+      </c>
     </row>
     <row r="122" ht="14.25" customHeight="1">
       <c r="AW122" s="13" t="n">
@@ -22992,6 +23280,9 @@
         <v>1179.2</v>
       </c>
       <c r="BZ122" s="15" t="n">
+        <v>1161.09</v>
+      </c>
+      <c r="CA122" s="15" t="n">
         <v>1161.09</v>
       </c>
     </row>
@@ -23026,6 +23317,7 @@
       <c r="BX123" s="15" t="n"/>
       <c r="BY123" s="15" t="n"/>
       <c r="BZ123" s="15" t="n"/>
+      <c r="CA123" s="15" t="n"/>
     </row>
     <row r="124" ht="14.25" customHeight="1">
       <c r="AW124" s="13" t="n">
@@ -23118,6 +23410,9 @@
       <c r="BZ124" s="15" t="n">
         <v>39.15</v>
       </c>
+      <c r="CA124" s="15" t="n">
+        <v>39.15</v>
+      </c>
     </row>
     <row r="125" ht="14.25" customHeight="1">
       <c r="AW125" s="13" t="n">
@@ -23208,6 +23503,9 @@
         <v>11132.25</v>
       </c>
       <c r="BZ125" s="15" t="n">
+        <v>11144.03</v>
+      </c>
+      <c r="CA125" s="15" t="n">
         <v>11144.03</v>
       </c>
     </row>
@@ -23242,6 +23540,7 @@
       <c r="BX126" s="15" t="n"/>
       <c r="BY126" s="15" t="n"/>
       <c r="BZ126" s="15" t="n"/>
+      <c r="CA126" s="15" t="n"/>
     </row>
     <row r="127" ht="14.25" customHeight="1">
       <c r="AW127" s="13" t="n">
@@ -23334,6 +23633,9 @@
       <c r="BZ127" s="15" t="n">
         <v>4.78</v>
       </c>
+      <c r="CA127" s="15" t="n">
+        <v>4.78</v>
+      </c>
     </row>
     <row r="128" ht="14.25" customHeight="1">
       <c r="AW128" s="13" t="n">
@@ -23424,6 +23726,9 @@
         <v>1823.05</v>
       </c>
       <c r="BZ128" s="15" t="n">
+        <v>1843.6</v>
+      </c>
+      <c r="CA128" s="15" t="n">
         <v>1843.6</v>
       </c>
     </row>
@@ -23458,6 +23763,7 @@
       <c r="BX129" s="15" t="n"/>
       <c r="BY129" s="15" t="n"/>
       <c r="BZ129" s="15" t="n"/>
+      <c r="CA129" s="15" t="n"/>
     </row>
     <row r="130" ht="14.25" customHeight="1">
       <c r="AW130" s="13" t="n">
@@ -23550,6 +23856,9 @@
       <c r="BZ130" s="15" t="n">
         <v>5.3</v>
       </c>
+      <c r="CA130" s="15" t="n">
+        <v>5.3</v>
+      </c>
     </row>
     <row r="131" ht="14.25" customHeight="1">
       <c r="AW131" s="13" t="n">
@@ -23640,6 +23949,9 @@
         <v>712.95</v>
       </c>
       <c r="BZ131" s="15" t="n">
+        <v>715.39</v>
+      </c>
+      <c r="CA131" s="15" t="n">
         <v>715.39</v>
       </c>
     </row>
@@ -23674,6 +23986,7 @@
       <c r="BX132" s="15" t="n"/>
       <c r="BY132" s="15" t="n"/>
       <c r="BZ132" s="15" t="n"/>
+      <c r="CA132" s="15" t="n"/>
     </row>
     <row r="133" ht="14.25" customHeight="1">
       <c r="AW133" s="13" t="n">
@@ -23766,6 +24079,9 @@
       <c r="BZ133" s="15" t="n">
         <v>45.48</v>
       </c>
+      <c r="CA133" s="15" t="n">
+        <v>45.48</v>
+      </c>
     </row>
     <row r="134" ht="14.25" customHeight="1">
       <c r="AW134" s="13" t="n">
@@ -23856,6 +24172,9 @@
         <v>2638.92</v>
       </c>
       <c r="BZ134" s="15" t="n">
+        <v>2638.92</v>
+      </c>
+      <c r="CA134" s="15" t="n">
         <v>2638.92</v>
       </c>
     </row>
@@ -23890,6 +24209,7 @@
       <c r="BX135" s="15" t="n"/>
       <c r="BY135" s="15" t="n"/>
       <c r="BZ135" s="15" t="n"/>
+      <c r="CA135" s="15" t="n"/>
     </row>
     <row r="136" ht="14.25" customHeight="1">
       <c r="AW136" s="13" t="n">
@@ -23982,6 +24302,9 @@
       <c r="BZ136" s="15" t="n">
         <v>21.18</v>
       </c>
+      <c r="CA136" s="15" t="n">
+        <v>21.18</v>
+      </c>
     </row>
     <row r="137" ht="14.25" customHeight="1">
       <c r="AW137" s="13" t="n">
@@ -24072,6 +24395,9 @@
         <v>3409.69</v>
       </c>
       <c r="BZ137" s="15" t="n">
+        <v>3452.7</v>
+      </c>
+      <c r="CA137" s="15" t="n">
         <v>3452.7</v>
       </c>
     </row>
@@ -24098,6 +24424,7 @@
       <c r="BX138" s="15" t="n"/>
       <c r="BY138" s="15" t="n"/>
       <c r="BZ138" s="15" t="n"/>
+      <c r="CA138" s="15" t="n"/>
     </row>
     <row r="139">
       <c r="BE139" s="15" t="n">
@@ -24166,6 +24493,9 @@
       <c r="BZ139" s="15" t="n">
         <v>5.7</v>
       </c>
+      <c r="CA139" s="15" t="n">
+        <v>5.7</v>
+      </c>
     </row>
     <row r="140">
       <c r="BE140" s="15" t="n">
@@ -24231,6 +24561,9 @@
       </c>
       <c r="BZ140" s="15" t="n">
         <v>2589.89</v>
+      </c>
+      <c r="CA140" s="15" t="n">
+        <v>2468.79</v>
       </c>
     </row>
     <row r="141">
@@ -24256,6 +24589,7 @@
       <c r="BX141" s="15" t="n"/>
       <c r="BY141" s="15" t="n"/>
       <c r="BZ141" s="15" t="n"/>
+      <c r="CA141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="BE142" s="15" t="n">
@@ -24324,6 +24658,9 @@
       <c r="BZ142" s="15" t="n">
         <v>11.17</v>
       </c>
+      <c r="CA142" s="15" t="n">
+        <v>11.17</v>
+      </c>
     </row>
     <row r="143">
       <c r="BE143" s="15" t="n">
@@ -24391,6 +24728,9 @@
       </c>
       <c r="BZ143" s="15" t="n">
         <v>5405.58</v>
+      </c>
+      <c r="CA143" s="15" t="n">
+        <v>5423.17</v>
       </c>
     </row>
     <row r="144">
@@ -24411,6 +24751,7 @@
       <c r="BX144" s="15" t="n"/>
       <c r="BY144" s="15" t="n"/>
       <c r="BZ144" s="15" t="n"/>
+      <c r="CA144" s="15" t="n"/>
     </row>
     <row r="145">
       <c r="BJ145" s="15" t="n">
@@ -24464,6 +24805,9 @@
       <c r="BZ145" s="15" t="n">
         <v>1.89</v>
       </c>
+      <c r="CA145" s="15" t="n">
+        <v>1.89</v>
+      </c>
     </row>
     <row r="146">
       <c r="BJ146" s="15" t="n">
@@ -24515,6 +24859,9 @@
         <v>2207.48</v>
       </c>
       <c r="BZ146" s="15" t="n">
+        <v>2207.65</v>
+      </c>
+      <c r="CA146" s="15" t="n">
         <v>2207.65</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-10-08 04:41:28]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CA146"/>
+  <dimension ref="A1:CB146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="51"/>
@@ -613,6 +613,7 @@
     <col width="15" customWidth="1" min="77" max="77"/>
     <col width="15" customWidth="1" min="78" max="78"/>
     <col width="15" customWidth="1" min="79" max="79"/>
+    <col width="15" customWidth="1" min="80" max="80"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -1011,6 +1012,11 @@
           <t>2026/10/05</t>
         </is>
       </c>
+      <c r="CB1" s="15" t="inlineStr">
+        <is>
+          <t>2026/10/08</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1408,6 +1414,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="CB2" s="16" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1647,6 +1658,9 @@
       <c r="CA3" s="15" t="n">
         <v>57.07</v>
       </c>
+      <c r="CB3" s="15" t="n">
+        <v>57.07</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1885,6 +1899,9 @@
       </c>
       <c r="CA4" s="15" t="n">
         <v>3842.19</v>
+      </c>
+      <c r="CB4" s="15" t="n">
+        <v>3831.84</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1967,6 +1984,7 @@
       <c r="BY5" s="15" t="n"/>
       <c r="BZ5" s="15" t="n"/>
       <c r="CA5" s="15" t="n"/>
+      <c r="CB5" s="15" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -2096,6 +2114,7 @@
       <c r="BY6" s="15" t="n"/>
       <c r="BZ6" s="15" t="n"/>
       <c r="CA6" s="15" t="n"/>
+      <c r="CB6" s="15" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -2333,6 +2352,9 @@
         <v>47.39</v>
       </c>
       <c r="CA7" s="15" t="n">
+        <v>47.39</v>
+      </c>
+      <c r="CB7" s="15" t="n">
         <v>47.39</v>
       </c>
     </row>
@@ -2525,6 +2547,9 @@
       </c>
       <c r="CA8" s="15" t="n">
         <v>5370.26</v>
+      </c>
+      <c r="CB8" s="15" t="n">
+        <v>5327.79</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
@@ -2655,6 +2680,7 @@
       <c r="BY9" s="15" t="n"/>
       <c r="BZ9" s="15" t="n"/>
       <c r="CA9" s="15" t="n"/>
+      <c r="CB9" s="15" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -2892,6 +2918,9 @@
         <v>43.3</v>
       </c>
       <c r="CA10" s="15" t="n">
+        <v>43.3</v>
+      </c>
+      <c r="CB10" s="15" t="n">
         <v>43.3</v>
       </c>
     </row>
@@ -3084,6 +3113,9 @@
       </c>
       <c r="CA11" s="15" t="n">
         <v>4357.62</v>
+      </c>
+      <c r="CB11" s="15" t="n">
+        <v>4338.67</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
@@ -3214,6 +3246,7 @@
       <c r="BY12" s="15" t="n"/>
       <c r="BZ12" s="15" t="n"/>
       <c r="CA12" s="15" t="n"/>
+      <c r="CB12" s="15" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -3451,6 +3484,9 @@
         <v>55.81</v>
       </c>
       <c r="CA13" s="15" t="n">
+        <v>55.81</v>
+      </c>
+      <c r="CB13" s="15" t="n">
         <v>55.81</v>
       </c>
     </row>
@@ -3643,6 +3679,9 @@
       </c>
       <c r="CA14" s="15" t="n">
         <v>7435.16</v>
+      </c>
+      <c r="CB14" s="15" t="n">
+        <v>7308.93</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
@@ -3773,6 +3812,7 @@
       <c r="BY15" s="15" t="n"/>
       <c r="BZ15" s="15" t="n"/>
       <c r="CA15" s="15" t="n"/>
+      <c r="CB15" s="15" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -4010,6 +4050,9 @@
         <v>25.62</v>
       </c>
       <c r="CA16" s="15" t="n">
+        <v>25.39</v>
+      </c>
+      <c r="CB16" s="15" t="n">
         <v>25.39</v>
       </c>
     </row>
@@ -4201,6 +4244,9 @@
         <v>2461.21</v>
       </c>
       <c r="CA17" s="15" t="n">
+        <v>2461.21</v>
+      </c>
+      <c r="CB17" s="15" t="n">
         <v>2461.21</v>
       </c>
     </row>
@@ -4332,6 +4378,7 @@
       <c r="BY18" s="15" t="n"/>
       <c r="BZ18" s="15" t="n"/>
       <c r="CA18" s="15" t="n"/>
+      <c r="CB18" s="15" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -4569,6 +4616,9 @@
         <v>79.77</v>
       </c>
       <c r="CA19" s="15" t="n">
+        <v>79.77</v>
+      </c>
+      <c r="CB19" s="15" t="n">
         <v>79.77</v>
       </c>
     </row>
@@ -4761,6 +4811,9 @@
       </c>
       <c r="CA20" s="15" t="n">
         <v>7722.72</v>
+      </c>
+      <c r="CB20" s="15" t="n">
+        <v>7801.77</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
@@ -4891,6 +4944,7 @@
       <c r="BY21" s="15" t="n"/>
       <c r="BZ21" s="15" t="n"/>
       <c r="CA21" s="15" t="n"/>
+      <c r="CB21" s="15" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -5126,6 +5180,9 @@
         <v>36.34</v>
       </c>
       <c r="CA22" s="15" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="CB22" s="15" t="n">
         <v>36.34</v>
       </c>
     </row>
@@ -5318,6 +5375,9 @@
       </c>
       <c r="CA23" s="15" t="n">
         <v>72382.47</v>
+      </c>
+      <c r="CB23" s="15" t="n">
+        <v>72253.3</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
@@ -5448,6 +5508,7 @@
       <c r="BY24" s="15" t="n"/>
       <c r="BZ24" s="15" t="n"/>
       <c r="CA24" s="15" t="n"/>
+      <c r="CB24" s="15" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -5685,6 +5746,9 @@
         <v>49.88</v>
       </c>
       <c r="CA25" s="15" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="CB25" s="15" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -5863,6 +5927,9 @@
       </c>
       <c r="CA26" s="15" t="n">
         <v>25194.01</v>
+      </c>
+      <c r="CB26" s="15" t="n">
+        <v>25104.36</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
@@ -5993,6 +6060,7 @@
       <c r="BY27" s="15" t="n"/>
       <c r="BZ27" s="15" t="n"/>
       <c r="CA27" s="15" t="n"/>
+      <c r="CB27" s="15" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -6230,6 +6298,9 @@
         <v>92.09</v>
       </c>
       <c r="CA28" s="15" t="n">
+        <v>92.09</v>
+      </c>
+      <c r="CB28" s="15" t="n">
         <v>92.09</v>
       </c>
     </row>
@@ -6422,6 +6493,9 @@
       </c>
       <c r="CA29" s="15" t="n">
         <v>69946.86</v>
+      </c>
+      <c r="CB29" s="15" t="n">
+        <v>69438.28</v>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
@@ -6552,6 +6626,7 @@
       <c r="BY30" s="15" t="n"/>
       <c r="BZ30" s="15" t="n"/>
       <c r="CA30" s="15" t="n"/>
+      <c r="CB30" s="15" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -6789,6 +6864,9 @@
         <v>97.44</v>
       </c>
       <c r="CA31" s="15" t="n">
+        <v>97.44</v>
+      </c>
+      <c r="CB31" s="15" t="n">
         <v>97.44</v>
       </c>
     </row>
@@ -6981,6 +7059,9 @@
       </c>
       <c r="CA32" s="15" t="n">
         <v>7003.74</v>
+      </c>
+      <c r="CB32" s="15" t="n">
+        <v>6693.27</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
@@ -7111,6 +7192,7 @@
       <c r="BY33" s="15" t="n"/>
       <c r="BZ33" s="15" t="n"/>
       <c r="CA33" s="15" t="n"/>
+      <c r="CB33" s="15" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -7348,6 +7430,9 @@
         <v>47.21</v>
       </c>
       <c r="CA34" s="15" t="n">
+        <v>47.21</v>
+      </c>
+      <c r="CB34" s="15" t="n">
         <v>47.21</v>
       </c>
     </row>
@@ -7540,6 +7625,9 @@
       </c>
       <c r="CA35" s="15" t="n">
         <v>5493.34</v>
+      </c>
+      <c r="CB35" s="15" t="n">
+        <v>5559.45</v>
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
@@ -7670,6 +7758,7 @@
       <c r="BY36" s="15" t="n"/>
       <c r="BZ36" s="15" t="n"/>
       <c r="CA36" s="15" t="n"/>
+      <c r="CB36" s="15" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -7907,6 +7996,9 @@
         <v>55.99</v>
       </c>
       <c r="CA37" s="15" t="n">
+        <v>55.99</v>
+      </c>
+      <c r="CB37" s="15" t="n">
         <v>55.99</v>
       </c>
     </row>
@@ -8098,6 +8190,9 @@
         <v>11285.61</v>
       </c>
       <c r="CA38" s="15" t="n">
+        <v>11285.61</v>
+      </c>
+      <c r="CB38" s="15" t="n">
         <v>11285.61</v>
       </c>
     </row>
@@ -8229,6 +8324,7 @@
       <c r="BY39" s="15" t="n"/>
       <c r="BZ39" s="15" t="n"/>
       <c r="CA39" s="15" t="n"/>
+      <c r="CB39" s="15" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -8466,6 +8562,9 @@
         <v>52.27</v>
       </c>
       <c r="CA40" s="15" t="n">
+        <v>52.27</v>
+      </c>
+      <c r="CB40" s="15" t="n">
         <v>52.27</v>
       </c>
     </row>
@@ -8657,6 +8756,9 @@
         <v>10971.43</v>
       </c>
       <c r="CA41" s="15" t="n">
+        <v>10971.43</v>
+      </c>
+      <c r="CB41" s="15" t="n">
         <v>10971.43</v>
       </c>
     </row>
@@ -8788,6 +8890,7 @@
       <c r="BY42" s="15" t="n"/>
       <c r="BZ42" s="15" t="n"/>
       <c r="CA42" s="15" t="n"/>
+      <c r="CB42" s="15" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -9025,6 +9128,9 @@
         <v>49.8</v>
       </c>
       <c r="CA43" s="15" t="n">
+        <v>49.8</v>
+      </c>
+      <c r="CB43" s="15" t="n">
         <v>49.8</v>
       </c>
     </row>
@@ -9216,6 +9322,9 @@
         <v>3271.9</v>
       </c>
       <c r="CA44" s="15" t="n">
+        <v>3271.9</v>
+      </c>
+      <c r="CB44" s="15" t="n">
         <v>3271.9</v>
       </c>
     </row>
@@ -9347,6 +9456,7 @@
       <c r="BY45" s="15" t="n"/>
       <c r="BZ45" s="15" t="n"/>
       <c r="CA45" s="15" t="n"/>
+      <c r="CB45" s="15" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -9584,6 +9694,9 @@
         <v>61.04</v>
       </c>
       <c r="CA46" s="15" t="n">
+        <v>61.04</v>
+      </c>
+      <c r="CB46" s="15" t="n">
         <v>61.04</v>
       </c>
     </row>
@@ -9775,6 +9888,9 @@
         <v>7025.76</v>
       </c>
       <c r="CA47" s="15" t="n">
+        <v>7025.76</v>
+      </c>
+      <c r="CB47" s="15" t="n">
         <v>7025.76</v>
       </c>
     </row>
@@ -9906,6 +10022,7 @@
       <c r="BY48" s="15" t="n"/>
       <c r="BZ48" s="15" t="n"/>
       <c r="CA48" s="15" t="n"/>
+      <c r="CB48" s="15" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -10143,6 +10260,9 @@
         <v>19.57</v>
       </c>
       <c r="CA49" s="15" t="n">
+        <v>19.57</v>
+      </c>
+      <c r="CB49" s="15" t="n">
         <v>19.57</v>
       </c>
     </row>
@@ -10334,6 +10454,9 @@
         <v>32172.27</v>
       </c>
       <c r="CA50" s="15" t="n">
+        <v>32172.27</v>
+      </c>
+      <c r="CB50" s="15" t="n">
         <v>32172.27</v>
       </c>
     </row>
@@ -10465,6 +10588,7 @@
       <c r="BY51" s="15" t="n"/>
       <c r="BZ51" s="15" t="n"/>
       <c r="CA51" s="15" t="n"/>
+      <c r="CB51" s="15" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -10702,6 +10826,9 @@
         <v>29.77</v>
       </c>
       <c r="CA52" s="15" t="n">
+        <v>29.77</v>
+      </c>
+      <c r="CB52" s="15" t="n">
         <v>29.77</v>
       </c>
     </row>
@@ -10894,6 +11021,9 @@
       </c>
       <c r="CA53" s="15" t="n">
         <v>3240.53</v>
+      </c>
+      <c r="CB53" s="15" t="n">
+        <v>3172.05</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
@@ -11024,6 +11154,7 @@
       <c r="BY54" s="15" t="n"/>
       <c r="BZ54" s="15" t="n"/>
       <c r="CA54" s="15" t="n"/>
+      <c r="CB54" s="15" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -11261,6 +11392,9 @@
         <v>38.37</v>
       </c>
       <c r="CA55" s="15" t="n">
+        <v>38.37</v>
+      </c>
+      <c r="CB55" s="15" t="n">
         <v>38.37</v>
       </c>
     </row>
@@ -11453,6 +11587,9 @@
       </c>
       <c r="CA56" s="15" t="n">
         <v>3135.28</v>
+      </c>
+      <c r="CB56" s="15" t="n">
+        <v>3068.62</v>
       </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
@@ -11583,6 +11720,7 @@
       <c r="BY57" s="15" t="n"/>
       <c r="BZ57" s="15" t="n"/>
       <c r="CA57" s="15" t="n"/>
+      <c r="CB57" s="15" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -11820,6 +11958,9 @@
         <v>19.41</v>
       </c>
       <c r="CA58" s="15" t="n">
+        <v>19.41</v>
+      </c>
+      <c r="CB58" s="15" t="n">
         <v>19.41</v>
       </c>
     </row>
@@ -12012,6 +12153,9 @@
       </c>
       <c r="CA59" s="15" t="n">
         <v>6883.56</v>
+      </c>
+      <c r="CB59" s="15" t="n">
+        <v>6778.05</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
@@ -12142,6 +12286,7 @@
       <c r="BY60" s="15" t="n"/>
       <c r="BZ60" s="15" t="n"/>
       <c r="CA60" s="15" t="n"/>
+      <c r="CB60" s="15" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -12379,6 +12524,9 @@
         <v>37.19</v>
       </c>
       <c r="CA61" s="15" t="n">
+        <v>37.19</v>
+      </c>
+      <c r="CB61" s="15" t="n">
         <v>37.19</v>
       </c>
     </row>
@@ -12571,6 +12719,9 @@
       </c>
       <c r="CA62" s="15" t="n">
         <v>8323.309999999999</v>
+      </c>
+      <c r="CB62" s="15" t="n">
+        <v>8258.719999999999</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
@@ -12701,6 +12852,7 @@
       <c r="BY63" s="15" t="n"/>
       <c r="BZ63" s="15" t="n"/>
       <c r="CA63" s="15" t="n"/>
+      <c r="CB63" s="15" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -12938,6 +13090,9 @@
         <v>6.29</v>
       </c>
       <c r="CA64" s="15" t="n">
+        <v>6.29</v>
+      </c>
+      <c r="CB64" s="15" t="n">
         <v>6.29</v>
       </c>
     </row>
@@ -13129,6 +13284,9 @@
         <v>10401.01</v>
       </c>
       <c r="CA65" s="15" t="n">
+        <v>10401.01</v>
+      </c>
+      <c r="CB65" s="15" t="n">
         <v>10401.01</v>
       </c>
     </row>
@@ -13260,6 +13418,7 @@
       <c r="BY66" s="15" t="n"/>
       <c r="BZ66" s="15" t="n"/>
       <c r="CA66" s="15" t="n"/>
+      <c r="CB66" s="15" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -13497,6 +13656,9 @@
         <v>15.25</v>
       </c>
       <c r="CA67" s="15" t="n">
+        <v>15.25</v>
+      </c>
+      <c r="CB67" s="15" t="n">
         <v>15.25</v>
       </c>
     </row>
@@ -13689,6 +13851,9 @@
       </c>
       <c r="CA68" s="15" t="n">
         <v>11058.05</v>
+      </c>
+      <c r="CB68" s="15" t="n">
+        <v>10986.17</v>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
@@ -13819,6 +13984,7 @@
       <c r="BY69" s="15" t="n"/>
       <c r="BZ69" s="15" t="n"/>
       <c r="CA69" s="15" t="n"/>
+      <c r="CB69" s="15" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -14056,6 +14222,9 @@
         <v>15.18</v>
       </c>
       <c r="CA70" s="15" t="n">
+        <v>15.18</v>
+      </c>
+      <c r="CB70" s="15" t="n">
         <v>15.18</v>
       </c>
     </row>
@@ -14248,6 +14417,9 @@
       </c>
       <c r="CA71" s="15" t="n">
         <v>6228.9</v>
+      </c>
+      <c r="CB71" s="15" t="n">
+        <v>6204.3</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
@@ -14378,6 +14550,7 @@
       <c r="BY72" s="15" t="n"/>
       <c r="BZ72" s="15" t="n"/>
       <c r="CA72" s="15" t="n"/>
+      <c r="CB72" s="15" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -14615,6 +14788,9 @@
         <v>17.67</v>
       </c>
       <c r="CA73" s="15" t="n">
+        <v>17.67</v>
+      </c>
+      <c r="CB73" s="15" t="n">
         <v>17.67</v>
       </c>
     </row>
@@ -14807,6 +14983,9 @@
       </c>
       <c r="CA74" s="15" t="n">
         <v>12295.96</v>
+      </c>
+      <c r="CB74" s="15" t="n">
+        <v>12290.17</v>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
@@ -14937,6 +15116,7 @@
       <c r="BY75" s="15" t="n"/>
       <c r="BZ75" s="15" t="n"/>
       <c r="CA75" s="15" t="n"/>
+      <c r="CB75" s="15" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -15174,6 +15354,9 @@
         <v>53.09</v>
       </c>
       <c r="CA76" s="15" t="n">
+        <v>53.36</v>
+      </c>
+      <c r="CB76" s="15" t="n">
         <v>53.36</v>
       </c>
     </row>
@@ -15365,6 +15548,9 @@
         <v>16651.14</v>
       </c>
       <c r="CA77" s="15" t="n">
+        <v>15569.82</v>
+      </c>
+      <c r="CB77" s="15" t="n">
         <v>15569.82</v>
       </c>
     </row>
@@ -15496,6 +15682,7 @@
       <c r="BY78" s="15" t="n"/>
       <c r="BZ78" s="15" t="n"/>
       <c r="CA78" s="15" t="n"/>
+      <c r="CB78" s="15" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -15733,6 +15920,9 @@
         <v>1.79</v>
       </c>
       <c r="CA79" s="15" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="CB79" s="15" t="n">
         <v>1.74</v>
       </c>
     </row>
@@ -15925,6 +16115,9 @@
       </c>
       <c r="CA80" s="15" t="n">
         <v>6406.02</v>
+      </c>
+      <c r="CB80" s="15" t="n">
+        <v>6277.54</v>
       </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
@@ -16055,6 +16248,7 @@
       <c r="BY81" s="15" t="n"/>
       <c r="BZ81" s="15" t="n"/>
       <c r="CA81" s="15" t="n"/>
+      <c r="CB81" s="15" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -16292,6 +16486,9 @@
         <v>3.58</v>
       </c>
       <c r="CA82" s="15" t="n">
+        <v>3.58</v>
+      </c>
+      <c r="CB82" s="15" t="n">
         <v>3.58</v>
       </c>
     </row>
@@ -16484,6 +16681,9 @@
       </c>
       <c r="CA83" s="15" t="n">
         <v>8284.629999999999</v>
+      </c>
+      <c r="CB83" s="15" t="n">
+        <v>8291.16</v>
       </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
@@ -16614,6 +16814,7 @@
       <c r="BY84" s="15" t="n"/>
       <c r="BZ84" s="15" t="n"/>
       <c r="CA84" s="15" t="n"/>
+      <c r="CB84" s="15" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -16851,6 +17052,9 @@
         <v>16.02</v>
       </c>
       <c r="CA85" s="15" t="n">
+        <v>14.91</v>
+      </c>
+      <c r="CB85" s="15" t="n">
         <v>14.91</v>
       </c>
     </row>
@@ -17043,6 +17247,9 @@
       </c>
       <c r="CA86" s="15" t="n">
         <v>2631.9</v>
+      </c>
+      <c r="CB86" s="15" t="n">
+        <v>1972.7</v>
       </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
@@ -17173,6 +17380,7 @@
       <c r="BY87" s="15" t="n"/>
       <c r="BZ87" s="15" t="n"/>
       <c r="CA87" s="15" t="n"/>
+      <c r="CB87" s="15" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -17410,6 +17618,9 @@
         <v>23.92</v>
       </c>
       <c r="CA88" s="15" t="n">
+        <v>22.01</v>
+      </c>
+      <c r="CB88" s="15" t="n">
         <v>22.01</v>
       </c>
     </row>
@@ -17602,6 +17813,9 @@
       </c>
       <c r="CA89" s="15" t="n">
         <v>5075.31</v>
+      </c>
+      <c r="CB89" s="15" t="n">
+        <v>4113.73</v>
       </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
@@ -17732,6 +17946,7 @@
       <c r="BY90" s="15" t="n"/>
       <c r="BZ90" s="15" t="n"/>
       <c r="CA90" s="15" t="n"/>
+      <c r="CB90" s="15" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -17969,6 +18184,9 @@
         <v>19.19</v>
       </c>
       <c r="CA91" s="15" t="n">
+        <v>19.19</v>
+      </c>
+      <c r="CB91" s="15" t="n">
         <v>19.19</v>
       </c>
     </row>
@@ -18161,6 +18379,9 @@
       </c>
       <c r="CA92" s="15" t="n">
         <v>8679.559999999999</v>
+      </c>
+      <c r="CB92" s="15" t="n">
+        <v>8544.57</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
@@ -18291,6 +18512,7 @@
       <c r="BY93" s="15" t="n"/>
       <c r="BZ93" s="15" t="n"/>
       <c r="CA93" s="15" t="n"/>
+      <c r="CB93" s="15" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -18528,6 +18750,9 @@
         <v>4.22</v>
       </c>
       <c r="CA94" s="15" t="n">
+        <v>4.22</v>
+      </c>
+      <c r="CB94" s="15" t="n">
         <v>4.22</v>
       </c>
     </row>
@@ -18719,6 +18944,9 @@
         <v>1174.56</v>
       </c>
       <c r="CA95" s="15" t="n">
+        <v>1174.56</v>
+      </c>
+      <c r="CB95" s="15" t="n">
         <v>1174.56</v>
       </c>
     </row>
@@ -18850,6 +19078,7 @@
       <c r="BY96" s="15" t="n"/>
       <c r="BZ96" s="15" t="n"/>
       <c r="CA96" s="15" t="n"/>
+      <c r="CB96" s="15" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -19087,6 +19316,9 @@
         <v>8.539999999999999</v>
       </c>
       <c r="CA97" s="15" t="n">
+        <v>8.539999999999999</v>
+      </c>
+      <c r="CB97" s="15" t="n">
         <v>8.539999999999999</v>
       </c>
     </row>
@@ -19278,6 +19510,9 @@
         <v>13618.21</v>
       </c>
       <c r="CA98" s="15" t="n">
+        <v>13618.21</v>
+      </c>
+      <c r="CB98" s="15" t="n">
         <v>13618.21</v>
       </c>
     </row>
@@ -19409,6 +19644,7 @@
       <c r="BY99" s="15" t="n"/>
       <c r="BZ99" s="15" t="n"/>
       <c r="CA99" s="15" t="n"/>
+      <c r="CB99" s="15" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -19646,6 +19882,9 @@
         <v>39.69</v>
       </c>
       <c r="CA100" s="15" t="n">
+        <v>39.69</v>
+      </c>
+      <c r="CB100" s="15" t="n">
         <v>39.69</v>
       </c>
     </row>
@@ -19837,6 +20076,9 @@
         <v>3360.25</v>
       </c>
       <c r="CA101" s="15" t="n">
+        <v>3360.25</v>
+      </c>
+      <c r="CB101" s="15" t="n">
         <v>3360.25</v>
       </c>
     </row>
@@ -19968,6 +20210,7 @@
       <c r="BY102" s="15" t="n"/>
       <c r="BZ102" s="15" t="n"/>
       <c r="CA102" s="15" t="n"/>
+      <c r="CB102" s="15" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -20205,6 +20448,9 @@
         <v>23.92</v>
       </c>
       <c r="CA103" s="15" t="n">
+        <v>23.92</v>
+      </c>
+      <c r="CB103" s="15" t="n">
         <v>23.92</v>
       </c>
     </row>
@@ -20397,6 +20643,9 @@
       </c>
       <c r="CA104" s="15" t="n">
         <v>2173.93</v>
+      </c>
+      <c r="CB104" s="15" t="n">
+        <v>2182.09</v>
       </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
@@ -20527,6 +20776,7 @@
       <c r="BY105" s="15" t="n"/>
       <c r="BZ105" s="15" t="n"/>
       <c r="CA105" s="15" t="n"/>
+      <c r="CB105" s="15" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -20764,6 +21014,9 @@
         <v>11.98</v>
       </c>
       <c r="CA106" s="15" t="n">
+        <v>11.98</v>
+      </c>
+      <c r="CB106" s="15" t="n">
         <v>11.98</v>
       </c>
     </row>
@@ -20956,6 +21209,9 @@
       </c>
       <c r="CA107" s="15" t="n">
         <v>2285.3</v>
+      </c>
+      <c r="CB107" s="15" t="n">
+        <v>2259.98</v>
       </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
@@ -21086,6 +21342,7 @@
       <c r="BY108" s="15" t="n"/>
       <c r="BZ108" s="15" t="n"/>
       <c r="CA108" s="15" t="n"/>
+      <c r="CB108" s="15" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -21323,6 +21580,9 @@
         <v>24.89</v>
       </c>
       <c r="CA109" s="15" t="n">
+        <v>24.89</v>
+      </c>
+      <c r="CB109" s="15" t="n">
         <v>24.89</v>
       </c>
     </row>
@@ -21514,6 +21774,9 @@
         <v>2312.43</v>
       </c>
       <c r="CA110" s="15" t="n">
+        <v>2312.43</v>
+      </c>
+      <c r="CB110" s="15" t="n">
         <v>2312.43</v>
       </c>
     </row>
@@ -21645,6 +21908,7 @@
       <c r="BY111" s="15" t="n"/>
       <c r="BZ111" s="15" t="n"/>
       <c r="CA111" s="15" t="n"/>
+      <c r="CB111" s="15" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -21882,6 +22146,9 @@
         <v>53.65</v>
       </c>
       <c r="CA112" s="15" t="n">
+        <v>53.65</v>
+      </c>
+      <c r="CB112" s="15" t="n">
         <v>53.65</v>
       </c>
     </row>
@@ -22071,6 +22338,9 @@
         <v>1963.8</v>
       </c>
       <c r="CA113" s="15" t="n">
+        <v>1963.8</v>
+      </c>
+      <c r="CB113" s="15" t="n">
         <v>1963.8</v>
       </c>
     </row>
@@ -22202,6 +22472,7 @@
       <c r="BY114" s="15" t="n"/>
       <c r="BZ114" s="15" t="n"/>
       <c r="CA114" s="15" t="n"/>
+      <c r="CB114" s="15" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -22439,6 +22710,9 @@
         <v>18.24</v>
       </c>
       <c r="CA115" s="15" t="n">
+        <v>18.24</v>
+      </c>
+      <c r="CB115" s="15" t="n">
         <v>18.24</v>
       </c>
     </row>
@@ -22616,6 +22890,9 @@
       </c>
       <c r="CA116" s="15" t="n">
         <v>8701.969999999999</v>
+      </c>
+      <c r="CB116" s="15" t="n">
+        <v>8670.76</v>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1">
@@ -22701,6 +22978,7 @@
       <c r="BY117" s="15" t="n"/>
       <c r="BZ117" s="15" t="n"/>
       <c r="CA117" s="15" t="n"/>
+      <c r="CB117" s="15" t="n"/>
     </row>
     <row r="118" ht="14.25" customHeight="1">
       <c r="P118" s="13" t="n">
@@ -22895,6 +23173,9 @@
       <c r="CA118" s="15" t="n">
         <v>69.3</v>
       </c>
+      <c r="CB118" s="15" t="n">
+        <v>69.3</v>
+      </c>
     </row>
     <row r="119" ht="14.25" customHeight="1">
       <c r="Y119" s="13" t="n">
@@ -23061,6 +23342,9 @@
       </c>
       <c r="CA119" s="15" t="n">
         <v>12036.57</v>
+      </c>
+      <c r="CB119" s="15" t="n">
+        <v>11702.13</v>
       </c>
     </row>
     <row r="120" ht="14.25" customHeight="1">
@@ -23095,6 +23379,7 @@
       <c r="BY120" s="15" t="n"/>
       <c r="BZ120" s="15" t="n"/>
       <c r="CA120" s="15" t="n"/>
+      <c r="CB120" s="15" t="n"/>
     </row>
     <row r="121" ht="14.25" customHeight="1">
       <c r="AW121" s="13" t="n">
@@ -23190,6 +23475,9 @@
       <c r="CA121" s="15" t="n">
         <v>21.06</v>
       </c>
+      <c r="CB121" s="15" t="n">
+        <v>21.06</v>
+      </c>
     </row>
     <row r="122" ht="14.25" customHeight="1">
       <c r="AW122" s="13" t="n">
@@ -23283,6 +23571,9 @@
         <v>1161.09</v>
       </c>
       <c r="CA122" s="15" t="n">
+        <v>1161.09</v>
+      </c>
+      <c r="CB122" s="15" t="n">
         <v>1161.09</v>
       </c>
     </row>
@@ -23318,6 +23609,7 @@
       <c r="BY123" s="15" t="n"/>
       <c r="BZ123" s="15" t="n"/>
       <c r="CA123" s="15" t="n"/>
+      <c r="CB123" s="15" t="n"/>
     </row>
     <row r="124" ht="14.25" customHeight="1">
       <c r="AW124" s="13" t="n">
@@ -23413,6 +23705,9 @@
       <c r="CA124" s="15" t="n">
         <v>39.15</v>
       </c>
+      <c r="CB124" s="15" t="n">
+        <v>39.15</v>
+      </c>
     </row>
     <row r="125" ht="14.25" customHeight="1">
       <c r="AW125" s="13" t="n">
@@ -23507,6 +23802,9 @@
       </c>
       <c r="CA125" s="15" t="n">
         <v>11144.03</v>
+      </c>
+      <c r="CB125" s="15" t="n">
+        <v>11216.93</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1">
@@ -23541,6 +23839,7 @@
       <c r="BY126" s="15" t="n"/>
       <c r="BZ126" s="15" t="n"/>
       <c r="CA126" s="15" t="n"/>
+      <c r="CB126" s="15" t="n"/>
     </row>
     <row r="127" ht="14.25" customHeight="1">
       <c r="AW127" s="13" t="n">
@@ -23636,6 +23935,9 @@
       <c r="CA127" s="15" t="n">
         <v>4.78</v>
       </c>
+      <c r="CB127" s="15" t="n">
+        <v>4.78</v>
+      </c>
     </row>
     <row r="128" ht="14.25" customHeight="1">
       <c r="AW128" s="13" t="n">
@@ -23729,6 +24031,9 @@
         <v>1843.6</v>
       </c>
       <c r="CA128" s="15" t="n">
+        <v>1843.6</v>
+      </c>
+      <c r="CB128" s="15" t="n">
         <v>1843.6</v>
       </c>
     </row>
@@ -23764,6 +24069,7 @@
       <c r="BY129" s="15" t="n"/>
       <c r="BZ129" s="15" t="n"/>
       <c r="CA129" s="15" t="n"/>
+      <c r="CB129" s="15" t="n"/>
     </row>
     <row r="130" ht="14.25" customHeight="1">
       <c r="AW130" s="13" t="n">
@@ -23859,6 +24165,9 @@
       <c r="CA130" s="15" t="n">
         <v>5.3</v>
       </c>
+      <c r="CB130" s="15" t="n">
+        <v>5.3</v>
+      </c>
     </row>
     <row r="131" ht="14.25" customHeight="1">
       <c r="AW131" s="13" t="n">
@@ -23953,6 +24262,9 @@
       </c>
       <c r="CA131" s="15" t="n">
         <v>715.39</v>
+      </c>
+      <c r="CB131" s="15" t="n">
+        <v>708.53</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1">
@@ -23987,6 +24299,7 @@
       <c r="BY132" s="15" t="n"/>
       <c r="BZ132" s="15" t="n"/>
       <c r="CA132" s="15" t="n"/>
+      <c r="CB132" s="15" t="n"/>
     </row>
     <row r="133" ht="14.25" customHeight="1">
       <c r="AW133" s="13" t="n">
@@ -24082,6 +24395,9 @@
       <c r="CA133" s="15" t="n">
         <v>45.48</v>
       </c>
+      <c r="CB133" s="15" t="n">
+        <v>45.48</v>
+      </c>
     </row>
     <row r="134" ht="14.25" customHeight="1">
       <c r="AW134" s="13" t="n">
@@ -24175,6 +24491,9 @@
         <v>2638.92</v>
       </c>
       <c r="CA134" s="15" t="n">
+        <v>2638.92</v>
+      </c>
+      <c r="CB134" s="15" t="n">
         <v>2638.92</v>
       </c>
     </row>
@@ -24210,6 +24529,7 @@
       <c r="BY135" s="15" t="n"/>
       <c r="BZ135" s="15" t="n"/>
       <c r="CA135" s="15" t="n"/>
+      <c r="CB135" s="15" t="n"/>
     </row>
     <row r="136" ht="14.25" customHeight="1">
       <c r="AW136" s="13" t="n">
@@ -24305,6 +24625,9 @@
       <c r="CA136" s="15" t="n">
         <v>21.18</v>
       </c>
+      <c r="CB136" s="15" t="n">
+        <v>21.18</v>
+      </c>
     </row>
     <row r="137" ht="14.25" customHeight="1">
       <c r="AW137" s="13" t="n">
@@ -24399,6 +24722,9 @@
       </c>
       <c r="CA137" s="15" t="n">
         <v>3452.7</v>
+      </c>
+      <c r="CB137" s="15" t="n">
+        <v>3457.37</v>
       </c>
     </row>
     <row r="138">
@@ -24425,6 +24751,7 @@
       <c r="BY138" s="15" t="n"/>
       <c r="BZ138" s="15" t="n"/>
       <c r="CA138" s="15" t="n"/>
+      <c r="CB138" s="15" t="n"/>
     </row>
     <row r="139">
       <c r="BE139" s="15" t="n">
@@ -24496,6 +24823,9 @@
       <c r="CA139" s="15" t="n">
         <v>5.7</v>
       </c>
+      <c r="CB139" s="15" t="n">
+        <v>5.7</v>
+      </c>
     </row>
     <row r="140">
       <c r="BE140" s="15" t="n">
@@ -24564,6 +24894,9 @@
       </c>
       <c r="CA140" s="15" t="n">
         <v>2468.79</v>
+      </c>
+      <c r="CB140" s="15" t="n">
+        <v>2589.89</v>
       </c>
     </row>
     <row r="141">
@@ -24590,6 +24923,7 @@
       <c r="BY141" s="15" t="n"/>
       <c r="BZ141" s="15" t="n"/>
       <c r="CA141" s="15" t="n"/>
+      <c r="CB141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="BE142" s="15" t="n">
@@ -24661,6 +24995,9 @@
       <c r="CA142" s="15" t="n">
         <v>11.17</v>
       </c>
+      <c r="CB142" s="15" t="n">
+        <v>11.17</v>
+      </c>
     </row>
     <row r="143">
       <c r="BE143" s="15" t="n">
@@ -24730,6 +25067,9 @@
         <v>5405.58</v>
       </c>
       <c r="CA143" s="15" t="n">
+        <v>5423.17</v>
+      </c>
+      <c r="CB143" s="15" t="n">
         <v>5423.17</v>
       </c>
     </row>
@@ -24752,6 +25092,7 @@
       <c r="BY144" s="15" t="n"/>
       <c r="BZ144" s="15" t="n"/>
       <c r="CA144" s="15" t="n"/>
+      <c r="CB144" s="15" t="n"/>
     </row>
     <row r="145">
       <c r="BJ145" s="15" t="n">
@@ -24808,6 +25149,9 @@
       <c r="CA145" s="15" t="n">
         <v>1.89</v>
       </c>
+      <c r="CB145" s="15" t="n">
+        <v>1.89</v>
+      </c>
     </row>
     <row r="146">
       <c r="BJ146" s="15" t="n">
@@ -24862,6 +25206,9 @@
         <v>2207.65</v>
       </c>
       <c r="CA146" s="15" t="n">
+        <v>2207.65</v>
+      </c>
+      <c r="CB146" s="15" t="n">
         <v>2207.65</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-10-08 10:57:06]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CB146"/>
+  <dimension ref="A1:CC146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="51"/>
@@ -614,6 +614,7 @@
     <col width="15" customWidth="1" min="78" max="78"/>
     <col width="15" customWidth="1" min="79" max="79"/>
     <col width="15" customWidth="1" min="80" max="80"/>
+    <col width="15" customWidth="1" min="81" max="81"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -1017,6 +1018,11 @@
           <t>2026/10/08</t>
         </is>
       </c>
+      <c r="CC1" s="15" t="inlineStr">
+        <is>
+          <t>2026/10/08</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1419,6 +1425,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="CC2" s="16" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1661,6 +1672,9 @@
       <c r="CB3" s="15" t="n">
         <v>57.07</v>
       </c>
+      <c r="CC3" s="15" t="n">
+        <v>57.07</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1902,6 +1916,9 @@
       </c>
       <c r="CB4" s="15" t="n">
         <v>3831.84</v>
+      </c>
+      <c r="CC4" s="15" t="n">
+        <v>3811.9</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1985,6 +2002,7 @@
       <c r="BZ5" s="15" t="n"/>
       <c r="CA5" s="15" t="n"/>
       <c r="CB5" s="15" t="n"/>
+      <c r="CC5" s="15" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -2115,6 +2133,7 @@
       <c r="BZ6" s="15" t="n"/>
       <c r="CA6" s="15" t="n"/>
       <c r="CB6" s="15" t="n"/>
+      <c r="CC6" s="15" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -2355,6 +2374,9 @@
         <v>47.39</v>
       </c>
       <c r="CB7" s="15" t="n">
+        <v>47.39</v>
+      </c>
+      <c r="CC7" s="15" t="n">
         <v>47.39</v>
       </c>
     </row>
@@ -2550,6 +2572,9 @@
       </c>
       <c r="CB8" s="15" t="n">
         <v>5327.79</v>
+      </c>
+      <c r="CC8" s="15" t="n">
+        <v>5289.44</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
@@ -2681,6 +2706,7 @@
       <c r="BZ9" s="15" t="n"/>
       <c r="CA9" s="15" t="n"/>
       <c r="CB9" s="15" t="n"/>
+      <c r="CC9" s="15" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -2921,6 +2947,9 @@
         <v>43.3</v>
       </c>
       <c r="CB10" s="15" t="n">
+        <v>43.3</v>
+      </c>
+      <c r="CC10" s="15" t="n">
         <v>43.3</v>
       </c>
     </row>
@@ -3116,6 +3145,9 @@
       </c>
       <c r="CB11" s="15" t="n">
         <v>4338.67</v>
+      </c>
+      <c r="CC11" s="15" t="n">
+        <v>4310.28</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
@@ -3247,6 +3279,7 @@
       <c r="BZ12" s="15" t="n"/>
       <c r="CA12" s="15" t="n"/>
       <c r="CB12" s="15" t="n"/>
+      <c r="CC12" s="15" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -3487,6 +3520,9 @@
         <v>55.81</v>
       </c>
       <c r="CB13" s="15" t="n">
+        <v>55.81</v>
+      </c>
+      <c r="CC13" s="15" t="n">
         <v>55.81</v>
       </c>
     </row>
@@ -3682,6 +3718,9 @@
       </c>
       <c r="CB14" s="15" t="n">
         <v>7308.93</v>
+      </c>
+      <c r="CC14" s="15" t="n">
+        <v>7248.43</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
@@ -3813,6 +3852,7 @@
       <c r="BZ15" s="15" t="n"/>
       <c r="CA15" s="15" t="n"/>
       <c r="CB15" s="15" t="n"/>
+      <c r="CC15" s="15" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -4053,6 +4093,9 @@
         <v>25.39</v>
       </c>
       <c r="CB16" s="15" t="n">
+        <v>25.39</v>
+      </c>
+      <c r="CC16" s="15" t="n">
         <v>25.39</v>
       </c>
     </row>
@@ -4248,6 +4291,9 @@
       </c>
       <c r="CB17" s="15" t="n">
         <v>2461.21</v>
+      </c>
+      <c r="CC17" s="15" t="n">
+        <v>2404.7</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
@@ -4379,6 +4425,7 @@
       <c r="BZ18" s="15" t="n"/>
       <c r="CA18" s="15" t="n"/>
       <c r="CB18" s="15" t="n"/>
+      <c r="CC18" s="15" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -4619,6 +4666,9 @@
         <v>79.77</v>
       </c>
       <c r="CB19" s="15" t="n">
+        <v>79.77</v>
+      </c>
+      <c r="CC19" s="15" t="n">
         <v>79.77</v>
       </c>
     </row>
@@ -4813,6 +4863,9 @@
         <v>7722.72</v>
       </c>
       <c r="CB20" s="15" t="n">
+        <v>7801.77</v>
+      </c>
+      <c r="CC20" s="15" t="n">
         <v>7801.77</v>
       </c>
     </row>
@@ -4945,6 +4998,7 @@
       <c r="BZ21" s="15" t="n"/>
       <c r="CA21" s="15" t="n"/>
       <c r="CB21" s="15" t="n"/>
+      <c r="CC21" s="15" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -5183,6 +5237,9 @@
         <v>36.34</v>
       </c>
       <c r="CB22" s="15" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="CC22" s="15" t="n">
         <v>36.34</v>
       </c>
     </row>
@@ -5378,6 +5435,9 @@
       </c>
       <c r="CB23" s="15" t="n">
         <v>72253.3</v>
+      </c>
+      <c r="CC23" s="15" t="n">
+        <v>71593.24000000001</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
@@ -5509,6 +5569,7 @@
       <c r="BZ24" s="15" t="n"/>
       <c r="CA24" s="15" t="n"/>
       <c r="CB24" s="15" t="n"/>
+      <c r="CC24" s="15" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -5749,6 +5810,9 @@
         <v>49.88</v>
       </c>
       <c r="CB25" s="15" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="CC25" s="15" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -5930,6 +5994,9 @@
       </c>
       <c r="CB26" s="15" t="n">
         <v>25104.36</v>
+      </c>
+      <c r="CC26" s="15" t="n">
+        <v>24808.03</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
@@ -6061,6 +6128,7 @@
       <c r="BZ27" s="15" t="n"/>
       <c r="CA27" s="15" t="n"/>
       <c r="CB27" s="15" t="n"/>
+      <c r="CC27" s="15" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -6301,6 +6369,9 @@
         <v>92.09</v>
       </c>
       <c r="CB28" s="15" t="n">
+        <v>92.09</v>
+      </c>
+      <c r="CC28" s="15" t="n">
         <v>92.09</v>
       </c>
     </row>
@@ -6496,6 +6567,9 @@
       </c>
       <c r="CB29" s="15" t="n">
         <v>69438.28</v>
+      </c>
+      <c r="CC29" s="15" t="n">
+        <v>69042.11</v>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
@@ -6627,6 +6701,7 @@
       <c r="BZ30" s="15" t="n"/>
       <c r="CA30" s="15" t="n"/>
       <c r="CB30" s="15" t="n"/>
+      <c r="CC30" s="15" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -6867,6 +6942,9 @@
         <v>97.44</v>
       </c>
       <c r="CB31" s="15" t="n">
+        <v>97.44</v>
+      </c>
+      <c r="CC31" s="15" t="n">
         <v>97.44</v>
       </c>
     </row>
@@ -7062,6 +7140,9 @@
       </c>
       <c r="CB32" s="15" t="n">
         <v>6693.27</v>
+      </c>
+      <c r="CC32" s="15" t="n">
+        <v>6625.93</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
@@ -7193,6 +7274,7 @@
       <c r="BZ33" s="15" t="n"/>
       <c r="CA33" s="15" t="n"/>
       <c r="CB33" s="15" t="n"/>
+      <c r="CC33" s="15" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -7433,6 +7515,9 @@
         <v>47.21</v>
       </c>
       <c r="CB34" s="15" t="n">
+        <v>47.21</v>
+      </c>
+      <c r="CC34" s="15" t="n">
         <v>47.21</v>
       </c>
     </row>
@@ -7628,6 +7713,9 @@
       </c>
       <c r="CB35" s="15" t="n">
         <v>5559.45</v>
+      </c>
+      <c r="CC35" s="15" t="n">
+        <v>5556.01</v>
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
@@ -7759,6 +7847,7 @@
       <c r="BZ36" s="15" t="n"/>
       <c r="CA36" s="15" t="n"/>
       <c r="CB36" s="15" t="n"/>
+      <c r="CC36" s="15" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -7999,6 +8088,9 @@
         <v>55.99</v>
       </c>
       <c r="CB37" s="15" t="n">
+        <v>55.99</v>
+      </c>
+      <c r="CC37" s="15" t="n">
         <v>55.99</v>
       </c>
     </row>
@@ -8193,6 +8285,9 @@
         <v>11285.61</v>
       </c>
       <c r="CB38" s="15" t="n">
+        <v>11285.61</v>
+      </c>
+      <c r="CC38" s="15" t="n">
         <v>11285.61</v>
       </c>
     </row>
@@ -8325,6 +8420,7 @@
       <c r="BZ39" s="15" t="n"/>
       <c r="CA39" s="15" t="n"/>
       <c r="CB39" s="15" t="n"/>
+      <c r="CC39" s="15" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -8565,6 +8661,9 @@
         <v>52.27</v>
       </c>
       <c r="CB40" s="15" t="n">
+        <v>52.27</v>
+      </c>
+      <c r="CC40" s="15" t="n">
         <v>52.27</v>
       </c>
     </row>
@@ -8759,6 +8858,9 @@
         <v>10971.43</v>
       </c>
       <c r="CB41" s="15" t="n">
+        <v>10971.43</v>
+      </c>
+      <c r="CC41" s="15" t="n">
         <v>10971.43</v>
       </c>
     </row>
@@ -8891,6 +8993,7 @@
       <c r="BZ42" s="15" t="n"/>
       <c r="CA42" s="15" t="n"/>
       <c r="CB42" s="15" t="n"/>
+      <c r="CC42" s="15" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -9131,6 +9234,9 @@
         <v>49.8</v>
       </c>
       <c r="CB43" s="15" t="n">
+        <v>49.8</v>
+      </c>
+      <c r="CC43" s="15" t="n">
         <v>49.8</v>
       </c>
     </row>
@@ -9326,6 +9432,9 @@
       </c>
       <c r="CB44" s="15" t="n">
         <v>3271.9</v>
+      </c>
+      <c r="CC44" s="15" t="n">
+        <v>3318.43</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
@@ -9457,6 +9566,7 @@
       <c r="BZ45" s="15" t="n"/>
       <c r="CA45" s="15" t="n"/>
       <c r="CB45" s="15" t="n"/>
+      <c r="CC45" s="15" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -9697,6 +9807,9 @@
         <v>61.04</v>
       </c>
       <c r="CB46" s="15" t="n">
+        <v>61.04</v>
+      </c>
+      <c r="CC46" s="15" t="n">
         <v>61.04</v>
       </c>
     </row>
@@ -9891,6 +10004,9 @@
         <v>7025.76</v>
       </c>
       <c r="CB47" s="15" t="n">
+        <v>7025.76</v>
+      </c>
+      <c r="CC47" s="15" t="n">
         <v>7025.76</v>
       </c>
     </row>
@@ -10023,6 +10139,7 @@
       <c r="BZ48" s="15" t="n"/>
       <c r="CA48" s="15" t="n"/>
       <c r="CB48" s="15" t="n"/>
+      <c r="CC48" s="15" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -10263,6 +10380,9 @@
         <v>19.57</v>
       </c>
       <c r="CB49" s="15" t="n">
+        <v>19.57</v>
+      </c>
+      <c r="CC49" s="15" t="n">
         <v>19.57</v>
       </c>
     </row>
@@ -10457,6 +10577,9 @@
         <v>32172.27</v>
       </c>
       <c r="CB50" s="15" t="n">
+        <v>32172.27</v>
+      </c>
+      <c r="CC50" s="15" t="n">
         <v>32172.27</v>
       </c>
     </row>
@@ -10589,6 +10712,7 @@
       <c r="BZ51" s="15" t="n"/>
       <c r="CA51" s="15" t="n"/>
       <c r="CB51" s="15" t="n"/>
+      <c r="CC51" s="15" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -10829,6 +10953,9 @@
         <v>29.77</v>
       </c>
       <c r="CB52" s="15" t="n">
+        <v>29.77</v>
+      </c>
+      <c r="CC52" s="15" t="n">
         <v>29.77</v>
       </c>
     </row>
@@ -11024,6 +11151,9 @@
       </c>
       <c r="CB53" s="15" t="n">
         <v>3172.05</v>
+      </c>
+      <c r="CC53" s="15" t="n">
+        <v>3141.09</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
@@ -11155,6 +11285,7 @@
       <c r="BZ54" s="15" t="n"/>
       <c r="CA54" s="15" t="n"/>
       <c r="CB54" s="15" t="n"/>
+      <c r="CC54" s="15" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -11395,6 +11526,9 @@
         <v>38.37</v>
       </c>
       <c r="CB55" s="15" t="n">
+        <v>38.37</v>
+      </c>
+      <c r="CC55" s="15" t="n">
         <v>38.37</v>
       </c>
     </row>
@@ -11590,6 +11724,9 @@
       </c>
       <c r="CB56" s="15" t="n">
         <v>3068.62</v>
+      </c>
+      <c r="CC56" s="15" t="n">
+        <v>3036.66</v>
       </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
@@ -11721,6 +11858,7 @@
       <c r="BZ57" s="15" t="n"/>
       <c r="CA57" s="15" t="n"/>
       <c r="CB57" s="15" t="n"/>
+      <c r="CC57" s="15" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -11961,6 +12099,9 @@
         <v>19.41</v>
       </c>
       <c r="CB58" s="15" t="n">
+        <v>19.41</v>
+      </c>
+      <c r="CC58" s="15" t="n">
         <v>19.41</v>
       </c>
     </row>
@@ -12156,6 +12297,9 @@
       </c>
       <c r="CB59" s="15" t="n">
         <v>6778.05</v>
+      </c>
+      <c r="CC59" s="15" t="n">
+        <v>6695.35</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
@@ -12287,6 +12431,7 @@
       <c r="BZ60" s="15" t="n"/>
       <c r="CA60" s="15" t="n"/>
       <c r="CB60" s="15" t="n"/>
+      <c r="CC60" s="15" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -12527,6 +12672,9 @@
         <v>37.19</v>
       </c>
       <c r="CB61" s="15" t="n">
+        <v>37.19</v>
+      </c>
+      <c r="CC61" s="15" t="n">
         <v>37.19</v>
       </c>
     </row>
@@ -12722,6 +12870,9 @@
       </c>
       <c r="CB62" s="15" t="n">
         <v>8258.719999999999</v>
+      </c>
+      <c r="CC62" s="15" t="n">
+        <v>8168.89</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
@@ -12853,6 +13004,7 @@
       <c r="BZ63" s="15" t="n"/>
       <c r="CA63" s="15" t="n"/>
       <c r="CB63" s="15" t="n"/>
+      <c r="CC63" s="15" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -13093,6 +13245,9 @@
         <v>6.29</v>
       </c>
       <c r="CB64" s="15" t="n">
+        <v>6.29</v>
+      </c>
+      <c r="CC64" s="15" t="n">
         <v>6.29</v>
       </c>
     </row>
@@ -13287,6 +13442,9 @@
         <v>10401.01</v>
       </c>
       <c r="CB65" s="15" t="n">
+        <v>10401.01</v>
+      </c>
+      <c r="CC65" s="15" t="n">
         <v>10401.01</v>
       </c>
     </row>
@@ -13419,6 +13577,7 @@
       <c r="BZ66" s="15" t="n"/>
       <c r="CA66" s="15" t="n"/>
       <c r="CB66" s="15" t="n"/>
+      <c r="CC66" s="15" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -13659,6 +13818,9 @@
         <v>15.25</v>
       </c>
       <c r="CB67" s="15" t="n">
+        <v>15.25</v>
+      </c>
+      <c r="CC67" s="15" t="n">
         <v>15.25</v>
       </c>
     </row>
@@ -13854,6 +14016,9 @@
       </c>
       <c r="CB68" s="15" t="n">
         <v>10986.17</v>
+      </c>
+      <c r="CC68" s="15" t="n">
+        <v>11058.05</v>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
@@ -13985,6 +14150,7 @@
       <c r="BZ69" s="15" t="n"/>
       <c r="CA69" s="15" t="n"/>
       <c r="CB69" s="15" t="n"/>
+      <c r="CC69" s="15" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -14225,6 +14391,9 @@
         <v>15.18</v>
       </c>
       <c r="CB70" s="15" t="n">
+        <v>15.18</v>
+      </c>
+      <c r="CC70" s="15" t="n">
         <v>15.18</v>
       </c>
     </row>
@@ -14420,6 +14589,9 @@
       </c>
       <c r="CB71" s="15" t="n">
         <v>6204.3</v>
+      </c>
+      <c r="CC71" s="15" t="n">
+        <v>6208.72</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
@@ -14551,6 +14723,7 @@
       <c r="BZ72" s="15" t="n"/>
       <c r="CA72" s="15" t="n"/>
       <c r="CB72" s="15" t="n"/>
+      <c r="CC72" s="15" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -14791,6 +14964,9 @@
         <v>17.67</v>
       </c>
       <c r="CB73" s="15" t="n">
+        <v>17.67</v>
+      </c>
+      <c r="CC73" s="15" t="n">
         <v>17.67</v>
       </c>
     </row>
@@ -14986,6 +15162,9 @@
       </c>
       <c r="CB74" s="15" t="n">
         <v>12290.17</v>
+      </c>
+      <c r="CC74" s="15" t="n">
+        <v>12256.81</v>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
@@ -15117,6 +15296,7 @@
       <c r="BZ75" s="15" t="n"/>
       <c r="CA75" s="15" t="n"/>
       <c r="CB75" s="15" t="n"/>
+      <c r="CC75" s="15" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -15357,6 +15537,9 @@
         <v>53.36</v>
       </c>
       <c r="CB76" s="15" t="n">
+        <v>53.36</v>
+      </c>
+      <c r="CC76" s="15" t="n">
         <v>53.36</v>
       </c>
     </row>
@@ -15552,6 +15735,9 @@
       </c>
       <c r="CB77" s="15" t="n">
         <v>15569.82</v>
+      </c>
+      <c r="CC77" s="15" t="n">
+        <v>15685.19</v>
       </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
@@ -15683,6 +15869,7 @@
       <c r="BZ78" s="15" t="n"/>
       <c r="CA78" s="15" t="n"/>
       <c r="CB78" s="15" t="n"/>
+      <c r="CC78" s="15" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -15923,6 +16110,9 @@
         <v>1.74</v>
       </c>
       <c r="CB79" s="15" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="CC79" s="15" t="n">
         <v>1.74</v>
       </c>
     </row>
@@ -16117,6 +16307,9 @@
         <v>6406.02</v>
       </c>
       <c r="CB80" s="15" t="n">
+        <v>6277.54</v>
+      </c>
+      <c r="CC80" s="15" t="n">
         <v>6277.54</v>
       </c>
     </row>
@@ -16249,6 +16442,7 @@
       <c r="BZ81" s="15" t="n"/>
       <c r="CA81" s="15" t="n"/>
       <c r="CB81" s="15" t="n"/>
+      <c r="CC81" s="15" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -16489,6 +16683,9 @@
         <v>3.58</v>
       </c>
       <c r="CB82" s="15" t="n">
+        <v>3.58</v>
+      </c>
+      <c r="CC82" s="15" t="n">
         <v>3.58</v>
       </c>
     </row>
@@ -16684,6 +16881,9 @@
       </c>
       <c r="CB83" s="15" t="n">
         <v>8291.16</v>
+      </c>
+      <c r="CC83" s="15" t="n">
+        <v>8280.549999999999</v>
       </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
@@ -16815,6 +17015,7 @@
       <c r="BZ84" s="15" t="n"/>
       <c r="CA84" s="15" t="n"/>
       <c r="CB84" s="15" t="n"/>
+      <c r="CC84" s="15" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -17055,6 +17256,9 @@
         <v>14.91</v>
       </c>
       <c r="CB85" s="15" t="n">
+        <v>14.91</v>
+      </c>
+      <c r="CC85" s="15" t="n">
         <v>14.91</v>
       </c>
     </row>
@@ -17250,6 +17454,9 @@
       </c>
       <c r="CB86" s="15" t="n">
         <v>1972.7</v>
+      </c>
+      <c r="CC86" s="15" t="n">
+        <v>2631.9</v>
       </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
@@ -17381,6 +17588,7 @@
       <c r="BZ87" s="15" t="n"/>
       <c r="CA87" s="15" t="n"/>
       <c r="CB87" s="15" t="n"/>
+      <c r="CC87" s="15" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -17621,6 +17829,9 @@
         <v>22.01</v>
       </c>
       <c r="CB88" s="15" t="n">
+        <v>22.01</v>
+      </c>
+      <c r="CC88" s="15" t="n">
         <v>22.01</v>
       </c>
     </row>
@@ -17816,6 +18027,9 @@
       </c>
       <c r="CB89" s="15" t="n">
         <v>4113.73</v>
+      </c>
+      <c r="CC89" s="15" t="n">
+        <v>4073.38</v>
       </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
@@ -17947,6 +18161,7 @@
       <c r="BZ90" s="15" t="n"/>
       <c r="CA90" s="15" t="n"/>
       <c r="CB90" s="15" t="n"/>
+      <c r="CC90" s="15" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -18187,6 +18402,9 @@
         <v>19.19</v>
       </c>
       <c r="CB91" s="15" t="n">
+        <v>19.19</v>
+      </c>
+      <c r="CC91" s="15" t="n">
         <v>19.19</v>
       </c>
     </row>
@@ -18382,6 +18600,9 @@
       </c>
       <c r="CB92" s="15" t="n">
         <v>8544.57</v>
+      </c>
+      <c r="CC92" s="15" t="n">
+        <v>8461.809999999999</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
@@ -18513,6 +18734,7 @@
       <c r="BZ93" s="15" t="n"/>
       <c r="CA93" s="15" t="n"/>
       <c r="CB93" s="15" t="n"/>
+      <c r="CC93" s="15" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -18753,6 +18975,9 @@
         <v>4.22</v>
       </c>
       <c r="CB94" s="15" t="n">
+        <v>4.22</v>
+      </c>
+      <c r="CC94" s="15" t="n">
         <v>4.22</v>
       </c>
     </row>
@@ -18948,6 +19173,9 @@
       </c>
       <c r="CB95" s="15" t="n">
         <v>1174.56</v>
+      </c>
+      <c r="CC95" s="15" t="n">
+        <v>1161.27</v>
       </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
@@ -19079,6 +19307,7 @@
       <c r="BZ96" s="15" t="n"/>
       <c r="CA96" s="15" t="n"/>
       <c r="CB96" s="15" t="n"/>
+      <c r="CC96" s="15" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -19319,6 +19548,9 @@
         <v>8.539999999999999</v>
       </c>
       <c r="CB97" s="15" t="n">
+        <v>8.539999999999999</v>
+      </c>
+      <c r="CC97" s="15" t="n">
         <v>8.539999999999999</v>
       </c>
     </row>
@@ -19514,6 +19746,9 @@
       </c>
       <c r="CB98" s="15" t="n">
         <v>13618.21</v>
+      </c>
+      <c r="CC98" s="15" t="n">
+        <v>13613.78</v>
       </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
@@ -19645,6 +19880,7 @@
       <c r="BZ99" s="15" t="n"/>
       <c r="CA99" s="15" t="n"/>
       <c r="CB99" s="15" t="n"/>
+      <c r="CC99" s="15" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -19885,6 +20121,9 @@
         <v>39.69</v>
       </c>
       <c r="CB100" s="15" t="n">
+        <v>39.69</v>
+      </c>
+      <c r="CC100" s="15" t="n">
         <v>39.69</v>
       </c>
     </row>
@@ -20079,6 +20318,9 @@
         <v>3360.25</v>
       </c>
       <c r="CB101" s="15" t="n">
+        <v>3360.25</v>
+      </c>
+      <c r="CC101" s="15" t="n">
         <v>3360.25</v>
       </c>
     </row>
@@ -20211,6 +20453,7 @@
       <c r="BZ102" s="15" t="n"/>
       <c r="CA102" s="15" t="n"/>
       <c r="CB102" s="15" t="n"/>
+      <c r="CC102" s="15" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -20451,6 +20694,9 @@
         <v>23.92</v>
       </c>
       <c r="CB103" s="15" t="n">
+        <v>23.92</v>
+      </c>
+      <c r="CC103" s="15" t="n">
         <v>23.92</v>
       </c>
     </row>
@@ -20646,6 +20892,9 @@
       </c>
       <c r="CB104" s="15" t="n">
         <v>2182.09</v>
+      </c>
+      <c r="CC104" s="15" t="n">
+        <v>2169.49</v>
       </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
@@ -20777,6 +21026,7 @@
       <c r="BZ105" s="15" t="n"/>
       <c r="CA105" s="15" t="n"/>
       <c r="CB105" s="15" t="n"/>
+      <c r="CC105" s="15" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -21017,6 +21267,9 @@
         <v>11.98</v>
       </c>
       <c r="CB106" s="15" t="n">
+        <v>11.98</v>
+      </c>
+      <c r="CC106" s="15" t="n">
         <v>11.98</v>
       </c>
     </row>
@@ -21212,6 +21465,9 @@
       </c>
       <c r="CB107" s="15" t="n">
         <v>2259.98</v>
+      </c>
+      <c r="CC107" s="15" t="n">
+        <v>2248.52</v>
       </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
@@ -21343,6 +21599,7 @@
       <c r="BZ108" s="15" t="n"/>
       <c r="CA108" s="15" t="n"/>
       <c r="CB108" s="15" t="n"/>
+      <c r="CC108" s="15" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -21583,6 +21840,9 @@
         <v>24.89</v>
       </c>
       <c r="CB109" s="15" t="n">
+        <v>24.89</v>
+      </c>
+      <c r="CC109" s="15" t="n">
         <v>24.89</v>
       </c>
     </row>
@@ -21778,6 +22038,9 @@
       </c>
       <c r="CB110" s="15" t="n">
         <v>2312.43</v>
+      </c>
+      <c r="CC110" s="15" t="n">
+        <v>2304.77</v>
       </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
@@ -21909,6 +22172,7 @@
       <c r="BZ111" s="15" t="n"/>
       <c r="CA111" s="15" t="n"/>
       <c r="CB111" s="15" t="n"/>
+      <c r="CC111" s="15" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -22149,6 +22413,9 @@
         <v>53.65</v>
       </c>
       <c r="CB112" s="15" t="n">
+        <v>53.65</v>
+      </c>
+      <c r="CC112" s="15" t="n">
         <v>53.65</v>
       </c>
     </row>
@@ -22342,6 +22609,9 @@
       </c>
       <c r="CB113" s="15" t="n">
         <v>1963.8</v>
+      </c>
+      <c r="CC113" s="15" t="n">
+        <v>1893.9</v>
       </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
@@ -22473,6 +22743,7 @@
       <c r="BZ114" s="15" t="n"/>
       <c r="CA114" s="15" t="n"/>
       <c r="CB114" s="15" t="n"/>
+      <c r="CC114" s="15" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -22713,6 +22984,9 @@
         <v>18.24</v>
       </c>
       <c r="CB115" s="15" t="n">
+        <v>18.24</v>
+      </c>
+      <c r="CC115" s="15" t="n">
         <v>18.24</v>
       </c>
     </row>
@@ -22893,6 +23167,9 @@
       </c>
       <c r="CB116" s="15" t="n">
         <v>8670.76</v>
+      </c>
+      <c r="CC116" s="15" t="n">
+        <v>8701.969999999999</v>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1">
@@ -22979,6 +23256,7 @@
       <c r="BZ117" s="15" t="n"/>
       <c r="CA117" s="15" t="n"/>
       <c r="CB117" s="15" t="n"/>
+      <c r="CC117" s="15" t="n"/>
     </row>
     <row r="118" ht="14.25" customHeight="1">
       <c r="P118" s="13" t="n">
@@ -23176,6 +23454,9 @@
       <c r="CB118" s="15" t="n">
         <v>69.3</v>
       </c>
+      <c r="CC118" s="15" t="n">
+        <v>69.3</v>
+      </c>
     </row>
     <row r="119" ht="14.25" customHeight="1">
       <c r="Y119" s="13" t="n">
@@ -23345,6 +23626,9 @@
       </c>
       <c r="CB119" s="15" t="n">
         <v>11702.13</v>
+      </c>
+      <c r="CC119" s="15" t="n">
+        <v>12036.57</v>
       </c>
     </row>
     <row r="120" ht="14.25" customHeight="1">
@@ -23380,6 +23664,7 @@
       <c r="BZ120" s="15" t="n"/>
       <c r="CA120" s="15" t="n"/>
       <c r="CB120" s="15" t="n"/>
+      <c r="CC120" s="15" t="n"/>
     </row>
     <row r="121" ht="14.25" customHeight="1">
       <c r="AW121" s="13" t="n">
@@ -23478,6 +23763,9 @@
       <c r="CB121" s="15" t="n">
         <v>21.06</v>
       </c>
+      <c r="CC121" s="15" t="n">
+        <v>21.06</v>
+      </c>
     </row>
     <row r="122" ht="14.25" customHeight="1">
       <c r="AW122" s="13" t="n">
@@ -23574,6 +23862,9 @@
         <v>1161.09</v>
       </c>
       <c r="CB122" s="15" t="n">
+        <v>1161.09</v>
+      </c>
+      <c r="CC122" s="15" t="n">
         <v>1161.09</v>
       </c>
     </row>
@@ -23610,6 +23901,7 @@
       <c r="BZ123" s="15" t="n"/>
       <c r="CA123" s="15" t="n"/>
       <c r="CB123" s="15" t="n"/>
+      <c r="CC123" s="15" t="n"/>
     </row>
     <row r="124" ht="14.25" customHeight="1">
       <c r="AW124" s="13" t="n">
@@ -23708,6 +24000,9 @@
       <c r="CB124" s="15" t="n">
         <v>39.15</v>
       </c>
+      <c r="CC124" s="15" t="n">
+        <v>39.15</v>
+      </c>
     </row>
     <row r="125" ht="14.25" customHeight="1">
       <c r="AW125" s="13" t="n">
@@ -23805,6 +24100,9 @@
       </c>
       <c r="CB125" s="15" t="n">
         <v>11216.93</v>
+      </c>
+      <c r="CC125" s="15" t="n">
+        <v>11098.74</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1">
@@ -23840,6 +24138,7 @@
       <c r="BZ126" s="15" t="n"/>
       <c r="CA126" s="15" t="n"/>
       <c r="CB126" s="15" t="n"/>
+      <c r="CC126" s="15" t="n"/>
     </row>
     <row r="127" ht="14.25" customHeight="1">
       <c r="AW127" s="13" t="n">
@@ -23938,6 +24237,9 @@
       <c r="CB127" s="15" t="n">
         <v>4.78</v>
       </c>
+      <c r="CC127" s="15" t="n">
+        <v>4.78</v>
+      </c>
     </row>
     <row r="128" ht="14.25" customHeight="1">
       <c r="AW128" s="13" t="n">
@@ -24034,6 +24336,9 @@
         <v>1843.6</v>
       </c>
       <c r="CB128" s="15" t="n">
+        <v>1843.6</v>
+      </c>
+      <c r="CC128" s="15" t="n">
         <v>1843.6</v>
       </c>
     </row>
@@ -24070,6 +24375,7 @@
       <c r="BZ129" s="15" t="n"/>
       <c r="CA129" s="15" t="n"/>
       <c r="CB129" s="15" t="n"/>
+      <c r="CC129" s="15" t="n"/>
     </row>
     <row r="130" ht="14.25" customHeight="1">
       <c r="AW130" s="13" t="n">
@@ -24168,6 +24474,9 @@
       <c r="CB130" s="15" t="n">
         <v>5.3</v>
       </c>
+      <c r="CC130" s="15" t="n">
+        <v>5.3</v>
+      </c>
     </row>
     <row r="131" ht="14.25" customHeight="1">
       <c r="AW131" s="13" t="n">
@@ -24265,6 +24574,9 @@
       </c>
       <c r="CB131" s="15" t="n">
         <v>708.53</v>
+      </c>
+      <c r="CC131" s="15" t="n">
+        <v>703.28</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1">
@@ -24300,6 +24612,7 @@
       <c r="BZ132" s="15" t="n"/>
       <c r="CA132" s="15" t="n"/>
       <c r="CB132" s="15" t="n"/>
+      <c r="CC132" s="15" t="n"/>
     </row>
     <row r="133" ht="14.25" customHeight="1">
       <c r="AW133" s="13" t="n">
@@ -24398,6 +24711,9 @@
       <c r="CB133" s="15" t="n">
         <v>45.48</v>
       </c>
+      <c r="CC133" s="15" t="n">
+        <v>45.48</v>
+      </c>
     </row>
     <row r="134" ht="14.25" customHeight="1">
       <c r="AW134" s="13" t="n">
@@ -24494,6 +24810,9 @@
         <v>2638.92</v>
       </c>
       <c r="CB134" s="15" t="n">
+        <v>2638.92</v>
+      </c>
+      <c r="CC134" s="15" t="n">
         <v>2638.92</v>
       </c>
     </row>
@@ -24530,6 +24849,7 @@
       <c r="BZ135" s="15" t="n"/>
       <c r="CA135" s="15" t="n"/>
       <c r="CB135" s="15" t="n"/>
+      <c r="CC135" s="15" t="n"/>
     </row>
     <row r="136" ht="14.25" customHeight="1">
       <c r="AW136" s="13" t="n">
@@ -24628,6 +24948,9 @@
       <c r="CB136" s="15" t="n">
         <v>21.18</v>
       </c>
+      <c r="CC136" s="15" t="n">
+        <v>21.18</v>
+      </c>
     </row>
     <row r="137" ht="14.25" customHeight="1">
       <c r="AW137" s="13" t="n">
@@ -24725,6 +25048,9 @@
       </c>
       <c r="CB137" s="15" t="n">
         <v>3457.37</v>
+      </c>
+      <c r="CC137" s="15" t="n">
+        <v>3441.79</v>
       </c>
     </row>
     <row r="138">
@@ -24752,6 +25078,7 @@
       <c r="BZ138" s="15" t="n"/>
       <c r="CA138" s="15" t="n"/>
       <c r="CB138" s="15" t="n"/>
+      <c r="CC138" s="15" t="n"/>
     </row>
     <row r="139">
       <c r="BE139" s="15" t="n">
@@ -24826,6 +25153,9 @@
       <c r="CB139" s="15" t="n">
         <v>5.7</v>
       </c>
+      <c r="CC139" s="15" t="n">
+        <v>5.7</v>
+      </c>
     </row>
     <row r="140">
       <c r="BE140" s="15" t="n">
@@ -24897,6 +25227,9 @@
       </c>
       <c r="CB140" s="15" t="n">
         <v>2589.89</v>
+      </c>
+      <c r="CC140" s="15" t="n">
+        <v>2561.58</v>
       </c>
     </row>
     <row r="141">
@@ -24924,6 +25257,7 @@
       <c r="BZ141" s="15" t="n"/>
       <c r="CA141" s="15" t="n"/>
       <c r="CB141" s="15" t="n"/>
+      <c r="CC141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="BE142" s="15" t="n">
@@ -24998,6 +25332,9 @@
       <c r="CB142" s="15" t="n">
         <v>11.17</v>
       </c>
+      <c r="CC142" s="15" t="n">
+        <v>11.17</v>
+      </c>
     </row>
     <row r="143">
       <c r="BE143" s="15" t="n">
@@ -25070,6 +25407,9 @@
         <v>5423.17</v>
       </c>
       <c r="CB143" s="15" t="n">
+        <v>5423.17</v>
+      </c>
+      <c r="CC143" s="15" t="n">
         <v>5423.17</v>
       </c>
     </row>
@@ -25093,6 +25433,7 @@
       <c r="BZ144" s="15" t="n"/>
       <c r="CA144" s="15" t="n"/>
       <c r="CB144" s="15" t="n"/>
+      <c r="CC144" s="15" t="n"/>
     </row>
     <row r="145">
       <c r="BJ145" s="15" t="n">
@@ -25152,6 +25493,9 @@
       <c r="CB145" s="15" t="n">
         <v>1.89</v>
       </c>
+      <c r="CC145" s="15" t="n">
+        <v>1.89</v>
+      </c>
     </row>
     <row r="146">
       <c r="BJ146" s="15" t="n">
@@ -25210,6 +25554,9 @@
       </c>
       <c r="CB146" s="15" t="n">
         <v>2207.65</v>
+      </c>
+      <c r="CC146" s="15" t="n">
+        <v>2172.18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-10-12 11:21:39]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CC146"/>
+  <dimension ref="A1:CD146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="51"/>
@@ -615,6 +615,7 @@
     <col width="15" customWidth="1" min="79" max="79"/>
     <col width="15" customWidth="1" min="80" max="80"/>
     <col width="15" customWidth="1" min="81" max="81"/>
+    <col width="15" customWidth="1" min="82" max="82"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -1023,6 +1024,11 @@
           <t>2026/10/08</t>
         </is>
       </c>
+      <c r="CD1" s="15" t="inlineStr">
+        <is>
+          <t>2026/10/12</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1430,6 +1436,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="CD2" s="16" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1675,6 +1686,9 @@
       <c r="CC3" s="15" t="n">
         <v>57.07</v>
       </c>
+      <c r="CD3" s="15" t="n">
+        <v>56.1</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1919,6 +1933,9 @@
       </c>
       <c r="CC4" s="15" t="n">
         <v>3811.9</v>
+      </c>
+      <c r="CD4" s="15" t="n">
+        <v>3797.24</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -2003,6 +2020,7 @@
       <c r="CA5" s="15" t="n"/>
       <c r="CB5" s="15" t="n"/>
       <c r="CC5" s="15" t="n"/>
+      <c r="CD5" s="15" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -2134,6 +2152,7 @@
       <c r="CA6" s="15" t="n"/>
       <c r="CB6" s="15" t="n"/>
       <c r="CC6" s="15" t="n"/>
+      <c r="CD6" s="15" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -2378,6 +2397,9 @@
       </c>
       <c r="CC7" s="15" t="n">
         <v>47.39</v>
+      </c>
+      <c r="CD7" s="15" t="n">
+        <v>45.74</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -2575,6 +2597,9 @@
       </c>
       <c r="CC8" s="15" t="n">
         <v>5289.44</v>
+      </c>
+      <c r="CD8" s="15" t="n">
+        <v>5235.37</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
@@ -2707,6 +2732,7 @@
       <c r="CA9" s="15" t="n"/>
       <c r="CB9" s="15" t="n"/>
       <c r="CC9" s="15" t="n"/>
+      <c r="CD9" s="15" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -2951,6 +2977,9 @@
       </c>
       <c r="CC10" s="15" t="n">
         <v>43.3</v>
+      </c>
+      <c r="CD10" s="15" t="n">
+        <v>42.77</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -3148,6 +3177,9 @@
       </c>
       <c r="CC11" s="15" t="n">
         <v>4310.28</v>
+      </c>
+      <c r="CD11" s="15" t="n">
+        <v>4287.98</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
@@ -3280,6 +3312,7 @@
       <c r="CA12" s="15" t="n"/>
       <c r="CB12" s="15" t="n"/>
       <c r="CC12" s="15" t="n"/>
+      <c r="CD12" s="15" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -3524,6 +3557,9 @@
       </c>
       <c r="CC13" s="15" t="n">
         <v>55.81</v>
+      </c>
+      <c r="CD13" s="15" t="n">
+        <v>52.82</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -3721,6 +3757,9 @@
       </c>
       <c r="CC14" s="15" t="n">
         <v>7248.43</v>
+      </c>
+      <c r="CD14" s="15" t="n">
+        <v>7093.02</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
@@ -3853,6 +3892,7 @@
       <c r="CA15" s="15" t="n"/>
       <c r="CB15" s="15" t="n"/>
       <c r="CC15" s="15" t="n"/>
+      <c r="CD15" s="15" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -4097,6 +4137,9 @@
       </c>
       <c r="CC16" s="15" t="n">
         <v>25.39</v>
+      </c>
+      <c r="CD16" s="15" t="n">
+        <v>25.69</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -4294,6 +4337,9 @@
       </c>
       <c r="CC17" s="15" t="n">
         <v>2404.7</v>
+      </c>
+      <c r="CD17" s="15" t="n">
+        <v>2417.22</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
@@ -4426,6 +4472,7 @@
       <c r="CA18" s="15" t="n"/>
       <c r="CB18" s="15" t="n"/>
       <c r="CC18" s="15" t="n"/>
+      <c r="CD18" s="15" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -4669,6 +4716,9 @@
         <v>79.77</v>
       </c>
       <c r="CC19" s="15" t="n">
+        <v>79.77</v>
+      </c>
+      <c r="CD19" s="15" t="n">
         <v>79.77</v>
       </c>
     </row>
@@ -4867,6 +4917,9 @@
       </c>
       <c r="CC20" s="15" t="n">
         <v>7801.77</v>
+      </c>
+      <c r="CD20" s="15" t="n">
+        <v>7811.54</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
@@ -4999,6 +5052,7 @@
       <c r="CA21" s="15" t="n"/>
       <c r="CB21" s="15" t="n"/>
       <c r="CC21" s="15" t="n"/>
+      <c r="CD21" s="15" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -5240,6 +5294,9 @@
         <v>36.34</v>
       </c>
       <c r="CC22" s="15" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="CD22" s="15" t="n">
         <v>36.34</v>
       </c>
     </row>
@@ -5438,6 +5495,9 @@
       </c>
       <c r="CC23" s="15" t="n">
         <v>71593.24000000001</v>
+      </c>
+      <c r="CD23" s="15" t="n">
+        <v>71924.67999999999</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
@@ -5570,6 +5630,7 @@
       <c r="CA24" s="15" t="n"/>
       <c r="CB24" s="15" t="n"/>
       <c r="CC24" s="15" t="n"/>
+      <c r="CD24" s="15" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -5813,6 +5874,9 @@
         <v>49.88</v>
       </c>
       <c r="CC25" s="15" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="CD25" s="15" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -5997,6 +6061,9 @@
       </c>
       <c r="CC26" s="15" t="n">
         <v>24808.03</v>
+      </c>
+      <c r="CD26" s="15" t="n">
+        <v>25257.04</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
@@ -6129,6 +6196,7 @@
       <c r="CA27" s="15" t="n"/>
       <c r="CB27" s="15" t="n"/>
       <c r="CC27" s="15" t="n"/>
+      <c r="CD27" s="15" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -6372,6 +6440,9 @@
         <v>92.09</v>
       </c>
       <c r="CC28" s="15" t="n">
+        <v>92.09</v>
+      </c>
+      <c r="CD28" s="15" t="n">
         <v>92.09</v>
       </c>
     </row>
@@ -6570,6 +6641,9 @@
       </c>
       <c r="CC29" s="15" t="n">
         <v>69042.11</v>
+      </c>
+      <c r="CD29" s="15" t="n">
+        <v>69030.92</v>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
@@ -6702,6 +6776,7 @@
       <c r="CA30" s="15" t="n"/>
       <c r="CB30" s="15" t="n"/>
       <c r="CC30" s="15" t="n"/>
+      <c r="CD30" s="15" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -6945,6 +7020,9 @@
         <v>97.44</v>
       </c>
       <c r="CC31" s="15" t="n">
+        <v>97.44</v>
+      </c>
+      <c r="CD31" s="15" t="n">
         <v>97.44</v>
       </c>
     </row>
@@ -7143,6 +7221,9 @@
       </c>
       <c r="CC32" s="15" t="n">
         <v>6625.93</v>
+      </c>
+      <c r="CD32" s="15" t="n">
+        <v>6384.24</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
@@ -7275,6 +7356,7 @@
       <c r="CA33" s="15" t="n"/>
       <c r="CB33" s="15" t="n"/>
       <c r="CC33" s="15" t="n"/>
+      <c r="CD33" s="15" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -7519,6 +7601,9 @@
       </c>
       <c r="CC34" s="15" t="n">
         <v>47.21</v>
+      </c>
+      <c r="CD34" s="15" t="n">
+        <v>46.97</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -7716,6 +7801,9 @@
       </c>
       <c r="CC35" s="15" t="n">
         <v>5556.01</v>
+      </c>
+      <c r="CD35" s="15" t="n">
+        <v>5618.87</v>
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
@@ -7848,6 +7936,7 @@
       <c r="CA36" s="15" t="n"/>
       <c r="CB36" s="15" t="n"/>
       <c r="CC36" s="15" t="n"/>
+      <c r="CD36" s="15" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -8092,6 +8181,9 @@
       </c>
       <c r="CC37" s="15" t="n">
         <v>55.99</v>
+      </c>
+      <c r="CD37" s="15" t="n">
+        <v>55.85</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -8289,6 +8381,9 @@
       </c>
       <c r="CC38" s="15" t="n">
         <v>11285.61</v>
+      </c>
+      <c r="CD38" s="15" t="n">
+        <v>11540.66</v>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
@@ -8421,6 +8516,7 @@
       <c r="CA39" s="15" t="n"/>
       <c r="CB39" s="15" t="n"/>
       <c r="CC39" s="15" t="n"/>
+      <c r="CD39" s="15" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -8665,6 +8761,9 @@
       </c>
       <c r="CC40" s="15" t="n">
         <v>52.27</v>
+      </c>
+      <c r="CD40" s="15" t="n">
+        <v>52.31</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -8862,6 +8961,9 @@
       </c>
       <c r="CC41" s="15" t="n">
         <v>10971.43</v>
+      </c>
+      <c r="CD41" s="15" t="n">
+        <v>11276.01</v>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
@@ -8994,6 +9096,7 @@
       <c r="CA42" s="15" t="n"/>
       <c r="CB42" s="15" t="n"/>
       <c r="CC42" s="15" t="n"/>
+      <c r="CD42" s="15" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -9238,6 +9341,9 @@
       </c>
       <c r="CC43" s="15" t="n">
         <v>49.8</v>
+      </c>
+      <c r="CD43" s="15" t="n">
+        <v>49.72</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -9435,6 +9541,9 @@
       </c>
       <c r="CC44" s="15" t="n">
         <v>3318.43</v>
+      </c>
+      <c r="CD44" s="15" t="n">
+        <v>3352.22</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
@@ -9567,6 +9676,7 @@
       <c r="CA45" s="15" t="n"/>
       <c r="CB45" s="15" t="n"/>
       <c r="CC45" s="15" t="n"/>
+      <c r="CD45" s="15" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -9811,6 +9921,9 @@
       </c>
       <c r="CC46" s="15" t="n">
         <v>61.04</v>
+      </c>
+      <c r="CD46" s="15" t="n">
+        <v>62.93</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -10008,6 +10121,9 @@
       </c>
       <c r="CC47" s="15" t="n">
         <v>7025.76</v>
+      </c>
+      <c r="CD47" s="15" t="n">
+        <v>7205.29</v>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
@@ -10140,6 +10256,7 @@
       <c r="CA48" s="15" t="n"/>
       <c r="CB48" s="15" t="n"/>
       <c r="CC48" s="15" t="n"/>
+      <c r="CD48" s="15" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -10384,6 +10501,9 @@
       </c>
       <c r="CC49" s="15" t="n">
         <v>19.57</v>
+      </c>
+      <c r="CD49" s="15" t="n">
+        <v>19.77</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -10581,6 +10701,9 @@
       </c>
       <c r="CC50" s="15" t="n">
         <v>32172.27</v>
+      </c>
+      <c r="CD50" s="15" t="n">
+        <v>31603.58</v>
       </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
@@ -10713,6 +10836,7 @@
       <c r="CA51" s="15" t="n"/>
       <c r="CB51" s="15" t="n"/>
       <c r="CC51" s="15" t="n"/>
+      <c r="CD51" s="15" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -10957,6 +11081,9 @@
       </c>
       <c r="CC52" s="15" t="n">
         <v>29.77</v>
+      </c>
+      <c r="CD52" s="15" t="n">
+        <v>27.51</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -11154,6 +11281,9 @@
       </c>
       <c r="CC53" s="15" t="n">
         <v>3141.09</v>
+      </c>
+      <c r="CD53" s="15" t="n">
+        <v>3057.91</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
@@ -11286,6 +11416,7 @@
       <c r="CA54" s="15" t="n"/>
       <c r="CB54" s="15" t="n"/>
       <c r="CC54" s="15" t="n"/>
+      <c r="CD54" s="15" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -11530,6 +11661,9 @@
       </c>
       <c r="CC55" s="15" t="n">
         <v>38.37</v>
+      </c>
+      <c r="CD55" s="15" t="n">
+        <v>34.71</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -11727,6 +11861,9 @@
       </c>
       <c r="CC56" s="15" t="n">
         <v>3036.66</v>
+      </c>
+      <c r="CD56" s="15" t="n">
+        <v>2963.82</v>
       </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
@@ -11859,6 +11996,7 @@
       <c r="CA57" s="15" t="n"/>
       <c r="CB57" s="15" t="n"/>
       <c r="CC57" s="15" t="n"/>
+      <c r="CD57" s="15" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -12103,6 +12241,9 @@
       </c>
       <c r="CC58" s="15" t="n">
         <v>19.41</v>
+      </c>
+      <c r="CD58" s="15" t="n">
+        <v>15.95</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -12300,6 +12441,9 @@
       </c>
       <c r="CC59" s="15" t="n">
         <v>6695.35</v>
+      </c>
+      <c r="CD59" s="15" t="n">
+        <v>6717.92</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
@@ -12432,6 +12576,7 @@
       <c r="CA60" s="15" t="n"/>
       <c r="CB60" s="15" t="n"/>
       <c r="CC60" s="15" t="n"/>
+      <c r="CD60" s="15" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -12676,6 +12821,9 @@
       </c>
       <c r="CC61" s="15" t="n">
         <v>37.19</v>
+      </c>
+      <c r="CD61" s="15" t="n">
+        <v>34.12</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -12873,6 +13021,9 @@
       </c>
       <c r="CC62" s="15" t="n">
         <v>8168.89</v>
+      </c>
+      <c r="CD62" s="15" t="n">
+        <v>8127.67</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
@@ -13005,6 +13156,7 @@
       <c r="CA63" s="15" t="n"/>
       <c r="CB63" s="15" t="n"/>
       <c r="CC63" s="15" t="n"/>
+      <c r="CD63" s="15" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -13249,6 +13401,9 @@
       </c>
       <c r="CC64" s="15" t="n">
         <v>6.29</v>
+      </c>
+      <c r="CD64" s="15" t="n">
+        <v>7.3</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -13446,6 +13601,9 @@
       </c>
       <c r="CC65" s="15" t="n">
         <v>10401.01</v>
+      </c>
+      <c r="CD65" s="15" t="n">
+        <v>10471.58</v>
       </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
@@ -13578,6 +13736,7 @@
       <c r="CA66" s="15" t="n"/>
       <c r="CB66" s="15" t="n"/>
       <c r="CC66" s="15" t="n"/>
+      <c r="CD66" s="15" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -13822,6 +13981,9 @@
       </c>
       <c r="CC67" s="15" t="n">
         <v>15.25</v>
+      </c>
+      <c r="CD67" s="15" t="n">
+        <v>16.26</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -14019,6 +14181,9 @@
       </c>
       <c r="CC68" s="15" t="n">
         <v>11058.05</v>
+      </c>
+      <c r="CD68" s="15" t="n">
+        <v>10962.63</v>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
@@ -14151,6 +14316,7 @@
       <c r="CA69" s="15" t="n"/>
       <c r="CB69" s="15" t="n"/>
       <c r="CC69" s="15" t="n"/>
+      <c r="CD69" s="15" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -14395,6 +14561,9 @@
       </c>
       <c r="CC70" s="15" t="n">
         <v>15.18</v>
+      </c>
+      <c r="CD70" s="15" t="n">
+        <v>15.57</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -14592,6 +14761,9 @@
       </c>
       <c r="CC71" s="15" t="n">
         <v>6208.72</v>
+      </c>
+      <c r="CD71" s="15" t="n">
+        <v>6260.98</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
@@ -14724,6 +14896,7 @@
       <c r="CA72" s="15" t="n"/>
       <c r="CB72" s="15" t="n"/>
       <c r="CC72" s="15" t="n"/>
+      <c r="CD72" s="15" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -14968,6 +15141,9 @@
       </c>
       <c r="CC73" s="15" t="n">
         <v>17.67</v>
+      </c>
+      <c r="CD73" s="15" t="n">
+        <v>18.7</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -15165,6 +15341,9 @@
       </c>
       <c r="CC74" s="15" t="n">
         <v>12256.81</v>
+      </c>
+      <c r="CD74" s="15" t="n">
+        <v>12469.15</v>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
@@ -15297,6 +15476,7 @@
       <c r="CA75" s="15" t="n"/>
       <c r="CB75" s="15" t="n"/>
       <c r="CC75" s="15" t="n"/>
+      <c r="CD75" s="15" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -15541,6 +15721,9 @@
       </c>
       <c r="CC76" s="15" t="n">
         <v>53.36</v>
+      </c>
+      <c r="CD76" s="15" t="n">
+        <v>52.26</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -15738,6 +15921,9 @@
       </c>
       <c r="CC77" s="15" t="n">
         <v>15685.19</v>
+      </c>
+      <c r="CD77" s="15" t="n">
+        <v>15594.78</v>
       </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
@@ -15870,6 +16056,7 @@
       <c r="CA78" s="15" t="n"/>
       <c r="CB78" s="15" t="n"/>
       <c r="CC78" s="15" t="n"/>
+      <c r="CD78" s="15" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -16114,6 +16301,9 @@
       </c>
       <c r="CC79" s="15" t="n">
         <v>1.74</v>
+      </c>
+      <c r="CD79" s="15" t="n">
+        <v>2.12</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -16310,6 +16500,9 @@
         <v>6277.54</v>
       </c>
       <c r="CC80" s="15" t="n">
+        <v>6277.54</v>
+      </c>
+      <c r="CD80" s="15" t="n">
         <v>6277.54</v>
       </c>
     </row>
@@ -16443,6 +16636,7 @@
       <c r="CA81" s="15" t="n"/>
       <c r="CB81" s="15" t="n"/>
       <c r="CC81" s="15" t="n"/>
+      <c r="CD81" s="15" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -16687,6 +16881,9 @@
       </c>
       <c r="CC82" s="15" t="n">
         <v>3.58</v>
+      </c>
+      <c r="CD82" s="15" t="n">
+        <v>5.02</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -16884,6 +17081,9 @@
       </c>
       <c r="CC83" s="15" t="n">
         <v>8280.549999999999</v>
+      </c>
+      <c r="CD83" s="15" t="n">
+        <v>8452.77</v>
       </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
@@ -17016,6 +17216,7 @@
       <c r="CA84" s="15" t="n"/>
       <c r="CB84" s="15" t="n"/>
       <c r="CC84" s="15" t="n"/>
+      <c r="CD84" s="15" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -17260,6 +17461,9 @@
       </c>
       <c r="CC85" s="15" t="n">
         <v>14.91</v>
+      </c>
+      <c r="CD85" s="15" t="n">
+        <v>15.86</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -17456,6 +17660,9 @@
         <v>1972.7</v>
       </c>
       <c r="CC86" s="15" t="n">
+        <v>2631.9</v>
+      </c>
+      <c r="CD86" s="15" t="n">
         <v>2631.9</v>
       </c>
     </row>
@@ -17589,6 +17796,7 @@
       <c r="CA87" s="15" t="n"/>
       <c r="CB87" s="15" t="n"/>
       <c r="CC87" s="15" t="n"/>
+      <c r="CD87" s="15" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -17833,6 +18041,9 @@
       </c>
       <c r="CC88" s="15" t="n">
         <v>22.01</v>
+      </c>
+      <c r="CD88" s="15" t="n">
+        <v>23.15</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -18030,6 +18241,9 @@
       </c>
       <c r="CC89" s="15" t="n">
         <v>4073.38</v>
+      </c>
+      <c r="CD89" s="15" t="n">
+        <v>4169.57</v>
       </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
@@ -18162,6 +18376,7 @@
       <c r="CA90" s="15" t="n"/>
       <c r="CB90" s="15" t="n"/>
       <c r="CC90" s="15" t="n"/>
+      <c r="CD90" s="15" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -18406,6 +18621,9 @@
       </c>
       <c r="CC91" s="15" t="n">
         <v>19.19</v>
+      </c>
+      <c r="CD91" s="15" t="n">
+        <v>15.91</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -18603,6 +18821,9 @@
       </c>
       <c r="CC92" s="15" t="n">
         <v>8461.809999999999</v>
+      </c>
+      <c r="CD92" s="15" t="n">
+        <v>8436.219999999999</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
@@ -18735,6 +18956,7 @@
       <c r="CA93" s="15" t="n"/>
       <c r="CB93" s="15" t="n"/>
       <c r="CC93" s="15" t="n"/>
+      <c r="CD93" s="15" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -18979,6 +19201,9 @@
       </c>
       <c r="CC94" s="15" t="n">
         <v>4.22</v>
+      </c>
+      <c r="CD94" s="15" t="n">
+        <v>3.65</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -19176,6 +19401,9 @@
       </c>
       <c r="CC95" s="15" t="n">
         <v>1161.27</v>
+      </c>
+      <c r="CD95" s="15" t="n">
+        <v>1175.05</v>
       </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
@@ -19308,6 +19536,7 @@
       <c r="CA96" s="15" t="n"/>
       <c r="CB96" s="15" t="n"/>
       <c r="CC96" s="15" t="n"/>
+      <c r="CD96" s="15" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -19552,6 +19781,9 @@
       </c>
       <c r="CC97" s="15" t="n">
         <v>8.539999999999999</v>
+      </c>
+      <c r="CD97" s="15" t="n">
+        <v>9.16</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -19749,6 +19981,9 @@
       </c>
       <c r="CC98" s="15" t="n">
         <v>13613.78</v>
+      </c>
+      <c r="CD98" s="15" t="n">
+        <v>13792.85</v>
       </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
@@ -19881,6 +20116,7 @@
       <c r="CA99" s="15" t="n"/>
       <c r="CB99" s="15" t="n"/>
       <c r="CC99" s="15" t="n"/>
+      <c r="CD99" s="15" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -20125,6 +20361,9 @@
       </c>
       <c r="CC100" s="15" t="n">
         <v>39.69</v>
+      </c>
+      <c r="CD100" s="15" t="n">
+        <v>33.47</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -20322,6 +20561,9 @@
       </c>
       <c r="CC101" s="15" t="n">
         <v>3360.25</v>
+      </c>
+      <c r="CD101" s="15" t="n">
+        <v>3225.74</v>
       </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
@@ -20454,6 +20696,7 @@
       <c r="CA102" s="15" t="n"/>
       <c r="CB102" s="15" t="n"/>
       <c r="CC102" s="15" t="n"/>
+      <c r="CD102" s="15" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -20698,6 +20941,9 @@
       </c>
       <c r="CC103" s="15" t="n">
         <v>23.92</v>
+      </c>
+      <c r="CD103" s="15" t="n">
+        <v>24.85</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -20895,6 +21141,9 @@
       </c>
       <c r="CC104" s="15" t="n">
         <v>2169.49</v>
+      </c>
+      <c r="CD104" s="15" t="n">
+        <v>2153.8</v>
       </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
@@ -21027,6 +21276,7 @@
       <c r="CA105" s="15" t="n"/>
       <c r="CB105" s="15" t="n"/>
       <c r="CC105" s="15" t="n"/>
+      <c r="CD105" s="15" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -21271,6 +21521,9 @@
       </c>
       <c r="CC106" s="15" t="n">
         <v>11.98</v>
+      </c>
+      <c r="CD106" s="15" t="n">
+        <v>10.33</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -21468,6 +21721,9 @@
       </c>
       <c r="CC107" s="15" t="n">
         <v>2248.52</v>
+      </c>
+      <c r="CD107" s="15" t="n">
+        <v>2235.18</v>
       </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
@@ -21600,6 +21856,7 @@
       <c r="CA108" s="15" t="n"/>
       <c r="CB108" s="15" t="n"/>
       <c r="CC108" s="15" t="n"/>
+      <c r="CD108" s="15" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -21844,6 +22101,9 @@
       </c>
       <c r="CC109" s="15" t="n">
         <v>24.89</v>
+      </c>
+      <c r="CD109" s="15" t="n">
+        <v>26.62</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -22041,6 +22301,9 @@
       </c>
       <c r="CC110" s="15" t="n">
         <v>2304.77</v>
+      </c>
+      <c r="CD110" s="15" t="n">
+        <v>2341.61</v>
       </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
@@ -22173,6 +22436,7 @@
       <c r="CA111" s="15" t="n"/>
       <c r="CB111" s="15" t="n"/>
       <c r="CC111" s="15" t="n"/>
+      <c r="CD111" s="15" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -22417,6 +22681,9 @@
       </c>
       <c r="CC112" s="15" t="n">
         <v>53.65</v>
+      </c>
+      <c r="CD112" s="15" t="n">
+        <v>46.91</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -22612,6 +22879,9 @@
       </c>
       <c r="CC113" s="15" t="n">
         <v>1893.9</v>
+      </c>
+      <c r="CD113" s="15" t="n">
+        <v>1870.76</v>
       </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
@@ -22744,6 +23014,7 @@
       <c r="CA114" s="15" t="n"/>
       <c r="CB114" s="15" t="n"/>
       <c r="CC114" s="15" t="n"/>
+      <c r="CD114" s="15" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -22988,6 +23259,9 @@
       </c>
       <c r="CC115" s="15" t="n">
         <v>18.24</v>
+      </c>
+      <c r="CD115" s="15" t="n">
+        <v>17.93</v>
       </c>
     </row>
     <row r="116" ht="14.25" customHeight="1">
@@ -23170,6 +23444,9 @@
       </c>
       <c r="CC116" s="15" t="n">
         <v>8701.969999999999</v>
+      </c>
+      <c r="CD116" s="15" t="n">
+        <v>8718.799999999999</v>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1">
@@ -23257,6 +23534,7 @@
       <c r="CA117" s="15" t="n"/>
       <c r="CB117" s="15" t="n"/>
       <c r="CC117" s="15" t="n"/>
+      <c r="CD117" s="15" t="n"/>
     </row>
     <row r="118" ht="14.25" customHeight="1">
       <c r="P118" s="13" t="n">
@@ -23457,6 +23735,9 @@
       <c r="CC118" s="15" t="n">
         <v>69.3</v>
       </c>
+      <c r="CD118" s="15" t="n">
+        <v>65.69</v>
+      </c>
     </row>
     <row r="119" ht="14.25" customHeight="1">
       <c r="Y119" s="13" t="n">
@@ -23629,6 +23910,9 @@
       </c>
       <c r="CC119" s="15" t="n">
         <v>12036.57</v>
+      </c>
+      <c r="CD119" s="15" t="n">
+        <v>11209.46</v>
       </c>
     </row>
     <row r="120" ht="14.25" customHeight="1">
@@ -23665,6 +23949,7 @@
       <c r="CA120" s="15" t="n"/>
       <c r="CB120" s="15" t="n"/>
       <c r="CC120" s="15" t="n"/>
+      <c r="CD120" s="15" t="n"/>
     </row>
     <row r="121" ht="14.25" customHeight="1">
       <c r="AW121" s="13" t="n">
@@ -23766,6 +24051,9 @@
       <c r="CC121" s="15" t="n">
         <v>21.06</v>
       </c>
+      <c r="CD121" s="15" t="n">
+        <v>24.77</v>
+      </c>
     </row>
     <row r="122" ht="14.25" customHeight="1">
       <c r="AW122" s="13" t="n">
@@ -23866,6 +24154,9 @@
       </c>
       <c r="CC122" s="15" t="n">
         <v>1161.09</v>
+      </c>
+      <c r="CD122" s="15" t="n">
+        <v>1200.52</v>
       </c>
     </row>
     <row r="123" ht="14.25" customHeight="1">
@@ -23902,6 +24193,7 @@
       <c r="CA123" s="15" t="n"/>
       <c r="CB123" s="15" t="n"/>
       <c r="CC123" s="15" t="n"/>
+      <c r="CD123" s="15" t="n"/>
     </row>
     <row r="124" ht="14.25" customHeight="1">
       <c r="AW124" s="13" t="n">
@@ -24003,6 +24295,9 @@
       <c r="CC124" s="15" t="n">
         <v>39.15</v>
       </c>
+      <c r="CD124" s="15" t="n">
+        <v>36.72</v>
+      </c>
     </row>
     <row r="125" ht="14.25" customHeight="1">
       <c r="AW125" s="13" t="n">
@@ -24103,6 +24398,9 @@
       </c>
       <c r="CC125" s="15" t="n">
         <v>11098.74</v>
+      </c>
+      <c r="CD125" s="15" t="n">
+        <v>10698.19</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1">
@@ -24139,6 +24437,7 @@
       <c r="CA126" s="15" t="n"/>
       <c r="CB126" s="15" t="n"/>
       <c r="CC126" s="15" t="n"/>
+      <c r="CD126" s="15" t="n"/>
     </row>
     <row r="127" ht="14.25" customHeight="1">
       <c r="AW127" s="13" t="n">
@@ -24240,6 +24539,9 @@
       <c r="CC127" s="15" t="n">
         <v>4.78</v>
       </c>
+      <c r="CD127" s="15" t="n">
+        <v>4.15</v>
+      </c>
     </row>
     <row r="128" ht="14.25" customHeight="1">
       <c r="AW128" s="13" t="n">
@@ -24340,6 +24642,9 @@
       </c>
       <c r="CC128" s="15" t="n">
         <v>1843.6</v>
+      </c>
+      <c r="CD128" s="15" t="n">
+        <v>1838.45</v>
       </c>
     </row>
     <row r="129" ht="14.25" customHeight="1">
@@ -24376,6 +24681,7 @@
       <c r="CA129" s="15" t="n"/>
       <c r="CB129" s="15" t="n"/>
       <c r="CC129" s="15" t="n"/>
+      <c r="CD129" s="15" t="n"/>
     </row>
     <row r="130" ht="14.25" customHeight="1">
       <c r="AW130" s="13" t="n">
@@ -24477,6 +24783,9 @@
       <c r="CC130" s="15" t="n">
         <v>5.3</v>
       </c>
+      <c r="CD130" s="15" t="n">
+        <v>5.2</v>
+      </c>
     </row>
     <row r="131" ht="14.25" customHeight="1">
       <c r="AW131" s="13" t="n">
@@ -24577,6 +24886,9 @@
       </c>
       <c r="CC131" s="15" t="n">
         <v>703.28</v>
+      </c>
+      <c r="CD131" s="15" t="n">
+        <v>721.09</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1">
@@ -24613,6 +24925,7 @@
       <c r="CA132" s="15" t="n"/>
       <c r="CB132" s="15" t="n"/>
       <c r="CC132" s="15" t="n"/>
+      <c r="CD132" s="15" t="n"/>
     </row>
     <row r="133" ht="14.25" customHeight="1">
       <c r="AW133" s="13" t="n">
@@ -24714,6 +25027,9 @@
       <c r="CC133" s="15" t="n">
         <v>45.48</v>
       </c>
+      <c r="CD133" s="15" t="n">
+        <v>47.64</v>
+      </c>
     </row>
     <row r="134" ht="14.25" customHeight="1">
       <c r="AW134" s="13" t="n">
@@ -24814,6 +25130,9 @@
       </c>
       <c r="CC134" s="15" t="n">
         <v>2638.92</v>
+      </c>
+      <c r="CD134" s="15" t="n">
+        <v>2641.45</v>
       </c>
     </row>
     <row r="135" ht="14.25" customHeight="1">
@@ -24850,6 +25169,7 @@
       <c r="CA135" s="15" t="n"/>
       <c r="CB135" s="15" t="n"/>
       <c r="CC135" s="15" t="n"/>
+      <c r="CD135" s="15" t="n"/>
     </row>
     <row r="136" ht="14.25" customHeight="1">
       <c r="AW136" s="13" t="n">
@@ -24951,6 +25271,9 @@
       <c r="CC136" s="15" t="n">
         <v>21.18</v>
       </c>
+      <c r="CD136" s="15" t="n">
+        <v>21.18</v>
+      </c>
     </row>
     <row r="137" ht="14.25" customHeight="1">
       <c r="AW137" s="13" t="n">
@@ -25051,6 +25374,9 @@
       </c>
       <c r="CC137" s="15" t="n">
         <v>3441.79</v>
+      </c>
+      <c r="CD137" s="15" t="n">
+        <v>3448.31</v>
       </c>
     </row>
     <row r="138">
@@ -25079,6 +25405,7 @@
       <c r="CA138" s="15" t="n"/>
       <c r="CB138" s="15" t="n"/>
       <c r="CC138" s="15" t="n"/>
+      <c r="CD138" s="15" t="n"/>
     </row>
     <row r="139">
       <c r="BE139" s="15" t="n">
@@ -25156,6 +25483,9 @@
       <c r="CC139" s="15" t="n">
         <v>5.7</v>
       </c>
+      <c r="CD139" s="15" t="n">
+        <v>5.41</v>
+      </c>
     </row>
     <row r="140">
       <c r="BE140" s="15" t="n">
@@ -25230,6 +25560,9 @@
       </c>
       <c r="CC140" s="15" t="n">
         <v>2561.58</v>
+      </c>
+      <c r="CD140" s="15" t="n">
+        <v>2480.67</v>
       </c>
     </row>
     <row r="141">
@@ -25258,6 +25591,7 @@
       <c r="CA141" s="15" t="n"/>
       <c r="CB141" s="15" t="n"/>
       <c r="CC141" s="15" t="n"/>
+      <c r="CD141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="BE142" s="15" t="n">
@@ -25335,6 +25669,9 @@
       <c r="CC142" s="15" t="n">
         <v>11.17</v>
       </c>
+      <c r="CD142" s="15" t="n">
+        <v>10.61</v>
+      </c>
     </row>
     <row r="143">
       <c r="BE143" s="15" t="n">
@@ -25411,6 +25748,9 @@
       </c>
       <c r="CC143" s="15" t="n">
         <v>5423.17</v>
+      </c>
+      <c r="CD143" s="15" t="n">
+        <v>5317.18</v>
       </c>
     </row>
     <row r="144">
@@ -25434,6 +25774,7 @@
       <c r="CA144" s="15" t="n"/>
       <c r="CB144" s="15" t="n"/>
       <c r="CC144" s="15" t="n"/>
+      <c r="CD144" s="15" t="n"/>
     </row>
     <row r="145">
       <c r="BJ145" s="15" t="n">
@@ -25496,6 +25837,9 @@
       <c r="CC145" s="15" t="n">
         <v>1.89</v>
       </c>
+      <c r="CD145" s="15" t="n">
+        <v>1.55</v>
+      </c>
     </row>
     <row r="146">
       <c r="BJ146" s="15" t="n">
@@ -25557,6 +25901,9 @@
       </c>
       <c r="CC146" s="15" t="n">
         <v>2172.18</v>
+      </c>
+      <c r="CD146" s="15" t="n">
+        <v>2172.48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-10-15 08:38:44]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CD146"/>
+  <dimension ref="A1:CE146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="51"/>
@@ -616,6 +616,7 @@
     <col width="15" customWidth="1" min="80" max="80"/>
     <col width="15" customWidth="1" min="81" max="81"/>
     <col width="15" customWidth="1" min="82" max="82"/>
+    <col width="15" customWidth="1" min="83" max="83"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -1029,6 +1030,11 @@
           <t>2026/10/12</t>
         </is>
       </c>
+      <c r="CE1" s="15" t="inlineStr">
+        <is>
+          <t>2026/10/15</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1441,6 +1447,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="CE2" s="16" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1689,6 +1700,9 @@
       <c r="CD3" s="15" t="n">
         <v>56.1</v>
       </c>
+      <c r="CE3" s="15" t="n">
+        <v>52.28</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1936,6 +1950,9 @@
       </c>
       <c r="CD4" s="15" t="n">
         <v>3797.24</v>
+      </c>
+      <c r="CE4" s="15" t="n">
+        <v>3707.48</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -2021,6 +2038,7 @@
       <c r="CB5" s="15" t="n"/>
       <c r="CC5" s="15" t="n"/>
       <c r="CD5" s="15" t="n"/>
+      <c r="CE5" s="15" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -2153,6 +2171,7 @@
       <c r="CB6" s="15" t="n"/>
       <c r="CC6" s="15" t="n"/>
       <c r="CD6" s="15" t="n"/>
+      <c r="CE6" s="15" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -2400,6 +2419,9 @@
       </c>
       <c r="CD7" s="15" t="n">
         <v>45.74</v>
+      </c>
+      <c r="CE7" s="15" t="n">
+        <v>43.95</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -2600,6 +2622,9 @@
       </c>
       <c r="CD8" s="15" t="n">
         <v>5235.37</v>
+      </c>
+      <c r="CE8" s="15" t="n">
+        <v>5057.08</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
@@ -2733,6 +2758,7 @@
       <c r="CB9" s="15" t="n"/>
       <c r="CC9" s="15" t="n"/>
       <c r="CD9" s="15" t="n"/>
+      <c r="CE9" s="15" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -2980,6 +3006,9 @@
       </c>
       <c r="CD10" s="15" t="n">
         <v>42.77</v>
+      </c>
+      <c r="CE10" s="15" t="n">
+        <v>41.38</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -3180,6 +3209,9 @@
       </c>
       <c r="CD11" s="15" t="n">
         <v>4287.98</v>
+      </c>
+      <c r="CE11" s="15" t="n">
+        <v>4166.01</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
@@ -3313,6 +3345,7 @@
       <c r="CB12" s="15" t="n"/>
       <c r="CC12" s="15" t="n"/>
       <c r="CD12" s="15" t="n"/>
+      <c r="CE12" s="15" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -3560,6 +3593,9 @@
       </c>
       <c r="CD13" s="15" t="n">
         <v>52.82</v>
+      </c>
+      <c r="CE13" s="15" t="n">
+        <v>47.77</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -3760,6 +3796,9 @@
       </c>
       <c r="CD14" s="15" t="n">
         <v>7093.02</v>
+      </c>
+      <c r="CE14" s="15" t="n">
+        <v>6769.25</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
@@ -3893,6 +3932,7 @@
       <c r="CB15" s="15" t="n"/>
       <c r="CC15" s="15" t="n"/>
       <c r="CD15" s="15" t="n"/>
+      <c r="CE15" s="15" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -4140,6 +4180,9 @@
       </c>
       <c r="CD16" s="15" t="n">
         <v>25.69</v>
+      </c>
+      <c r="CE16" s="15" t="n">
+        <v>24.99</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -4339,6 +4382,9 @@
         <v>2404.7</v>
       </c>
       <c r="CD17" s="15" t="n">
+        <v>2417.22</v>
+      </c>
+      <c r="CE17" s="15" t="n">
         <v>2417.22</v>
       </c>
     </row>
@@ -4473,6 +4519,7 @@
       <c r="CB18" s="15" t="n"/>
       <c r="CC18" s="15" t="n"/>
       <c r="CD18" s="15" t="n"/>
+      <c r="CE18" s="15" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -4720,6 +4767,9 @@
       </c>
       <c r="CD19" s="15" t="n">
         <v>79.77</v>
+      </c>
+      <c r="CE19" s="15" t="n">
+        <v>79.69</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -4920,6 +4970,9 @@
       </c>
       <c r="CD20" s="15" t="n">
         <v>7811.54</v>
+      </c>
+      <c r="CE20" s="15" t="n">
+        <v>7718.94</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
@@ -5053,6 +5106,7 @@
       <c r="CB21" s="15" t="n"/>
       <c r="CC21" s="15" t="n"/>
       <c r="CD21" s="15" t="n"/>
+      <c r="CE21" s="15" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -5297,6 +5351,9 @@
         <v>36.34</v>
       </c>
       <c r="CD22" s="15" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="CE22" s="15" t="n">
         <v>36.34</v>
       </c>
     </row>
@@ -5498,6 +5555,9 @@
       </c>
       <c r="CD23" s="15" t="n">
         <v>71924.67999999999</v>
+      </c>
+      <c r="CE23" s="15" t="n">
+        <v>74262.87</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
@@ -5631,6 +5691,7 @@
       <c r="CB24" s="15" t="n"/>
       <c r="CC24" s="15" t="n"/>
       <c r="CD24" s="15" t="n"/>
+      <c r="CE24" s="15" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -5877,6 +5938,9 @@
         <v>49.88</v>
       </c>
       <c r="CD25" s="15" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="CE25" s="15" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -6064,6 +6128,9 @@
       </c>
       <c r="CD26" s="15" t="n">
         <v>25257.04</v>
+      </c>
+      <c r="CE26" s="15" t="n">
+        <v>25216.44</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
@@ -6197,6 +6264,7 @@
       <c r="CB27" s="15" t="n"/>
       <c r="CC27" s="15" t="n"/>
       <c r="CD27" s="15" t="n"/>
+      <c r="CE27" s="15" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -6443,6 +6511,9 @@
         <v>92.09</v>
       </c>
       <c r="CD28" s="15" t="n">
+        <v>92.09</v>
+      </c>
+      <c r="CE28" s="15" t="n">
         <v>92.09</v>
       </c>
     </row>
@@ -6644,6 +6715,9 @@
       </c>
       <c r="CD29" s="15" t="n">
         <v>69030.92</v>
+      </c>
+      <c r="CE29" s="15" t="n">
+        <v>64425.95</v>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
@@ -6777,6 +6851,7 @@
       <c r="CB30" s="15" t="n"/>
       <c r="CC30" s="15" t="n"/>
       <c r="CD30" s="15" t="n"/>
+      <c r="CE30" s="15" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -7023,6 +7098,9 @@
         <v>97.44</v>
       </c>
       <c r="CD31" s="15" t="n">
+        <v>97.44</v>
+      </c>
+      <c r="CE31" s="15" t="n">
         <v>97.44</v>
       </c>
     </row>
@@ -7224,6 +7302,9 @@
       </c>
       <c r="CD32" s="15" t="n">
         <v>6384.24</v>
+      </c>
+      <c r="CE32" s="15" t="n">
+        <v>5554.22</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
@@ -7357,6 +7438,7 @@
       <c r="CB33" s="15" t="n"/>
       <c r="CC33" s="15" t="n"/>
       <c r="CD33" s="15" t="n"/>
+      <c r="CE33" s="15" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -7604,6 +7686,9 @@
       </c>
       <c r="CD34" s="15" t="n">
         <v>46.97</v>
+      </c>
+      <c r="CE34" s="15" t="n">
+        <v>47.89</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -7804,6 +7889,9 @@
       </c>
       <c r="CD35" s="15" t="n">
         <v>5618.87</v>
+      </c>
+      <c r="CE35" s="15" t="n">
+        <v>5535.58</v>
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
@@ -7937,6 +8025,7 @@
       <c r="CB36" s="15" t="n"/>
       <c r="CC36" s="15" t="n"/>
       <c r="CD36" s="15" t="n"/>
+      <c r="CE36" s="15" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -8184,6 +8273,9 @@
       </c>
       <c r="CD37" s="15" t="n">
         <v>55.85</v>
+      </c>
+      <c r="CE37" s="15" t="n">
+        <v>56.13</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -8384,6 +8476,9 @@
       </c>
       <c r="CD38" s="15" t="n">
         <v>11540.66</v>
+      </c>
+      <c r="CE38" s="15" t="n">
+        <v>11589.36</v>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
@@ -8517,6 +8612,7 @@
       <c r="CB39" s="15" t="n"/>
       <c r="CC39" s="15" t="n"/>
       <c r="CD39" s="15" t="n"/>
+      <c r="CE39" s="15" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -8764,6 +8860,9 @@
       </c>
       <c r="CD40" s="15" t="n">
         <v>52.31</v>
+      </c>
+      <c r="CE40" s="15" t="n">
+        <v>50.61</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -8964,6 +9063,9 @@
       </c>
       <c r="CD41" s="15" t="n">
         <v>11276.01</v>
+      </c>
+      <c r="CE41" s="15" t="n">
+        <v>11295.34</v>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
@@ -9097,6 +9199,7 @@
       <c r="CB42" s="15" t="n"/>
       <c r="CC42" s="15" t="n"/>
       <c r="CD42" s="15" t="n"/>
+      <c r="CE42" s="15" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -9344,6 +9447,9 @@
       </c>
       <c r="CD43" s="15" t="n">
         <v>49.72</v>
+      </c>
+      <c r="CE43" s="15" t="n">
+        <v>47.59</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -9544,6 +9650,9 @@
       </c>
       <c r="CD44" s="15" t="n">
         <v>3352.22</v>
+      </c>
+      <c r="CE44" s="15" t="n">
+        <v>3399.77</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
@@ -9677,6 +9786,7 @@
       <c r="CB45" s="15" t="n"/>
       <c r="CC45" s="15" t="n"/>
       <c r="CD45" s="15" t="n"/>
+      <c r="CE45" s="15" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -9924,6 +10034,9 @@
       </c>
       <c r="CD46" s="15" t="n">
         <v>62.93</v>
+      </c>
+      <c r="CE46" s="15" t="n">
+        <v>62.55</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -10124,6 +10237,9 @@
       </c>
       <c r="CD47" s="15" t="n">
         <v>7205.29</v>
+      </c>
+      <c r="CE47" s="15" t="n">
+        <v>7249.41</v>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
@@ -10257,6 +10373,7 @@
       <c r="CB48" s="15" t="n"/>
       <c r="CC48" s="15" t="n"/>
       <c r="CD48" s="15" t="n"/>
+      <c r="CE48" s="15" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -10504,6 +10621,9 @@
       </c>
       <c r="CD49" s="15" t="n">
         <v>19.77</v>
+      </c>
+      <c r="CE49" s="15" t="n">
+        <v>21.37</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -10704,6 +10824,9 @@
       </c>
       <c r="CD50" s="15" t="n">
         <v>31603.58</v>
+      </c>
+      <c r="CE50" s="15" t="n">
+        <v>32092.73</v>
       </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
@@ -10837,6 +10960,7 @@
       <c r="CB51" s="15" t="n"/>
       <c r="CC51" s="15" t="n"/>
       <c r="CD51" s="15" t="n"/>
+      <c r="CE51" s="15" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -11084,6 +11208,9 @@
       </c>
       <c r="CD52" s="15" t="n">
         <v>27.51</v>
+      </c>
+      <c r="CE52" s="15" t="n">
+        <v>24.38</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -11284,6 +11411,9 @@
       </c>
       <c r="CD53" s="15" t="n">
         <v>3057.91</v>
+      </c>
+      <c r="CE53" s="15" t="n">
+        <v>2866.7</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
@@ -11417,6 +11547,7 @@
       <c r="CB54" s="15" t="n"/>
       <c r="CC54" s="15" t="n"/>
       <c r="CD54" s="15" t="n"/>
+      <c r="CE54" s="15" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -11664,6 +11795,9 @@
       </c>
       <c r="CD55" s="15" t="n">
         <v>34.71</v>
+      </c>
+      <c r="CE55" s="15" t="n">
+        <v>30.5</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -11864,6 +11998,9 @@
       </c>
       <c r="CD56" s="15" t="n">
         <v>2963.82</v>
+      </c>
+      <c r="CE56" s="15" t="n">
+        <v>2783.17</v>
       </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
@@ -11997,6 +12134,7 @@
       <c r="CB57" s="15" t="n"/>
       <c r="CC57" s="15" t="n"/>
       <c r="CD57" s="15" t="n"/>
+      <c r="CE57" s="15" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -12244,6 +12382,9 @@
       </c>
       <c r="CD58" s="15" t="n">
         <v>15.95</v>
+      </c>
+      <c r="CE58" s="15" t="n">
+        <v>12.67</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -12444,6 +12585,9 @@
       </c>
       <c r="CD59" s="15" t="n">
         <v>6717.92</v>
+      </c>
+      <c r="CE59" s="15" t="n">
+        <v>6509.75</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
@@ -12577,6 +12721,7 @@
       <c r="CB60" s="15" t="n"/>
       <c r="CC60" s="15" t="n"/>
       <c r="CD60" s="15" t="n"/>
+      <c r="CE60" s="15" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -12824,6 +12969,9 @@
       </c>
       <c r="CD61" s="15" t="n">
         <v>34.12</v>
+      </c>
+      <c r="CE61" s="15" t="n">
+        <v>31.49</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -13024,6 +13172,9 @@
       </c>
       <c r="CD62" s="15" t="n">
         <v>8127.67</v>
+      </c>
+      <c r="CE62" s="15" t="n">
+        <v>8081.97</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
@@ -13157,6 +13308,7 @@
       <c r="CB63" s="15" t="n"/>
       <c r="CC63" s="15" t="n"/>
       <c r="CD63" s="15" t="n"/>
+      <c r="CE63" s="15" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -13404,6 +13556,9 @@
       </c>
       <c r="CD64" s="15" t="n">
         <v>7.3</v>
+      </c>
+      <c r="CE64" s="15" t="n">
+        <v>8.470000000000001</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -13604,6 +13759,9 @@
       </c>
       <c r="CD65" s="15" t="n">
         <v>10471.58</v>
+      </c>
+      <c r="CE65" s="15" t="n">
+        <v>10500.32</v>
       </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
@@ -13737,6 +13895,7 @@
       <c r="CB66" s="15" t="n"/>
       <c r="CC66" s="15" t="n"/>
       <c r="CD66" s="15" t="n"/>
+      <c r="CE66" s="15" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -13984,6 +14143,9 @@
       </c>
       <c r="CD67" s="15" t="n">
         <v>16.26</v>
+      </c>
+      <c r="CE67" s="15" t="n">
+        <v>14.76</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -14184,6 +14346,9 @@
       </c>
       <c r="CD68" s="15" t="n">
         <v>10962.63</v>
+      </c>
+      <c r="CE68" s="15" t="n">
+        <v>10639.68</v>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
@@ -14317,6 +14482,7 @@
       <c r="CB69" s="15" t="n"/>
       <c r="CC69" s="15" t="n"/>
       <c r="CD69" s="15" t="n"/>
+      <c r="CE69" s="15" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -14564,6 +14730,9 @@
       </c>
       <c r="CD70" s="15" t="n">
         <v>15.57</v>
+      </c>
+      <c r="CE70" s="15" t="n">
+        <v>16.89</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -14764,6 +14933,9 @@
       </c>
       <c r="CD71" s="15" t="n">
         <v>6260.98</v>
+      </c>
+      <c r="CE71" s="15" t="n">
+        <v>6264.52</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
@@ -14897,6 +15069,7 @@
       <c r="CB72" s="15" t="n"/>
       <c r="CC72" s="15" t="n"/>
       <c r="CD72" s="15" t="n"/>
+      <c r="CE72" s="15" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -15144,6 +15317,9 @@
       </c>
       <c r="CD73" s="15" t="n">
         <v>18.7</v>
+      </c>
+      <c r="CE73" s="15" t="n">
+        <v>18.8</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -15344,6 +15520,9 @@
       </c>
       <c r="CD74" s="15" t="n">
         <v>12469.15</v>
+      </c>
+      <c r="CE74" s="15" t="n">
+        <v>12310.32</v>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
@@ -15477,6 +15656,7 @@
       <c r="CB75" s="15" t="n"/>
       <c r="CC75" s="15" t="n"/>
       <c r="CD75" s="15" t="n"/>
+      <c r="CE75" s="15" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -15724,6 +15904,9 @@
       </c>
       <c r="CD76" s="15" t="n">
         <v>52.26</v>
+      </c>
+      <c r="CE76" s="15" t="n">
+        <v>51.21</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -15924,6 +16107,9 @@
       </c>
       <c r="CD77" s="15" t="n">
         <v>15594.78</v>
+      </c>
+      <c r="CE77" s="15" t="n">
+        <v>15569.82</v>
       </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
@@ -16057,6 +16243,7 @@
       <c r="CB78" s="15" t="n"/>
       <c r="CC78" s="15" t="n"/>
       <c r="CD78" s="15" t="n"/>
+      <c r="CE78" s="15" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -16304,6 +16491,9 @@
       </c>
       <c r="CD79" s="15" t="n">
         <v>2.12</v>
+      </c>
+      <c r="CE79" s="15" t="n">
+        <v>2.51</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -16504,6 +16694,9 @@
       </c>
       <c r="CD80" s="15" t="n">
         <v>6277.54</v>
+      </c>
+      <c r="CE80" s="15" t="n">
+        <v>6420.75</v>
       </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
@@ -16637,6 +16830,7 @@
       <c r="CB81" s="15" t="n"/>
       <c r="CC81" s="15" t="n"/>
       <c r="CD81" s="15" t="n"/>
+      <c r="CE81" s="15" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -16884,6 +17078,9 @@
       </c>
       <c r="CD82" s="15" t="n">
         <v>5.02</v>
+      </c>
+      <c r="CE82" s="15" t="n">
+        <v>5.58</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -17084,6 +17281,9 @@
       </c>
       <c r="CD83" s="15" t="n">
         <v>8452.77</v>
+      </c>
+      <c r="CE83" s="15" t="n">
+        <v>8455.75</v>
       </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
@@ -17217,6 +17417,7 @@
       <c r="CB84" s="15" t="n"/>
       <c r="CC84" s="15" t="n"/>
       <c r="CD84" s="15" t="n"/>
+      <c r="CE84" s="15" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -17464,6 +17665,9 @@
       </c>
       <c r="CD85" s="15" t="n">
         <v>15.86</v>
+      </c>
+      <c r="CE85" s="15" t="n">
+        <v>16.14</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -17663,6 +17867,9 @@
         <v>2631.9</v>
       </c>
       <c r="CD86" s="15" t="n">
+        <v>2631.9</v>
+      </c>
+      <c r="CE86" s="15" t="n">
         <v>2631.9</v>
       </c>
     </row>
@@ -17797,6 +18004,7 @@
       <c r="CB87" s="15" t="n"/>
       <c r="CC87" s="15" t="n"/>
       <c r="CD87" s="15" t="n"/>
+      <c r="CE87" s="15" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -18044,6 +18252,9 @@
       </c>
       <c r="CD88" s="15" t="n">
         <v>23.15</v>
+      </c>
+      <c r="CE88" s="15" t="n">
+        <v>23.03</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -18244,6 +18455,9 @@
       </c>
       <c r="CD89" s="15" t="n">
         <v>4169.57</v>
+      </c>
+      <c r="CE89" s="15" t="n">
+        <v>4060.99</v>
       </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
@@ -18377,6 +18591,7 @@
       <c r="CB90" s="15" t="n"/>
       <c r="CC90" s="15" t="n"/>
       <c r="CD90" s="15" t="n"/>
+      <c r="CE90" s="15" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -18624,6 +18839,9 @@
       </c>
       <c r="CD91" s="15" t="n">
         <v>15.91</v>
+      </c>
+      <c r="CE91" s="15" t="n">
+        <v>12.42</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -18824,6 +19042,9 @@
       </c>
       <c r="CD92" s="15" t="n">
         <v>8436.219999999999</v>
+      </c>
+      <c r="CE92" s="15" t="n">
+        <v>8280.559999999999</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
@@ -18957,6 +19178,7 @@
       <c r="CB93" s="15" t="n"/>
       <c r="CC93" s="15" t="n"/>
       <c r="CD93" s="15" t="n"/>
+      <c r="CE93" s="15" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -19204,6 +19426,9 @@
       </c>
       <c r="CD94" s="15" t="n">
         <v>3.65</v>
+      </c>
+      <c r="CE94" s="15" t="n">
+        <v>2.98</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -19404,6 +19629,9 @@
       </c>
       <c r="CD95" s="15" t="n">
         <v>1175.05</v>
+      </c>
+      <c r="CE95" s="15" t="n">
+        <v>1123.24</v>
       </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
@@ -19537,6 +19765,7 @@
       <c r="CB96" s="15" t="n"/>
       <c r="CC96" s="15" t="n"/>
       <c r="CD96" s="15" t="n"/>
+      <c r="CE96" s="15" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -19784,6 +20013,9 @@
       </c>
       <c r="CD97" s="15" t="n">
         <v>9.16</v>
+      </c>
+      <c r="CE97" s="15" t="n">
+        <v>9.52</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -19984,6 +20216,9 @@
       </c>
       <c r="CD98" s="15" t="n">
         <v>13792.85</v>
+      </c>
+      <c r="CE98" s="15" t="n">
+        <v>13749.28</v>
       </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
@@ -20117,6 +20352,7 @@
       <c r="CB99" s="15" t="n"/>
       <c r="CC99" s="15" t="n"/>
       <c r="CD99" s="15" t="n"/>
+      <c r="CE99" s="15" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -20364,6 +20600,9 @@
       </c>
       <c r="CD100" s="15" t="n">
         <v>33.47</v>
+      </c>
+      <c r="CE100" s="15" t="n">
+        <v>28.39</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -20564,6 +20803,9 @@
       </c>
       <c r="CD101" s="15" t="n">
         <v>3225.74</v>
+      </c>
+      <c r="CE101" s="15" t="n">
+        <v>3128.43</v>
       </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
@@ -20697,6 +20939,7 @@
       <c r="CB102" s="15" t="n"/>
       <c r="CC102" s="15" t="n"/>
       <c r="CD102" s="15" t="n"/>
+      <c r="CE102" s="15" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -20944,6 +21187,9 @@
       </c>
       <c r="CD103" s="15" t="n">
         <v>24.85</v>
+      </c>
+      <c r="CE103" s="15" t="n">
+        <v>19.2</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -21144,6 +21390,9 @@
       </c>
       <c r="CD104" s="15" t="n">
         <v>2153.8</v>
+      </c>
+      <c r="CE104" s="15" t="n">
+        <v>2007.76</v>
       </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
@@ -21277,6 +21526,7 @@
       <c r="CB105" s="15" t="n"/>
       <c r="CC105" s="15" t="n"/>
       <c r="CD105" s="15" t="n"/>
+      <c r="CE105" s="15" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -21524,6 +21774,9 @@
       </c>
       <c r="CD106" s="15" t="n">
         <v>10.33</v>
+      </c>
+      <c r="CE106" s="15" t="n">
+        <v>7.19</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -21724,6 +21977,9 @@
       </c>
       <c r="CD107" s="15" t="n">
         <v>2235.18</v>
+      </c>
+      <c r="CE107" s="15" t="n">
+        <v>2101.93</v>
       </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
@@ -21857,6 +22113,7 @@
       <c r="CB108" s="15" t="n"/>
       <c r="CC108" s="15" t="n"/>
       <c r="CD108" s="15" t="n"/>
+      <c r="CE108" s="15" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -22104,6 +22361,9 @@
       </c>
       <c r="CD109" s="15" t="n">
         <v>26.62</v>
+      </c>
+      <c r="CE109" s="15" t="n">
+        <v>21.33</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -22303,6 +22563,9 @@
         <v>2304.77</v>
       </c>
       <c r="CD110" s="15" t="n">
+        <v>2341.61</v>
+      </c>
+      <c r="CE110" s="15" t="n">
         <v>2341.61</v>
       </c>
     </row>
@@ -22437,6 +22700,7 @@
       <c r="CB111" s="15" t="n"/>
       <c r="CC111" s="15" t="n"/>
       <c r="CD111" s="15" t="n"/>
+      <c r="CE111" s="15" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -22684,6 +22948,9 @@
       </c>
       <c r="CD112" s="15" t="n">
         <v>46.91</v>
+      </c>
+      <c r="CE112" s="15" t="n">
+        <v>39.66</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -22882,6 +23149,9 @@
       </c>
       <c r="CD113" s="15" t="n">
         <v>1870.76</v>
+      </c>
+      <c r="CE113" s="15" t="n">
+        <v>1816.17</v>
       </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
@@ -23015,6 +23285,7 @@
       <c r="CB114" s="15" t="n"/>
       <c r="CC114" s="15" t="n"/>
       <c r="CD114" s="15" t="n"/>
+      <c r="CE114" s="15" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -23262,6 +23533,9 @@
       </c>
       <c r="CD115" s="15" t="n">
         <v>17.93</v>
+      </c>
+      <c r="CE115" s="15" t="n">
+        <v>16.12</v>
       </c>
     </row>
     <row r="116" ht="14.25" customHeight="1">
@@ -23447,6 +23721,9 @@
       </c>
       <c r="CD116" s="15" t="n">
         <v>8718.799999999999</v>
+      </c>
+      <c r="CE116" s="15" t="n">
+        <v>8773.190000000001</v>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1">
@@ -23535,6 +23812,7 @@
       <c r="CB117" s="15" t="n"/>
       <c r="CC117" s="15" t="n"/>
       <c r="CD117" s="15" t="n"/>
+      <c r="CE117" s="15" t="n"/>
     </row>
     <row r="118" ht="14.25" customHeight="1">
       <c r="P118" s="13" t="n">
@@ -23738,6 +24016,9 @@
       <c r="CD118" s="15" t="n">
         <v>65.69</v>
       </c>
+      <c r="CE118" s="15" t="n">
+        <v>61.04</v>
+      </c>
     </row>
     <row r="119" ht="14.25" customHeight="1">
       <c r="Y119" s="13" t="n">
@@ -23913,6 +24194,9 @@
       </c>
       <c r="CD119" s="15" t="n">
         <v>11209.46</v>
+      </c>
+      <c r="CE119" s="15" t="n">
+        <v>10590.92</v>
       </c>
     </row>
     <row r="120" ht="14.25" customHeight="1">
@@ -23950,6 +24234,7 @@
       <c r="CB120" s="15" t="n"/>
       <c r="CC120" s="15" t="n"/>
       <c r="CD120" s="15" t="n"/>
+      <c r="CE120" s="15" t="n"/>
     </row>
     <row r="121" ht="14.25" customHeight="1">
       <c r="AW121" s="13" t="n">
@@ -24054,6 +24339,9 @@
       <c r="CD121" s="15" t="n">
         <v>24.77</v>
       </c>
+      <c r="CE121" s="15" t="n">
+        <v>27.71</v>
+      </c>
     </row>
     <row r="122" ht="14.25" customHeight="1">
       <c r="AW122" s="13" t="n">
@@ -24157,6 +24445,9 @@
       </c>
       <c r="CD122" s="15" t="n">
         <v>1200.52</v>
+      </c>
+      <c r="CE122" s="15" t="n">
+        <v>1211.93</v>
       </c>
     </row>
     <row r="123" ht="14.25" customHeight="1">
@@ -24194,6 +24485,7 @@
       <c r="CB123" s="15" t="n"/>
       <c r="CC123" s="15" t="n"/>
       <c r="CD123" s="15" t="n"/>
+      <c r="CE123" s="15" t="n"/>
     </row>
     <row r="124" ht="14.25" customHeight="1">
       <c r="AW124" s="13" t="n">
@@ -24298,6 +24590,9 @@
       <c r="CD124" s="15" t="n">
         <v>36.72</v>
       </c>
+      <c r="CE124" s="15" t="n">
+        <v>37.48</v>
+      </c>
     </row>
     <row r="125" ht="14.25" customHeight="1">
       <c r="AW125" s="13" t="n">
@@ -24401,6 +24696,9 @@
       </c>
       <c r="CD125" s="15" t="n">
         <v>10698.19</v>
+      </c>
+      <c r="CE125" s="15" t="n">
+        <v>10429.97</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1">
@@ -24438,6 +24736,7 @@
       <c r="CB126" s="15" t="n"/>
       <c r="CC126" s="15" t="n"/>
       <c r="CD126" s="15" t="n"/>
+      <c r="CE126" s="15" t="n"/>
     </row>
     <row r="127" ht="14.25" customHeight="1">
       <c r="AW127" s="13" t="n">
@@ -24542,6 +24841,9 @@
       <c r="CD127" s="15" t="n">
         <v>4.15</v>
       </c>
+      <c r="CE127" s="15" t="n">
+        <v>3.49</v>
+      </c>
     </row>
     <row r="128" ht="14.25" customHeight="1">
       <c r="AW128" s="13" t="n">
@@ -24645,6 +24947,9 @@
       </c>
       <c r="CD128" s="15" t="n">
         <v>1838.45</v>
+      </c>
+      <c r="CE128" s="15" t="n">
+        <v>1767.42</v>
       </c>
     </row>
     <row r="129" ht="14.25" customHeight="1">
@@ -24682,6 +24987,7 @@
       <c r="CB129" s="15" t="n"/>
       <c r="CC129" s="15" t="n"/>
       <c r="CD129" s="15" t="n"/>
+      <c r="CE129" s="15" t="n"/>
     </row>
     <row r="130" ht="14.25" customHeight="1">
       <c r="AW130" s="13" t="n">
@@ -24786,6 +25092,9 @@
       <c r="CD130" s="15" t="n">
         <v>5.2</v>
       </c>
+      <c r="CE130" s="15" t="n">
+        <v>6.29</v>
+      </c>
     </row>
     <row r="131" ht="14.25" customHeight="1">
       <c r="AW131" s="13" t="n">
@@ -24889,6 +25198,9 @@
       </c>
       <c r="CD131" s="15" t="n">
         <v>721.09</v>
+      </c>
+      <c r="CE131" s="15" t="n">
+        <v>721.53</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1">
@@ -24926,6 +25238,7 @@
       <c r="CB132" s="15" t="n"/>
       <c r="CC132" s="15" t="n"/>
       <c r="CD132" s="15" t="n"/>
+      <c r="CE132" s="15" t="n"/>
     </row>
     <row r="133" ht="14.25" customHeight="1">
       <c r="AW133" s="13" t="n">
@@ -25030,6 +25343,9 @@
       <c r="CD133" s="15" t="n">
         <v>47.64</v>
       </c>
+      <c r="CE133" s="15" t="n">
+        <v>42.44</v>
+      </c>
     </row>
     <row r="134" ht="14.25" customHeight="1">
       <c r="AW134" s="13" t="n">
@@ -25133,6 +25449,9 @@
       </c>
       <c r="CD134" s="15" t="n">
         <v>2641.45</v>
+      </c>
+      <c r="CE134" s="15" t="n">
+        <v>2506.83</v>
       </c>
     </row>
     <row r="135" ht="14.25" customHeight="1">
@@ -25170,6 +25489,7 @@
       <c r="CB135" s="15" t="n"/>
       <c r="CC135" s="15" t="n"/>
       <c r="CD135" s="15" t="n"/>
+      <c r="CE135" s="15" t="n"/>
     </row>
     <row r="136" ht="14.25" customHeight="1">
       <c r="AW136" s="13" t="n">
@@ -25274,6 +25594,9 @@
       <c r="CD136" s="15" t="n">
         <v>21.18</v>
       </c>
+      <c r="CE136" s="15" t="n">
+        <v>21.17</v>
+      </c>
     </row>
     <row r="137" ht="14.25" customHeight="1">
       <c r="AW137" s="13" t="n">
@@ -25377,6 +25700,9 @@
       </c>
       <c r="CD137" s="15" t="n">
         <v>3448.31</v>
+      </c>
+      <c r="CE137" s="15" t="n">
+        <v>3336.46</v>
       </c>
     </row>
     <row r="138">
@@ -25406,6 +25732,7 @@
       <c r="CB138" s="15" t="n"/>
       <c r="CC138" s="15" t="n"/>
       <c r="CD138" s="15" t="n"/>
+      <c r="CE138" s="15" t="n"/>
     </row>
     <row r="139">
       <c r="BE139" s="15" t="n">
@@ -25486,6 +25813,9 @@
       <c r="CD139" s="15" t="n">
         <v>5.41</v>
       </c>
+      <c r="CE139" s="15" t="n">
+        <v>4.55</v>
+      </c>
     </row>
     <row r="140">
       <c r="BE140" s="15" t="n">
@@ -25563,6 +25893,9 @@
       </c>
       <c r="CD140" s="15" t="n">
         <v>2480.67</v>
+      </c>
+      <c r="CE140" s="15" t="n">
+        <v>2343.25</v>
       </c>
     </row>
     <row r="141">
@@ -25592,6 +25925,7 @@
       <c r="CB141" s="15" t="n"/>
       <c r="CC141" s="15" t="n"/>
       <c r="CD141" s="15" t="n"/>
+      <c r="CE141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="BE142" s="15" t="n">
@@ -25672,6 +26006,9 @@
       <c r="CD142" s="15" t="n">
         <v>10.61</v>
       </c>
+      <c r="CE142" s="15" t="n">
+        <v>15.38</v>
+      </c>
     </row>
     <row r="143">
       <c r="BE143" s="15" t="n">
@@ -25751,6 +26088,9 @@
       </c>
       <c r="CD143" s="15" t="n">
         <v>5317.18</v>
+      </c>
+      <c r="CE143" s="15" t="n">
+        <v>5386.01</v>
       </c>
     </row>
     <row r="144">
@@ -25775,6 +26115,7 @@
       <c r="CB144" s="15" t="n"/>
       <c r="CC144" s="15" t="n"/>
       <c r="CD144" s="15" t="n"/>
+      <c r="CE144" s="15" t="n"/>
     </row>
     <row r="145">
       <c r="BJ145" s="15" t="n">
@@ -25840,6 +26181,9 @@
       <c r="CD145" s="15" t="n">
         <v>1.55</v>
       </c>
+      <c r="CE145" s="15" t="n">
+        <v>1.31</v>
+      </c>
     </row>
     <row r="146">
       <c r="BJ146" s="15" t="n">
@@ -25904,6 +26248,9 @@
       </c>
       <c r="CD146" s="15" t="n">
         <v>2172.48</v>
+      </c>
+      <c r="CE146" s="15" t="n">
+        <v>2174.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-10-19 09:19:11]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CE146"/>
+  <dimension ref="A1:CF146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="51"/>
@@ -617,6 +617,7 @@
     <col width="15" customWidth="1" min="81" max="81"/>
     <col width="15" customWidth="1" min="82" max="82"/>
     <col width="15" customWidth="1" min="83" max="83"/>
+    <col width="15" customWidth="1" min="84" max="84"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -1035,6 +1036,11 @@
           <t>2026/10/15</t>
         </is>
       </c>
+      <c r="CF1" s="15" t="inlineStr">
+        <is>
+          <t>2026/10/19</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1452,6 +1458,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="CF2" s="16" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1703,6 +1714,9 @@
       <c r="CE3" s="15" t="n">
         <v>52.28</v>
       </c>
+      <c r="CF3" s="15" t="n">
+        <v>48.84</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1953,6 +1967,9 @@
       </c>
       <c r="CE4" s="15" t="n">
         <v>3707.48</v>
+      </c>
+      <c r="CF4" s="15" t="n">
+        <v>3730.92</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -2039,6 +2056,7 @@
       <c r="CC5" s="15" t="n"/>
       <c r="CD5" s="15" t="n"/>
       <c r="CE5" s="15" t="n"/>
+      <c r="CF5" s="15" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -2172,6 +2190,7 @@
       <c r="CC6" s="15" t="n"/>
       <c r="CD6" s="15" t="n"/>
       <c r="CE6" s="15" t="n"/>
+      <c r="CF6" s="15" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -2422,6 +2441,9 @@
       </c>
       <c r="CE7" s="15" t="n">
         <v>43.95</v>
+      </c>
+      <c r="CF7" s="15" t="n">
+        <v>42.08</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -2625,6 +2647,9 @@
       </c>
       <c r="CE8" s="15" t="n">
         <v>5057.08</v>
+      </c>
+      <c r="CF8" s="15" t="n">
+        <v>5070.19</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
@@ -2759,6 +2784,7 @@
       <c r="CC9" s="15" t="n"/>
       <c r="CD9" s="15" t="n"/>
       <c r="CE9" s="15" t="n"/>
+      <c r="CF9" s="15" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -3009,6 +3035,9 @@
       </c>
       <c r="CE10" s="15" t="n">
         <v>41.38</v>
+      </c>
+      <c r="CF10" s="15" t="n">
+        <v>39.73</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -3212,6 +3241,9 @@
       </c>
       <c r="CE11" s="15" t="n">
         <v>4166.01</v>
+      </c>
+      <c r="CF11" s="15" t="n">
+        <v>4174.53</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
@@ -3346,6 +3378,7 @@
       <c r="CC12" s="15" t="n"/>
       <c r="CD12" s="15" t="n"/>
       <c r="CE12" s="15" t="n"/>
+      <c r="CF12" s="15" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -3596,6 +3629,9 @@
       </c>
       <c r="CE13" s="15" t="n">
         <v>47.77</v>
+      </c>
+      <c r="CF13" s="15" t="n">
+        <v>44.05</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -3799,6 +3835,9 @@
       </c>
       <c r="CE14" s="15" t="n">
         <v>6769.25</v>
+      </c>
+      <c r="CF14" s="15" t="n">
+        <v>6800.66</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
@@ -3933,6 +3972,7 @@
       <c r="CC15" s="15" t="n"/>
       <c r="CD15" s="15" t="n"/>
       <c r="CE15" s="15" t="n"/>
+      <c r="CF15" s="15" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -4183,6 +4223,9 @@
       </c>
       <c r="CE16" s="15" t="n">
         <v>24.99</v>
+      </c>
+      <c r="CF16" s="15" t="n">
+        <v>24.23</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -4386,6 +4429,9 @@
       </c>
       <c r="CE17" s="15" t="n">
         <v>2417.22</v>
+      </c>
+      <c r="CF17" s="15" t="n">
+        <v>2372.31</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
@@ -4520,6 +4566,7 @@
       <c r="CC18" s="15" t="n"/>
       <c r="CD18" s="15" t="n"/>
       <c r="CE18" s="15" t="n"/>
+      <c r="CF18" s="15" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -4770,6 +4817,9 @@
       </c>
       <c r="CE19" s="15" t="n">
         <v>79.69</v>
+      </c>
+      <c r="CF19" s="15" t="n">
+        <v>78.52</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -4973,6 +5023,9 @@
       </c>
       <c r="CE20" s="15" t="n">
         <v>7718.94</v>
+      </c>
+      <c r="CF20" s="15" t="n">
+        <v>7659.44</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
@@ -5107,6 +5160,7 @@
       <c r="CC21" s="15" t="n"/>
       <c r="CD21" s="15" t="n"/>
       <c r="CE21" s="15" t="n"/>
+      <c r="CF21" s="15" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -5354,6 +5408,9 @@
         <v>36.34</v>
       </c>
       <c r="CE22" s="15" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="CF22" s="15" t="n">
         <v>36.34</v>
       </c>
     </row>
@@ -5558,6 +5615,9 @@
       </c>
       <c r="CE23" s="15" t="n">
         <v>74262.87</v>
+      </c>
+      <c r="CF23" s="15" t="n">
+        <v>73736.45</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
@@ -5692,6 +5752,7 @@
       <c r="CC24" s="15" t="n"/>
       <c r="CD24" s="15" t="n"/>
       <c r="CE24" s="15" t="n"/>
+      <c r="CF24" s="15" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -5941,6 +6002,9 @@
         <v>49.88</v>
       </c>
       <c r="CE25" s="15" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="CF25" s="15" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -6131,6 +6195,9 @@
       </c>
       <c r="CE26" s="15" t="n">
         <v>25216.44</v>
+      </c>
+      <c r="CF26" s="15" t="n">
+        <v>25329.55</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
@@ -6265,6 +6332,7 @@
       <c r="CC27" s="15" t="n"/>
       <c r="CD27" s="15" t="n"/>
       <c r="CE27" s="15" t="n"/>
+      <c r="CF27" s="15" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -6514,6 +6582,9 @@
         <v>92.09</v>
       </c>
       <c r="CE28" s="15" t="n">
+        <v>92.09</v>
+      </c>
+      <c r="CF28" s="15" t="n">
         <v>92.09</v>
       </c>
     </row>
@@ -6718,6 +6789,9 @@
       </c>
       <c r="CE29" s="15" t="n">
         <v>64425.95</v>
+      </c>
+      <c r="CF29" s="15" t="n">
+        <v>64916.7</v>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
@@ -6852,6 +6926,7 @@
       <c r="CC30" s="15" t="n"/>
       <c r="CD30" s="15" t="n"/>
       <c r="CE30" s="15" t="n"/>
+      <c r="CF30" s="15" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -7101,6 +7176,9 @@
         <v>97.44</v>
       </c>
       <c r="CE31" s="15" t="n">
+        <v>97.44</v>
+      </c>
+      <c r="CF31" s="15" t="n">
         <v>97.44</v>
       </c>
     </row>
@@ -7305,6 +7383,9 @@
       </c>
       <c r="CE32" s="15" t="n">
         <v>5554.22</v>
+      </c>
+      <c r="CF32" s="15" t="n">
+        <v>5768.01</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
@@ -7439,6 +7520,7 @@
       <c r="CC33" s="15" t="n"/>
       <c r="CD33" s="15" t="n"/>
       <c r="CE33" s="15" t="n"/>
+      <c r="CF33" s="15" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -7689,6 +7771,9 @@
       </c>
       <c r="CE34" s="15" t="n">
         <v>47.89</v>
+      </c>
+      <c r="CF34" s="15" t="n">
+        <v>49.93</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -7892,6 +7977,9 @@
       </c>
       <c r="CE35" s="15" t="n">
         <v>5535.58</v>
+      </c>
+      <c r="CF35" s="15" t="n">
+        <v>5623.37</v>
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
@@ -8026,6 +8114,7 @@
       <c r="CC36" s="15" t="n"/>
       <c r="CD36" s="15" t="n"/>
       <c r="CE36" s="15" t="n"/>
+      <c r="CF36" s="15" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -8276,6 +8365,9 @@
       </c>
       <c r="CE37" s="15" t="n">
         <v>56.13</v>
+      </c>
+      <c r="CF37" s="15" t="n">
+        <v>55.89</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -8479,6 +8571,9 @@
       </c>
       <c r="CE38" s="15" t="n">
         <v>11589.36</v>
+      </c>
+      <c r="CF38" s="15" t="n">
+        <v>11605.41</v>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
@@ -8613,6 +8708,7 @@
       <c r="CC39" s="15" t="n"/>
       <c r="CD39" s="15" t="n"/>
       <c r="CE39" s="15" t="n"/>
+      <c r="CF39" s="15" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -8863,6 +8959,9 @@
       </c>
       <c r="CE40" s="15" t="n">
         <v>50.61</v>
+      </c>
+      <c r="CF40" s="15" t="n">
+        <v>52.9</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -9066,6 +9165,9 @@
       </c>
       <c r="CE41" s="15" t="n">
         <v>11295.34</v>
+      </c>
+      <c r="CF41" s="15" t="n">
+        <v>11191.38</v>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
@@ -9200,6 +9302,7 @@
       <c r="CC42" s="15" t="n"/>
       <c r="CD42" s="15" t="n"/>
       <c r="CE42" s="15" t="n"/>
+      <c r="CF42" s="15" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -9450,6 +9553,9 @@
       </c>
       <c r="CE43" s="15" t="n">
         <v>47.59</v>
+      </c>
+      <c r="CF43" s="15" t="n">
+        <v>52.02</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -9653,6 +9759,9 @@
       </c>
       <c r="CE44" s="15" t="n">
         <v>3399.77</v>
+      </c>
+      <c r="CF44" s="15" t="n">
+        <v>3337.49</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
@@ -9787,6 +9896,7 @@
       <c r="CC45" s="15" t="n"/>
       <c r="CD45" s="15" t="n"/>
       <c r="CE45" s="15" t="n"/>
+      <c r="CF45" s="15" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -10037,6 +10147,9 @@
       </c>
       <c r="CE46" s="15" t="n">
         <v>62.55</v>
+      </c>
+      <c r="CF46" s="15" t="n">
+        <v>62.33</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -10240,6 +10353,9 @@
       </c>
       <c r="CE47" s="15" t="n">
         <v>7249.41</v>
+      </c>
+      <c r="CF47" s="15" t="n">
+        <v>7229.66</v>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
@@ -10374,6 +10490,7 @@
       <c r="CC48" s="15" t="n"/>
       <c r="CD48" s="15" t="n"/>
       <c r="CE48" s="15" t="n"/>
+      <c r="CF48" s="15" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -10624,6 +10741,9 @@
       </c>
       <c r="CE49" s="15" t="n">
         <v>21.37</v>
+      </c>
+      <c r="CF49" s="15" t="n">
+        <v>15.87</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -10827,6 +10947,9 @@
       </c>
       <c r="CE50" s="15" t="n">
         <v>32092.73</v>
+      </c>
+      <c r="CF50" s="15" t="n">
+        <v>31175.73</v>
       </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
@@ -10961,6 +11084,7 @@
       <c r="CC51" s="15" t="n"/>
       <c r="CD51" s="15" t="n"/>
       <c r="CE51" s="15" t="n"/>
+      <c r="CF51" s="15" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -11211,6 +11335,9 @@
       </c>
       <c r="CE52" s="15" t="n">
         <v>24.38</v>
+      </c>
+      <c r="CF52" s="15" t="n">
+        <v>22.83</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -11414,6 +11541,9 @@
       </c>
       <c r="CE53" s="15" t="n">
         <v>2866.7</v>
+      </c>
+      <c r="CF53" s="15" t="n">
+        <v>2825.99</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
@@ -11548,6 +11678,7 @@
       <c r="CC54" s="15" t="n"/>
       <c r="CD54" s="15" t="n"/>
       <c r="CE54" s="15" t="n"/>
+      <c r="CF54" s="15" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -11798,6 +11929,9 @@
       </c>
       <c r="CE55" s="15" t="n">
         <v>30.5</v>
+      </c>
+      <c r="CF55" s="15" t="n">
+        <v>27.31</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -12001,6 +12135,9 @@
       </c>
       <c r="CE56" s="15" t="n">
         <v>2783.17</v>
+      </c>
+      <c r="CF56" s="15" t="n">
+        <v>2746.29</v>
       </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
@@ -12135,6 +12272,7 @@
       <c r="CC57" s="15" t="n"/>
       <c r="CD57" s="15" t="n"/>
       <c r="CE57" s="15" t="n"/>
+      <c r="CF57" s="15" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -12385,6 +12523,9 @@
       </c>
       <c r="CE58" s="15" t="n">
         <v>12.67</v>
+      </c>
+      <c r="CF58" s="15" t="n">
+        <v>8.5</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -12588,6 +12729,9 @@
       </c>
       <c r="CE59" s="15" t="n">
         <v>6509.75</v>
+      </c>
+      <c r="CF59" s="15" t="n">
+        <v>6436.71</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
@@ -12722,6 +12866,7 @@
       <c r="CC60" s="15" t="n"/>
       <c r="CD60" s="15" t="n"/>
       <c r="CE60" s="15" t="n"/>
+      <c r="CF60" s="15" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -12972,6 +13117,9 @@
       </c>
       <c r="CE61" s="15" t="n">
         <v>31.49</v>
+      </c>
+      <c r="CF61" s="15" t="n">
+        <v>30.42</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -13175,6 +13323,9 @@
       </c>
       <c r="CE62" s="15" t="n">
         <v>8081.97</v>
+      </c>
+      <c r="CF62" s="15" t="n">
+        <v>7983.99</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
@@ -13309,6 +13460,7 @@
       <c r="CC63" s="15" t="n"/>
       <c r="CD63" s="15" t="n"/>
       <c r="CE63" s="15" t="n"/>
+      <c r="CF63" s="15" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -13559,6 +13711,9 @@
       </c>
       <c r="CE64" s="15" t="n">
         <v>8.470000000000001</v>
+      </c>
+      <c r="CF64" s="15" t="n">
+        <v>10.03</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -13762,6 +13917,9 @@
       </c>
       <c r="CE65" s="15" t="n">
         <v>10500.32</v>
+      </c>
+      <c r="CF65" s="15" t="n">
+        <v>10577.64</v>
       </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
@@ -13896,6 +14054,7 @@
       <c r="CC66" s="15" t="n"/>
       <c r="CD66" s="15" t="n"/>
       <c r="CE66" s="15" t="n"/>
+      <c r="CF66" s="15" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -14146,6 +14305,9 @@
       </c>
       <c r="CE67" s="15" t="n">
         <v>14.76</v>
+      </c>
+      <c r="CF67" s="15" t="n">
+        <v>13.16</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -14349,6 +14511,9 @@
       </c>
       <c r="CE68" s="15" t="n">
         <v>10639.68</v>
+      </c>
+      <c r="CF68" s="15" t="n">
+        <v>10832.7</v>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
@@ -14483,6 +14648,7 @@
       <c r="CC69" s="15" t="n"/>
       <c r="CD69" s="15" t="n"/>
       <c r="CE69" s="15" t="n"/>
+      <c r="CF69" s="15" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -14733,6 +14899,9 @@
       </c>
       <c r="CE70" s="15" t="n">
         <v>16.89</v>
+      </c>
+      <c r="CF70" s="15" t="n">
+        <v>20.52</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -14936,6 +15105,9 @@
       </c>
       <c r="CE71" s="15" t="n">
         <v>6264.52</v>
+      </c>
+      <c r="CF71" s="15" t="n">
+        <v>6399.37</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
@@ -15070,6 +15242,7 @@
       <c r="CC72" s="15" t="n"/>
       <c r="CD72" s="15" t="n"/>
       <c r="CE72" s="15" t="n"/>
+      <c r="CF72" s="15" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -15320,6 +15493,9 @@
       </c>
       <c r="CE73" s="15" t="n">
         <v>18.8</v>
+      </c>
+      <c r="CF73" s="15" t="n">
+        <v>20.82</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -15523,6 +15699,9 @@
       </c>
       <c r="CE74" s="15" t="n">
         <v>12310.32</v>
+      </c>
+      <c r="CF74" s="15" t="n">
+        <v>12467.08</v>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
@@ -15657,6 +15836,7 @@
       <c r="CC75" s="15" t="n"/>
       <c r="CD75" s="15" t="n"/>
       <c r="CE75" s="15" t="n"/>
+      <c r="CF75" s="15" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -15907,6 +16087,9 @@
       </c>
       <c r="CE76" s="15" t="n">
         <v>51.21</v>
+      </c>
+      <c r="CF76" s="15" t="n">
+        <v>51.34</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -16110,6 +16293,9 @@
       </c>
       <c r="CE77" s="15" t="n">
         <v>15569.82</v>
+      </c>
+      <c r="CF77" s="15" t="n">
+        <v>14858.25</v>
       </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
@@ -16244,6 +16430,7 @@
       <c r="CC78" s="15" t="n"/>
       <c r="CD78" s="15" t="n"/>
       <c r="CE78" s="15" t="n"/>
+      <c r="CF78" s="15" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -16494,6 +16681,9 @@
       </c>
       <c r="CE79" s="15" t="n">
         <v>2.51</v>
+      </c>
+      <c r="CF79" s="15" t="n">
+        <v>2.09</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -16697,6 +16887,9 @@
       </c>
       <c r="CE80" s="15" t="n">
         <v>6420.75</v>
+      </c>
+      <c r="CF80" s="15" t="n">
+        <v>6524.39</v>
       </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
@@ -16831,6 +17024,7 @@
       <c r="CC81" s="15" t="n"/>
       <c r="CD81" s="15" t="n"/>
       <c r="CE81" s="15" t="n"/>
+      <c r="CF81" s="15" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -17081,6 +17275,9 @@
       </c>
       <c r="CE82" s="15" t="n">
         <v>5.58</v>
+      </c>
+      <c r="CF82" s="15" t="n">
+        <v>5.12</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -17283,6 +17480,9 @@
         <v>8452.77</v>
       </c>
       <c r="CE83" s="15" t="n">
+        <v>8455.75</v>
+      </c>
+      <c r="CF83" s="15" t="n">
         <v>8455.75</v>
       </c>
     </row>
@@ -17418,6 +17618,7 @@
       <c r="CC84" s="15" t="n"/>
       <c r="CD84" s="15" t="n"/>
       <c r="CE84" s="15" t="n"/>
+      <c r="CF84" s="15" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -17668,6 +17869,9 @@
       </c>
       <c r="CE85" s="15" t="n">
         <v>16.14</v>
+      </c>
+      <c r="CF85" s="15" t="n">
+        <v>15.32</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -17871,6 +18075,9 @@
       </c>
       <c r="CE86" s="15" t="n">
         <v>2631.9</v>
+      </c>
+      <c r="CF86" s="15" t="n">
+        <v>2018.26</v>
       </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
@@ -18005,6 +18212,7 @@
       <c r="CC87" s="15" t="n"/>
       <c r="CD87" s="15" t="n"/>
       <c r="CE87" s="15" t="n"/>
+      <c r="CF87" s="15" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -18255,6 +18463,9 @@
       </c>
       <c r="CE88" s="15" t="n">
         <v>23.03</v>
+      </c>
+      <c r="CF88" s="15" t="n">
+        <v>21.52</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -18458,6 +18669,9 @@
       </c>
       <c r="CE89" s="15" t="n">
         <v>4060.99</v>
+      </c>
+      <c r="CF89" s="15" t="n">
+        <v>4108.24</v>
       </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
@@ -18592,6 +18806,7 @@
       <c r="CC90" s="15" t="n"/>
       <c r="CD90" s="15" t="n"/>
       <c r="CE90" s="15" t="n"/>
+      <c r="CF90" s="15" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -18842,6 +19057,9 @@
       </c>
       <c r="CE91" s="15" t="n">
         <v>12.42</v>
+      </c>
+      <c r="CF91" s="15" t="n">
+        <v>11.34</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -19045,6 +19263,9 @@
       </c>
       <c r="CE92" s="15" t="n">
         <v>8280.559999999999</v>
+      </c>
+      <c r="CF92" s="15" t="n">
+        <v>8248.190000000001</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
@@ -19179,6 +19400,7 @@
       <c r="CC93" s="15" t="n"/>
       <c r="CD93" s="15" t="n"/>
       <c r="CE93" s="15" t="n"/>
+      <c r="CF93" s="15" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -19429,6 +19651,9 @@
       </c>
       <c r="CE94" s="15" t="n">
         <v>2.98</v>
+      </c>
+      <c r="CF94" s="15" t="n">
+        <v>2.9</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -19632,6 +19857,9 @@
       </c>
       <c r="CE95" s="15" t="n">
         <v>1123.24</v>
+      </c>
+      <c r="CF95" s="15" t="n">
+        <v>1132.34</v>
       </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
@@ -19766,6 +19994,7 @@
       <c r="CC96" s="15" t="n"/>
       <c r="CD96" s="15" t="n"/>
       <c r="CE96" s="15" t="n"/>
+      <c r="CF96" s="15" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -20016,6 +20245,9 @@
       </c>
       <c r="CE97" s="15" t="n">
         <v>9.52</v>
+      </c>
+      <c r="CF97" s="15" t="n">
+        <v>11.14</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -20219,6 +20451,9 @@
       </c>
       <c r="CE98" s="15" t="n">
         <v>13749.28</v>
+      </c>
+      <c r="CF98" s="15" t="n">
+        <v>13964.02</v>
       </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
@@ -20353,6 +20588,7 @@
       <c r="CC99" s="15" t="n"/>
       <c r="CD99" s="15" t="n"/>
       <c r="CE99" s="15" t="n"/>
+      <c r="CF99" s="15" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -20603,6 +20839,9 @@
       </c>
       <c r="CE100" s="15" t="n">
         <v>28.39</v>
+      </c>
+      <c r="CF100" s="15" t="n">
+        <v>27.32</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -20806,6 +21045,9 @@
       </c>
       <c r="CE101" s="15" t="n">
         <v>3128.43</v>
+      </c>
+      <c r="CF101" s="15" t="n">
+        <v>3063.29</v>
       </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
@@ -20940,6 +21182,7 @@
       <c r="CC102" s="15" t="n"/>
       <c r="CD102" s="15" t="n"/>
       <c r="CE102" s="15" t="n"/>
+      <c r="CF102" s="15" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -21190,6 +21433,9 @@
       </c>
       <c r="CE103" s="15" t="n">
         <v>19.2</v>
+      </c>
+      <c r="CF103" s="15" t="n">
+        <v>16.2</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -21393,6 +21639,9 @@
       </c>
       <c r="CE104" s="15" t="n">
         <v>2007.76</v>
+      </c>
+      <c r="CF104" s="15" t="n">
+        <v>1994.68</v>
       </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
@@ -21527,6 +21776,7 @@
       <c r="CC105" s="15" t="n"/>
       <c r="CD105" s="15" t="n"/>
       <c r="CE105" s="15" t="n"/>
+      <c r="CF105" s="15" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -21777,6 +22027,9 @@
       </c>
       <c r="CE106" s="15" t="n">
         <v>7.19</v>
+      </c>
+      <c r="CF106" s="15" t="n">
+        <v>5.93</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -21980,6 +22233,9 @@
       </c>
       <c r="CE107" s="15" t="n">
         <v>2101.93</v>
+      </c>
+      <c r="CF107" s="15" t="n">
+        <v>2129.26</v>
       </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
@@ -22114,6 +22370,7 @@
       <c r="CC108" s="15" t="n"/>
       <c r="CD108" s="15" t="n"/>
       <c r="CE108" s="15" t="n"/>
+      <c r="CF108" s="15" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -22364,6 +22621,9 @@
       </c>
       <c r="CE109" s="15" t="n">
         <v>21.33</v>
+      </c>
+      <c r="CF109" s="15" t="n">
+        <v>20.41</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -22567,6 +22827,9 @@
       </c>
       <c r="CE110" s="15" t="n">
         <v>2341.61</v>
+      </c>
+      <c r="CF110" s="15" t="n">
+        <v>2126.96</v>
       </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
@@ -22701,6 +22964,7 @@
       <c r="CC111" s="15" t="n"/>
       <c r="CD111" s="15" t="n"/>
       <c r="CE111" s="15" t="n"/>
+      <c r="CF111" s="15" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -22951,6 +23215,9 @@
       </c>
       <c r="CE112" s="15" t="n">
         <v>39.66</v>
+      </c>
+      <c r="CF112" s="15" t="n">
+        <v>37.97</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -23152,6 +23419,9 @@
       </c>
       <c r="CE113" s="15" t="n">
         <v>1816.17</v>
+      </c>
+      <c r="CF113" s="15" t="n">
+        <v>1812.24</v>
       </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
@@ -23286,6 +23556,7 @@
       <c r="CC114" s="15" t="n"/>
       <c r="CD114" s="15" t="n"/>
       <c r="CE114" s="15" t="n"/>
+      <c r="CF114" s="15" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -23536,6 +23807,9 @@
       </c>
       <c r="CE115" s="15" t="n">
         <v>16.12</v>
+      </c>
+      <c r="CF115" s="15" t="n">
+        <v>14.82</v>
       </c>
     </row>
     <row r="116" ht="14.25" customHeight="1">
@@ -23724,6 +23998,9 @@
       </c>
       <c r="CE116" s="15" t="n">
         <v>8773.190000000001</v>
+      </c>
+      <c r="CF116" s="15" t="n">
+        <v>8453.4</v>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1">
@@ -23813,6 +24090,7 @@
       <c r="CC117" s="15" t="n"/>
       <c r="CD117" s="15" t="n"/>
       <c r="CE117" s="15" t="n"/>
+      <c r="CF117" s="15" t="n"/>
     </row>
     <row r="118" ht="14.25" customHeight="1">
       <c r="P118" s="13" t="n">
@@ -24019,6 +24297,9 @@
       <c r="CE118" s="15" t="n">
         <v>61.04</v>
       </c>
+      <c r="CF118" s="15" t="n">
+        <v>59.09</v>
+      </c>
     </row>
     <row r="119" ht="14.25" customHeight="1">
       <c r="Y119" s="13" t="n">
@@ -24197,6 +24478,9 @@
       </c>
       <c r="CE119" s="15" t="n">
         <v>10590.92</v>
+      </c>
+      <c r="CF119" s="15" t="n">
+        <v>10334.16</v>
       </c>
     </row>
     <row r="120" ht="14.25" customHeight="1">
@@ -24235,6 +24519,7 @@
       <c r="CC120" s="15" t="n"/>
       <c r="CD120" s="15" t="n"/>
       <c r="CE120" s="15" t="n"/>
+      <c r="CF120" s="15" t="n"/>
     </row>
     <row r="121" ht="14.25" customHeight="1">
       <c r="AW121" s="13" t="n">
@@ -24342,6 +24627,9 @@
       <c r="CE121" s="15" t="n">
         <v>27.71</v>
       </c>
+      <c r="CF121" s="15" t="n">
+        <v>22.27</v>
+      </c>
     </row>
     <row r="122" ht="14.25" customHeight="1">
       <c r="AW122" s="13" t="n">
@@ -24448,6 +24736,9 @@
       </c>
       <c r="CE122" s="15" t="n">
         <v>1211.93</v>
+      </c>
+      <c r="CF122" s="15" t="n">
+        <v>1158.42</v>
       </c>
     </row>
     <row r="123" ht="14.25" customHeight="1">
@@ -24486,6 +24777,7 @@
       <c r="CC123" s="15" t="n"/>
       <c r="CD123" s="15" t="n"/>
       <c r="CE123" s="15" t="n"/>
+      <c r="CF123" s="15" t="n"/>
     </row>
     <row r="124" ht="14.25" customHeight="1">
       <c r="AW124" s="13" t="n">
@@ -24593,6 +24885,9 @@
       <c r="CE124" s="15" t="n">
         <v>37.48</v>
       </c>
+      <c r="CF124" s="15" t="n">
+        <v>35.53</v>
+      </c>
     </row>
     <row r="125" ht="14.25" customHeight="1">
       <c r="AW125" s="13" t="n">
@@ -24699,6 +24994,9 @@
       </c>
       <c r="CE125" s="15" t="n">
         <v>10429.97</v>
+      </c>
+      <c r="CF125" s="15" t="n">
+        <v>10840.09</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1">
@@ -24737,6 +25035,7 @@
       <c r="CC126" s="15" t="n"/>
       <c r="CD126" s="15" t="n"/>
       <c r="CE126" s="15" t="n"/>
+      <c r="CF126" s="15" t="n"/>
     </row>
     <row r="127" ht="14.25" customHeight="1">
       <c r="AW127" s="13" t="n">
@@ -24844,6 +25143,9 @@
       <c r="CE127" s="15" t="n">
         <v>3.49</v>
       </c>
+      <c r="CF127" s="15" t="n">
+        <v>2.83</v>
+      </c>
     </row>
     <row r="128" ht="14.25" customHeight="1">
       <c r="AW128" s="13" t="n">
@@ -24950,6 +25252,9 @@
       </c>
       <c r="CE128" s="15" t="n">
         <v>1767.42</v>
+      </c>
+      <c r="CF128" s="15" t="n">
+        <v>1807.17</v>
       </c>
     </row>
     <row r="129" ht="14.25" customHeight="1">
@@ -24988,6 +25293,7 @@
       <c r="CC129" s="15" t="n"/>
       <c r="CD129" s="15" t="n"/>
       <c r="CE129" s="15" t="n"/>
+      <c r="CF129" s="15" t="n"/>
     </row>
     <row r="130" ht="14.25" customHeight="1">
       <c r="AW130" s="13" t="n">
@@ -25095,6 +25401,9 @@
       <c r="CE130" s="15" t="n">
         <v>6.29</v>
       </c>
+      <c r="CF130" s="15" t="n">
+        <v>5.5</v>
+      </c>
     </row>
     <row r="131" ht="14.25" customHeight="1">
       <c r="AW131" s="13" t="n">
@@ -25201,6 +25510,9 @@
       </c>
       <c r="CE131" s="15" t="n">
         <v>721.53</v>
+      </c>
+      <c r="CF131" s="15" t="n">
+        <v>714.64</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1">
@@ -25239,6 +25551,7 @@
       <c r="CC132" s="15" t="n"/>
       <c r="CD132" s="15" t="n"/>
       <c r="CE132" s="15" t="n"/>
+      <c r="CF132" s="15" t="n"/>
     </row>
     <row r="133" ht="14.25" customHeight="1">
       <c r="AW133" s="13" t="n">
@@ -25346,6 +25659,9 @@
       <c r="CE133" s="15" t="n">
         <v>42.44</v>
       </c>
+      <c r="CF133" s="15" t="n">
+        <v>39.54</v>
+      </c>
     </row>
     <row r="134" ht="14.25" customHeight="1">
       <c r="AW134" s="13" t="n">
@@ -25451,6 +25767,9 @@
         <v>2641.45</v>
       </c>
       <c r="CE134" s="15" t="n">
+        <v>2506.83</v>
+      </c>
+      <c r="CF134" s="15" t="n">
         <v>2506.83</v>
       </c>
     </row>
@@ -25490,6 +25809,7 @@
       <c r="CC135" s="15" t="n"/>
       <c r="CD135" s="15" t="n"/>
       <c r="CE135" s="15" t="n"/>
+      <c r="CF135" s="15" t="n"/>
     </row>
     <row r="136" ht="14.25" customHeight="1">
       <c r="AW136" s="13" t="n">
@@ -25597,6 +25917,9 @@
       <c r="CE136" s="15" t="n">
         <v>21.17</v>
       </c>
+      <c r="CF136" s="15" t="n">
+        <v>20.72</v>
+      </c>
     </row>
     <row r="137" ht="14.25" customHeight="1">
       <c r="AW137" s="13" t="n">
@@ -25703,6 +26026,9 @@
       </c>
       <c r="CE137" s="15" t="n">
         <v>3336.46</v>
+      </c>
+      <c r="CF137" s="15" t="n">
+        <v>3358.86</v>
       </c>
     </row>
     <row r="138">
@@ -25733,6 +26059,7 @@
       <c r="CC138" s="15" t="n"/>
       <c r="CD138" s="15" t="n"/>
       <c r="CE138" s="15" t="n"/>
+      <c r="CF138" s="15" t="n"/>
     </row>
     <row r="139">
       <c r="BE139" s="15" t="n">
@@ -25816,6 +26143,9 @@
       <c r="CE139" s="15" t="n">
         <v>4.55</v>
       </c>
+      <c r="CF139" s="15" t="n">
+        <v>4.35</v>
+      </c>
     </row>
     <row r="140">
       <c r="BE140" s="15" t="n">
@@ -25896,6 +26226,9 @@
       </c>
       <c r="CE140" s="15" t="n">
         <v>2343.25</v>
+      </c>
+      <c r="CF140" s="15" t="n">
+        <v>2357.2</v>
       </c>
     </row>
     <row r="141">
@@ -25926,6 +26259,7 @@
       <c r="CC141" s="15" t="n"/>
       <c r="CD141" s="15" t="n"/>
       <c r="CE141" s="15" t="n"/>
+      <c r="CF141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="BE142" s="15" t="n">
@@ -26009,6 +26343,9 @@
       <c r="CE142" s="15" t="n">
         <v>15.38</v>
       </c>
+      <c r="CF142" s="15" t="n">
+        <v>16.61</v>
+      </c>
     </row>
     <row r="143">
       <c r="BE143" s="15" t="n">
@@ -26091,6 +26428,9 @@
       </c>
       <c r="CE143" s="15" t="n">
         <v>5386.01</v>
+      </c>
+      <c r="CF143" s="15" t="n">
+        <v>5403.94</v>
       </c>
     </row>
     <row r="144">
@@ -26116,6 +26456,7 @@
       <c r="CC144" s="15" t="n"/>
       <c r="CD144" s="15" t="n"/>
       <c r="CE144" s="15" t="n"/>
+      <c r="CF144" s="15" t="n"/>
     </row>
     <row r="145">
       <c r="BJ145" s="15" t="n">
@@ -26184,6 +26525,9 @@
       <c r="CE145" s="15" t="n">
         <v>1.31</v>
       </c>
+      <c r="CF145" s="15" t="n">
+        <v>1.2</v>
+      </c>
     </row>
     <row r="146">
       <c r="BJ146" s="15" t="n">
@@ -26251,6 +26595,9 @@
       </c>
       <c r="CE146" s="15" t="n">
         <v>2174.1</v>
+      </c>
+      <c r="CF146" s="15" t="n">
+        <v>2142.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-10-22 08:57:51]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CF146"/>
+  <dimension ref="A1:CG146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="51"/>
@@ -618,6 +618,7 @@
     <col width="15" customWidth="1" min="82" max="82"/>
     <col width="15" customWidth="1" min="83" max="83"/>
     <col width="15" customWidth="1" min="84" max="84"/>
+    <col width="15" customWidth="1" min="85" max="85"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -1041,6 +1042,11 @@
           <t>2026/10/19</t>
         </is>
       </c>
+      <c r="CG1" s="15" t="inlineStr">
+        <is>
+          <t>2026/10/22</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1463,6 +1469,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="CG2" s="16" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1717,6 +1728,9 @@
       <c r="CF3" s="15" t="n">
         <v>48.84</v>
       </c>
+      <c r="CG3" s="15" t="n">
+        <v>48.26</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1970,6 +1984,9 @@
       </c>
       <c r="CF4" s="15" t="n">
         <v>3730.92</v>
+      </c>
+      <c r="CG4" s="15" t="n">
+        <v>3658.03</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -2057,6 +2074,7 @@
       <c r="CD5" s="15" t="n"/>
       <c r="CE5" s="15" t="n"/>
       <c r="CF5" s="15" t="n"/>
+      <c r="CG5" s="15" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -2191,6 +2209,7 @@
       <c r="CD6" s="15" t="n"/>
       <c r="CE6" s="15" t="n"/>
       <c r="CF6" s="15" t="n"/>
+      <c r="CG6" s="15" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -2444,6 +2463,9 @@
       </c>
       <c r="CF7" s="15" t="n">
         <v>42.08</v>
+      </c>
+      <c r="CG7" s="15" t="n">
+        <v>41.17</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -2650,6 +2672,9 @@
       </c>
       <c r="CF8" s="15" t="n">
         <v>5070.19</v>
+      </c>
+      <c r="CG8" s="15" t="n">
+        <v>4911.33</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
@@ -2785,6 +2810,7 @@
       <c r="CD9" s="15" t="n"/>
       <c r="CE9" s="15" t="n"/>
       <c r="CF9" s="15" t="n"/>
+      <c r="CG9" s="15" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -3038,6 +3064,9 @@
       </c>
       <c r="CF10" s="15" t="n">
         <v>39.73</v>
+      </c>
+      <c r="CG10" s="15" t="n">
+        <v>37.75</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -3244,6 +3273,9 @@
       </c>
       <c r="CF11" s="15" t="n">
         <v>4174.53</v>
+      </c>
+      <c r="CG11" s="15" t="n">
+        <v>4036.3</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
@@ -3379,6 +3411,7 @@
       <c r="CD12" s="15" t="n"/>
       <c r="CE12" s="15" t="n"/>
       <c r="CF12" s="15" t="n"/>
+      <c r="CG12" s="15" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -3632,6 +3665,9 @@
       </c>
       <c r="CF13" s="15" t="n">
         <v>44.05</v>
+      </c>
+      <c r="CG13" s="15" t="n">
+        <v>45.39</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -3838,6 +3874,9 @@
       </c>
       <c r="CF14" s="15" t="n">
         <v>6800.66</v>
+      </c>
+      <c r="CG14" s="15" t="n">
+        <v>6655.25</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
@@ -3973,6 +4012,7 @@
       <c r="CD15" s="15" t="n"/>
       <c r="CE15" s="15" t="n"/>
       <c r="CF15" s="15" t="n"/>
+      <c r="CG15" s="15" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -4226,6 +4266,9 @@
       </c>
       <c r="CF16" s="15" t="n">
         <v>24.23</v>
+      </c>
+      <c r="CG16" s="15" t="n">
+        <v>22.46</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -4432,6 +4475,9 @@
       </c>
       <c r="CF17" s="15" t="n">
         <v>2372.31</v>
+      </c>
+      <c r="CG17" s="15" t="n">
+        <v>2404.7</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
@@ -4567,6 +4613,7 @@
       <c r="CD18" s="15" t="n"/>
       <c r="CE18" s="15" t="n"/>
       <c r="CF18" s="15" t="n"/>
+      <c r="CG18" s="15" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -4820,6 +4867,9 @@
       </c>
       <c r="CF19" s="15" t="n">
         <v>78.52</v>
+      </c>
+      <c r="CG19" s="15" t="n">
+        <v>78.97</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -5026,6 +5076,9 @@
       </c>
       <c r="CF20" s="15" t="n">
         <v>7659.44</v>
+      </c>
+      <c r="CG20" s="15" t="n">
+        <v>7757.17</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
@@ -5161,6 +5214,7 @@
       <c r="CD21" s="15" t="n"/>
       <c r="CE21" s="15" t="n"/>
       <c r="CF21" s="15" t="n"/>
+      <c r="CG21" s="15" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -5411,6 +5465,9 @@
         <v>36.34</v>
       </c>
       <c r="CF22" s="15" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="CG22" s="15" t="n">
         <v>36.34</v>
       </c>
     </row>
@@ -5618,6 +5675,9 @@
       </c>
       <c r="CF23" s="15" t="n">
         <v>73736.45</v>
+      </c>
+      <c r="CG23" s="15" t="n">
+        <v>73221.31</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
@@ -5753,6 +5813,7 @@
       <c r="CD24" s="15" t="n"/>
       <c r="CE24" s="15" t="n"/>
       <c r="CF24" s="15" t="n"/>
+      <c r="CG24" s="15" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -6005,6 +6066,9 @@
         <v>49.88</v>
       </c>
       <c r="CF25" s="15" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="CG25" s="15" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -6198,6 +6262,9 @@
       </c>
       <c r="CF26" s="15" t="n">
         <v>25329.55</v>
+      </c>
+      <c r="CG26" s="15" t="n">
+        <v>25382.48</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
@@ -6333,6 +6400,7 @@
       <c r="CD27" s="15" t="n"/>
       <c r="CE27" s="15" t="n"/>
       <c r="CF27" s="15" t="n"/>
+      <c r="CG27" s="15" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -6585,6 +6653,9 @@
         <v>92.09</v>
       </c>
       <c r="CF28" s="15" t="n">
+        <v>92.09</v>
+      </c>
+      <c r="CG28" s="15" t="n">
         <v>92.09</v>
       </c>
     </row>
@@ -6792,6 +6863,9 @@
       </c>
       <c r="CF29" s="15" t="n">
         <v>64916.7</v>
+      </c>
+      <c r="CG29" s="15" t="n">
+        <v>62907.84</v>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
@@ -6927,6 +7001,7 @@
       <c r="CD30" s="15" t="n"/>
       <c r="CE30" s="15" t="n"/>
       <c r="CF30" s="15" t="n"/>
+      <c r="CG30" s="15" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -7179,6 +7254,9 @@
         <v>97.44</v>
       </c>
       <c r="CF31" s="15" t="n">
+        <v>97.44</v>
+      </c>
+      <c r="CG31" s="15" t="n">
         <v>97.44</v>
       </c>
     </row>
@@ -7386,6 +7464,9 @@
       </c>
       <c r="CF32" s="15" t="n">
         <v>5768.01</v>
+      </c>
+      <c r="CG32" s="15" t="n">
+        <v>5533.77</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
@@ -7521,6 +7602,7 @@
       <c r="CD33" s="15" t="n"/>
       <c r="CE33" s="15" t="n"/>
       <c r="CF33" s="15" t="n"/>
+      <c r="CG33" s="15" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -7774,6 +7856,9 @@
       </c>
       <c r="CF34" s="15" t="n">
         <v>49.93</v>
+      </c>
+      <c r="CG34" s="15" t="n">
+        <v>53.72</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -7980,6 +8065,9 @@
       </c>
       <c r="CF35" s="15" t="n">
         <v>5623.37</v>
+      </c>
+      <c r="CG35" s="15" t="n">
+        <v>5405.75</v>
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
@@ -8115,6 +8203,7 @@
       <c r="CD36" s="15" t="n"/>
       <c r="CE36" s="15" t="n"/>
       <c r="CF36" s="15" t="n"/>
+      <c r="CG36" s="15" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -8368,6 +8457,9 @@
       </c>
       <c r="CF37" s="15" t="n">
         <v>55.89</v>
+      </c>
+      <c r="CG37" s="15" t="n">
+        <v>66.67</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -8574,6 +8666,9 @@
       </c>
       <c r="CF38" s="15" t="n">
         <v>11605.41</v>
+      </c>
+      <c r="CG38" s="15" t="n">
+        <v>11296.62</v>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
@@ -8709,6 +8804,7 @@
       <c r="CD39" s="15" t="n"/>
       <c r="CE39" s="15" t="n"/>
       <c r="CF39" s="15" t="n"/>
+      <c r="CG39" s="15" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -8962,6 +9058,9 @@
       </c>
       <c r="CF40" s="15" t="n">
         <v>52.9</v>
+      </c>
+      <c r="CG40" s="15" t="n">
+        <v>57.34</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -9168,6 +9267,9 @@
       </c>
       <c r="CF41" s="15" t="n">
         <v>11191.38</v>
+      </c>
+      <c r="CG41" s="15" t="n">
+        <v>11097.06</v>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
@@ -9303,6 +9405,7 @@
       <c r="CD42" s="15" t="n"/>
       <c r="CE42" s="15" t="n"/>
       <c r="CF42" s="15" t="n"/>
+      <c r="CG42" s="15" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -9556,6 +9659,9 @@
       </c>
       <c r="CF43" s="15" t="n">
         <v>52.02</v>
+      </c>
+      <c r="CG43" s="15" t="n">
+        <v>55.89</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -9762,6 +9868,9 @@
       </c>
       <c r="CF44" s="15" t="n">
         <v>3337.49</v>
+      </c>
+      <c r="CG44" s="15" t="n">
+        <v>3287.02</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
@@ -9897,6 +10006,7 @@
       <c r="CD45" s="15" t="n"/>
       <c r="CE45" s="15" t="n"/>
       <c r="CF45" s="15" t="n"/>
+      <c r="CG45" s="15" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -10150,6 +10260,9 @@
       </c>
       <c r="CF46" s="15" t="n">
         <v>62.33</v>
+      </c>
+      <c r="CG46" s="15" t="n">
+        <v>70.61</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -10356,6 +10469,9 @@
       </c>
       <c r="CF47" s="15" t="n">
         <v>7229.66</v>
+      </c>
+      <c r="CG47" s="15" t="n">
+        <v>7139.86</v>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
@@ -10491,6 +10607,7 @@
       <c r="CD48" s="15" t="n"/>
       <c r="CE48" s="15" t="n"/>
       <c r="CF48" s="15" t="n"/>
+      <c r="CG48" s="15" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -10744,6 +10861,9 @@
       </c>
       <c r="CF49" s="15" t="n">
         <v>15.87</v>
+      </c>
+      <c r="CG49" s="15" t="n">
+        <v>15.52</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -10949,6 +11069,9 @@
         <v>32092.73</v>
       </c>
       <c r="CF50" s="15" t="n">
+        <v>31175.73</v>
+      </c>
+      <c r="CG50" s="15" t="n">
         <v>31175.73</v>
       </c>
     </row>
@@ -11085,6 +11208,7 @@
       <c r="CD51" s="15" t="n"/>
       <c r="CE51" s="15" t="n"/>
       <c r="CF51" s="15" t="n"/>
+      <c r="CG51" s="15" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -11338,6 +11462,9 @@
       </c>
       <c r="CF52" s="15" t="n">
         <v>22.83</v>
+      </c>
+      <c r="CG52" s="15" t="n">
+        <v>18.62</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -11544,6 +11671,9 @@
       </c>
       <c r="CF53" s="15" t="n">
         <v>2825.99</v>
+      </c>
+      <c r="CG53" s="15" t="n">
+        <v>2614.37</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
@@ -11679,6 +11809,7 @@
       <c r="CD54" s="15" t="n"/>
       <c r="CE54" s="15" t="n"/>
       <c r="CF54" s="15" t="n"/>
+      <c r="CG54" s="15" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -11932,6 +12063,9 @@
       </c>
       <c r="CF55" s="15" t="n">
         <v>27.31</v>
+      </c>
+      <c r="CG55" s="15" t="n">
+        <v>23.25</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -12138,6 +12272,9 @@
       </c>
       <c r="CF56" s="15" t="n">
         <v>2746.29</v>
+      </c>
+      <c r="CG56" s="15" t="n">
+        <v>2576.9</v>
       </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
@@ -12273,6 +12410,7 @@
       <c r="CD57" s="15" t="n"/>
       <c r="CE57" s="15" t="n"/>
       <c r="CF57" s="15" t="n"/>
+      <c r="CG57" s="15" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -12526,6 +12664,9 @@
       </c>
       <c r="CF58" s="15" t="n">
         <v>8.5</v>
+      </c>
+      <c r="CG58" s="15" t="n">
+        <v>11.43</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -12732,6 +12873,9 @@
       </c>
       <c r="CF59" s="15" t="n">
         <v>6436.71</v>
+      </c>
+      <c r="CG59" s="15" t="n">
+        <v>6433.89</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
@@ -12867,6 +13011,7 @@
       <c r="CD60" s="15" t="n"/>
       <c r="CE60" s="15" t="n"/>
       <c r="CF60" s="15" t="n"/>
+      <c r="CG60" s="15" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -13120,6 +13265,9 @@
       </c>
       <c r="CF61" s="15" t="n">
         <v>30.42</v>
+      </c>
+      <c r="CG61" s="15" t="n">
+        <v>34.96</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -13326,6 +13474,9 @@
       </c>
       <c r="CF62" s="15" t="n">
         <v>7983.99</v>
+      </c>
+      <c r="CG62" s="15" t="n">
+        <v>7887.89</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
@@ -13461,6 +13612,7 @@
       <c r="CD63" s="15" t="n"/>
       <c r="CE63" s="15" t="n"/>
       <c r="CF63" s="15" t="n"/>
+      <c r="CG63" s="15" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -13714,6 +13866,9 @@
       </c>
       <c r="CF64" s="15" t="n">
         <v>10.03</v>
+      </c>
+      <c r="CG64" s="15" t="n">
+        <v>7.82</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -13920,6 +14075,9 @@
       </c>
       <c r="CF65" s="15" t="n">
         <v>10577.64</v>
+      </c>
+      <c r="CG65" s="15" t="n">
+        <v>10387.03</v>
       </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
@@ -14055,6 +14213,7 @@
       <c r="CD66" s="15" t="n"/>
       <c r="CE66" s="15" t="n"/>
       <c r="CF66" s="15" t="n"/>
+      <c r="CG66" s="15" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -14308,6 +14467,9 @@
       </c>
       <c r="CF67" s="15" t="n">
         <v>13.16</v>
+      </c>
+      <c r="CG67" s="15" t="n">
+        <v>12.12</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -14514,6 +14676,9 @@
       </c>
       <c r="CF68" s="15" t="n">
         <v>10832.7</v>
+      </c>
+      <c r="CG68" s="15" t="n">
+        <v>10541.68</v>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
@@ -14649,6 +14814,7 @@
       <c r="CD69" s="15" t="n"/>
       <c r="CE69" s="15" t="n"/>
       <c r="CF69" s="15" t="n"/>
+      <c r="CG69" s="15" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -14902,6 +15068,9 @@
       </c>
       <c r="CF70" s="15" t="n">
         <v>20.52</v>
+      </c>
+      <c r="CG70" s="15" t="n">
+        <v>18.32</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -15108,6 +15277,9 @@
       </c>
       <c r="CF71" s="15" t="n">
         <v>6399.37</v>
+      </c>
+      <c r="CG71" s="15" t="n">
+        <v>6124</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
@@ -15243,6 +15415,7 @@
       <c r="CD72" s="15" t="n"/>
       <c r="CE72" s="15" t="n"/>
       <c r="CF72" s="15" t="n"/>
+      <c r="CG72" s="15" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -15496,6 +15669,9 @@
       </c>
       <c r="CF73" s="15" t="n">
         <v>20.82</v>
+      </c>
+      <c r="CG73" s="15" t="n">
+        <v>19.09</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -15702,6 +15878,9 @@
       </c>
       <c r="CF74" s="15" t="n">
         <v>12467.08</v>
+      </c>
+      <c r="CG74" s="15" t="n">
+        <v>12248.57</v>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
@@ -15837,6 +16016,7 @@
       <c r="CD75" s="15" t="n"/>
       <c r="CE75" s="15" t="n"/>
       <c r="CF75" s="15" t="n"/>
+      <c r="CG75" s="15" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -16090,6 +16270,9 @@
       </c>
       <c r="CF76" s="15" t="n">
         <v>51.34</v>
+      </c>
+      <c r="CG76" s="15" t="n">
+        <v>51.69</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -16296,6 +16479,9 @@
       </c>
       <c r="CF77" s="15" t="n">
         <v>14858.25</v>
+      </c>
+      <c r="CG77" s="15" t="n">
+        <v>14180.18</v>
       </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
@@ -16431,6 +16617,7 @@
       <c r="CD78" s="15" t="n"/>
       <c r="CE78" s="15" t="n"/>
       <c r="CF78" s="15" t="n"/>
+      <c r="CG78" s="15" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -16684,6 +16871,9 @@
       </c>
       <c r="CF79" s="15" t="n">
         <v>2.09</v>
+      </c>
+      <c r="CG79" s="15" t="n">
+        <v>0.85</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -16890,6 +17080,9 @@
       </c>
       <c r="CF80" s="15" t="n">
         <v>6524.39</v>
+      </c>
+      <c r="CG80" s="15" t="n">
+        <v>5973.47</v>
       </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
@@ -17025,6 +17218,7 @@
       <c r="CD81" s="15" t="n"/>
       <c r="CE81" s="15" t="n"/>
       <c r="CF81" s="15" t="n"/>
+      <c r="CG81" s="15" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -17278,6 +17472,9 @@
       </c>
       <c r="CF82" s="15" t="n">
         <v>5.12</v>
+      </c>
+      <c r="CG82" s="15" t="n">
+        <v>5.53</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -17484,6 +17681,9 @@
       </c>
       <c r="CF83" s="15" t="n">
         <v>8455.75</v>
+      </c>
+      <c r="CG83" s="15" t="n">
+        <v>8481.950000000001</v>
       </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
@@ -17619,6 +17819,7 @@
       <c r="CD84" s="15" t="n"/>
       <c r="CE84" s="15" t="n"/>
       <c r="CF84" s="15" t="n"/>
+      <c r="CG84" s="15" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -17872,6 +18073,9 @@
       </c>
       <c r="CF85" s="15" t="n">
         <v>15.32</v>
+      </c>
+      <c r="CG85" s="15" t="n">
+        <v>13.06</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -18078,6 +18282,9 @@
       </c>
       <c r="CF86" s="15" t="n">
         <v>2018.26</v>
+      </c>
+      <c r="CG86" s="15" t="n">
+        <v>1873.97</v>
       </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
@@ -18213,6 +18420,7 @@
       <c r="CD87" s="15" t="n"/>
       <c r="CE87" s="15" t="n"/>
       <c r="CF87" s="15" t="n"/>
+      <c r="CG87" s="15" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -18466,6 +18674,9 @@
       </c>
       <c r="CF88" s="15" t="n">
         <v>21.52</v>
+      </c>
+      <c r="CG88" s="15" t="n">
+        <v>17.59</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -18672,6 +18883,9 @@
       </c>
       <c r="CF89" s="15" t="n">
         <v>4108.24</v>
+      </c>
+      <c r="CG89" s="15" t="n">
+        <v>3793.93</v>
       </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
@@ -18807,6 +19021,7 @@
       <c r="CD90" s="15" t="n"/>
       <c r="CE90" s="15" t="n"/>
       <c r="CF90" s="15" t="n"/>
+      <c r="CG90" s="15" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -19060,6 +19275,9 @@
       </c>
       <c r="CF91" s="15" t="n">
         <v>11.34</v>
+      </c>
+      <c r="CG91" s="15" t="n">
+        <v>14.8</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -19266,6 +19484,9 @@
       </c>
       <c r="CF92" s="15" t="n">
         <v>8248.190000000001</v>
+      </c>
+      <c r="CG92" s="15" t="n">
+        <v>8136.47</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
@@ -19401,6 +19622,7 @@
       <c r="CD93" s="15" t="n"/>
       <c r="CE93" s="15" t="n"/>
       <c r="CF93" s="15" t="n"/>
+      <c r="CG93" s="15" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -19654,6 +19876,9 @@
       </c>
       <c r="CF94" s="15" t="n">
         <v>2.9</v>
+      </c>
+      <c r="CG94" s="15" t="n">
+        <v>2.88</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -19860,6 +20085,9 @@
       </c>
       <c r="CF95" s="15" t="n">
         <v>1132.34</v>
+      </c>
+      <c r="CG95" s="15" t="n">
+        <v>1115.29</v>
       </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
@@ -19995,6 +20223,7 @@
       <c r="CD96" s="15" t="n"/>
       <c r="CE96" s="15" t="n"/>
       <c r="CF96" s="15" t="n"/>
+      <c r="CG96" s="15" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -20248,6 +20477,9 @@
       </c>
       <c r="CF97" s="15" t="n">
         <v>11.14</v>
+      </c>
+      <c r="CG97" s="15" t="n">
+        <v>9.27</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -20454,6 +20686,9 @@
       </c>
       <c r="CF98" s="15" t="n">
         <v>13964.02</v>
+      </c>
+      <c r="CG98" s="15" t="n">
+        <v>13708.46</v>
       </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
@@ -20589,6 +20824,7 @@
       <c r="CD99" s="15" t="n"/>
       <c r="CE99" s="15" t="n"/>
       <c r="CF99" s="15" t="n"/>
+      <c r="CG99" s="15" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -20842,6 +21078,9 @@
       </c>
       <c r="CF100" s="15" t="n">
         <v>27.32</v>
+      </c>
+      <c r="CG100" s="15" t="n">
+        <v>31.19</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -21048,6 +21287,9 @@
       </c>
       <c r="CF101" s="15" t="n">
         <v>3063.29</v>
+      </c>
+      <c r="CG101" s="15" t="n">
+        <v>3135.6</v>
       </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
@@ -21183,6 +21425,7 @@
       <c r="CD102" s="15" t="n"/>
       <c r="CE102" s="15" t="n"/>
       <c r="CF102" s="15" t="n"/>
+      <c r="CG102" s="15" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -21436,6 +21679,9 @@
       </c>
       <c r="CF103" s="15" t="n">
         <v>16.2</v>
+      </c>
+      <c r="CG103" s="15" t="n">
+        <v>10.29</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -21642,6 +21888,9 @@
       </c>
       <c r="CF104" s="15" t="n">
         <v>1994.68</v>
+      </c>
+      <c r="CG104" s="15" t="n">
+        <v>1884.73</v>
       </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
@@ -21777,6 +22026,7 @@
       <c r="CD105" s="15" t="n"/>
       <c r="CE105" s="15" t="n"/>
       <c r="CF105" s="15" t="n"/>
+      <c r="CG105" s="15" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -22030,6 +22280,9 @@
       </c>
       <c r="CF106" s="15" t="n">
         <v>5.93</v>
+      </c>
+      <c r="CG106" s="15" t="n">
+        <v>5.86</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -22236,6 +22489,9 @@
       </c>
       <c r="CF107" s="15" t="n">
         <v>2129.26</v>
+      </c>
+      <c r="CG107" s="15" t="n">
+        <v>2078.53</v>
       </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
@@ -22371,6 +22627,7 @@
       <c r="CD108" s="15" t="n"/>
       <c r="CE108" s="15" t="n"/>
       <c r="CF108" s="15" t="n"/>
+      <c r="CG108" s="15" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -22624,6 +22881,9 @@
       </c>
       <c r="CF109" s="15" t="n">
         <v>20.41</v>
+      </c>
+      <c r="CG109" s="15" t="n">
+        <v>15.75</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -22830,6 +23090,9 @@
       </c>
       <c r="CF110" s="15" t="n">
         <v>2126.96</v>
+      </c>
+      <c r="CG110" s="15" t="n">
+        <v>2068.3</v>
       </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
@@ -22965,6 +23228,7 @@
       <c r="CD111" s="15" t="n"/>
       <c r="CE111" s="15" t="n"/>
       <c r="CF111" s="15" t="n"/>
+      <c r="CG111" s="15" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -23218,6 +23482,9 @@
       </c>
       <c r="CF112" s="15" t="n">
         <v>37.97</v>
+      </c>
+      <c r="CG112" s="15" t="n">
+        <v>44.36</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -23422,6 +23689,9 @@
       </c>
       <c r="CF113" s="15" t="n">
         <v>1812.24</v>
+      </c>
+      <c r="CG113" s="15" t="n">
+        <v>1799.37</v>
       </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
@@ -23557,6 +23827,7 @@
       <c r="CD114" s="15" t="n"/>
       <c r="CE114" s="15" t="n"/>
       <c r="CF114" s="15" t="n"/>
+      <c r="CG114" s="15" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -23810,6 +24081,9 @@
       </c>
       <c r="CF115" s="15" t="n">
         <v>14.82</v>
+      </c>
+      <c r="CG115" s="15" t="n">
+        <v>16.61</v>
       </c>
     </row>
     <row r="116" ht="14.25" customHeight="1">
@@ -24001,6 +24275,9 @@
       </c>
       <c r="CF116" s="15" t="n">
         <v>8453.4</v>
+      </c>
+      <c r="CG116" s="15" t="n">
+        <v>8531.5</v>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1">
@@ -24091,6 +24368,7 @@
       <c r="CD117" s="15" t="n"/>
       <c r="CE117" s="15" t="n"/>
       <c r="CF117" s="15" t="n"/>
+      <c r="CG117" s="15" t="n"/>
     </row>
     <row r="118" ht="14.25" customHeight="1">
       <c r="P118" s="13" t="n">
@@ -24300,6 +24578,9 @@
       <c r="CF118" s="15" t="n">
         <v>59.09</v>
       </c>
+      <c r="CG118" s="15" t="n">
+        <v>58.19</v>
+      </c>
     </row>
     <row r="119" ht="14.25" customHeight="1">
       <c r="Y119" s="13" t="n">
@@ -24481,6 +24762,9 @@
       </c>
       <c r="CF119" s="15" t="n">
         <v>10334.16</v>
+      </c>
+      <c r="CG119" s="15" t="n">
+        <v>10204.26</v>
       </c>
     </row>
     <row r="120" ht="14.25" customHeight="1">
@@ -24520,6 +24804,7 @@
       <c r="CD120" s="15" t="n"/>
       <c r="CE120" s="15" t="n"/>
       <c r="CF120" s="15" t="n"/>
+      <c r="CG120" s="15" t="n"/>
     </row>
     <row r="121" ht="14.25" customHeight="1">
       <c r="AW121" s="13" t="n">
@@ -24630,6 +24915,9 @@
       <c r="CF121" s="15" t="n">
         <v>22.27</v>
       </c>
+      <c r="CG121" s="15" t="n">
+        <v>22.17</v>
+      </c>
     </row>
     <row r="122" ht="14.25" customHeight="1">
       <c r="AW122" s="13" t="n">
@@ -24739,6 +25027,9 @@
       </c>
       <c r="CF122" s="15" t="n">
         <v>1158.42</v>
+      </c>
+      <c r="CG122" s="15" t="n">
+        <v>1161.26</v>
       </c>
     </row>
     <row r="123" ht="14.25" customHeight="1">
@@ -24778,6 +25069,7 @@
       <c r="CD123" s="15" t="n"/>
       <c r="CE123" s="15" t="n"/>
       <c r="CF123" s="15" t="n"/>
+      <c r="CG123" s="15" t="n"/>
     </row>
     <row r="124" ht="14.25" customHeight="1">
       <c r="AW124" s="13" t="n">
@@ -24888,6 +25180,9 @@
       <c r="CF124" s="15" t="n">
         <v>35.53</v>
       </c>
+      <c r="CG124" s="15" t="n">
+        <v>36.2</v>
+      </c>
     </row>
     <row r="125" ht="14.25" customHeight="1">
       <c r="AW125" s="13" t="n">
@@ -24997,6 +25292,9 @@
       </c>
       <c r="CF125" s="15" t="n">
         <v>10840.09</v>
+      </c>
+      <c r="CG125" s="15" t="n">
+        <v>10518.38</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1">
@@ -25036,6 +25334,7 @@
       <c r="CD126" s="15" t="n"/>
       <c r="CE126" s="15" t="n"/>
       <c r="CF126" s="15" t="n"/>
+      <c r="CG126" s="15" t="n"/>
     </row>
     <row r="127" ht="14.25" customHeight="1">
       <c r="AW127" s="13" t="n">
@@ -25146,6 +25445,9 @@
       <c r="CF127" s="15" t="n">
         <v>2.83</v>
       </c>
+      <c r="CG127" s="15" t="n">
+        <v>4.81</v>
+      </c>
     </row>
     <row r="128" ht="14.25" customHeight="1">
       <c r="AW128" s="13" t="n">
@@ -25255,6 +25557,9 @@
       </c>
       <c r="CF128" s="15" t="n">
         <v>1807.17</v>
+      </c>
+      <c r="CG128" s="15" t="n">
+        <v>1835.65</v>
       </c>
     </row>
     <row r="129" ht="14.25" customHeight="1">
@@ -25294,6 +25599,7 @@
       <c r="CD129" s="15" t="n"/>
       <c r="CE129" s="15" t="n"/>
       <c r="CF129" s="15" t="n"/>
+      <c r="CG129" s="15" t="n"/>
     </row>
     <row r="130" ht="14.25" customHeight="1">
       <c r="AW130" s="13" t="n">
@@ -25404,6 +25710,9 @@
       <c r="CF130" s="15" t="n">
         <v>5.5</v>
       </c>
+      <c r="CG130" s="15" t="n">
+        <v>2.7</v>
+      </c>
     </row>
     <row r="131" ht="14.25" customHeight="1">
       <c r="AW131" s="13" t="n">
@@ -25513,6 +25822,9 @@
       </c>
       <c r="CF131" s="15" t="n">
         <v>714.64</v>
+      </c>
+      <c r="CG131" s="15" t="n">
+        <v>691.47</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1">
@@ -25552,6 +25864,7 @@
       <c r="CD132" s="15" t="n"/>
       <c r="CE132" s="15" t="n"/>
       <c r="CF132" s="15" t="n"/>
+      <c r="CG132" s="15" t="n"/>
     </row>
     <row r="133" ht="14.25" customHeight="1">
       <c r="AW133" s="13" t="n">
@@ -25662,6 +25975,9 @@
       <c r="CF133" s="15" t="n">
         <v>39.54</v>
       </c>
+      <c r="CG133" s="15" t="n">
+        <v>36.31</v>
+      </c>
     </row>
     <row r="134" ht="14.25" customHeight="1">
       <c r="AW134" s="13" t="n">
@@ -25771,6 +26087,9 @@
       </c>
       <c r="CF134" s="15" t="n">
         <v>2506.83</v>
+      </c>
+      <c r="CG134" s="15" t="n">
+        <v>2420.65</v>
       </c>
     </row>
     <row r="135" ht="14.25" customHeight="1">
@@ -25810,6 +26129,7 @@
       <c r="CD135" s="15" t="n"/>
       <c r="CE135" s="15" t="n"/>
       <c r="CF135" s="15" t="n"/>
+      <c r="CG135" s="15" t="n"/>
     </row>
     <row r="136" ht="14.25" customHeight="1">
       <c r="AW136" s="13" t="n">
@@ -25920,6 +26240,9 @@
       <c r="CF136" s="15" t="n">
         <v>20.72</v>
       </c>
+      <c r="CG136" s="15" t="n">
+        <v>20.4</v>
+      </c>
     </row>
     <row r="137" ht="14.25" customHeight="1">
       <c r="AW137" s="13" t="n">
@@ -26029,6 +26352,9 @@
       </c>
       <c r="CF137" s="15" t="n">
         <v>3358.86</v>
+      </c>
+      <c r="CG137" s="15" t="n">
+        <v>3278.67</v>
       </c>
     </row>
     <row r="138">
@@ -26060,6 +26386,7 @@
       <c r="CD138" s="15" t="n"/>
       <c r="CE138" s="15" t="n"/>
       <c r="CF138" s="15" t="n"/>
+      <c r="CG138" s="15" t="n"/>
     </row>
     <row r="139">
       <c r="BE139" s="15" t="n">
@@ -26146,6 +26473,9 @@
       <c r="CF139" s="15" t="n">
         <v>4.35</v>
       </c>
+      <c r="CG139" s="15" t="n">
+        <v>4.07</v>
+      </c>
     </row>
     <row r="140">
       <c r="BE140" s="15" t="n">
@@ -26229,6 +26559,9 @@
       </c>
       <c r="CF140" s="15" t="n">
         <v>2357.2</v>
+      </c>
+      <c r="CG140" s="15" t="n">
+        <v>2287.18</v>
       </c>
     </row>
     <row r="141">
@@ -26260,6 +26593,7 @@
       <c r="CD141" s="15" t="n"/>
       <c r="CE141" s="15" t="n"/>
       <c r="CF141" s="15" t="n"/>
+      <c r="CG141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="BE142" s="15" t="n">
@@ -26346,6 +26680,9 @@
       <c r="CF142" s="15" t="n">
         <v>16.61</v>
       </c>
+      <c r="CG142" s="15" t="n">
+        <v>18.35</v>
+      </c>
     </row>
     <row r="143">
       <c r="BE143" s="15" t="n">
@@ -26431,6 +26768,9 @@
       </c>
       <c r="CF143" s="15" t="n">
         <v>5403.94</v>
+      </c>
+      <c r="CG143" s="15" t="n">
+        <v>5471.95</v>
       </c>
     </row>
     <row r="144">
@@ -26457,6 +26797,7 @@
       <c r="CD144" s="15" t="n"/>
       <c r="CE144" s="15" t="n"/>
       <c r="CF144" s="15" t="n"/>
+      <c r="CG144" s="15" t="n"/>
     </row>
     <row r="145">
       <c r="BJ145" s="15" t="n">
@@ -26528,6 +26869,9 @@
       <c r="CF145" s="15" t="n">
         <v>1.2</v>
       </c>
+      <c r="CG145" s="15" t="n">
+        <v>0.63</v>
+      </c>
     </row>
     <row r="146">
       <c r="BJ146" s="15" t="n">
@@ -26598,6 +26942,9 @@
       </c>
       <c r="CF146" s="15" t="n">
         <v>2142.8</v>
+      </c>
+      <c r="CG146" s="15" t="n">
+        <v>2113.91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-10-26 09:22:31]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CG146"/>
+  <dimension ref="A1:CH146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="51"/>
@@ -619,6 +619,7 @@
     <col width="15" customWidth="1" min="83" max="83"/>
     <col width="15" customWidth="1" min="84" max="84"/>
     <col width="15" customWidth="1" min="85" max="85"/>
+    <col width="15" customWidth="1" min="86" max="86"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -1047,6 +1048,11 @@
           <t>2026/10/22</t>
         </is>
       </c>
+      <c r="CH1" s="15" t="inlineStr">
+        <is>
+          <t>2026/10/26</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1474,6 +1480,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="CH2" s="16" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1731,6 +1742,9 @@
       <c r="CG3" s="15" t="n">
         <v>48.26</v>
       </c>
+      <c r="CH3" s="15" t="n">
+        <v>15.06</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1987,6 +2001,9 @@
       </c>
       <c r="CG4" s="15" t="n">
         <v>3658.03</v>
+      </c>
+      <c r="CH4" s="15" t="n">
+        <v>3697.52</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -2075,6 +2092,7 @@
       <c r="CE5" s="15" t="n"/>
       <c r="CF5" s="15" t="n"/>
       <c r="CG5" s="15" t="n"/>
+      <c r="CH5" s="15" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -2210,6 +2228,7 @@
       <c r="CE6" s="15" t="n"/>
       <c r="CF6" s="15" t="n"/>
       <c r="CG6" s="15" t="n"/>
+      <c r="CH6" s="15" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -2466,6 +2485,9 @@
       </c>
       <c r="CG7" s="15" t="n">
         <v>41.17</v>
+      </c>
+      <c r="CH7" s="15" t="n">
+        <v>40.05</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -2675,6 +2697,9 @@
       </c>
       <c r="CG8" s="15" t="n">
         <v>4911.33</v>
+      </c>
+      <c r="CH8" s="15" t="n">
+        <v>4989.34</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
@@ -2811,6 +2836,7 @@
       <c r="CE9" s="15" t="n"/>
       <c r="CF9" s="15" t="n"/>
       <c r="CG9" s="15" t="n"/>
+      <c r="CH9" s="15" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -3067,6 +3093,9 @@
       </c>
       <c r="CG10" s="15" t="n">
         <v>37.75</v>
+      </c>
+      <c r="CH10" s="15" t="n">
+        <v>37.23</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -3276,6 +3305,9 @@
       </c>
       <c r="CG11" s="15" t="n">
         <v>4036.3</v>
+      </c>
+      <c r="CH11" s="15" t="n">
+        <v>4103.54</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
@@ -3412,6 +3444,7 @@
       <c r="CE12" s="15" t="n"/>
       <c r="CF12" s="15" t="n"/>
       <c r="CG12" s="15" t="n"/>
+      <c r="CH12" s="15" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -3668,6 +3701,9 @@
       </c>
       <c r="CG13" s="15" t="n">
         <v>45.39</v>
+      </c>
+      <c r="CH13" s="15" t="n">
+        <v>45.09</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -3877,6 +3913,9 @@
       </c>
       <c r="CG14" s="15" t="n">
         <v>6655.25</v>
+      </c>
+      <c r="CH14" s="15" t="n">
+        <v>6712.73</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
@@ -4013,6 +4052,7 @@
       <c r="CE15" s="15" t="n"/>
       <c r="CF15" s="15" t="n"/>
       <c r="CG15" s="15" t="n"/>
+      <c r="CH15" s="15" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -4269,6 +4309,9 @@
       </c>
       <c r="CG16" s="15" t="n">
         <v>22.46</v>
+      </c>
+      <c r="CH16" s="15" t="n">
+        <v>21.37</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -4478,6 +4521,9 @@
       </c>
       <c r="CG17" s="15" t="n">
         <v>2404.7</v>
+      </c>
+      <c r="CH17" s="15" t="n">
+        <v>2304.53</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
@@ -4614,6 +4660,7 @@
       <c r="CE18" s="15" t="n"/>
       <c r="CF18" s="15" t="n"/>
       <c r="CG18" s="15" t="n"/>
+      <c r="CH18" s="15" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -4870,6 +4917,9 @@
       </c>
       <c r="CG19" s="15" t="n">
         <v>78.97</v>
+      </c>
+      <c r="CH19" s="15" t="n">
+        <v>77.92</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -5079,6 +5129,9 @@
       </c>
       <c r="CG20" s="15" t="n">
         <v>7757.17</v>
+      </c>
+      <c r="CH20" s="15" t="n">
+        <v>7623.68</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
@@ -5215,6 +5268,7 @@
       <c r="CE21" s="15" t="n"/>
       <c r="CF21" s="15" t="n"/>
       <c r="CG21" s="15" t="n"/>
+      <c r="CH21" s="15" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -5468,6 +5522,9 @@
         <v>36.34</v>
       </c>
       <c r="CG22" s="15" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="CH22" s="15" t="n">
         <v>36.34</v>
       </c>
     </row>
@@ -5678,6 +5735,9 @@
       </c>
       <c r="CG23" s="15" t="n">
         <v>73221.31</v>
+      </c>
+      <c r="CH23" s="15" t="n">
+        <v>73435.72</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
@@ -5814,6 +5874,7 @@
       <c r="CE24" s="15" t="n"/>
       <c r="CF24" s="15" t="n"/>
       <c r="CG24" s="15" t="n"/>
+      <c r="CH24" s="15" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -6069,6 +6130,9 @@
         <v>49.88</v>
       </c>
       <c r="CG25" s="15" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="CH25" s="15" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -6265,6 +6329,9 @@
       </c>
       <c r="CG26" s="15" t="n">
         <v>25382.48</v>
+      </c>
+      <c r="CH26" s="15" t="n">
+        <v>25369.8</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
@@ -6401,6 +6468,7 @@
       <c r="CE27" s="15" t="n"/>
       <c r="CF27" s="15" t="n"/>
       <c r="CG27" s="15" t="n"/>
+      <c r="CH27" s="15" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -6656,6 +6724,9 @@
         <v>92.09</v>
       </c>
       <c r="CG28" s="15" t="n">
+        <v>92.09</v>
+      </c>
+      <c r="CH28" s="15" t="n">
         <v>92.09</v>
       </c>
     </row>
@@ -6866,6 +6937,9 @@
       </c>
       <c r="CG29" s="15" t="n">
         <v>62907.84</v>
+      </c>
+      <c r="CH29" s="15" t="n">
+        <v>62189.65</v>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
@@ -7002,6 +7076,7 @@
       <c r="CE30" s="15" t="n"/>
       <c r="CF30" s="15" t="n"/>
       <c r="CG30" s="15" t="n"/>
+      <c r="CH30" s="15" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -7257,6 +7332,9 @@
         <v>97.44</v>
       </c>
       <c r="CG31" s="15" t="n">
+        <v>97.44</v>
+      </c>
+      <c r="CH31" s="15" t="n">
         <v>97.44</v>
       </c>
     </row>
@@ -7467,6 +7545,9 @@
       </c>
       <c r="CG32" s="15" t="n">
         <v>5533.77</v>
+      </c>
+      <c r="CH32" s="15" t="n">
+        <v>5469.47</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
@@ -7603,6 +7684,7 @@
       <c r="CE33" s="15" t="n"/>
       <c r="CF33" s="15" t="n"/>
       <c r="CG33" s="15" t="n"/>
+      <c r="CH33" s="15" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -7859,6 +7941,9 @@
       </c>
       <c r="CG34" s="15" t="n">
         <v>53.72</v>
+      </c>
+      <c r="CH34" s="15" t="n">
+        <v>54.3</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -8068,6 +8153,9 @@
       </c>
       <c r="CG35" s="15" t="n">
         <v>5405.75</v>
+      </c>
+      <c r="CH35" s="15" t="n">
+        <v>5465.01</v>
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
@@ -8204,6 +8292,7 @@
       <c r="CE36" s="15" t="n"/>
       <c r="CF36" s="15" t="n"/>
       <c r="CG36" s="15" t="n"/>
+      <c r="CH36" s="15" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -8460,6 +8549,9 @@
       </c>
       <c r="CG37" s="15" t="n">
         <v>66.67</v>
+      </c>
+      <c r="CH37" s="15" t="n">
+        <v>66.54000000000001</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -8669,6 +8761,9 @@
       </c>
       <c r="CG38" s="15" t="n">
         <v>11296.62</v>
+      </c>
+      <c r="CH38" s="15" t="n">
+        <v>11466.63</v>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
@@ -8805,6 +8900,7 @@
       <c r="CE39" s="15" t="n"/>
       <c r="CF39" s="15" t="n"/>
       <c r="CG39" s="15" t="n"/>
+      <c r="CH39" s="15" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -9061,6 +9157,9 @@
       </c>
       <c r="CG40" s="15" t="n">
         <v>57.34</v>
+      </c>
+      <c r="CH40" s="15" t="n">
+        <v>57.73</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -9270,6 +9369,9 @@
       </c>
       <c r="CG41" s="15" t="n">
         <v>11097.06</v>
+      </c>
+      <c r="CH41" s="15" t="n">
+        <v>10952.98</v>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
@@ -9406,6 +9508,7 @@
       <c r="CE42" s="15" t="n"/>
       <c r="CF42" s="15" t="n"/>
       <c r="CG42" s="15" t="n"/>
+      <c r="CH42" s="15" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -9662,6 +9765,9 @@
       </c>
       <c r="CG43" s="15" t="n">
         <v>55.89</v>
+      </c>
+      <c r="CH43" s="15" t="n">
+        <v>56.51</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -9871,6 +9977,9 @@
       </c>
       <c r="CG44" s="15" t="n">
         <v>3287.02</v>
+      </c>
+      <c r="CH44" s="15" t="n">
+        <v>3209.4</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
@@ -10007,6 +10116,7 @@
       <c r="CE45" s="15" t="n"/>
       <c r="CF45" s="15" t="n"/>
       <c r="CG45" s="15" t="n"/>
+      <c r="CH45" s="15" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -10263,6 +10373,9 @@
       </c>
       <c r="CG46" s="15" t="n">
         <v>70.61</v>
+      </c>
+      <c r="CH46" s="15" t="n">
+        <v>70.53</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -10472,6 +10585,9 @@
       </c>
       <c r="CG47" s="15" t="n">
         <v>7139.86</v>
+      </c>
+      <c r="CH47" s="15" t="n">
+        <v>7092</v>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
@@ -10608,6 +10724,7 @@
       <c r="CE48" s="15" t="n"/>
       <c r="CF48" s="15" t="n"/>
       <c r="CG48" s="15" t="n"/>
+      <c r="CH48" s="15" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -10864,6 +10981,9 @@
       </c>
       <c r="CG49" s="15" t="n">
         <v>15.52</v>
+      </c>
+      <c r="CH49" s="15" t="n">
+        <v>13.29</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -11073,6 +11193,9 @@
       </c>
       <c r="CG50" s="15" t="n">
         <v>31175.73</v>
+      </c>
+      <c r="CH50" s="15" t="n">
+        <v>30617.14</v>
       </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
@@ -11209,6 +11332,7 @@
       <c r="CE51" s="15" t="n"/>
       <c r="CF51" s="15" t="n"/>
       <c r="CG51" s="15" t="n"/>
+      <c r="CH51" s="15" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -11465,6 +11589,9 @@
       </c>
       <c r="CG52" s="15" t="n">
         <v>18.62</v>
+      </c>
+      <c r="CH52" s="15" t="n">
+        <v>18.17</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -11674,6 +11801,9 @@
       </c>
       <c r="CG53" s="15" t="n">
         <v>2614.37</v>
+      </c>
+      <c r="CH53" s="15" t="n">
+        <v>2679.92</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
@@ -11810,6 +11940,7 @@
       <c r="CE54" s="15" t="n"/>
       <c r="CF54" s="15" t="n"/>
       <c r="CG54" s="15" t="n"/>
+      <c r="CH54" s="15" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -12066,6 +12197,9 @@
       </c>
       <c r="CG55" s="15" t="n">
         <v>23.25</v>
+      </c>
+      <c r="CH55" s="15" t="n">
+        <v>23.46</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -12275,6 +12409,9 @@
       </c>
       <c r="CG56" s="15" t="n">
         <v>2576.9</v>
+      </c>
+      <c r="CH56" s="15" t="n">
+        <v>2638.23</v>
       </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
@@ -12411,6 +12548,7 @@
       <c r="CE57" s="15" t="n"/>
       <c r="CF57" s="15" t="n"/>
       <c r="CG57" s="15" t="n"/>
+      <c r="CH57" s="15" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -12667,6 +12805,9 @@
       </c>
       <c r="CG58" s="15" t="n">
         <v>11.43</v>
+      </c>
+      <c r="CH58" s="15" t="n">
+        <v>11.9</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -12876,6 +13017,9 @@
       </c>
       <c r="CG59" s="15" t="n">
         <v>6433.89</v>
+      </c>
+      <c r="CH59" s="15" t="n">
+        <v>6713.03</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
@@ -13012,6 +13156,7 @@
       <c r="CE60" s="15" t="n"/>
       <c r="CF60" s="15" t="n"/>
       <c r="CG60" s="15" t="n"/>
+      <c r="CH60" s="15" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -13268,6 +13413,9 @@
       </c>
       <c r="CG61" s="15" t="n">
         <v>34.96</v>
+      </c>
+      <c r="CH61" s="15" t="n">
+        <v>36.13</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -13477,6 +13625,9 @@
       </c>
       <c r="CG62" s="15" t="n">
         <v>7887.89</v>
+      </c>
+      <c r="CH62" s="15" t="n">
+        <v>8183.44</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
@@ -13613,6 +13764,7 @@
       <c r="CE63" s="15" t="n"/>
       <c r="CF63" s="15" t="n"/>
       <c r="CG63" s="15" t="n"/>
+      <c r="CH63" s="15" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -13869,6 +14021,9 @@
       </c>
       <c r="CG64" s="15" t="n">
         <v>7.82</v>
+      </c>
+      <c r="CH64" s="15" t="n">
+        <v>10.13</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -14078,6 +14233,9 @@
       </c>
       <c r="CG65" s="15" t="n">
         <v>10387.03</v>
+      </c>
+      <c r="CH65" s="15" t="n">
+        <v>10588.76</v>
       </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
@@ -14214,6 +14372,7 @@
       <c r="CE66" s="15" t="n"/>
       <c r="CF66" s="15" t="n"/>
       <c r="CG66" s="15" t="n"/>
+      <c r="CH66" s="15" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -14470,6 +14629,9 @@
       </c>
       <c r="CG67" s="15" t="n">
         <v>12.12</v>
+      </c>
+      <c r="CH67" s="15" t="n">
+        <v>14.67</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -14679,6 +14841,9 @@
       </c>
       <c r="CG68" s="15" t="n">
         <v>10541.68</v>
+      </c>
+      <c r="CH68" s="15" t="n">
+        <v>10616.81</v>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
@@ -14815,6 +14980,7 @@
       <c r="CE69" s="15" t="n"/>
       <c r="CF69" s="15" t="n"/>
       <c r="CG69" s="15" t="n"/>
+      <c r="CH69" s="15" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -15071,6 +15237,9 @@
       </c>
       <c r="CG70" s="15" t="n">
         <v>18.32</v>
+      </c>
+      <c r="CH70" s="15" t="n">
+        <v>20.89</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -15280,6 +15449,9 @@
       </c>
       <c r="CG71" s="15" t="n">
         <v>6124</v>
+      </c>
+      <c r="CH71" s="15" t="n">
+        <v>6434.81</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
@@ -15416,6 +15588,7 @@
       <c r="CE72" s="15" t="n"/>
       <c r="CF72" s="15" t="n"/>
       <c r="CG72" s="15" t="n"/>
+      <c r="CH72" s="15" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -15672,6 +15845,9 @@
       </c>
       <c r="CG73" s="15" t="n">
         <v>19.09</v>
+      </c>
+      <c r="CH73" s="15" t="n">
+        <v>21.12</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -15881,6 +16057,9 @@
       </c>
       <c r="CG74" s="15" t="n">
         <v>12248.57</v>
+      </c>
+      <c r="CH74" s="15" t="n">
+        <v>12540.33</v>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
@@ -16017,6 +16196,7 @@
       <c r="CE75" s="15" t="n"/>
       <c r="CF75" s="15" t="n"/>
       <c r="CG75" s="15" t="n"/>
+      <c r="CH75" s="15" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -16273,6 +16453,9 @@
       </c>
       <c r="CG76" s="15" t="n">
         <v>51.69</v>
+      </c>
+      <c r="CH76" s="15" t="n">
+        <v>50.84</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -16482,6 +16665,9 @@
       </c>
       <c r="CG77" s="15" t="n">
         <v>14180.18</v>
+      </c>
+      <c r="CH77" s="15" t="n">
+        <v>14317.76</v>
       </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
@@ -16618,6 +16804,7 @@
       <c r="CE78" s="15" t="n"/>
       <c r="CF78" s="15" t="n"/>
       <c r="CG78" s="15" t="n"/>
+      <c r="CH78" s="15" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -16874,6 +17061,9 @@
       </c>
       <c r="CG79" s="15" t="n">
         <v>0.85</v>
+      </c>
+      <c r="CH79" s="15" t="n">
+        <v>0.5</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -17083,6 +17273,9 @@
       </c>
       <c r="CG80" s="15" t="n">
         <v>5973.47</v>
+      </c>
+      <c r="CH80" s="15" t="n">
+        <v>6061.76</v>
       </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
@@ -17219,6 +17412,7 @@
       <c r="CE81" s="15" t="n"/>
       <c r="CF81" s="15" t="n"/>
       <c r="CG81" s="15" t="n"/>
+      <c r="CH81" s="15" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -17475,6 +17669,9 @@
       </c>
       <c r="CG82" s="15" t="n">
         <v>5.53</v>
+      </c>
+      <c r="CH82" s="15" t="n">
+        <v>5.42</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -17684,6 +17881,9 @@
       </c>
       <c r="CG83" s="15" t="n">
         <v>8481.950000000001</v>
+      </c>
+      <c r="CH83" s="15" t="n">
+        <v>8442.360000000001</v>
       </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
@@ -17820,6 +18020,7 @@
       <c r="CE84" s="15" t="n"/>
       <c r="CF84" s="15" t="n"/>
       <c r="CG84" s="15" t="n"/>
+      <c r="CH84" s="15" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -18076,6 +18277,9 @@
       </c>
       <c r="CG85" s="15" t="n">
         <v>13.06</v>
+      </c>
+      <c r="CH85" s="15" t="n">
+        <v>11.92</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -18285,6 +18489,9 @@
       </c>
       <c r="CG86" s="15" t="n">
         <v>1873.97</v>
+      </c>
+      <c r="CH86" s="15" t="n">
+        <v>2631.9</v>
       </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
@@ -18421,6 +18628,7 @@
       <c r="CE87" s="15" t="n"/>
       <c r="CF87" s="15" t="n"/>
       <c r="CG87" s="15" t="n"/>
+      <c r="CH87" s="15" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -18677,6 +18885,9 @@
       </c>
       <c r="CG88" s="15" t="n">
         <v>17.59</v>
+      </c>
+      <c r="CH88" s="15" t="n">
+        <v>15.35</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -18886,6 +19097,9 @@
       </c>
       <c r="CG89" s="15" t="n">
         <v>3793.93</v>
+      </c>
+      <c r="CH89" s="15" t="n">
+        <v>3857.53</v>
       </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
@@ -19022,6 +19236,7 @@
       <c r="CE90" s="15" t="n"/>
       <c r="CF90" s="15" t="n"/>
       <c r="CG90" s="15" t="n"/>
+      <c r="CH90" s="15" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -19278,6 +19493,9 @@
       </c>
       <c r="CG91" s="15" t="n">
         <v>14.8</v>
+      </c>
+      <c r="CH91" s="15" t="n">
+        <v>15.86</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -19487,6 +19705,9 @@
       </c>
       <c r="CG92" s="15" t="n">
         <v>8136.47</v>
+      </c>
+      <c r="CH92" s="15" t="n">
+        <v>8402.59</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
@@ -19623,6 +19844,7 @@
       <c r="CE93" s="15" t="n"/>
       <c r="CF93" s="15" t="n"/>
       <c r="CG93" s="15" t="n"/>
+      <c r="CH93" s="15" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -19879,6 +20101,9 @@
       </c>
       <c r="CG94" s="15" t="n">
         <v>2.88</v>
+      </c>
+      <c r="CH94" s="15" t="n">
+        <v>3.19</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -20088,6 +20313,9 @@
       </c>
       <c r="CG95" s="15" t="n">
         <v>1115.29</v>
+      </c>
+      <c r="CH95" s="15" t="n">
+        <v>1125.75</v>
       </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
@@ -20224,6 +20452,7 @@
       <c r="CE96" s="15" t="n"/>
       <c r="CF96" s="15" t="n"/>
       <c r="CG96" s="15" t="n"/>
+      <c r="CH96" s="15" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -20480,6 +20709,9 @@
       </c>
       <c r="CG97" s="15" t="n">
         <v>9.27</v>
+      </c>
+      <c r="CH97" s="15" t="n">
+        <v>10.68</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -20689,6 +20921,9 @@
       </c>
       <c r="CG98" s="15" t="n">
         <v>13708.46</v>
+      </c>
+      <c r="CH98" s="15" t="n">
+        <v>13885.15</v>
       </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
@@ -20825,6 +21060,7 @@
       <c r="CE99" s="15" t="n"/>
       <c r="CF99" s="15" t="n"/>
       <c r="CG99" s="15" t="n"/>
+      <c r="CH99" s="15" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -21081,6 +21317,9 @@
       </c>
       <c r="CG100" s="15" t="n">
         <v>31.19</v>
+      </c>
+      <c r="CH100" s="15" t="n">
+        <v>31.52</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -21290,6 +21529,9 @@
       </c>
       <c r="CG101" s="15" t="n">
         <v>3135.6</v>
+      </c>
+      <c r="CH101" s="15" t="n">
+        <v>3135.45</v>
       </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
@@ -21426,6 +21668,7 @@
       <c r="CE102" s="15" t="n"/>
       <c r="CF102" s="15" t="n"/>
       <c r="CG102" s="15" t="n"/>
+      <c r="CH102" s="15" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -21682,6 +21925,9 @@
       </c>
       <c r="CG103" s="15" t="n">
         <v>10.29</v>
+      </c>
+      <c r="CH103" s="15" t="n">
+        <v>11.12</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -21891,6 +22137,9 @@
       </c>
       <c r="CG104" s="15" t="n">
         <v>1884.73</v>
+      </c>
+      <c r="CH104" s="15" t="n">
+        <v>1939.87</v>
       </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
@@ -22027,6 +22276,7 @@
       <c r="CE105" s="15" t="n"/>
       <c r="CF105" s="15" t="n"/>
       <c r="CG105" s="15" t="n"/>
+      <c r="CH105" s="15" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -22283,6 +22533,9 @@
       </c>
       <c r="CG106" s="15" t="n">
         <v>5.86</v>
+      </c>
+      <c r="CH106" s="15" t="n">
+        <v>5.82</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -22492,6 +22745,9 @@
       </c>
       <c r="CG107" s="15" t="n">
         <v>2078.53</v>
+      </c>
+      <c r="CH107" s="15" t="n">
+        <v>2097.68</v>
       </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
@@ -22628,6 +22884,7 @@
       <c r="CE108" s="15" t="n"/>
       <c r="CF108" s="15" t="n"/>
       <c r="CG108" s="15" t="n"/>
+      <c r="CH108" s="15" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -22884,6 +23141,9 @@
       </c>
       <c r="CG109" s="15" t="n">
         <v>15.75</v>
+      </c>
+      <c r="CH109" s="15" t="n">
+        <v>17.14</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -23093,6 +23353,9 @@
       </c>
       <c r="CG110" s="15" t="n">
         <v>2068.3</v>
+      </c>
+      <c r="CH110" s="15" t="n">
+        <v>2106.06</v>
       </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
@@ -23229,6 +23492,7 @@
       <c r="CE111" s="15" t="n"/>
       <c r="CF111" s="15" t="n"/>
       <c r="CG111" s="15" t="n"/>
+      <c r="CH111" s="15" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -23485,6 +23749,9 @@
       </c>
       <c r="CG112" s="15" t="n">
         <v>44.36</v>
+      </c>
+      <c r="CH112" s="15" t="n">
+        <v>44.31</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -23692,6 +23959,9 @@
       </c>
       <c r="CG113" s="15" t="n">
         <v>1799.37</v>
+      </c>
+      <c r="CH113" s="15" t="n">
+        <v>1830.13</v>
       </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
@@ -23828,6 +24098,7 @@
       <c r="CE114" s="15" t="n"/>
       <c r="CF114" s="15" t="n"/>
       <c r="CG114" s="15" t="n"/>
+      <c r="CH114" s="15" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -24084,6 +24355,9 @@
       </c>
       <c r="CG115" s="15" t="n">
         <v>16.61</v>
+      </c>
+      <c r="CH115" s="15" t="n">
+        <v>17.75</v>
       </c>
     </row>
     <row r="116" ht="14.25" customHeight="1">
@@ -24278,6 +24552,9 @@
       </c>
       <c r="CG116" s="15" t="n">
         <v>8531.5</v>
+      </c>
+      <c r="CH116" s="15" t="n">
+        <v>8786.73</v>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1">
@@ -24369,6 +24646,7 @@
       <c r="CE117" s="15" t="n"/>
       <c r="CF117" s="15" t="n"/>
       <c r="CG117" s="15" t="n"/>
+      <c r="CH117" s="15" t="n"/>
     </row>
     <row r="118" ht="14.25" customHeight="1">
       <c r="P118" s="13" t="n">
@@ -24581,6 +24859,9 @@
       <c r="CG118" s="15" t="n">
         <v>58.19</v>
       </c>
+      <c r="CH118" s="15" t="n">
+        <v>58.26</v>
+      </c>
     </row>
     <row r="119" ht="14.25" customHeight="1">
       <c r="Y119" s="13" t="n">
@@ -24765,6 +25046,9 @@
       </c>
       <c r="CG119" s="15" t="n">
         <v>10204.26</v>
+      </c>
+      <c r="CH119" s="15" t="n">
+        <v>10146.48</v>
       </c>
     </row>
     <row r="120" ht="14.25" customHeight="1">
@@ -24805,6 +25089,7 @@
       <c r="CE120" s="15" t="n"/>
       <c r="CF120" s="15" t="n"/>
       <c r="CG120" s="15" t="n"/>
+      <c r="CH120" s="15" t="n"/>
     </row>
     <row r="121" ht="14.25" customHeight="1">
       <c r="AW121" s="13" t="n">
@@ -24918,6 +25203,9 @@
       <c r="CG121" s="15" t="n">
         <v>22.17</v>
       </c>
+      <c r="CH121" s="15" t="n">
+        <v>21.11</v>
+      </c>
     </row>
     <row r="122" ht="14.25" customHeight="1">
       <c r="AW122" s="13" t="n">
@@ -25030,6 +25318,9 @@
       </c>
       <c r="CG122" s="15" t="n">
         <v>1161.26</v>
+      </c>
+      <c r="CH122" s="15" t="n">
+        <v>1157.63</v>
       </c>
     </row>
     <row r="123" ht="14.25" customHeight="1">
@@ -25070,6 +25361,7 @@
       <c r="CE123" s="15" t="n"/>
       <c r="CF123" s="15" t="n"/>
       <c r="CG123" s="15" t="n"/>
+      <c r="CH123" s="15" t="n"/>
     </row>
     <row r="124" ht="14.25" customHeight="1">
       <c r="AW124" s="13" t="n">
@@ -25183,6 +25475,9 @@
       <c r="CG124" s="15" t="n">
         <v>36.2</v>
       </c>
+      <c r="CH124" s="15" t="n">
+        <v>36.78</v>
+      </c>
     </row>
     <row r="125" ht="14.25" customHeight="1">
       <c r="AW125" s="13" t="n">
@@ -25295,6 +25590,9 @@
       </c>
       <c r="CG125" s="15" t="n">
         <v>10518.38</v>
+      </c>
+      <c r="CH125" s="15" t="n">
+        <v>10655.96</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1">
@@ -25335,6 +25633,7 @@
       <c r="CE126" s="15" t="n"/>
       <c r="CF126" s="15" t="n"/>
       <c r="CG126" s="15" t="n"/>
+      <c r="CH126" s="15" t="n"/>
     </row>
     <row r="127" ht="14.25" customHeight="1">
       <c r="AW127" s="13" t="n">
@@ -25448,6 +25747,9 @@
       <c r="CG127" s="15" t="n">
         <v>4.81</v>
       </c>
+      <c r="CH127" s="15" t="n">
+        <v>4.64</v>
+      </c>
     </row>
     <row r="128" ht="14.25" customHeight="1">
       <c r="AW128" s="13" t="n">
@@ -25560,6 +25862,9 @@
       </c>
       <c r="CG128" s="15" t="n">
         <v>1835.65</v>
+      </c>
+      <c r="CH128" s="15" t="n">
+        <v>1818.43</v>
       </c>
     </row>
     <row r="129" ht="14.25" customHeight="1">
@@ -25600,6 +25905,7 @@
       <c r="CE129" s="15" t="n"/>
       <c r="CF129" s="15" t="n"/>
       <c r="CG129" s="15" t="n"/>
+      <c r="CH129" s="15" t="n"/>
     </row>
     <row r="130" ht="14.25" customHeight="1">
       <c r="AW130" s="13" t="n">
@@ -25713,6 +26019,9 @@
       <c r="CG130" s="15" t="n">
         <v>2.7</v>
       </c>
+      <c r="CH130" s="15" t="n">
+        <v>3.34</v>
+      </c>
     </row>
     <row r="131" ht="14.25" customHeight="1">
       <c r="AW131" s="13" t="n">
@@ -25825,6 +26134,9 @@
       </c>
       <c r="CG131" s="15" t="n">
         <v>691.47</v>
+      </c>
+      <c r="CH131" s="15" t="n">
+        <v>707.62</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1">
@@ -25865,6 +26177,7 @@
       <c r="CE132" s="15" t="n"/>
       <c r="CF132" s="15" t="n"/>
       <c r="CG132" s="15" t="n"/>
+      <c r="CH132" s="15" t="n"/>
     </row>
     <row r="133" ht="14.25" customHeight="1">
       <c r="AW133" s="13" t="n">
@@ -25978,6 +26291,9 @@
       <c r="CG133" s="15" t="n">
         <v>36.31</v>
       </c>
+      <c r="CH133" s="15" t="n">
+        <v>34.84</v>
+      </c>
     </row>
     <row r="134" ht="14.25" customHeight="1">
       <c r="AW134" s="13" t="n">
@@ -26090,6 +26406,9 @@
       </c>
       <c r="CG134" s="15" t="n">
         <v>2420.65</v>
+      </c>
+      <c r="CH134" s="15" t="n">
+        <v>2379.81</v>
       </c>
     </row>
     <row r="135" ht="14.25" customHeight="1">
@@ -26130,6 +26449,7 @@
       <c r="CE135" s="15" t="n"/>
       <c r="CF135" s="15" t="n"/>
       <c r="CG135" s="15" t="n"/>
+      <c r="CH135" s="15" t="n"/>
     </row>
     <row r="136" ht="14.25" customHeight="1">
       <c r="AW136" s="13" t="n">
@@ -26243,6 +26563,9 @@
       <c r="CG136" s="15" t="n">
         <v>20.4</v>
       </c>
+      <c r="CH136" s="15" t="n">
+        <v>20.14</v>
+      </c>
     </row>
     <row r="137" ht="14.25" customHeight="1">
       <c r="AW137" s="13" t="n">
@@ -26355,6 +26678,9 @@
       </c>
       <c r="CG137" s="15" t="n">
         <v>3278.67</v>
+      </c>
+      <c r="CH137" s="15" t="n">
+        <v>3287.91</v>
       </c>
     </row>
     <row r="138">
@@ -26387,6 +26713,7 @@
       <c r="CE138" s="15" t="n"/>
       <c r="CF138" s="15" t="n"/>
       <c r="CG138" s="15" t="n"/>
+      <c r="CH138" s="15" t="n"/>
     </row>
     <row r="139">
       <c r="BE139" s="15" t="n">
@@ -26476,6 +26803,9 @@
       <c r="CG139" s="15" t="n">
         <v>4.07</v>
       </c>
+      <c r="CH139" s="15" t="n">
+        <v>3.2</v>
+      </c>
     </row>
     <row r="140">
       <c r="BE140" s="15" t="n">
@@ -26562,6 +26892,9 @@
       </c>
       <c r="CG140" s="15" t="n">
         <v>2287.18</v>
+      </c>
+      <c r="CH140" s="15" t="n">
+        <v>2359.67</v>
       </c>
     </row>
     <row r="141">
@@ -26594,6 +26927,7 @@
       <c r="CE141" s="15" t="n"/>
       <c r="CF141" s="15" t="n"/>
       <c r="CG141" s="15" t="n"/>
+      <c r="CH141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="BE142" s="15" t="n">
@@ -26683,6 +27017,9 @@
       <c r="CG142" s="15" t="n">
         <v>18.35</v>
       </c>
+      <c r="CH142" s="15" t="n">
+        <v>18.81</v>
+      </c>
     </row>
     <row r="143">
       <c r="BE143" s="15" t="n">
@@ -26771,6 +27108,9 @@
       </c>
       <c r="CG143" s="15" t="n">
         <v>5471.95</v>
+      </c>
+      <c r="CH143" s="15" t="n">
+        <v>5451.55</v>
       </c>
     </row>
     <row r="144">
@@ -26798,6 +27138,7 @@
       <c r="CE144" s="15" t="n"/>
       <c r="CF144" s="15" t="n"/>
       <c r="CG144" s="15" t="n"/>
+      <c r="CH144" s="15" t="n"/>
     </row>
     <row r="145">
       <c r="BJ145" s="15" t="n">
@@ -26872,6 +27213,9 @@
       <c r="CG145" s="15" t="n">
         <v>0.63</v>
       </c>
+      <c r="CH145" s="15" t="n">
+        <v>0.65</v>
+      </c>
     </row>
     <row r="146">
       <c r="BJ146" s="15" t="n">
@@ -26945,6 +27289,9 @@
       </c>
       <c r="CG146" s="15" t="n">
         <v>2113.91</v>
+      </c>
+      <c r="CH146" s="15" t="n">
+        <v>2112.85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-10-29 10:25:53]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CH146"/>
+  <dimension ref="A1:CI146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="51"/>
@@ -620,6 +620,7 @@
     <col width="15" customWidth="1" min="84" max="84"/>
     <col width="15" customWidth="1" min="85" max="85"/>
     <col width="15" customWidth="1" min="86" max="86"/>
+    <col width="15" customWidth="1" min="87" max="87"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -1053,6 +1054,11 @@
           <t>2026/10/26</t>
         </is>
       </c>
+      <c r="CI1" s="15" t="inlineStr">
+        <is>
+          <t>2026/10/29</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1485,6 +1491,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="CI2" s="16" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1745,6 +1756,9 @@
       <c r="CH3" s="15" t="n">
         <v>15.06</v>
       </c>
+      <c r="CI3" s="15" t="n">
+        <v>45.41</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -2004,6 +2018,9 @@
       </c>
       <c r="CH4" s="15" t="n">
         <v>3697.52</v>
+      </c>
+      <c r="CI4" s="15" t="n">
+        <v>3651.43</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -2093,6 +2110,7 @@
       <c r="CF5" s="15" t="n"/>
       <c r="CG5" s="15" t="n"/>
       <c r="CH5" s="15" t="n"/>
+      <c r="CI5" s="15" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -2229,6 +2247,7 @@
       <c r="CF6" s="15" t="n"/>
       <c r="CG6" s="15" t="n"/>
       <c r="CH6" s="15" t="n"/>
+      <c r="CI6" s="15" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -2488,6 +2507,9 @@
       </c>
       <c r="CH7" s="15" t="n">
         <v>40.05</v>
+      </c>
+      <c r="CI7" s="15" t="n">
+        <v>39.95</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -2700,6 +2722,9 @@
       </c>
       <c r="CH8" s="15" t="n">
         <v>4989.34</v>
+      </c>
+      <c r="CI8" s="15" t="n">
+        <v>4884.9</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
@@ -2837,6 +2862,7 @@
       <c r="CF9" s="15" t="n"/>
       <c r="CG9" s="15" t="n"/>
       <c r="CH9" s="15" t="n"/>
+      <c r="CI9" s="15" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -3096,6 +3122,9 @@
       </c>
       <c r="CH10" s="15" t="n">
         <v>37.23</v>
+      </c>
+      <c r="CI10" s="15" t="n">
+        <v>37.97</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -3308,6 +3337,9 @@
       </c>
       <c r="CH11" s="15" t="n">
         <v>4103.54</v>
+      </c>
+      <c r="CI11" s="15" t="n">
+        <v>4041.84</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
@@ -3445,6 +3477,7 @@
       <c r="CF12" s="15" t="n"/>
       <c r="CG12" s="15" t="n"/>
       <c r="CH12" s="15" t="n"/>
+      <c r="CI12" s="15" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -3704,6 +3737,9 @@
       </c>
       <c r="CH13" s="15" t="n">
         <v>45.09</v>
+      </c>
+      <c r="CI13" s="15" t="n">
+        <v>38</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -3916,6 +3952,9 @@
       </c>
       <c r="CH14" s="15" t="n">
         <v>6712.73</v>
+      </c>
+      <c r="CI14" s="15" t="n">
+        <v>6453.72</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
@@ -4053,6 +4092,7 @@
       <c r="CF15" s="15" t="n"/>
       <c r="CG15" s="15" t="n"/>
       <c r="CH15" s="15" t="n"/>
+      <c r="CI15" s="15" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -4312,6 +4352,9 @@
       </c>
       <c r="CH16" s="15" t="n">
         <v>21.37</v>
+      </c>
+      <c r="CI16" s="15" t="n">
+        <v>21.73</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -4524,6 +4567,9 @@
       </c>
       <c r="CH17" s="15" t="n">
         <v>2304.53</v>
+      </c>
+      <c r="CI17" s="15" t="n">
+        <v>2271.08</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
@@ -4661,6 +4707,7 @@
       <c r="CF18" s="15" t="n"/>
       <c r="CG18" s="15" t="n"/>
       <c r="CH18" s="15" t="n"/>
+      <c r="CI18" s="15" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -4920,6 +4967,9 @@
       </c>
       <c r="CH19" s="15" t="n">
         <v>77.92</v>
+      </c>
+      <c r="CI19" s="15" t="n">
+        <v>78.25</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -5132,6 +5182,9 @@
       </c>
       <c r="CH20" s="15" t="n">
         <v>7623.68</v>
+      </c>
+      <c r="CI20" s="15" t="n">
+        <v>7743.98</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
@@ -5269,6 +5322,7 @@
       <c r="CF21" s="15" t="n"/>
       <c r="CG21" s="15" t="n"/>
       <c r="CH21" s="15" t="n"/>
+      <c r="CI21" s="15" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -5525,6 +5579,9 @@
         <v>36.34</v>
       </c>
       <c r="CH22" s="15" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="CI22" s="15" t="n">
         <v>36.34</v>
       </c>
     </row>
@@ -5738,6 +5795,9 @@
       </c>
       <c r="CH23" s="15" t="n">
         <v>73435.72</v>
+      </c>
+      <c r="CI23" s="15" t="n">
+        <v>74151.03999999999</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
@@ -5875,6 +5935,7 @@
       <c r="CF24" s="15" t="n"/>
       <c r="CG24" s="15" t="n"/>
       <c r="CH24" s="15" t="n"/>
+      <c r="CI24" s="15" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -6133,6 +6194,9 @@
         <v>49.88</v>
       </c>
       <c r="CH25" s="15" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="CI25" s="15" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -6332,6 +6396,9 @@
       </c>
       <c r="CH26" s="15" t="n">
         <v>25369.8</v>
+      </c>
+      <c r="CI26" s="15" t="n">
+        <v>25987.92</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
@@ -6469,6 +6536,7 @@
       <c r="CF27" s="15" t="n"/>
       <c r="CG27" s="15" t="n"/>
       <c r="CH27" s="15" t="n"/>
+      <c r="CI27" s="15" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -6727,6 +6795,9 @@
         <v>92.09</v>
       </c>
       <c r="CH28" s="15" t="n">
+        <v>92.09</v>
+      </c>
+      <c r="CI28" s="15" t="n">
         <v>92.09</v>
       </c>
     </row>
@@ -6940,6 +7011,9 @@
       </c>
       <c r="CH29" s="15" t="n">
         <v>62189.65</v>
+      </c>
+      <c r="CI29" s="15" t="n">
+        <v>64659.47</v>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
@@ -7077,6 +7151,7 @@
       <c r="CF30" s="15" t="n"/>
       <c r="CG30" s="15" t="n"/>
       <c r="CH30" s="15" t="n"/>
+      <c r="CI30" s="15" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -7335,6 +7410,9 @@
         <v>97.44</v>
       </c>
       <c r="CH31" s="15" t="n">
+        <v>97.44</v>
+      </c>
+      <c r="CI31" s="15" t="n">
         <v>97.44</v>
       </c>
     </row>
@@ -7548,6 +7626,9 @@
       </c>
       <c r="CH32" s="15" t="n">
         <v>5469.47</v>
+      </c>
+      <c r="CI32" s="15" t="n">
+        <v>5937.66</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
@@ -7685,6 +7766,7 @@
       <c r="CF33" s="15" t="n"/>
       <c r="CG33" s="15" t="n"/>
       <c r="CH33" s="15" t="n"/>
+      <c r="CI33" s="15" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -7944,6 +8026,9 @@
       </c>
       <c r="CH34" s="15" t="n">
         <v>54.3</v>
+      </c>
+      <c r="CI34" s="15" t="n">
+        <v>54.01</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -8156,6 +8241,9 @@
       </c>
       <c r="CH35" s="15" t="n">
         <v>5465.01</v>
+      </c>
+      <c r="CI35" s="15" t="n">
+        <v>5546.77</v>
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
@@ -8293,6 +8381,7 @@
       <c r="CF36" s="15" t="n"/>
       <c r="CG36" s="15" t="n"/>
       <c r="CH36" s="15" t="n"/>
+      <c r="CI36" s="15" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -8552,6 +8641,9 @@
       </c>
       <c r="CH37" s="15" t="n">
         <v>66.54000000000001</v>
+      </c>
+      <c r="CI37" s="15" t="n">
+        <v>66.90000000000001</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -8764,6 +8856,9 @@
       </c>
       <c r="CH38" s="15" t="n">
         <v>11466.63</v>
+      </c>
+      <c r="CI38" s="15" t="n">
+        <v>11412.48</v>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
@@ -8901,6 +8996,7 @@
       <c r="CF39" s="15" t="n"/>
       <c r="CG39" s="15" t="n"/>
       <c r="CH39" s="15" t="n"/>
+      <c r="CI39" s="15" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -9160,6 +9256,9 @@
       </c>
       <c r="CH40" s="15" t="n">
         <v>57.73</v>
+      </c>
+      <c r="CI40" s="15" t="n">
+        <v>55.81</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -9372,6 +9471,9 @@
       </c>
       <c r="CH41" s="15" t="n">
         <v>10952.98</v>
+      </c>
+      <c r="CI41" s="15" t="n">
+        <v>11306.19</v>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
@@ -9509,6 +9611,7 @@
       <c r="CF42" s="15" t="n"/>
       <c r="CG42" s="15" t="n"/>
       <c r="CH42" s="15" t="n"/>
+      <c r="CI42" s="15" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -9768,6 +9871,9 @@
       </c>
       <c r="CH43" s="15" t="n">
         <v>56.51</v>
+      </c>
+      <c r="CI43" s="15" t="n">
+        <v>56.77</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -9980,6 +10086,9 @@
       </c>
       <c r="CH44" s="15" t="n">
         <v>3209.4</v>
+      </c>
+      <c r="CI44" s="15" t="n">
+        <v>3310.6</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
@@ -10117,6 +10226,7 @@
       <c r="CF45" s="15" t="n"/>
       <c r="CG45" s="15" t="n"/>
       <c r="CH45" s="15" t="n"/>
+      <c r="CI45" s="15" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -10376,6 +10486,9 @@
       </c>
       <c r="CH46" s="15" t="n">
         <v>70.53</v>
+      </c>
+      <c r="CI46" s="15" t="n">
+        <v>69.7</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -10588,6 +10701,9 @@
       </c>
       <c r="CH47" s="15" t="n">
         <v>7092</v>
+      </c>
+      <c r="CI47" s="15" t="n">
+        <v>7268.36</v>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
@@ -10725,6 +10841,7 @@
       <c r="CF48" s="15" t="n"/>
       <c r="CG48" s="15" t="n"/>
       <c r="CH48" s="15" t="n"/>
+      <c r="CI48" s="15" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -10984,6 +11101,9 @@
       </c>
       <c r="CH49" s="15" t="n">
         <v>13.29</v>
+      </c>
+      <c r="CI49" s="15" t="n">
+        <v>13.16</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -11195,6 +11315,9 @@
         <v>31175.73</v>
       </c>
       <c r="CH50" s="15" t="n">
+        <v>30617.14</v>
+      </c>
+      <c r="CI50" s="15" t="n">
         <v>30617.14</v>
       </c>
     </row>
@@ -11333,6 +11456,7 @@
       <c r="CF51" s="15" t="n"/>
       <c r="CG51" s="15" t="n"/>
       <c r="CH51" s="15" t="n"/>
+      <c r="CI51" s="15" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -11592,6 +11716,9 @@
       </c>
       <c r="CH52" s="15" t="n">
         <v>18.17</v>
+      </c>
+      <c r="CI52" s="15" t="n">
+        <v>14.77</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -11804,6 +11931,9 @@
       </c>
       <c r="CH53" s="15" t="n">
         <v>2679.92</v>
+      </c>
+      <c r="CI53" s="15" t="n">
+        <v>2551.72</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
@@ -11941,6 +12071,7 @@
       <c r="CF54" s="15" t="n"/>
       <c r="CG54" s="15" t="n"/>
       <c r="CH54" s="15" t="n"/>
+      <c r="CI54" s="15" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -12200,6 +12331,9 @@
       </c>
       <c r="CH55" s="15" t="n">
         <v>23.46</v>
+      </c>
+      <c r="CI55" s="15" t="n">
+        <v>19.18</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -12412,6 +12546,9 @@
       </c>
       <c r="CH56" s="15" t="n">
         <v>2638.23</v>
+      </c>
+      <c r="CI56" s="15" t="n">
+        <v>2517.59</v>
       </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
@@ -12549,6 +12686,7 @@
       <c r="CF57" s="15" t="n"/>
       <c r="CG57" s="15" t="n"/>
       <c r="CH57" s="15" t="n"/>
+      <c r="CI57" s="15" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -12808,6 +12946,9 @@
       </c>
       <c r="CH58" s="15" t="n">
         <v>11.9</v>
+      </c>
+      <c r="CI58" s="15" t="n">
+        <v>6.61</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -13020,6 +13161,9 @@
       </c>
       <c r="CH59" s="15" t="n">
         <v>6713.03</v>
+      </c>
+      <c r="CI59" s="15" t="n">
+        <v>6542.52</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
@@ -13157,6 +13301,7 @@
       <c r="CF60" s="15" t="n"/>
       <c r="CG60" s="15" t="n"/>
       <c r="CH60" s="15" t="n"/>
+      <c r="CI60" s="15" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -13416,6 +13561,9 @@
       </c>
       <c r="CH61" s="15" t="n">
         <v>36.13</v>
+      </c>
+      <c r="CI61" s="15" t="n">
+        <v>19.3</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -13628,6 +13776,9 @@
       </c>
       <c r="CH62" s="15" t="n">
         <v>8183.44</v>
+      </c>
+      <c r="CI62" s="15" t="n">
+        <v>8057.83</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
@@ -13765,6 +13916,7 @@
       <c r="CF63" s="15" t="n"/>
       <c r="CG63" s="15" t="n"/>
       <c r="CH63" s="15" t="n"/>
+      <c r="CI63" s="15" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -14024,6 +14176,9 @@
       </c>
       <c r="CH64" s="15" t="n">
         <v>10.13</v>
+      </c>
+      <c r="CI64" s="15" t="n">
+        <v>10.42</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -14236,6 +14391,9 @@
       </c>
       <c r="CH65" s="15" t="n">
         <v>10588.76</v>
+      </c>
+      <c r="CI65" s="15" t="n">
+        <v>10579.02</v>
       </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
@@ -14373,6 +14531,7 @@
       <c r="CF66" s="15" t="n"/>
       <c r="CG66" s="15" t="n"/>
       <c r="CH66" s="15" t="n"/>
+      <c r="CI66" s="15" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -14632,6 +14791,9 @@
       </c>
       <c r="CH67" s="15" t="n">
         <v>14.67</v>
+      </c>
+      <c r="CI67" s="15" t="n">
+        <v>18.11</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -14844,6 +15006,9 @@
       </c>
       <c r="CH68" s="15" t="n">
         <v>10616.81</v>
+      </c>
+      <c r="CI68" s="15" t="n">
+        <v>10491.44</v>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
@@ -14981,6 +15146,7 @@
       <c r="CF69" s="15" t="n"/>
       <c r="CG69" s="15" t="n"/>
       <c r="CH69" s="15" t="n"/>
+      <c r="CI69" s="15" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -15240,6 +15406,9 @@
       </c>
       <c r="CH70" s="15" t="n">
         <v>20.89</v>
+      </c>
+      <c r="CI70" s="15" t="n">
+        <v>20.16</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -15452,6 +15621,9 @@
       </c>
       <c r="CH71" s="15" t="n">
         <v>6434.81</v>
+      </c>
+      <c r="CI71" s="15" t="n">
+        <v>6312.68</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
@@ -15589,6 +15761,7 @@
       <c r="CF72" s="15" t="n"/>
       <c r="CG72" s="15" t="n"/>
       <c r="CH72" s="15" t="n"/>
+      <c r="CI72" s="15" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -15848,6 +16021,9 @@
       </c>
       <c r="CH73" s="15" t="n">
         <v>21.12</v>
+      </c>
+      <c r="CI73" s="15" t="n">
+        <v>19.11</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -16060,6 +16236,9 @@
       </c>
       <c r="CH74" s="15" t="n">
         <v>12540.33</v>
+      </c>
+      <c r="CI74" s="15" t="n">
+        <v>12389.55</v>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
@@ -16197,6 +16376,7 @@
       <c r="CF75" s="15" t="n"/>
       <c r="CG75" s="15" t="n"/>
       <c r="CH75" s="15" t="n"/>
+      <c r="CI75" s="15" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -16456,6 +16636,9 @@
       </c>
       <c r="CH76" s="15" t="n">
         <v>50.84</v>
+      </c>
+      <c r="CI76" s="15" t="n">
+        <v>48.64</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -16668,6 +16851,9 @@
       </c>
       <c r="CH77" s="15" t="n">
         <v>14317.76</v>
+      </c>
+      <c r="CI77" s="15" t="n">
+        <v>15569.82</v>
       </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
@@ -16805,6 +16991,7 @@
       <c r="CF78" s="15" t="n"/>
       <c r="CG78" s="15" t="n"/>
       <c r="CH78" s="15" t="n"/>
+      <c r="CI78" s="15" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -17064,6 +17251,9 @@
       </c>
       <c r="CH79" s="15" t="n">
         <v>0.5</v>
+      </c>
+      <c r="CI79" s="15" t="n">
+        <v>0.46</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -17275,6 +17465,9 @@
         <v>5973.47</v>
       </c>
       <c r="CH80" s="15" t="n">
+        <v>6061.76</v>
+      </c>
+      <c r="CI80" s="15" t="n">
         <v>6061.76</v>
       </c>
     </row>
@@ -17413,6 +17606,7 @@
       <c r="CF81" s="15" t="n"/>
       <c r="CG81" s="15" t="n"/>
       <c r="CH81" s="15" t="n"/>
+      <c r="CI81" s="15" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -17672,6 +17866,9 @@
       </c>
       <c r="CH82" s="15" t="n">
         <v>5.42</v>
+      </c>
+      <c r="CI82" s="15" t="n">
+        <v>5.12</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -17884,6 +18081,9 @@
       </c>
       <c r="CH83" s="15" t="n">
         <v>8442.360000000001</v>
+      </c>
+      <c r="CI83" s="15" t="n">
+        <v>8340.09</v>
       </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
@@ -18021,6 +18221,7 @@
       <c r="CF84" s="15" t="n"/>
       <c r="CG84" s="15" t="n"/>
       <c r="CH84" s="15" t="n"/>
+      <c r="CI84" s="15" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -18280,6 +18481,9 @@
       </c>
       <c r="CH85" s="15" t="n">
         <v>11.92</v>
+      </c>
+      <c r="CI85" s="15" t="n">
+        <v>11.95</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -18492,6 +18696,9 @@
       </c>
       <c r="CH86" s="15" t="n">
         <v>2631.9</v>
+      </c>
+      <c r="CI86" s="15" t="n">
+        <v>1859</v>
       </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
@@ -18629,6 +18836,7 @@
       <c r="CF87" s="15" t="n"/>
       <c r="CG87" s="15" t="n"/>
       <c r="CH87" s="15" t="n"/>
+      <c r="CI87" s="15" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -18888,6 +19096,9 @@
       </c>
       <c r="CH88" s="15" t="n">
         <v>15.35</v>
+      </c>
+      <c r="CI88" s="15" t="n">
+        <v>15.3</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -19100,6 +19311,9 @@
       </c>
       <c r="CH89" s="15" t="n">
         <v>3857.53</v>
+      </c>
+      <c r="CI89" s="15" t="n">
+        <v>5075.31</v>
       </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
@@ -19237,6 +19451,7 @@
       <c r="CF90" s="15" t="n"/>
       <c r="CG90" s="15" t="n"/>
       <c r="CH90" s="15" t="n"/>
+      <c r="CI90" s="15" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -19496,6 +19711,9 @@
       </c>
       <c r="CH91" s="15" t="n">
         <v>15.86</v>
+      </c>
+      <c r="CI91" s="15" t="n">
+        <v>7.39</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -19708,6 +19926,9 @@
       </c>
       <c r="CH92" s="15" t="n">
         <v>8402.59</v>
+      </c>
+      <c r="CI92" s="15" t="n">
+        <v>8183.56</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
@@ -19845,6 +20066,7 @@
       <c r="CF93" s="15" t="n"/>
       <c r="CG93" s="15" t="n"/>
       <c r="CH93" s="15" t="n"/>
+      <c r="CI93" s="15" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -20104,6 +20326,9 @@
       </c>
       <c r="CH94" s="15" t="n">
         <v>3.19</v>
+      </c>
+      <c r="CI94" s="15" t="n">
+        <v>3.32</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -20316,6 +20541,9 @@
       </c>
       <c r="CH95" s="15" t="n">
         <v>1125.75</v>
+      </c>
+      <c r="CI95" s="15" t="n">
+        <v>1158.98</v>
       </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
@@ -20453,6 +20681,7 @@
       <c r="CF96" s="15" t="n"/>
       <c r="CG96" s="15" t="n"/>
       <c r="CH96" s="15" t="n"/>
+      <c r="CI96" s="15" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -20712,6 +20941,9 @@
       </c>
       <c r="CH97" s="15" t="n">
         <v>10.68</v>
+      </c>
+      <c r="CI97" s="15" t="n">
+        <v>9.65</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -20924,6 +21156,9 @@
       </c>
       <c r="CH98" s="15" t="n">
         <v>13885.15</v>
+      </c>
+      <c r="CI98" s="15" t="n">
+        <v>13784.37</v>
       </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
@@ -21061,6 +21296,7 @@
       <c r="CF99" s="15" t="n"/>
       <c r="CG99" s="15" t="n"/>
       <c r="CH99" s="15" t="n"/>
+      <c r="CI99" s="15" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -21320,6 +21556,9 @@
       </c>
       <c r="CH100" s="15" t="n">
         <v>31.52</v>
+      </c>
+      <c r="CI100" s="15" t="n">
+        <v>19.56</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -21532,6 +21771,9 @@
       </c>
       <c r="CH101" s="15" t="n">
         <v>3135.45</v>
+      </c>
+      <c r="CI101" s="15" t="n">
+        <v>3047.65</v>
       </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
@@ -21669,6 +21911,7 @@
       <c r="CF102" s="15" t="n"/>
       <c r="CG102" s="15" t="n"/>
       <c r="CH102" s="15" t="n"/>
+      <c r="CI102" s="15" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -21928,6 +22171,9 @@
       </c>
       <c r="CH103" s="15" t="n">
         <v>11.12</v>
+      </c>
+      <c r="CI103" s="15" t="n">
+        <v>9.210000000000001</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -22140,6 +22386,9 @@
       </c>
       <c r="CH104" s="15" t="n">
         <v>1939.87</v>
+      </c>
+      <c r="CI104" s="15" t="n">
+        <v>1875.33</v>
       </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
@@ -22277,6 +22526,7 @@
       <c r="CF105" s="15" t="n"/>
       <c r="CG105" s="15" t="n"/>
       <c r="CH105" s="15" t="n"/>
+      <c r="CI105" s="15" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -22536,6 +22786,9 @@
       </c>
       <c r="CH106" s="15" t="n">
         <v>5.82</v>
+      </c>
+      <c r="CI106" s="15" t="n">
+        <v>4.84</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -22748,6 +23001,9 @@
       </c>
       <c r="CH107" s="15" t="n">
         <v>2097.68</v>
+      </c>
+      <c r="CI107" s="15" t="n">
+        <v>2037.53</v>
       </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
@@ -22885,6 +23141,7 @@
       <c r="CF108" s="15" t="n"/>
       <c r="CG108" s="15" t="n"/>
       <c r="CH108" s="15" t="n"/>
+      <c r="CI108" s="15" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -23144,6 +23401,9 @@
       </c>
       <c r="CH109" s="15" t="n">
         <v>17.14</v>
+      </c>
+      <c r="CI109" s="15" t="n">
+        <v>16.65</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -23356,6 +23616,9 @@
       </c>
       <c r="CH110" s="15" t="n">
         <v>2106.06</v>
+      </c>
+      <c r="CI110" s="15" t="n">
+        <v>2047.93</v>
       </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
@@ -23493,6 +23756,7 @@
       <c r="CF111" s="15" t="n"/>
       <c r="CG111" s="15" t="n"/>
       <c r="CH111" s="15" t="n"/>
+      <c r="CI111" s="15" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -23752,6 +24016,9 @@
       </c>
       <c r="CH112" s="15" t="n">
         <v>44.31</v>
+      </c>
+      <c r="CI112" s="15" t="n">
+        <v>28.75</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -23962,6 +24229,9 @@
       </c>
       <c r="CH113" s="15" t="n">
         <v>1830.13</v>
+      </c>
+      <c r="CI113" s="15" t="n">
+        <v>1767.7</v>
       </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
@@ -24099,6 +24369,7 @@
       <c r="CF114" s="15" t="n"/>
       <c r="CG114" s="15" t="n"/>
       <c r="CH114" s="15" t="n"/>
+      <c r="CI114" s="15" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -24358,6 +24629,9 @@
       </c>
       <c r="CH115" s="15" t="n">
         <v>17.75</v>
+      </c>
+      <c r="CI115" s="15" t="n">
+        <v>16.8</v>
       </c>
     </row>
     <row r="116" ht="14.25" customHeight="1">
@@ -24555,6 +24829,9 @@
       </c>
       <c r="CH116" s="15" t="n">
         <v>8786.73</v>
+      </c>
+      <c r="CI116" s="15" t="n">
+        <v>8693.709999999999</v>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1">
@@ -24647,6 +24924,7 @@
       <c r="CF117" s="15" t="n"/>
       <c r="CG117" s="15" t="n"/>
       <c r="CH117" s="15" t="n"/>
+      <c r="CI117" s="15" t="n"/>
     </row>
     <row r="118" ht="14.25" customHeight="1">
       <c r="P118" s="13" t="n">
@@ -24862,6 +25140,9 @@
       <c r="CH118" s="15" t="n">
         <v>58.26</v>
       </c>
+      <c r="CI118" s="15" t="n">
+        <v>52.67</v>
+      </c>
     </row>
     <row r="119" ht="14.25" customHeight="1">
       <c r="Y119" s="13" t="n">
@@ -25049,6 +25330,9 @@
       </c>
       <c r="CH119" s="15" t="n">
         <v>10146.48</v>
+      </c>
+      <c r="CI119" s="15" t="n">
+        <v>9627.639999999999</v>
       </c>
     </row>
     <row r="120" ht="14.25" customHeight="1">
@@ -25090,6 +25374,7 @@
       <c r="CF120" s="15" t="n"/>
       <c r="CG120" s="15" t="n"/>
       <c r="CH120" s="15" t="n"/>
+      <c r="CI120" s="15" t="n"/>
     </row>
     <row r="121" ht="14.25" customHeight="1">
       <c r="AW121" s="13" t="n">
@@ -25206,6 +25491,9 @@
       <c r="CH121" s="15" t="n">
         <v>21.11</v>
       </c>
+      <c r="CI121" s="15" t="n">
+        <v>22.65</v>
+      </c>
     </row>
     <row r="122" ht="14.25" customHeight="1">
       <c r="AW122" s="13" t="n">
@@ -25321,6 +25609,9 @@
       </c>
       <c r="CH122" s="15" t="n">
         <v>1157.63</v>
+      </c>
+      <c r="CI122" s="15" t="n">
+        <v>1142.49</v>
       </c>
     </row>
     <row r="123" ht="14.25" customHeight="1">
@@ -25362,6 +25653,7 @@
       <c r="CF123" s="15" t="n"/>
       <c r="CG123" s="15" t="n"/>
       <c r="CH123" s="15" t="n"/>
+      <c r="CI123" s="15" t="n"/>
     </row>
     <row r="124" ht="14.25" customHeight="1">
       <c r="AW124" s="13" t="n">
@@ -25478,6 +25770,9 @@
       <c r="CH124" s="15" t="n">
         <v>36.78</v>
       </c>
+      <c r="CI124" s="15" t="n">
+        <v>31.26</v>
+      </c>
     </row>
     <row r="125" ht="14.25" customHeight="1">
       <c r="AW125" s="13" t="n">
@@ -25593,6 +25888,9 @@
       </c>
       <c r="CH125" s="15" t="n">
         <v>10655.96</v>
+      </c>
+      <c r="CI125" s="15" t="n">
+        <v>10296.94</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1">
@@ -25634,6 +25932,7 @@
       <c r="CF126" s="15" t="n"/>
       <c r="CG126" s="15" t="n"/>
       <c r="CH126" s="15" t="n"/>
+      <c r="CI126" s="15" t="n"/>
     </row>
     <row r="127" ht="14.25" customHeight="1">
       <c r="AW127" s="13" t="n">
@@ -25750,6 +26049,9 @@
       <c r="CH127" s="15" t="n">
         <v>4.64</v>
       </c>
+      <c r="CI127" s="15" t="n">
+        <v>2.54</v>
+      </c>
     </row>
     <row r="128" ht="14.25" customHeight="1">
       <c r="AW128" s="13" t="n">
@@ -25865,6 +26167,9 @@
       </c>
       <c r="CH128" s="15" t="n">
         <v>1818.43</v>
+      </c>
+      <c r="CI128" s="15" t="n">
+        <v>1792.22</v>
       </c>
     </row>
     <row r="129" ht="14.25" customHeight="1">
@@ -25906,6 +26211,7 @@
       <c r="CF129" s="15" t="n"/>
       <c r="CG129" s="15" t="n"/>
       <c r="CH129" s="15" t="n"/>
+      <c r="CI129" s="15" t="n"/>
     </row>
     <row r="130" ht="14.25" customHeight="1">
       <c r="AW130" s="13" t="n">
@@ -26022,6 +26328,9 @@
       <c r="CH130" s="15" t="n">
         <v>3.34</v>
       </c>
+      <c r="CI130" s="15" t="n">
+        <v>2.09</v>
+      </c>
     </row>
     <row r="131" ht="14.25" customHeight="1">
       <c r="AW131" s="13" t="n">
@@ -26137,6 +26446,9 @@
       </c>
       <c r="CH131" s="15" t="n">
         <v>707.62</v>
+      </c>
+      <c r="CI131" s="15" t="n">
+        <v>674.87</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1">
@@ -26178,6 +26490,7 @@
       <c r="CF132" s="15" t="n"/>
       <c r="CG132" s="15" t="n"/>
       <c r="CH132" s="15" t="n"/>
+      <c r="CI132" s="15" t="n"/>
     </row>
     <row r="133" ht="14.25" customHeight="1">
       <c r="AW133" s="13" t="n">
@@ -26294,6 +26607,9 @@
       <c r="CH133" s="15" t="n">
         <v>34.84</v>
       </c>
+      <c r="CI133" s="15" t="n">
+        <v>31.58</v>
+      </c>
     </row>
     <row r="134" ht="14.25" customHeight="1">
       <c r="AW134" s="13" t="n">
@@ -26409,6 +26725,9 @@
       </c>
       <c r="CH134" s="15" t="n">
         <v>2379.81</v>
+      </c>
+      <c r="CI134" s="15" t="n">
+        <v>2348.56</v>
       </c>
     </row>
     <row r="135" ht="14.25" customHeight="1">
@@ -26450,6 +26769,7 @@
       <c r="CF135" s="15" t="n"/>
       <c r="CG135" s="15" t="n"/>
       <c r="CH135" s="15" t="n"/>
+      <c r="CI135" s="15" t="n"/>
     </row>
     <row r="136" ht="14.25" customHeight="1">
       <c r="AW136" s="13" t="n">
@@ -26566,6 +26886,9 @@
       <c r="CH136" s="15" t="n">
         <v>20.14</v>
       </c>
+      <c r="CI136" s="15" t="n">
+        <v>20.08</v>
+      </c>
     </row>
     <row r="137" ht="14.25" customHeight="1">
       <c r="AW137" s="13" t="n">
@@ -26681,6 +27004,9 @@
       </c>
       <c r="CH137" s="15" t="n">
         <v>3287.91</v>
+      </c>
+      <c r="CI137" s="15" t="n">
+        <v>3227.98</v>
       </c>
     </row>
     <row r="138">
@@ -26714,6 +27040,7 @@
       <c r="CF138" s="15" t="n"/>
       <c r="CG138" s="15" t="n"/>
       <c r="CH138" s="15" t="n"/>
+      <c r="CI138" s="15" t="n"/>
     </row>
     <row r="139">
       <c r="BE139" s="15" t="n">
@@ -26806,6 +27133,9 @@
       <c r="CH139" s="15" t="n">
         <v>3.2</v>
       </c>
+      <c r="CI139" s="15" t="n">
+        <v>3.29</v>
+      </c>
     </row>
     <row r="140">
       <c r="BE140" s="15" t="n">
@@ -26895,6 +27225,9 @@
       </c>
       <c r="CH140" s="15" t="n">
         <v>2359.67</v>
+      </c>
+      <c r="CI140" s="15" t="n">
+        <v>2249.64</v>
       </c>
     </row>
     <row r="141">
@@ -26928,6 +27261,7 @@
       <c r="CF141" s="15" t="n"/>
       <c r="CG141" s="15" t="n"/>
       <c r="CH141" s="15" t="n"/>
+      <c r="CI141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="BE142" s="15" t="n">
@@ -27020,6 +27354,9 @@
       <c r="CH142" s="15" t="n">
         <v>18.81</v>
       </c>
+      <c r="CI142" s="15" t="n">
+        <v>13.62</v>
+      </c>
     </row>
     <row r="143">
       <c r="BE143" s="15" t="n">
@@ -27111,6 +27448,9 @@
       </c>
       <c r="CH143" s="15" t="n">
         <v>5451.55</v>
+      </c>
+      <c r="CI143" s="15" t="n">
+        <v>5263.22</v>
       </c>
     </row>
     <row r="144">
@@ -27139,6 +27479,7 @@
       <c r="CF144" s="15" t="n"/>
       <c r="CG144" s="15" t="n"/>
       <c r="CH144" s="15" t="n"/>
+      <c r="CI144" s="15" t="n"/>
     </row>
     <row r="145">
       <c r="BJ145" s="15" t="n">
@@ -27216,6 +27557,9 @@
       <c r="CH145" s="15" t="n">
         <v>0.65</v>
       </c>
+      <c r="CI145" s="15" t="n">
+        <v>0.96</v>
+      </c>
     </row>
     <row r="146">
       <c r="BJ146" s="15" t="n">
@@ -27292,6 +27636,9 @@
       </c>
       <c r="CH146" s="15" t="n">
         <v>2112.85</v>
+      </c>
+      <c r="CI146" s="15" t="n">
+        <v>2107.29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>